<commit_message>
Updated OpenAI niche generation with 100 high-ticket diverse niches
</commit_message>
<xml_diff>
--- a/output/master.xlsx
+++ b/output/master.xlsx
@@ -448,42 +448,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hey, I'm Lawrence - Welcome to Stay Ready To 3D Print 👋
-I've tested tons of printers and logged thousands of hours troubleshooting, tuning, and
-figuring out what actually works in 3D printing.
-Now I run my own 3D printing business while helping you avoid the expensive lessons I learned the hard way.
-Here’s what you’ll actually learn here:
-✅ Tutorials - from first print to advanced tuning
-✅ Printer mods that actually make a difference
-✅ Honest gear reviews 
-✅ Step-by-step project builds you can follow
-✅ Side hustle lessons from running my own 3D printing business
-✅ Regular live streams solving print problems together and live giveaways! 
-Subscribe and join the community. 
-Email Chris (Production Manager) at stayreadyto3dprint@gmail.com for all business, brands, reviews, and collaboration inquiries. 
- Visit our website to check out our products at 
-www.stayreadyto3dprint.com
+          <t xml:space="preserve">The Realest Tax &amp; Business Strategist You Will Ever Meet™️
+I’m Patrice L Stewart—Experienced Entrepreneur &amp; Financial Literacy Advocate 💼
+📊 22 Years in Tax, Accounting, Banking, &amp; Finance industries.
+💡 Knowing Your Numbers is the Key to Business Success! 💡
+I teach Business Owners how to leverage tax laws and loopholes 🏛️ so you can keep more of your hard-earned money 💵 and use strategies the wealthy swear by 💎.
+My Passion: Education &amp; Coaching 🎓
+Join my Online Financial Academy—a monthly Group Coaching Program 📈
+👉 Learn More: plstewart.info/WSWTY
+🚀 Work with me or join an Event/Workshop!
+👉 Book Now: Plstewart.info/help
 </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>47700</t>
+          <t>27100</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>1294</t>
         </is>
       </c>
     </row>
@@ -571,56 +566,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MQ2Cb2a8hJQ</t>
+          <t>_jxLIKW9dQk</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Slicer Ninja is launching soon on kickstarter! Don’t miss out! #3dprinter #3dprinted  #trending</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sign up for free here:  http://kickstarter.com/projects/slicerninja/slicer-ninja-ai-3d-print-file-optimizer
-What Is Slicer Ninja?
-Slicer Ninja is a web-based tool designed to take the guesswork out of slicer settings.
-Instead of digging through menus, forums, and trial-and-error prints, Slicer Ninja analyzes your model, your printer, and your filament, then recommends optimized slicer settings automatically. The goal is simple: better prints, less waste, and less time spent fighting your slicer.
-You upload a model, select your printer and material, and Slicer Ninja helps optimize things like orientation, layer height, walls, infill, flow, and speed—based on real-world printing logic, not generic presets. It’s built to work with your existing slicer, not replace it.
-Whether you’re new to 3D printing or you’ve been doing this for years, Slicer Ninja is meant to save time, reduce failed prints, and help you get consistent results without overthinking every setting.</t>
-        </is>
-      </c>
+          <t>We told Blacks to wait your turn! After 1.2 Billion gone #chicago #cityofchicago #politics</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-02T17:06:08Z</t>
+          <t>2026-01-30T07:07:28Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1113</t>
+          <t>1457</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.02965</v>
+        <v>0.055594</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -629,76 +615,59 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>running into problems like this, they get old really fast when you're 3D printing, especially when you're new. Because let's face it, in slicers, there are a ton of settings and some of which I still to this day don't know exactly what they do. So, I created a software, it's called Slicer Ninja, and it's launching on Kickstarter here pretty soon. And it basically allows anyone to 3D print without even knowing a single thing about the slicer. You can simply upload your STL file, give it to Slicer Ninja, it'll optimize it, give it back to you with all the settings set, all your supports, everything is done for you. Even if you're not a beginner like myself, it'll save you a ton of time. But the only way it's ever going to make it is with the community support, and that's you. Now, Slicer Ninja is fully functioning. It just needs some finishing touches from actual developers. My plan is to bring in a dev team to finish out Slicer Ninja and make it the best software possible. With your help, I think we can do it. No problem. If you want to get a really good deal on Slicer Ninja and stay in touch with what's going on with it, check out the link in the description. I'll pin it in the comments so you won't miss a</t>
+          <t>I don't blame the migrants for coming here. We left a trail for them to come. I don't hate on my immigrants. My parents are immigrants to this country. I'm a first generation American. I don't hate on any of these people who came here. They had no choice. But we left a trail for them to come. We gave them over a billion dollars to come here. We invited them with free food, free clothing, free rent, free education. &gt;&gt; That's why we're here today. Yeah, &gt;&gt; we can keep talking about whatever head tax and gambling is bad and all this other stuff. We made the gamble. &gt;&gt; We gambled on the migrants and we lost. We put over a billion dollars into into people who've never paid a nickel into the system. &gt;&gt; Meanwhile, Meanwhile, we told the black community, "Wait your turn. [screaming] &gt;&gt; Wait your turn. Yes. &gt;&gt; Sergeant at arms. Sergeant at arms.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>http://kickstarter.com/projects/slicerninja/slicer-ninja-ai-3d-print-file-optimizer || what is the cost to back this project?  I am a teacher, and a slice like this could be a great alternative for my younger students.  we us Mac M1, M2 and M4 computers, will this software be Mac Compatible?  thanks || It’s going to be several methods of backing as low as $10 on up to a few hundred. It’s a web based software so it’ll work as long as you have internet and a browser. || If it’s fully functioning, what does the dev team need to do? || Make it better. We want to add features such as filament management, batch optimization, and more. I’m not a developer so I need help to finish it and make sure it’s going to work as expected when thousands of people are using it. It’s not as simple as it may seem.</t>
+          <t>Yes a billion dollars...and they STOLE 19 BILLION. || Frfr makes no sense but to cause division still today they are making new free programs for migrants but still no reparation… but black ppl protesting in the streets… I don’t know what to say 😑😑😑 || The left destroys everything they live in a bs reality ! || For President ! || Nobody remembers when everybody was erupting in city hall about them putting migrant hotels in black neighborhoods during Biden. If they could fix it with the migrants, they could of fixed it with the blacks for the last 20 years. || Enjoy the race to the bottom. Instead of solidarity with immigrants, you want to sew division. They're coming for you too you degenerate || And there they go trying to turn us on each other coming from a klan man sounds amazing..never paid a nickel he dosnt know his facts at all do the math and add up how much immigrant paid into the system actual FACTS BILLIONS,  BLACKS HAVE BEEN HERE WAY BEFORE IMMIGRANTS OR DO YOU FORGET "SLAVERY" OR IS THAT NOT IMPORTANT BECAUSE U GUYS ARE TRYING TO ERASE THERE HISTORY.  WHAT A LOOSER || Vote them suckers out! || 0:19 they had no choice to come here? || Ain't that a blip...smh... || I sincerely hope we get pritzker out in 2026 &amp; johnson out in 2027 &amp; most of these liberal Chicago aldermen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>YiMevD99WKE</t>
+          <t>hi9MmOTlWGo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The Truth: Bambu Lab Finally Clears The Air</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>🎉 PROMO ALERT
-Use PROMO CODE: STAY20 and get 20% OFF our all-new MorphX TPU filament.
-⏰ Offer ends 2-10-26 — limited supply available, so don’t wait.
-In this video, I directly question Bambu Lab about recent changes to their Terms &amp; Conditions and Terms of Use, and what those updates really mean for everyday users. Link to Bambu lab ToS Document's.....https://bambulab.com/en-us/policies/terms
-Specifically, we break down:
-How the new software and firmware terms affect Bambu Lab 3D printers
-Whether enabling Developer Mode can impact warranty coverage
-If refusing firmware updates could void your warranty
-Concerns around data collection and user privacy
-Claims of hidden changes and whether anything was intentionally buried
-Allegations of unethical business practices — fact vs rumor
-The goal of this video is to clear the air, separate truth from speculation, and provide on-the-record answers so the community can make informed decisions instead of reacting to misinformation.
-If you’ve been confused by the recent controversy, worried about losing warranty protection, or unsure how these updates affect the way you use your printer — this video is for you.
-If this video helped you, consider liking, subscribing, and sharing it with other makers who may still be confused by the situation. My goal is transparency — not hype.</t>
-        </is>
-      </c>
+          <t>Are you really in business? #business #taxdeductions #taxes #credit #cashflow #income #entrepreneur</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-01-28T10:30:19Z</t>
+          <t>2026-01-12T19:11:29Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>19689</t>
+          <t>995</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>46</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>317</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.046981</v>
+        <v>0.053266</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -707,83 +676,59 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>So, let's stop right there. We all know who they're talking about. What? So, you knew about this over a year? You were selling paper weights? Premium paper weights is what you were doing. Not cool. As a business owner, I would never do that. So, in this video, we'll cover some of the questions that I asked Bamboo and the answers that I got. Like, why'd you change your terms of service? Did you try to hide it? And if I don't update to the latest firmware, will I lose warranty or will I lose warranty if I stay on developer mode or LAN mode? There was a ton of questions that were floating around the internet. A lot of them just left everybody confused, not knowing what to believe, including me. And come to find out, some of the stuff that I believe it was actually not even true. So, I'm going to cover several different topics around this whole controversy of firmware, the ecosystem, locking out third-party softwares, and oh, speaking of thirdparty software, there's another company in this whole thing that deserves your attention way more than Bamboo Lab does. I can't wait to tell you about that. So, real quick, let me tell you about today's sponsor, and it's me. Stay Ready to 3D Print has come out with Morphex TPU. We launched it a couple of weeks ago, and the sales have been absolutely nuts. Everybody loves this stuff. It's a super easy to print TPU. So, it makes printing shoes like these a breeze. And they're super comfortable, too. I was so tired of dealing with TPUs and being forced to print with a super stiff 95A TPU just to get the 3D printer to print the TPU. And what's the point in printing a shoe in 95A? It'll be so stiff that you won't even be able to wear it comfortably. But with Morphex, all those problems are over. It's the best of both worlds. It starts out as a 90A, so it's easy to print, and then after it's heated and extruded, it morphs into a 70A, so it's super soft. I mean, you can take this whole shoe right here that's done in 15% infill and you can bend it everywhere. It's soft. I wore these exact shoes to BitSummit 2025 and let me tell you, they were great. So, if you want to get Morphex TPU, go to stay readyto3dprint.com and check it out. And I'll leave a promo code in the description to give you 20% off. So, go check them out because that code will only be good for a limited time. So, real quick, let's go back a little bit so I can explain how we got here today. So, some of you might remember I went to Rapid TCT up in Detroit a few months ago. I built Creality's 11th anniversary motorcycle. I took it up to Detroit and I actually went around all of Rapid TCT and I interviewed several different brands, Bamboo being one of them. And while I was at their booth, I was asking about their new H2D machine. And one of the Bamboo reps, he was just going on and on and explaining all about the H2D machine. And then towards the end of the interview, he brought up software. And so I thought it was a great opportunity to actually ask some follow-up questions and that is when this happened. &gt;&gt; So speaking of developer mode, I think some people were worried about with Huh. &gt;&gt; Do you chat with &gt;&gt; I'm sorry. &gt;&gt; Are you asking about authorization stuff? &gt;&gt; The the land mode &gt;&gt; land developer mode. &gt;&gt; The developer mode. Yeah. Huntington has also. &gt;&gt; Now, keep in mind, this happened right in the middle of that whole controversy thing, right after they had announced the terms of service changes and all that good stuff. So, this didn't look good at all. And to me, it looked like, what are you hiding, right? Why would you abruptly stop an interview like that and do it so rudely? That was the main problem that I had with the whole thing. It wasn't that you didn't want us to talk about software, cuz I get it. you want to do that in a controlled way, especially with all the controversy bouncing around. So, I understood that. But for me, it was just the way that they went about doing it. It rubbed me the wrong way, especially when I was there to talk about their H2D machine and I was promoting it on my channel for free. &gt;&gt; Oh, okay. Okay. We'll cut that out. Don't worry about it. &gt;&gt; Yeah. &gt;&gt; So, I know in the video I said, "Okay, don't worry. I won't post it." But honestly, when I got back home, I thought long and hard and I had decided, you know what? No, I need to post this and let people make their own decision. I didn't try to influence anybody's decision in that video. I simply posted it and just gave the facts. Now, if you look at some of the comments, people got pretty heated about that whole thing, and that video got over 10,000 views in the first few hours. But if you look at it as a whole, like I do, when I look at my analytics, it was over 75% likes and only like 25% dislikes. So, the video resonated with most people. So, about a week after the video had been out on YouTube, I got an email and it was Bamboo actually replying to an email that I sent them asking to review a machine. And needless to say, they were a bit confused. They were wondering, "Hey, we see you want to review one of our machines, but we're a little confused cuz now we see this video." I'm glad that they did because if they wouldn't have reached out, this video never would have happened and I would never have been able to bring you guys the actual truth. And I think that's what everybody needs. And honestly, it's kind of sad because a lot of those people made decisions just like I did based on rumors that mostly weren't true. And a lot of those rumors, they were just simply misconstrued and baseless. So, after a few emails back and forth with the Bamboo Lab rep, we came to an agreement. He sent out an X1C and he gave me a $400 Bamboo Lab gift card where I could go on their store and buy pretty much everything I needed to basically test out their printer over the next couple of months. And that's exactly what I did. So, needless to say, me and Bamboo Lab started off on a really good foot considering the video I had just posted. I was a little confused at this point and I was definitely on my guard because I was like, "Wait a minute. I just posted this video basically bashing you and you reply to an email and at first you're confused and at the end of a couple of emails now you're sending me a $1,000 printer and giving me a $400 gift card. So I was wondering, okay, wait a minute. Are they trying to buy my opinion or like what's going on here? And I've had the printer several months now and I've been using it pretty much almost every day. I just got busy and I couldn't just jump on the video right away. But honestly, it's been a good thing because it's allowed me to use the printer over a long period of time and really get to know the Bamboo ecosystem and test out all the stuff that everyone's saying to see for myself, is it true? And then the things that I wasn't sure about, I reached out to Bamboo Lab directly with a whole laundry list of questions and they answered them. All right, so I'm not even going to pretend like I memorized this whole email because I didn't. So, I got my phone here. I'm going to go over with you the questions that I presented to Bamboo and then as you'll see on the screen here, my questions will be in white and their answers will be in red. So, the first question I asked was what support and warranty coverage do you get if you're using the cloud on the latest firmware, if you're in LAN mode with no internet, if you're in developer mode, or even if you're on an older firmware. And here's what they said. Support and warranty are provided for all publicly released models and firmware. Naturally, if a user requests support for a bug or feature that has already been fixed, the only recommendation support can provide is to update to the version where that fix was implemented. So, that was their answer on that. Pretty much you've got support and you've got warranty. So, the second question was about terms of service and updates. So, my question was, if a user declines an update, can functionality, support, or warranty be reduced or blocked under the current terms of service? and they basically said please read above basically refer me to the answer for the first question. So in other words no you won't be blocked and it won't be reduced you will have warranty and they will provide support. So number three is authorization control and thirdparty tools and this is where it gets interesting. This next question is Bigtree Tech/Panda Touch support. And my question was, Bigtree Tech has publicly stated that some of their devices, including Panda Touch, will lose functionality after recent Bamboo updates. What is Bamboo's position on this? And is there a plan to maintain compatibility or provide an alternative? Here's the answer they gave. Once again, this is old news. They had over a year's notice. In fact, their release of Touch was one of the triggers for us to be transparent about closing these exploits. We don't want people purchasing something without knowing it won't work in the future. Outside of developer mode, we will not allow this functionality as it involves an unauthorized device. And again, the reason why Bamboo is doing this is to protect you. And Big Tree Tech is only concerned about selling you a third party device. That's the only reason they care if Bamboo patches some of these security exploits. And Bamboo has pretty much said that if it means compromising security that they're going to patch it and they're not really worried about what Big Tree Tech thinks about it. They let them know about this a long time ago and they chose to continually sell these third-party devices. Blows my mind. My question was, will Bamboo provide an official pathway API program for thirdparty controllers like Home Assistant or Panda Touch to retain full functionality? And if so, what is the plan or timeline? And here's what they said. API access will only be allowed through authorized license partners. Now, for the community, the available option is developer mode. As mentioned in my previous emails, we gave more than a year and a half of advanced warning about this change. In Panda Touch's case, we cannot take responsibility if a manufacturer chose to rely on a known exploit and still decided to sell hardware that was bound to stop functioning at some point. So, let's stop right there. I want you to think about this. Who are they talking about? We all know who they're talking about. They're talking about Big Tree Tech who makes all the panda stuff. And here's where a lot of this controversy came into play. Because guess who played dumb? Whenever this whole controversy came about, Big Tree Tech, they acted surprised. Oh, I can't believe this. Oh, this doesn't work now. What? So, you knew about this over a year? You knew Bamboo was going to push out an update that basically rendered your product useless and you continued to sell those products to the public? I don't understand that. Now, I could get if you announced like, "Hey, these products might be coming useless. Here's what we're going to do with products that we already have manufactured in stock. We're going to go ahead and reduce the price down to basically build price and push them out at super low prices just to get rid of them and stop manufacturing them." But that's not what they did. They continued to build these products for Bamboo Lab machines knowing that at some point a firmware update was coming out that would render their products useless. So, like I said earlier, I think there's a company here that deserves our attention way more than Bamboo Lab does at this point. Yeah, it just blew my mind when I heard that. Now, you might be thinking like, "Oh man, Bamboo Lab is throwing Big Tree under the bus." But really, they're not. Bamboo Lab is covering theirelves at this point. and really big tree tech threw them under the bus. By continually selling these products, you set users expectations that they'll be able to use these products. So, of course, these users got mad when Bamboo Lab did this that everybody looked at Bamboo Lab like, "Hey, what's going on here?" Right? when in all actuality, Big Tree Tech should have put out something along with Bamboo Lab when they found that out, letting people know, hey, you might not want to buy these devices because they probably won't work here in the next 6 months to a year. So, Big Tree Tech, if you're watching, I think you owe everybody an apology for one, acting surprised when you already knew what the game was, and for two, for continuing to sell a product that you knew was going to be useless. you were selling paper weights. Premium paper weights is what you were doing. So yeah, to me not cool as a business owner I would never do that. So for my question number four is about LAN only mode. Now my question was will LAN via Bamboo connect always work without internet or an account? Which features differ from cloud mode and is any telemetry collected in LAN mode? And the answer was yes. On current hardware, there will be no changes to how things work. As always, I can't speak to future hardware or software. Those remain unknowns, which is, and that's fair. Developer mode. Now, here's one that I heard all the time from various different people. And honestly, somewhere along the line, I adopted it and I actually believed it, too. So trust me, if you got caught up in this whole controversy, you're not alone because there's a lot of stuff that I believed and now looking back, I didn't even do my homework and I just adopted certain things. And I don't typically do that. I'm a very, very curious and investigated person, but I heard it from a reliable source, so I didn't even think about it. So, on to developer mode. I asked, "Does enabling developer mode affect support or warranty by itself or only if issues are directly caused by changes made while using that mode?" And the answer was, as stated above, running this mode does not void warranty or support. They're basically saying that you can use developer mode and you're not going to lose support or warranty, as a lot of people believe before, including myself. So, question number six I asked was about firmware roll back. And the question I asked was, will Bamboo provide a supported roll back option to older firmware that keeps first-party apps functional for users who need compatibility? So basically, will they offer a firmware roll back that allows you to continue using those big tree tech products? And the answer was yes, unless stated otherwise in release notes. So that's kind of left open. It it's like yeah, unless we decide not to. So, that one, I mean, I wouldn't bank on it. I really wouldn't bank on it. Cuz let me tell you this, a lot of the reason why Bamboo Lab did the whole terms of service thing boils down to their new machine. And here's why. They released the H2D. And in the H2D, there's a laser inside that machine. And what the bamboo rep had explained to me during an email was that we're basically putting a laser inside people's living rooms, inside their bedrooms, inside their garages, and we have to do everything that we can to protect those people and not allow some person with ill intentions to hack into their system using an exploit that, let's say, Big Tree Tech used in order for that Panda Touch to work. Someone else can use that same exploit to get into your machine and do nefarious things such as turning on your laser in the middle of the night or while you're away on vacation or get access to your camera and be able to, you know, look around or whatever. But the biggest thing was was safety. You don't want someone to be able to get into your machine and turn on that laser in the middle of the night and burn down your whole dang house. And honestly, big props to Bamboo Labs for not caving in to those companies, those third party companies that, you know, out of selfish reasons, they wanted those accesses to be left open. They wanted those exploits to not be patched. That way, they could continue selling you their little third-party products. And Bamboo Lab decided to choose their customer and their customer safety over all of those companies. And that's kind of how this whole thing started. So, I just want to give props to Bamboo Lab for that. And I see why they did it now and honestly it was the right move 100%. So we're going to move on to question number seven and that is future gating of core functions. So my question here was can you confirm that core printer operation start stop jogging temps job uploads etc will not be gated behind proprietary authorization except where necessary for documented security reasons. And that kind of plays to what I just said. Can you confirm that you're going to allow us basically allow us freedom unless security reasons require you to shut it down basically is what I was asking and he said nothing will change with current hardware but to be clear the only mode that currently allows this is developer mode and that's something we already knew and that's great. So in developer mode you have a lot more freedom. All right now moving on to number nine public documentation. So my question on this was, "Can you point me to the official pages covering terms of service, authorization, control, land mode, developer mode, and warranty so I can cite them directly in my video?" Their answer was, "Once again, since all of these modes are supported, I can only refer you to our terms of service." And then he gave me the link. And so I'll include that link in the description for you guys to go check out for yourself. Okay. Now, next, it's kind of a paragraph, so bear with me. I asked the Bamboo rep. I said, "Hey, I'm not sure if you've seen Lewis Rossman's video about this a few months back." I'm asking some of the questions he brought up as well, but one thing I'd like to know is, did Bamboo delete the web archives of the terms of service changes made? If so, why? Why not just tell everyone they made changes versus trying to hide it? Was it just to avoid confusion? I'm curious because if that truly happened, then it just seems odd without a logical explanation. and his answer was, "Please refer back to my original email." And then he reiterated, "The only change was a minor clarification regarding forced updates. We would only ever apply or force an update if a public safety issue arose from a firmware version. That's the simple fact. Despite how some may want to portray it otherwise, we openly reported this change, but after being accused of gaslighting, we chose not to make further comment. In my opinion, that was probably not the greatest choice, but hey, that's a choice that Bamboo Lab made, and honestly, I think they'll be okay. So, my response was, "Well, I'm sure you have some very logical explanations for a lot of this, and I look forward to hearing them." And he went on to say that we had hoped that clear-minded users would understand why these changes became necessary once we began integrating features like a laser into the printer. Unauthorized 3D print commands are one thing, but triggering a laser unattended could put lives at risk. So, like I had explained earlier, Bamboo instituted a lot of these changes due to the fact that they're putting a laser in people's living room. So, just let that sink in and maybe some of this will make sense now because before to me, yeah, I was with you guys. A lot of it didn't make sense. And I'm an avid Creity user up until recently. Of course, I will be selling off all my Create machines and changing brands. I don't know if that's going to be Bamboo or Prussa, but it will be one of the two. And that has nothing to do with this video. It just happens to be that I'm no longer promoting Create as a brand. So, he goes on to say, "As a company, we have a responsibility to protect not only the best interest of our customer, but also the best interest of the company itself." With that said, most if not all of the accusations made back in January have proven untrue. We were not hiding anything. We were simply closing a known protocol exploit. Even then, we provided our user base with options and continue to support developer mode. At this point, it's baseless for anyone to continue pushing this narrative. So, yeah, there you have it. A lot of the hard questions were asked and every single time they came back with a solid answer. Now, I didn't take these as just straight up fact. When I got the machine, I've tested the machine over a period of several months. Now, let me give you my thoughts on the machine, right? I've always thought that Bamboo Lab had a great product from day one. I just never used a machine for the simple fact that previously I enjoyed modding my machines and to a degree that you just couldn't do it on a bamboo machine. And now a few years down the road, I'm just not at that point anymore where I want to do mods like that. Honestly, now I just want to be able to print with a printer that works 9 out of 10. And yeah, I like to add the occasional light kit, the occasional flowtech hotend, uh different extruder gears, minor stuff like that, but I'm not doing those in-depth mods that I was doing before. I'm just not doing them anymore. And that was one of the biggest things holding me back from using bamboo. And of course, now that they've clarified this, it really has put my mind at ease. And I feel 100% okay going out and just buying bamboo machines if that's the brand that I decide to go with. I'm not sure yet. It might be Prussa or who knows, it might be another brand, but those are the two brands that are, you know, number one and number two. I'm just not sure which one it'll be just yet. But I can tell you with the X1C, my experience with the X1C, it was basically just like any other printer that I've had. I always put all these printers basically in the same category pretty much. Nine out of 10 printers, they just work and they all have little minor issues. Like my X1C, it's been phenomenal until recently whenever the extruder stopped working and it just kept jamming after jam after jam. I didn't know what was wrong with it. I reached out to the rep like, "Hey," he was on vacation, but like he went and made sure the next day I had an extruder in the mail and I got the extruder. it solved the problem. I don't know what happened and maybe it's something I did. I'm not sure. But honestly, I mean, I don't get upset at those things because those are simple 3D printing issues that from time to time, you're going to have them even with the best machine. And I think the sooner people realize that and stop putting certain brands on these pedestals that they really don't belong. I mean, after all, these are robots. They only do what you tell them to do. And very very rarely do they just up and do something on their own that they weren't told to do. So n out of 10 if your machine is messing up or it's printing bad. It's usually something you're doing and that's just the raw truth. It's usually usually something you're doing you're doing. But overall the X1C has been a good machine and honestly the print quality is actually phenomenal. And I really love the way that you can basically just use your Bamboo Handy app and you don't even have to connect to a PC. That's been my biggest thing with the X1C is it's kind of how I use the X1C. Now, I have a bunch of other printers, but the X1C, it's kind of like my running gun machine. I'll be on Bamboo Handy and I find something that I want to print real quick. I'll just pull it up, hit start print, and and there it goes. So, I leave that machine on pretty much 24/7 and I'll just shut off the lights from my phone or whatever the case may be. So, that's one of the biggest things that I like about the Bamboo whole ecosystem thing is the way they require people to upload their files basically in a 3MF format to where someone's already printed that file. It's ready to go. All I have to do is hit print and make sure that I have that filament in my printer. And honestly, you don't even have to make sure you have that filament in your printer. You can select, let's say it's a PLA model and you all you have is PET G in your printer. You can actually select Pet G and it'll actually print it in Pet G for you. All the settings are already pre-done. You don't have to do anything. And as far as print profiles, oh, I haven't done any of that with the Bamboo machine. It's been great. And really, Bamboo has really been innovating here lately. So, obviously, they're coming out with the H2S, which has already hit, and then they're coming out with the H2C. And from what I understand, it's going to be six tool head changer. And that thing is going to be absolutely phenomenal. I mean, wireless induction hotends, it's got some high-tech stuff in there, and it's going to change the way we do color printing. And the future is tool changers. So, if you're thinking about buying a machine, you need to consider, if you want to do multicolor, you need to highly consider getting a tool changer. Whether it's the Bamboo H2D with the upgrade or the Bamboo H2C or even the Snapmaker U1. There's several brands coming out with multi-tool head machines. I even heard that Creity is finally thinking about doing one after I decide to get rid of all my Creity machines. Now, I'll make a video on that later on why I'm leaving Creity and I'm no longer promoting their brand. They didn't treat us very nicely and they allowed some stuff to happen that I'm just not okay with as a human being and I have to do what's best for the channel. And at the same time, they weren't innovating like other brands were. Other brands were coming out with tool changers and all this new stuff. And it seemed to me that Creality was basically just slapping another letter on on a printer and saying, "Oh, here's our new printer." Like the K1 Max and then they released the K2 and then the K2 Plus and then the K2 Pro and the K2. And honestly, the only thing different in the whole K2 lineup is size. They didn't change much of anything. If anything, they just took away features and put out another printer. And so that is part of the reason why I left Creity was lack of innovation. Well, now they're coming out with the multi-tool head supposedly. I guess we'll see. But one thing in this game, I'm always open ears to anything new. If it's a new brand or a new product, I'm not married to anybody. And I go where the innovation is and where we're being treated fairly. One thing I can say about the Bamboo community is that their users are dieh hard. Because when I made that rapid TCT video, man, were they in the comments. They were in the comments bashing me and talking all kinds of smack and saying that I was a Creity fanboy and all this stuff. Well, what do you have to say now? I own a bamboo machine and I'm even considering bringing bamboo products throughout my whole studio. They're in my top two as two brands that I'm considering of bringing into my studio. So, now I know what they'll say. They'll probably say, "Oh, you're just riding on bamboo or whatever the case may be." So, I know what to do with all that. I just don't listen to it. I know at the end of the day, I just want a solid brand in my studio and Bamboo is a solid brand and I really respect what they've done with the terms of service, how they handled it, how they answered all these questions and it just really opened up my eyes about them and so yeah, I really appreciate that. Thank you, Bamboo. And with that, until next time, stay ready to 3D</t>
+          <t>Many of you all think just because you are a business or you're a sole proprietor that you don't have to have paperwork and that's not true. You should still have a profit and loss statement that you are providing to us. Every business, if you are a real legitimate business, you should know your numbers and you should have a profit and loss statement at minimum that you are providing to us as well as a balance sheet as well as bank statements to show your transactions. When you are an LLC or a corporation, we are required to get that [music] information from you. Real tax professionals are like myself, someone who was registered as an IRS efile agent. All right? I have a EIN number. I can electronically file your taxes for the last 3 years. So, there are certain documentation and paperwork that the IRS requires me to get from you being a legal legitimate business. All right. Patrice L. Stewart here, the realist tax and business strategist. Follow my page and channel for more tax, credit, and business tips.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Win A Laser! Anyone who purchases MorphX TPU will be entered into a giveaway for an ACMER 7w Diode Laser! We will announce the giveaway on Discord so be sure to join our server here. 
-https://discord.gg/ZGgcwk7eWt || says this link has expired? || @TheGhinishok let me refresh it. || https://discord.gg/ZGgcwk7eWt || So, they did not lock the printer, but rather their cloud. As long as they stay out of their cloud, anybody can use do whatever they want with the printer. || OMG, dude get to the point…..could have made a 2 minute video… || $11.50 for standard shipping for one roll of TPU? IDK bro, seems pretty steep. || BTT had a disclaimer on the product description well before the controversy began.. They were not trying to pull a fast one on anybody. And to your point of "they should have sold at cost and quit manufacturing". Why?? Their product is still useable. || They def did not.  There are tools that allow you to look at the internet from the past. They def did not. || @stayreadyto3dprint  Do let me know if you post the CFS for sale anywhere. I need a second one. || Not the first time an update or firmware update screwed over people. Cough nvidia, samsung, apple, sony, even LG etc. || True || The security excuse is fiction. The issue was all in their cloud. Nobody was connecting to your printer, except Bambu. They did have that in ident where THEY sent reprint commands that cause people problems. 
-My fix, printer no net access. Delete Bambu handy and slicer. Install Orca slicer and use home assistant for secure remote.  Turn on LAN mode and it is on a version before they crippled the printer. || We knew ALL this except the future laser, at the time - if you bothered to read and listen instead of jumping on a Reddit/YouTube bandwagon. || PUBLIC SAFETY ISSUE MEANS COMPLYING TO THE GOVERNMENTS NEW RULES AND REGULATIONS! ALL FOR YOUR SAFETY TRUST US. || How about contacting Luke from BigTreeTech for their side of the situation, not doing so is showing your bias. Luke is on record refuting the slant you present. There is more to it than you make out. || What record is he on refuting it? And I did reach out. They stopped replying to my emails a long time ago. So I don’t owe them anything at this point. They’ve done other things that inspired them of mentioning publicly. Let’s just say they aren’t very ethically motivated as a brand. That’s all I’ll say on that. || Wtf is that sh1t on your head?
-so stupid ape try to look bada$$ || this whole situation just confirms why i’m stepping away from bambu. the printers might be great on the hardware side, but locking things down after the sale and calling it “security” really doesnt sit right with me. if firmware updates can sudenly take away tools or limit how i use a machine i paid for, thats a hard no... || I understand that completely || Bambulab never more! Not gonna lie, I’m more disappointed than satisfied with Bambu. || where can i find  the stl for those shoes? || Go to my website and the TPU sale will pop up. Tap Get MorphX.  Scroll to the bottom and I included a few files for free. Those are the whaleberry sport shoes. 
-www.stayreadyto3dprint.com || Are you bias on Bambu? What brand should I go with chat? I need support and freedom here. Coming from an ender 3 years ago! || I think Bambu or Prusa would be great options. Prusa has a better customer service. Price is higher but you pay for the customer service and quality of the build. The Nextruder system is why those machines are so rock solid. Depends on your needs really. || The issue for me at least is 3d printing was built on open source.  Bambu has gone closed source with all the Intellectual Property many brilliant engineers and tinkers have given to the community to bring it where it is today. Bambu took all of that and started a business and doesn't give back to the community which build their business.  Then hides behind our security as the reasons to go closed.  Even when it is an obvious rip off of open source projects. || Yeah I don’t agree with how they did that for sure. One of the reasons I don’t own bambu machines. But I think I’m over it now. Cause I really want the H2C lol😅 || this video sounds really one sided + they make claims but you don't verify or explain why it could be like that yes or no. Don't get me wrong here, you might be right, but I feel it lacks a bit of rigor :) || Maybe so. Hindsight is always 20/20. I tried to just provide facts I found and allow viewers to form their own opinions || They just want to be able to not let you print “prohibited items” later on… || Hope not || @stayreadyto3dprint lol that's like pulling your pants down. Putting your head in the sand and your ass up in the air and saying "i hope no one is gonna fuck my ah" || Bullshit. I had the shittiest experience in my first two weeks and they ran me around in circles with "What did you do?" "Can you send me 5 MORE photos of the same 5 photos you sent". I've ran mine offline since I heard about the firmware update and since then I have scanned my printer with an ESP32 Marauder I built and guess what it gives off wifi and bluetooth - I hate that BBL marketing suckered me and now I am the wiser for having made that mistake, one I won't make again. American or Canadian made and wifi as an option. || Duly noted. I’m wanting to come out with a us made printer brand. We will see if I can pull it off. With actual customer service as well. I think it’s high time || 😂😂😂"customer safety". Fucking shill. 😂😂😂 || The answer to question 6 is just No, with extra words. 😅😅 || About the answer to Question 3. 🤦 Using a protocol/API as intended is in no way an EXPLOIT! I don't buy that Bambu warned BTT. According to Bambu, they also allegedly reached out to the makers of Orca, but no one from the Orca slicer dev team had been contacted by Bambu. Not to forget how Bambu kept insisting that MQTT was turned off for safety reasons, and it was an exploit, and unless you know what it was and how it worked, you don't know if that is a lie. Also, remember that the security of YOUR local network is YOUR responsibility, not Bambu Labs. Even if you have a fully open Wi-Fi, it’s still not Bambu’s responsibility what happens on your network. The only responsibility of Bambu Labs is that I can’t access your printer over the internet, and that's it! || BTT was using more than just api access. FYI || About the answer to Question 2, in my book beeing forced to update firmware to get support is the same as no or limited support. For example, Lidar is having trouble scanning the QR code, bambu see i dont run the latest firmware, they will not assist me in any way before that is fixed! || To be clear, they said you would receive support no matter if you’re using dev mode or what firmware you’re running, but sometimes updating firmware is a fix for some things. They made it very clear. They weren’t abandoning users who decide not to upgrade or use dev mode because that was one of my biggest issues with them before and they did clarify that for me. || Brother this is bullshit. They could have made a new TOS for the new machines and left the old ones alone. This is the dumbest take in the world. Oh they put in a laser. So fucking what? Change the TOS for that machine leave the rest alone. The older machines dont need those updates. || Good video but just a shame he couldn't spell Bambu correctly 😂 || The biggest reason I went to bambu, as an engineer, I hated messing with my printer before I could use them, tweak them, etc... I wanted a printer to just work. || Do you have your BL machine air gapped? || I grabbed my A1 Mini about a year ago as a hobbyist due to recommendations on ease of use.  Since then, I grabbed a Comgrow T300 secondhand to print larger items.
-Suffice to say, my tax refund is going to a P2S.  HOPEFULLY, it'll work with OrcaSlicer out of the box, if not, than in Dev Mode. || They bought off another influencer 😢 || Well that was cheap! Lol a printer buys a guy who has a ton of them and give stuff away all the time? I’m still not a full blown bambu user. Just sharing what I discovered. Nothing more || so why didn't bambu labs design the own 5inch screen for the p1s etc || They did now. It’s the p2S. || Bigtree's animated LCD screen adds more mass to the A1's toolhead - that accelerates wear over the warrany period. The Panda Touch is not using an API that Bambu provided for devs, it's using a clever hack, that inevitably would be patched. I don't blame Bambu for locking them out, but I don't see why they need to lock out 3rd-party slicers. I think they could have developed the secured communications protocol to enable the laser cutting functionality while leaving the 3d printing alone. || I think you’re the first one that actually realizes that BTT is not using just an API authorized by Bambu. They’re also using as you stated, clever, hacks, and exploits to gain access. Obviously, if they were only using an API, there would be no patching and their device devices would just work. || So, then why didn’t they just make those changes for the H2D? || Maybe it was easier to make a blanket change versus just the H2d. Idk? || Короче Крупная фирма с своей экосистемой агрессивно ее навязывают, перекрывая доступ к любым сторонним улучшениям говоря нам: "Это для вашей безопасности". Ничто не ново под луной. || Big Tree did the expedient thing... "We're getting ours!" || so....you sold out? || No. I’m still not a bambu user. Wdym? I’m a prusa user just stating facts here to share with the community. || ​@stayreadyto3dprintk || Talking too much, saying little.
-Anyway, when Bambu decided to close its system, I didn't update my printers. I disconnected them from the internet and use them with a memory card. I don't mind. I started with an Ender 3 and I'm fine with it. What I am very clear about is that when they reach the end of their useful life, I will replace them with another brand. No more Bambu for me. || better to have the option than not. let people decide what security options to enable. no conspiracy about it. I'm looking elsewhere || I was almost tempted to pick up a Bambu just to see if it lives up to the hype. I'm so glad I went with my gut and decided it'd be more sensible to stick with Creality. I have to say it's disappointing that your video is awfully disingenuous when you're effectivly saying that if the manufacturer of your car makes it impossible to use after market  parts or modifications, the fault lies totally on the producers of the parts. Personally, if I bought a Toyota Corolla and for some dumb reason I want a chrome skull as a shifter knob, Toyota doesn't get to to veto my poor life choices. I really regret having purchased from your site. || Well Ferrari and big brands do it do it all the time. I never said I liked it. I was simply explaining why they did it and that if they truly did things for security reasons they I can see why and if it was to protect their customer I think it was the right move. Note if they had ill intentions then obviously I don’t agree with it. I’m sorry you regret purchasing from me just because our opinions don’t align. I’m more than happy to offer you a refund if you’d like to send back whatever it is you bought. Unlike other brands I actually care about my customers and I pride myself on excellent customer service. || It is a bunch of lies! (not you Bambu Labs) Bambu Labs had tons of sales for Christmas the year before last then right after the return window closed in the new year pushed out new terms of service quietly and new firmware that then required you to sign in to their cloud server but they got caught and it became a huge deal and they walked it back and made the lan mode thing AFTER they got caught. I was one of the ones burned by this crap. They set it up this way so that they can approve or disallow your prints. It may not currently be being used, but it was the ground work for it. The Biden White House and Alvin Bragg was also part of this because they where pushing 3D printer companies about 3d printed guns at the same time this happened. (Look up Alvin Bragg 3d print letter) They are still not done look at the 3d printer ban laws that are currently being proposed across the country. They are trying to pose it as a safety issue but it is really going to be about control and DRM on 3d printers.  The so called exploits were written into the firmware and were a feature until they needed to be able to control who used your printer and how. As other have said if it really was about security, local authentication using industry standards would have been far superior than trying to develop a whole new cloud system that now involved user name and password being sent across the internet and stored in databases in the cloud waiting to be compromised. || Yes, Biqu/BTT DID know the touch MIGHT be locked down, they released a specific video about it and that they were in talks with Bambu.  They was posted here on youtube and it does have the option to flash your Touch to a Klipper Touch IF it happened.  
-Bambu needs to be clear IF behind the scenes PARTNERED with BIQU after the talks between them happened about the Panda Touch.  BIQU somehow has more than 10x the amount of PANDA gear as it did before "talks" between them happened.  Just food for thought. || But once they found out stuff was going south they didn’t announce that part I don’t think. If they did I didn’t find it. Bambu told me that they gave them plenty of warning. About a year to be exact and they just kept selling products. To be fair they now have a disclaimer on their website. But they didn’t have it before. lol
-Nice to see you stopped by. Haven’t seen your vids lately bud. Idk if the algorithm just stopped showing me or if you’re not posting. Say hi to the misses. Hope you all ate doing well || Just bought 2 rolls of the tpu. Running a bbl p1s. Any idea on what profile would be best to run on it? It's gonna ask what filament type. I'm guessing generic tpu settings? || I wouldn’t use tpu settings. It’ll work but be a lot slower than it has to be. I would import the Prusa Flex profile. It works great. No changes needed. But I also recommend doing material calibrations for your specific machine. Thanks for the support by the way! || ​@stayreadyto3dprintI'm really new to the 3d printing world. Only had my machine about a month now. Don't know how i would import the settings you are talking about. Any help in that area would be greatly appreciated. And did i order a day too early to be entered in the drawing?! || @westsidecracker1nope you’re good to go. Anyone who orders will be entered. 
-As for the profile goes if you don’t know how. Just get prusa slicer and look at the flex profile and take photos. Then go to your slicer of choice and make the changes. Or join discord and I can get on and help you personally. Just tag me in the chat somewhere. https://mee6.xyz/i/4YMcjZjNO6 || ​@stayreadyto3dprintsounds good. Thanks for the help. This will be my first try with tpu. Hoping for the best! Lol || Try this link if the other one’s broken. https://discord.gg/ZGgcwk7eWt || First ever video of you that I've watched coz I was interested in buying a bambulab printer. And you were in my recommendeds. Well. Not anymore. I have NO idea what big tech is or does or did but what I DID notice is that you're tryna sweet talk us like they sweet talked you. They paid you off with a printer &amp; gift card first to sweeten you up, since you (apparently) dissed them after the in person interview at (wherever you were, which was really REALLy rude of that guy btw. I'd hate for someone to represent MY company like that!). .. anyway....... free printer, free filament, email worded to protect their company. I read other comments and have to agree. This is a paid ad for a company who's printer I'm no longer interested in. I guess I can thank you for that. I'll stick with the current brand I'm using. Stay offline and hope for the best 😂 || So the first video someone makes you don’t agree with they are shunned huh? lol can’t please everyone all the time. Impossible. But thanks for insinuating I have no morals and I’m a piece of shit bribe taker. Thats awesome. Nice to meet you too || At the end of the day, it comes down to this. If I don't control it (root) I don't OWN it. It's not mine and can be modified or taken away at any time by the manufacturer. This is an intolerable situation when I still am expected to pay full price. 
-If they want to provide me with the hardware and I only pay for filament, maybe. But probably not. Frankly, if Bambu decides to shut down or similar, you own a paperweight. And outside of replacing the control board, nothing you can do about it. This is why my X1C has X1Plus installed, and is completely blocked from the internet. And I can still monitor it, and my other printers, thanks to Octoanywhere. 
-My other issue with this, is that they modified the device AFTER THE SALE. I bought it knowing I could use various tools. They forced those tools to break. They can call it security, but there are other ways to secure things. Again, unreasonable. If they wanted to do it for new machines only, and were very clear about the change, fine. But that's not what happened.
-I think you are legit trying to be objective. This has a LOT of backstory that you aren't going to get from Bambu. As for BTT, they could be letting potential customers know about the issues a bit more clearly. But it's also not unreasonable for them to be irritated at Bambu.
-As a result, I don't recommend Bambu to people anymore. I used to suggest them to people all the time. It sucks, but I won't put my reputation on the line for backstabbers.
-As a programmer who has custom built printers and modified the software. There are better ways to handle security that would work and still allow users to use their printers. This, like most so-called safety restrictions are not about safety. They are about control. || Well put. Thanks for your insight. Also, we’re looking for people who can build printers because I think it’s high time we have a USA made printer with USA style customer service. So if you’re interested send us an email. || you got the shore hardness backwards bro. 95A is super flexible  and harder to print || lol def not. 95a is pretty stiff and if you print shoes with it you’ll see it sucks for shoes. 70a is much softer. As is 60a and so on and so forth. || So, you can only access the API via developer mode. However if your licenced you can use the API with out your user needing to use turn on developer. So they closed a 'bug/security'. TBF they allow you to roll firmware back, which seems ok. With that said, there is no reason to stop Bambu from 'pair' API's like alot of other software (looking at EvE Online API access) , so you only allow API's the customer has chosen. I think I am still on the fence for both companys. || I honestly don’t feel that BL has any ill intent in doing what they are doing. I truly believe they’re doing it to cover their own butts in case of an accident or something. || Love the explanation. I agree IF they had the heads up that's pretty slimey for them to roll the dice. Really wanna try the morph flex but it's first time I've seen it here...any samples or anything? 50$+ is a bit steep for me for something I haven't tested (no shade meant) || I wish we could afford to send out samples like these big companies. But if you go on my page, there’s a few videos that I posted of shoes that I printed. It prints flawlessly using the Prusa slicer flex profile. With the 20% off it comes out to around 40 bucks. It was 49. I dropped it down to 44 and added 20% off of that. || ​@stayreadyto3dprinthonestly it beats many of the other filaments of this style, think I'm gonna cop a roll! Ty sir || Ty as well || I'm with you, thats why i buy Bambu printers i'm tired of working on and modding then fixing, i just want to fill orders and keep my farm running || I used to enjoy modding my machines, but I’m just kind of over it I guess lol || I've never seen a video of yours. This would be the first. My general impression is that you're not very professional. || That would be correct. I’m just a guy who enjoys 3d printing and I make videos. I’m not a professional videographer. I provide my opinion on things and review machines and do giveaways when I can. Def not a professional at this. Just having fun and giving away as much stuff from brands that I can and always replying to comments unlike most YouTubers. Thanks for watching though. || BTT should certainly be transparent regarding on what firmware their devices function and in what modes.  From what I understand all of BTT's products that have been developed for bambu lab printers still function correctly on the latest firmware in developer mode.  Personally I own a p1s, and I run it in lan mode with developer mode enabled.  I keep my printer on my iot vlan and block external network access to all of my printers (the rest of the printers that I have run klipper (voron v2, voron v0, creality k1 max)) just like I do for the rest of the IOT devices that run on my network (because I don't trust anything these days to not phone home, and it limits remote attack surface). while still allowing me to do anything that a printer is capable of just by using an authorized computer on my network.  if someone wanted to access my printers and iot devices they would either have to gain access via the administrative vpn that I run (which would require my username, password, AND a key file (so reasonably unlikely) or they would have to be inside my house using one of the computers that i've authorized to talk to said devices OR i suppose they could manage to get on my user lan and then either hack my network switch or my firewall to allow access (pretty unlikely... i'm not that sweet of a target).  so even if I were to buy a network enabled laser machine (I honesly just might at some point), I trust that if I configured it that same as my printers network-wise that I'm pretty safe regarding the network security aspects.  but it should NOT be up to my device manufacturers to tell me that I can't use a device that I purchased and own with other equipment or software in any manner that I like.  THAT'S the part that I find obscene.  equipment that I own should be made to work in any manner that I see fit that is technically doable.  my klipper machines do exactly what they're told when they're told, my marlin machines (when I ran them) used to do the same (with a little help from some raspberry pis for wifi and frontend administration in that case), my bambu labs printer needs to do what I want when I want, and when it doesn't, I'll resell it and buy something new and tell everybody exactly why I did so.  it's NOT an exploit to use undocumented APIs to gather data end control a product if that's the owner's intent.  that's not a bug, that's a feature, and removing features (even untentional ones) because bambu simply doesn't want users to be able to inexpensively expand capabilities and undercut bambu's more expensive models doesn't mean that they should be able to get away with locking down their ecosystem.  at this point I don't care how well they work, I am *MUCH* happier with my creality k1 max than my p1s because of the direction bambu is going with their firmware. - with the k1 max, I can go right on the front panel and if I want (and only if I want) enable the root account of the computer that drives the thing and do literally anything that I want with the printer's underlying operating system... creality CLEARLY will not warrant any changes I choose to make, but they'll still honor the warranty of the hardware (assuming I didn't cause physical damage through modifying the software or hardware) and they'll still support me (so long as I didn't create the problem at hand via my modifications).  it enabled me to use shaketune (which is advanced belt tensioning and resonance compensation), KAMP so I can choose to do finer meshing in just the print area and have more control over purging as well, I can add various hardware and other software components, directly live stream from the printer if I want to, added a bunch of macros for various bits of calibration, etc.  does anyone have to do these things to enjoy their k1 max? no.  does is significantly add value to that machine for me and other hobbiests? absolutely!
-right now I'm mostly happy with my p1s in lan only + developer mode. it does mostly what I tell it to do. if they choose to remove or cripple that functionality, that'll be the day that I no longer own a bambu machine.  Prusa is a bit more open, but still pretty expensive for what you get... the core one is a nice printer but I can't stand factory unenclosed printers, and the enclosure design for the prusa xl is pretty terrible overall.  these closed printers are trouble though (bambu, elegoo centauri carbon, etc.)... I really wish more brands would just use klipper and call it a day. || Someone sounds like the got pissed off and then just complains and waffles back and forth. The point is lost somewhere. || Will maybe you can find it lol let me know if you do 😅 || This video blows MY mind... you obviously have zero knowledge about cybersecurity and what constitutes and exploit. At the very least try to understand what you're talking about and verify facts before making broad statements and reading Bambu's response word for word. You're getting played.  I hope to see a video in the future on your channel where you take an objective approach to this topic. Its a very serious issue especially with US States starting to introduce Bills that would force all of your prints to be scanned by AI and tracked forever. Off grid printing is about to become very important and this video helps push a dangerous narrative cloaked, per usual, as being for your safety when its really about control and influence. || I’m sure there will be more videos on this topic. This video was simply to ask Bambu questions and provide the community with their answers verbatim in order for people to form their own opinions. I’m not really taking sides. I also recently posted a video about what Washington lawmakers are doing, and trying to force printer companies to alter their software to scan for gun models. I don’t know if you saw that it’s in my short videos. || For the record, I do not agree with them trying to dictate what we can and can’t print, but thankfully printing off-line is an option and they can never ever control that || I'm like you.  I've been printing for years, and I've worked through my tinkering phase and I'm sick of it.  Now, I just want a printer that works.  Since I got my H2D in December, I've done lots of printing, and only one was less than perfect.  That one turned out to be a problem with the model and the designer's profile, not the printer.
-I bought the printer in full knowledge that it is a closed-source printer.  I would prefer open-source, but not one other commodity item in my house is open source.  My central heating, my microwave, my coffee maker, washing machine, TV, none of my music hardware like keyboards, effects pedals, electronic drums, none of my workshop tools, or my car, nothing.  Why do we demand our printers and only our printers are open source?  It's because until Bambu Labs came along, they weren't good enough.  We needed to mod them endlessly to get them to perform well.  Bambu Labs made the first printers that were good enough out of the box to get great prints.
-My only reservation is that, if a time comes when Bambu decide it's not economical to continue to support the product, that they should then open source the product.  I've spent a lot on this printer, I don't want to be left with a brick, or have to downgrade it in order to continue using it.  If by such a time they still have IP worth protecting, then they can open source most of the product, but continue to support the library containing their secret sauce.  Open source code can call the API for the library without knowing what magic it's doing.  If Bambu don't do this, and I am left with a useless printer, I will never buy from Bambu again, and I dare say most others would say the same, so it's in their own commercial interest to look after their customers. || Well said. I agree. I don’t think it will come to that though. || Exactly! || WTF is land mode? Its LAN mode... . || It’s a typo from the editors. Geez. 😅 || screw warranties, I'll take open source and physical ownership over warranty any day of the week. || Honestly, wtf security issue is a hardware device plugged into it? If you have physical access to a printer, what are they afraid of - stealing files from the onboard memory? They literally have a secure model of printer for this stuff. It should not apply to general consumer printers. This is seriously one of the reasons I am not buying Bambu for my first printer. I do not want to buy into a closed ecosystem. || wonder why it needs to connect to the internet at all.  Do you really believe that they wont shut down printing certain "models"  I prefer being able to print what i want without being monitored. || I do believe they are trying to shut down being able to print certain models. I recently posted a short video talking about this showing a US law maker talking about how doing that is basic common sense if you look at my recent videos, you’ll see it. For the record, I do not agree with that at all. || Bull. All they had to do was add a level of security to the “exploit “ so it could still be used by you and third party but secure it from those scary “hackers”. This is not about security. It’s about protecting their walled garden and their ability to stop you from using your machine how you want || Wait, so this whole video is basically saying "We have 100% irrefutable proof that BambuLabs was acting in bad faith and lied repeatedly, but trust me bro, they said it wasn't their fault it was BTT." That's a weird take. I hope the free machine was worth it lol. MQTT isn't an exploit. || It was actually me just sharing questions I asked bambu lab directly. To clear the air and all the misinformation out there from people who haven’t even spoken to a bambu lab rep. And to allow ppl to form their own opinion after that based on remarks from bambu themselves. That’s all. || For me, this clarifies nothing. I'm still not buying it. Bambu Lab have offered NO assurance that they won't remove developer mode at a later date. Then we're into things like loss of our IP and having to pay a subscription to use our own hardware! This whole issue of trust (because we don't trust them) could have been avoided if they had put ethernet ports on their H series machines and made the use of the Laser LAN mode only. Personally I'm still a bit pissed that a simple ethernet port is still missing from nearly all of their machines.  Thanks for trying on our behalf. I still believe that we are the ones being exploited though. || Hey I tried. I just wanted to get some questions answered directly from Bambu because I know a lot of people, including myself or relying on information from other people on the Internet and even I was wrong on some of it. || Just got into this hobby and am finding more and more how much I dislike Bambu and am glad I didn't go with them. That interview bullshit just sealed the deal with me. But it's good to see Bambu can fight negative press one free machine at a time.. I guess. || Just bought a roll of the TPU. || Nice!!! You will love it. The best starting point for a profile is Prusa’s flex profile. It prints MorphX perfectly. || Just to be clear here, they only restrict API touch functions of these panda screens right?
-My panda knomi will still work? || It all depends on what firmware you are running, and if that firmware is blocking key things, your device needs to function. From what I was told basically at any point if they find a Security reason to patch it, they will do so without warning. But they aren’t doing it just to render those devices useless they would only do that if needed for security reasons so it’s kind of up in the air I guess. || ​@stayreadyto3dprintoh I thought that it was safe because it's just displays information and it doesn't have any input/ touch screen like the regular knomi v2 || @anthonyrossetti7509it may be. I’m not 100% sure what allows it to function tbh. || Ok so what is driving the dropping creality? || Coming soon. They suck that’s why. Lol and they treated us pretty shitty. Details coming soon. Plus they aren’t innovating. They keep coming out with machines, basically changing a few things and </t>
+          <t>❤❤❤❤ || 💪🏾💪🏾 || 💯 || 💪🏾💪🏾 || Yep, please don't wait until you are 3 years in to start generating P&amp;L statements. || Right I see this wayyyy to often with folks || ​@PATRICELSTEWART, this would have saved me a few thousand dollars.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>OReSdBUIe3A</t>
+          <t>GK6JhMq6vSQ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Is 3D Printing About To Take a Dive?</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Lawmakers are trying to invade makers privacy and dictate what we can and cannot 3-D print on a machine that we bought and paid for in a home that we own as a free American. 
-Make it illegal, but you don’t get to install software that spies on me. 
-What’s next? Will they install cameras in our house to make sure we’re not committing a crime?</t>
-        </is>
-      </c>
+          <t>Self Prepared is No Liability #patricelstewart #business #taxdeductions #tax #taxpreparation #taxes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-01-23T22:37:10Z</t>
+          <t>2026-01-10T07:31:35Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1293</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>199</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.051817</v>
+        <v>0.108483</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -792,69 +737,65 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Well, this is going to blow your mind. And honestly, I can't believe this is where we're at in life. But check this out. &gt;&gt; I'm proposing the first in the nation law requiring all 3D printers sold in the state of New York to include software that blocks the printer from creating a gun. It's just common sense. Just common sense. &gt;&gt; Common sense. It's funny they mentioned that. So, if you're using common sense, common sense would say to go after the real guns that's had millions of cases in the past 5 years versus 3D printed weapons that's had in the hundreds in the past 5 years. I mean, come on. Do you really think that criminals are going to buy a 3D printer, sitting down, taking the time to learn the software, figure out how to 3D print, how to get a print to come out good, and do all of that to get a 3D printed weapon when they could just go on the street and buy a weapon on the black market or steal one or do whatever they do to get unregistered firearms or illegal weapons, whatever it is. So, this stuff about 3D printed weapons and all that, they're they're going after this. To me, that is not common sense. To me, there there's an underlying agenda here, and I'm pretty sure you guys can see through it. So, what do you think about this? Do you think they should continue to do this and basically invade our privacy by watching our 3D printers and dictating what we can 3D</t>
+          <t>When you are filing your taxes, you are supposed to receive a full copy of your tax return. All pages, not just the 1040 page, which is two pages. A lot of you all only receive no paperwork or you receive one or two or three pages. An average tax return is about anywhere between 12 to 25 to 30 pages with all of your worksheets, all of your forms, everything. Also, it should not say self-prepared if you are going to a tax professional who says that they can file you professionally and you're paying them to file your taxes. All right? A lot of you all go to people who do your taxes on Turboax and that may be cool with you, but there is a process and there's a difference between someone who is a real tax professional like myself who is an eile agent. We are registered with the IRS. I have an EIN number with the IRS. I also have to have a P10 number. So on the bottom of your paperwork when I give it to you, it has all of my company information because that means I am responsible for the tax return that I filed on your behalf. A lot of people you all go to are doing all of this extra stuff because they have no liability for the tax return. If it says self-prepared, then that means you are responsible for that tax return. Patrice L. Stewart here, the realist tax and business strategist.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>How would ai even be able to correctly identify a part and what it’s intended for? BTW I support gun restrictions, but this is just Looney Tunes. || Yeah I agree. || Open source software/hardware wins again || Yup. They can’t stop
-That. It’s a waste of time. We all know that. All smoke and mirrors || GOP is proposing a bill to fine women $17 thousand dollars if they aren’t married by 30 years of age. || Oh nice. How about that. LOL || I'd outlaw home depot selling pipe bomb components... Idiots || Why not just outlaw installing those components (a.k.a water pipes) into any politician's home? They would surely enjoy the pre-industrial lifestyle without running water. || Yesh what about that? Geez. || Umm. Yeah. And how are you going to identify that....
-And this is what you're going for? Oh dear gods. || Right? How will they? By invading our privacy is how. Ugh || Look, I'm not in favor of 3D printing guns, and I'm no 2A advocate, but I am a certified drafter, and I worked 20 years in silicon Valley, and I have NO IDEA how this "software" could be written. 
-I don't think it's possible. || I think if they do it’s way more to do with spying on citizens of interest versus caring about guns. || hi Lawrence why was my comment taken down ? Or not showing up cheers mate || Yeah I do not know. I didn’t do it. Probably YouTube pushing a narrative or blocking one. 😝 || @debraSam2012strange. Not surprised || Its LEGAL for american citizens to manufacture their own firearms for personal use without an FFL. It's the states that are illegally taking their rights away.
-But what if they sell it? Theres already a law for that.
-But what if a falon makes a gun? Theres already a law for that.
-What if its used in a crime? ..... really?.... || Exactly. Make a law. If they break it lock them up. Simple. But they don’t get to dictate what a machine we bought does or doesn’t do. Thats bs. || I was just watching videos about it so dumb || Crazy huh? What do you think will happen ? || Knowing the way things are they'll probably do it but i hope not</t>
+          <t>Good morning Beautiful Queen😍...Thanks for the love and information🥂 || Great information! || Thank you for keeping it 💯 || 😊 || Thankyou || You’re welcome 😊 || 💯 || 💪🏾💪🏾 || ❤❤❤ || ❤❤ || ❤️✊🏾 || ❤❤</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5ipo5Vlc7tU</t>
+          <t>26JhrkttRwY</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>My Fav’s From CES 2026 #3dprinter #tech #ces #laser @xToollaser</t>
+          <t>Tax Time let's talk do's and don'ts</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>I went to the world’s largest tech event, CES 2026 in Las Vegas where I found some of the newest tech to come in the 3d printing world in 2026. Enjoy!!!</t>
+          <t>Work with Patrice 
+plstewart.info/bookme
+#taxdeductions #business #realestate #chicago #taxes #credit #entrepreneur #tax #taxtips #taxtipsandtricks #taxrefunds #taxreporting #taxtips2026 #w2s #1099 #selfemployed #entrepreneurship #taxwriteoffs #taxwriteoff #taxplanning #taxwithholding #realestateinvesting #1099k #taxhelp #irs #smallbusiness #schedule1 #schedulec #llc #partnership #scorporation #corporate #taxcredits #bigbeautifulbill #bbb #trump #trending #financeeducation #financialfreedom #financialliteracy #finance #mindset</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-01-15T20:02:50Z</t>
+          <t>2026-01-10T01:11:18Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>152</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.036041</v>
+        <v>0.118421</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -863,529 +804,430 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Here's some of the coolest things that I found at CES 2026, [music] like this circuit board printer. It prints a conductive liquid directly on the PCB board. Very cool. [music] But check out this metal 3D printer. It takes liquid cartridges and turns it into hard metal. Depending on which cartridge you put into it, whether it be aluminum, copper, steel, nickel, and as you can see, it can print intricate designs. But check out how you load this thing. I've never seen one like [music] this. It takes these liquid filled syringes full of liquid metal, and you just simply load it up and go. Now, I did a video on this one already, but this is the Atom Form Pallet 300 made by MOA. It's a 12 nozzle changer with [music] 36 colors. Pretty cool, and it's coming soon. Now, this isn't a printer. This is a software [music] from AF Research where they basically took machine learning and jammed it into a printer. It takes a $5 webcam and some high-tech software where it can basically [music] teach itself how to print quality prints from nothing. So, no more programming filament profiles. XL had a humongous booth. This is their apparel printer. It's a DTF printer that prints on [music] these plastic films here and it prints super vibrant color and then you just hit it with a heat press. But they're really known for their lasers and they brought [music] the F2 Ultra again with the rotary attachment and the passer attachment on the UV model. Now, the UV model is the one that can actually laser inside of crystal blocks and do the glass and [music] clear stuff. It's really nice, and so is the M1 Ultra. It's not brand new, but it's [music] still awesome. It's a laser that actually has a inkjet printer built into it that can print on top of the wood, which [music] creates endless possibilities. But this one was the talk of the show. This is their all-new UV additive printer. Unlike a UV laser that subtracts [music] material, this one adds material and it's full color. I mean, it looks absolutely wonderful. All of these were done on the new machine, and [music] I can't wait for it to launch. Then we have Create, who brought the Create High and disguised it as the allnew Sparks i7 and kind of made a new CFS. And I don't know, but the Falcon team is still on my good side because they're actually innovating and making new products. [music] And this is the allnew T1 5 in1 laser. And this is the Falcon A1C 20 watt desktop.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Liquid metal? This is T2 stuff. || That metal 3d printer is sweet || It’s like 30k though ughhhhh😢 || Dang ​@stayreadyto3dprint</t>
-        </is>
-      </c>
+          <t>I don't know why this still pops up here. Make sure my volume is on. Make sure my volume is up. Good evening. Good evening. Good evening. Good evening. I'm on a few platforms, so I'm just going to allow a minute or two before I get started. Um, tonight I wanted to come on to briefly talk to you about tax updates, especially with these advances right now. Kind of wanted to explain to you all um how these advances work. I know a lot of people are promoting advances and things right now. So, I wanted to actually make sure that you all know the proper process on this and how it all works because you have a lot of people, you know how it is. Every year you get all these hustlers, as I like to call them, you get all the hustlers that's hustling taxes and tax time. And a lot of y'all don't know or get the real information. So, I am also filming on my YouTube channel. As always, YouTube is my number one platform. So, the replay to this video uh will be on my YouTube channel. I will not have this replay on Instagram or on Facebook. I am Patrice L. Stewart on all platforms. The name that you see on on whatever channel you're watching me on is the same name on my YouTube channel. Okay. So, good evening. Good evening. Good evening. It is Thursday night, I believe. Yeah. I don't even remember the days of the week. It's Thursday night. And so, I've been getting a bunch of calls right now around this whole tax advance, right? So, I wanted to share you with you all how this whole tax time season works right now. Okay. Um, and let me just make sure before I say that because I know yesterday, I didn't check today, but as of yesterday, the IRS has not announced the opening filing date for 2026 tax season. So, let me just make sure before I say that that Oh, we got a date. See, things change every single year. So that's why you have to check every single day. So yesterday I checked, we didn't have a date. We actually have a IRS open and filing date. As of right now is Monday, January 26. So I'm glad I decided to check before I said anything. So let's go ahead and get into this update. Um, hello, welcome. My name is Patrice L. Stewart. If you are new here to my page and my channel, better known as the realist tax and business strategist. Um I have over 20 years in the tax accounting banking industry and I am a tax strategist. Okay. Um right now we are in tax season. I want one of the things I want to say is taxes is all year round, right? It's it's only called a season right now because that's the time that majority of you all are filing which is between January and April, right? But just so you know, taxes is all year round. I filed taxes from January to December. The last tax return that I submitted was December 26, okay? A couple of weeks ago. That's why I'm not rushing to file taxes today. Um because I just got through filing the last tax return December 26. So people like me who are real professionals in this industry, uh we file all year. It's it's not seasonal. Taxes does not start um does not stop, excuse me, after April 15th. Right? So, I wanted to put that out there. Taxes is all year round. You can file taxes after April. I have some clients that wait to file their taxes until September, October, November. They want to get their refund closer to the holiday time. All right? So, that's up to you. Just want to put that out there. two, now that we have a IRS date, because I was [clears throat] just getting ready to come on here and say the the IRS is not even open right now, but they have officially now put a opening season date. So, every year, um, the IRS shuts down at the end of the year, usually whatever the last day is of that we filed a tax return. So, this year we were able to file t last year, I'm sorry, we were able to file taxes up until December 26, right? So, the IRS shuts down about a week and then in January they open back up. So, right now you all may be seeing people promoting, "Oh, you can get a cash advance. You can get a cash advance. You can get a cash advance because I've already had four calls today about this cash advance." I wanted to explain that to you all. All right. What is this cash advance and how does it actually work? One, the IRS is not officially open. Okay? They literally just put on here today because I like I said I checked yesterday and they did not have a open seasoning date. Now they have a open seasoning date for 2026 which will be January 26. January 26 is the official day that the IRS actually opens for tax season. Now you all may see people promoting and saying, "Hey, you can get a cash advance. I mean, you can get you can get an advance on your taxes. Let me explain this to you because a lot of people will not explain this to you because again, uh, a lot of them be thirsty to get your money. Real quick, um, I personally don't like to file taxes early January. My office, we're not actually opening until Monday the 12th, and I only file uh, advances for a specific client base, not for everybody. But one with the cash advance, in order for you to apply for a cash advance, you still need all of your forms and documents. Okay? So, the worst thing for you to do is if you have three W2s and you only have one W2 right now and you go and you let somebody prepare your taxes and file for a cash advance, one, the IRS is not open. So, what you're getting, you're doing a pre-agnowledgement advance. Okay? So, there's two different types of acknowledgements. You have a pre-agnowledgement and then you have the post acknowledgement, which means the IRS is actually open. Okay? Right now, any of you all that are working with somebody and you are doing a cash advance today, today is January 8th. All right? You are in a pre-agnowledgement. So that means your taxes are going to be sitting in a uh basically in a waiting pot, okay, till the IRS opens. Now, will they give you that advance? That advance is not through the IRS. That advance is through whatever tax office company that you're using. Their bank is allowing you to offer cash advances. All right? So, I want to explain that cash advances do not come through the IRS. They are not from the IRS. They are actually from whoever you're working with that that office is uh is registered with a bank. That bank is giving you all the cash advance. Okay. But the biggest thing I see when people apply for these cash advances or or give or give me feedback, let me say that because we ask a lot of questions before we push through an advance for somebody. Um, the biggest thing that I've seen that people do is you all go to these offices that are pushing to for you to do these cash advances and you don't have all of your paperwork. Right? That's the biggest first mistake I would say. Do not apply for these cash advances and you are missing paperwork. A lot of you all do not have your W TWS right now. Yes, companies do go online and you have access to your uh portals and W2 information for some of you online, but a lot of employers are still getting your W2s and paperwork together. If you know that you own a home and you file your house, your your mortgage company probably does not have your uh 1098 on there yet, right? If your child goes to school and you need to claim school credit, you probably don't have that school form on there yet. Okay? Most of the time, we are allowed as employers and companies up until January 31st to mail out your W2s, your 1099s, your 1099 KS, your your any form, right? Whether it's investing, whether it's your school form, whether it's your W2s, whether it's 1099s, the companies have up until January 31st to get those mailed out to you. So, the biggest thing that I see is you all are applying for these cash advances with these people that are promoting these things to you, but they're not explaining that to you. You need all of your paperwork before you file for that cash advance. Okay? And again, the official opening date that the IRS will begin processing tax returns officially is January 26. Okay, that's the date. Um, the deadline date this year, and again, deadline is for people who normally owe. All right. They the IRS would like for you to pay by April 15th, but it does not mean that you cannot file taxes after April 15th. You actually have up to three years to file a tax return. Okay? Um if you did not file taxes last year, if you didn't file 2024 taxes, if you haven't filed 2023 taxes, you can still file those. You can still file those electronically. With my office, we can file up to your last three years electronically. So, now that we're in 2026, we're filing 2025 taxes. You have 2024 taxes and 2023 taxes. Any prior years to that would have to be mailed in or uh my office, we have a department that we try to fax in prior year taxes and get them processed through a little bit quicker. Okay. Um but again, you can file taxes after April, you all. Um, all US citizens have the right to do a six-month extension. Okay? So, if you need an extension and you need more time to pay, if you know that you owe and you are not ready to pay that by April 15th, that's where the filing the extension comes in at. All right. Um, and again, all American US cit all US citizens um have the right to file a six-month extension. Okay. Uh, what else did I want to say? What else did I want to say? Tomorrow I am going over the big beautiful bill in my private community and also on the uh YouTube page for members only. So, the big beautiful bill that they um turned into law last year, there are some new updates, all right, for you all. Um, so we'll be going over those in the private community, what school won't teach you. Those of you all who are in the private community, make sure that you sign uh that you join in, that you log in into the Zoom because I will be going live to go over what's in the big beautiful bill and how you can take advantage of some of these tax updates that um the government has set up for you in the big beautiful bill. That's really it. What time is it? I don't have I didn't want to be on here a extra long time. Okay, perfect. 13 minutes I've been on here. So, I will review any questions that you all have now at this time and especially on my YouTube channel. Uh, thank you, Train. What's going on? Happy New Year. Chad, you say, "Can you give us tips on skipping them?" When you say, "Can you give us tips on skipping them?" I don't understand. You need to ask a a better question, Chad. Skipping what? Bid spotter say, "Patrice, I'm just seeing you. [laughter] We're live. Let me listen." Yes, Big Spotter. Go ahead and listen. Take a couple of notes. Like I said, I didn't I'm not going heavy tonight. I just wanted to really bring that up because we do have I had a couple of people call my office today about that whole cash advance thing and I think a lot of times you all get all of these promoters, you know, not knocking anybody, but it is what it is. I mean, I'm I'm a professional in this space. I'm a tax expert. I'm a tax strategist. So, this is my lane. Take it how you want to take it. But we have a you have a lot of people that at this time like to side hustle taxes, right? And they love to promote certain things to you all, give you all these astronomical dollar amounts that you could get. And I'm going just say this like I always say. If it sounds too good to be true, it normally is. Every single week, my office gets calls from you all who have been audited or being audited because you have credits on your tax returns that you should not have. If you normally get back $1,000, $500, whatever you normally get back, and now somebody is telling you, "Oh, I can get you back five to 10 bands, uh, hello." Clearly, they're not doing what you normally do. It's just that simple. So, I don't want to hear that fake weak ass excuse that y'all like to come on here and say, "Oh, well that somebody just put whatever they wanted on my taxes. You was good with it when you was about to get that $5,000, right? You was good with it when you got that five or $10,000. But now that the IRS has audited you, cuz the IRS will give you that money. Let's let's be clear. They will send you that money. People be thinking like, "Oh, well, I got my refund." Yeah, you get that refund and in two to three years you'll be calling my office crying like the rest of these people are, right? And that's what it is. The IRS will give you that money. Let's be clear, right? Sometimes whatever they put on you all's taxes, fraudulent credits and stuff, sometimes it goes through. Yes, it does. But I guarantee you, I bet money on it. Within two to three years, you will be getting a letter saying that you owe this dollar amount, [laughter] saying that you owe this dollar amount. And then you'll be crying talking about, "Oh, the person put on whatever they, you know, put whatever they put on my taxes." Yeah. All right. So, don't come on here with them sad stories lying because you was fine with it. Okay. Just know and understand half of these people that are promoting that stuff, they're not real professionals. Real professionals, we don't even promote stuff like that, right? We're not promoting five, $10,000 refunds. People that promote dollar amounts and numbers usually are hustlers. Hustlers and I like to call them. Real tax professionals don't do that. Real experts don't do that. We don't have to do that. We don't have to do that. It's not a This is not a numbers game, right? This is real. Your finances is real. Your money and your taxes is real. Okay? This is not a game for you to be playing with. And a lot of people who have done it in the last couple of years are seeing that. Everybody going to promote and say, you know, hey, I got the money, but nobody ever comes back on to tell y'all that now they under investigation, right? Uh so that's the reality of it. Um is the big beautiful bill going to help us get a bigger refund? So many people the big beautiful bill will help. Every single one of you all are different individuals. So there's no um you know one sizefits all to taxes. That's what I love to say. Every single person's tax return is different. So is it going to help people who receive tips? Yes, it is. Those of you all who rely on tip jobs, you will be able to have a nice dollar amount that you'll be writing off. seniors. It is helping seniors. Seniors have a whole new tax uh deduction that they've never had before. So again, certain people will benefit from the bill. Certain people won't. Um the standard deduction goes up every single year. That's not nothing new, but the standard deduction has gone up this year. So, some people should see should again I don't know your situation, your paperwork. Also, taxes are based off of what you paid into the system. Okay? So, if you have a W2 and you didn't pay any federal taxes, I'm Let me say this to y'all. Let me get a little closer in the screen when I say this one. Those of you all who pay no federal taxes throughout the whole year and expect the refund, did your mama drop you on your head? Because I really don't understand that. All right. One thing my dad always taught me was either you going to pay taxes throughout the year and you get some money back or you pay or you do not pay taxes and you get your money during the year. All right. But to pay zero in federal taxes, you made a h 100,000 and you paid zero in federal taxes and you expect a tax refund. Why? Does that make any sense to you? Okay, you didn't pay any taxes into the system. So 99.9% of the time you're going to owe. All right. Now, if you have other things like maybe real estate investments, right? Maybe some other things going on that help you with that tax deficit. But those of you all who know that you paid zero in taxes through the whole year and expect a refund, I don't understand your logic behind that. You have none. You don't understand how the system works. Okay? So, I'm I'm on here to tell you that today. If you are a W2 wage earner, you all pay taxes out of your paychecks. Now, if you are someone like me who is a business, I'm a corporation, but I'm also an escorp. I don't pay taxes throughout the year. businesses. We pay our taxes when we file our business taxes at the end of the year, especially service-based businesses like myself. Now, if you are a productbased business or maybe you have a store, a retail location, maybe you sell clothes or maybe you have a grocery store or something like that. A lot of you all pay taxes throughout the year. All right? And this is why I said every single business is different and there's no one-sizefitit all to it when it comes down to taxes. Everybody's situation is different. But I definitely need to put that out there because we have way too many people who pay zero in federal taxes from a W2 that expect the refund. And that just makes no sense to me. I just don't understand why you all think that that you should get that. Especially when you grown grown. You grown. You've been filing taxes for 20 years and you still have that misconception in your head that you should be getting a refund. So maybe you've never gone to a tax professional that knows how to explain this type of stuff to you. And that is the reason why I trademark I'm the realest tax and business strategist because I'm real. I'm honest. I'mma tell you the truth. It ain't no sugar coating over here. We going to get straight to it. I'mma tell you what it is and that's what it is. So, uh, any questions? I'm not going over the big beautiful bill tonight. I'm going over that tomorrow and I'm going over that in the private community. Um, the private community right now for what school won't teach you, it's only $37 a month. So, those of y'all that want to get in class tomorrow night, we'll be on at 6:00, 6:00 to 7:00 p.m. Um, you can get in, you can text me to the phone number and you can get into the private community. It's a membership community that I have and that's where I do all my educating. All of the classes and the workshops that we host are in the in the private community. Um YouTube, do you have any other questions on here? It's been 22 minutes. I I will be on here another eight minutes. Oh, I saw somebody on Instagram. I'm sorry, Instagram. I'm not purposely um ignoring you. I just am not on here much. I really just come on here to let y'all know that I'm live. But I would recommend that you go to my YouTube page and channel. Alan, you say, "Patrice, is it true that Social Security will go untacked in 2026?" Um, it's part of the big beautiful bill. I'mma say that. It is part of the big beautiful bill for Social Security. Um, so that's the most I'm going to say, Allan. It is part of the big beautiful wheel. So people who are on social security, that is something that um that is that will that will be beneficial for you. that is something that will be beneficial for you. But I'm going to go over that in a lot more detail um for you all like I said in class. And then those of you all who are members on my YouTube channel, I do have a membership here on my YouTube channel. So you all also will get access to that as well. And like I said, people who are in tip based industry, you all will be happy. Um, those of you all who are seniors, uh, our seniors will be happy because there is a brand new deduction for our seniors. And it's a couple other things. It's a lot actually. It's a lot, excuse me, that they have added in this big beautiful bill. So, we are going to go over some of those things um tomorrow during the class. And like I said, somebody asked me earlier or inboxed me earlier about the um standard deduction. So, the standard deduction increases every single year. Um every single year. So, it has increased this year. So, a lot of you all should see depend again should I won't say should it could it could be you might see an increase in your tax return you might not it really depends on what your W2s look like right because again everybody pays different amounts in federal taxes those of you all who claim zero all year um you might want to stop doing that because again people who claim zero all year normally you all owe you are welcome Welcome, Alan. Thank you for waiting and being patient cuz I saw your question come in, but I was talking and looking over here at the YouTube uh screen and channel. So, Miss Dos, you said the link won't work, huh? I don't know what's going on. We'll I'll type it in the um I'll type it in the comments. I'll type it in on here. So then that way you could just click it. PL Stewart PL Stewart. But it's that time of the year, so I'll be like back on the back on here doing these live sessions with you all from time to time. [clears throat] Uh they'll be short. Like I say, I give more information in the private community. I have gone into community. We've been on the internet for free for 10 plus years. So now I only focus on people who are serious and people who serious get into the community. Uh, okay, Miss Doss, I just typed it in the comments, so I don't know if it gonna come up right away then. There you go. Oh, and I didn't send it to you. I didn't text you either yet, Miss Dawson. I'm I'mma text it to your phone. I got distracted once we got off the phone. So, I'll send it to your phone cuz I told you I'll text the link to you. Um, okay. I knew YouTube has somebody else. YouTube, y'all always got questions. That's why I love y'all. Uh, how often do we meet in the private community once subscribed? So we meet weekly and then I also put video content up in there as well. So we drop video content and when you join it's it's about 40 different modules in there already for you to watch. So when you join the community it's already 40 different modules in there but that's all from last year. So now I'll be updating um you know more newer information for you. But in the private community, if I don't come on, then we have a guest speaker or somebody else come on. But at minimum, I go live once a month at minimum. But you do we we do normally meet weekly. I do have another coach in there, Chuck Finance. He's in there. So, he does study hall. Um, and then we normally do an interview with a professional to teach you all and educate you all on a different type of topic. So, 2026, we got a lot planned and to roll out. So, the biggest thing that I'm working on for 2026, which I'm really excited about, is my male community. You my YouTube channel is mostly 75% men. And we have 75% men as followers and 25% women. So, I am very big with educating the men, the male. We need the men fully aware, fully financially handsome. If you all remember, I had these shirts, financially sexy for women, financially handsome for men. Um, but this year, 2026, I am completely focused on making more men financially handsome. I am tired [laughter] tired of this whole back and forth 5050 conversation that I see online. Um, a lot of the young guys are driving their girlfriend car, lived in their girlfriend house. So, my goal is to empower more men financially. Um, so I'm really excited about that and especially in the sports and entertainment space. Um, so I definitely have some things that I am working on that we'll be rolling out. Um, and I'm actually going to be hosting a workshop for the male youth. So, if you have a son that's between 13 to 19, within the next 30 days, I will be talking about that. Um, I know it's sports, so I'm trying to figure out and talk to a couple of men on what's the best day to host this in-person workshop, but I am hosting an in-person workshop here in Chicago for the male youth between the ages of 13 to 19. Um, and it's a course. It's a ongoing course. It's not a one-time thing. This first event will be a one time a one day event but moving forward it will be an actual um course a 8 to 12 week course where we are empowering the male youth regarding different financial topics and setting up their retirement account making sure that they understand credit business entrepreneurship um it's a lot geared towards women got everything women empowerment this women empower department that, but I don't really see a lot of information out here for the men and specifically talking to the men. So, I'm meeting with two great fellas this weekend to help me um finalize the curriculum for the course so we can make sure that it's something that the men will, you know, take away from it and get out of it. But yeah, that's that's that's the thing for 2026. I'm I'm real excited to hear about I'm really excited to push this whole program out because this will be nationwide. Y'all will eventually see me traveling from state to state to different locations to talk to the men and the male youth specifically. I'm only focusing on men. It will not be females in these classrooms. It will only be men. So, if you in Chicago and you have a young son that is between 13 and 19, he needs to be in the room. All right? He needs to be in the room so he can learn this. Learn how to get this money, baby. All right? Learn how to get this money cuz once we have the men empowered, once all of our men are back empowered financially, then we can get back get back in equilibrium as a community cuz everything is off whack right now. All right. That's why I said boy my god baby 23 and she talking about her friends friends boyfriends and how are these boys living with girls driving girls cars like nom. I'mma need y'all to get y'all weight up fellas. So we going to focus on that. We're not going to talk about the men. We going to empower the men. So I'm ready. Let's go. Let's roll. Doing that would definitely help provide structure. Exactly. You see another that's the whole point, right? That's the whole point. We we need we need to bring back structure and order. And I'm I've always been a person that's about how do we change things? I'm not a complainer. I'm not on here complaining about nothing. Uh I'm always in how can we fix this, right? What's what can we do? So me being in financial services for the last 23 years, that's what I know that I could do to help out, right? That's what I could do is help share the knowledge and information that I have to the men and also guide you through it. Right? We're helping you set up your investment account. We helping you fix your credit. We helping you start your businesses. Um I got two clients that I helped last year in Florida do they NIL deal. Right? So again, I'm really focusing on the male youth and especially the ones that are in sports and entertainment. Um because I feel like we have a huge need there. If we have 30 boys in a room, the reality is one of them is going to the league. The other 29 is not. Right? So in my mind, y'all setting these kids up for failure because what are we doing if you only teaching them to do football and basketball and you know in a room of 30 kids only one is going to the league the other 29 what are we doing? Right? So in my mind I'm like this this is whack. [laughter] We need to fix this. That's a problem. Right? So, for me, that's that's one of the things I'm going to do. And it's a it's an untapped market. I have literally talked to about 50 different coaches, mentors, teachers, educators, men that work with the male youth already. And I literally asked that question, do you have a financial literacy program for these young boys? And they, every single one of them, right hand to God, every single one of them said no. Every single one. 50 coaches. And that's just in Chicago or the South Suburbs. 50. Every single one said, "No, we do not have a financial literacy program." Baby, how? Why? Okay. Well, here I am. Let's get it going. Let's start it. So, if you are a male or know a male and you got friends that's coaches and all that, tap in. get with me cuz I will be moving around. I'mma start in Chicago, but the goal is to definitely at some point this year, travel to other states, travel to other cities, get in the room with you all, get in the room with these young men. Um, and teach them cuz it's it's time. It's overtime. Exactly. [laughter] I like that. Uh see another you say we need more trays and less dough boys. Exactly. Exactly. Exactly. We need way more trades and less dough boys. And college and and all of that is not for everybody. You know what I'm saying? Every young man doesn't want to go to college. But we also have trades. We don't talk about that enough. And we actually have a lack of men, specifically black men in the trades. I have a friend that uh he runs the program for the trucking, no for for the electrical um apprenticeship for com. And he said the last what probably four [snorts] years it's like no black men in there. Like all Hispanic. It's like I think he said the last class that they did it was one black man in there. That's crazy. You know, some of these classes have 50 to 75 people in them and we only and you only got one black man to learn electrical to learn electrical trade. That's crazy to me. Crazy. So, we need to start having these conversations. And on that football field, in that basketball field, there's like a hundred other positions, right? I just said only one of them go into the league. Everybody can't be a quarterback. Everybody can't be the line running back or whatever these, right? It's it's so many other positions within that same industry. But why are we not talking to these young men about that? Right? Why are we not talking about that? Why are we not empowering them to do more? cuz I have seen so many grown men who were once young boys trying to go to the league and once they don't make it to the league they depressed and then their life is over. They don't do nothing else. They don't do nothing else with themselves. That's horrible. So that's why I said when I reached out to those men and asked them about if they have a financial literacy program for their um you know mentees and and all 50 of them said no. I knew then that that was a need that that was a need that needs to be serviced. So I'm excited to to service it. Let's get in the room and change some lives. What's Dawson see another? I'm still learning. I don't know sports too well. I got a I still I'm still learning a lot since I'm about to be talking to these kids. I've been studying and learning some stuff. But what's at Dawson? Is that a location or a school? I saw somebody say something about their sons. Dedra, you said, "Love that for the boys. Our young men need this. I have two sons. I hope they will be able to participate. So that's what I really need to find out like if I wanted to host a workshop within the next 30 days like it would is a Saturday. Okay? Cuz I know a lot of you all I don't have kids so I don't know when y'all are practicing. Are y'all practicing? Are they practicing on Saturdays? You know, uh Sunday everybody sitting there watching football. So I don't want to do a Sunday. But I need to find out from these coaches that I'll be reaching back out to this year as far as like what's the best day to do that? If I did an hour workshop once a week, every you know once a week for an hour to two hours, what would be the best day to host that? Right? So that's that's been my biggest question now is like what would be the best day to provide that service to them. And I do actually have a fullfledged 501c3. So I will be on here at some point asking y'all for donations and donors because again we need to get this information to the kids and the youth. Um, but yeah, 2026 we rolling. So, Dedra, I'll be posting more about it. I'm getting ready to sit down with two fellas this weekend that I'm meeting on Sunday. Um, so probably on Monday, I'll be talking more about an actual date, but the goal is to have our first one day event within the next 30 days at minimum. within the next 30 days. And I'm open to it could be the evening, it could be, you know, a weekend. I just don't know what's what is the best what's a good day to do this for those of you all that are in sports and entertainment. So, Dedra, if you got two sons, then let me know that. Give me that feedback. What day will they be available to meet for one or two hours to learn this information? And the program is called financially handsome because again we are changing it's raining like casting dogs right now. Jeez. We are changing the mindset of the youth. Changing the mindset of the youth. Okay. You say Dawson is the tech school on 39th and state. Okay, let me write that down. Somebody gave me the le the um somebody gave me the information to Leo, the principal at Leo High School on 79th Street. So, 39th in State Dawson. I'mma write that down. Dawson Tech. Thank you. C Nether. Yeah, they gave me Leo High School infor</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lwi_rKRQx54</t>
+          <t>geilOn3K8ks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Uniformation GK3 PRO Printer Giveaway! 1/11/26 @6  pm CST</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>FILL THE FORM HERE
-https://forms.gle/7BDED7YRwbos1wwdA
-https://uniformation3d.com/
-follow on instagram here
-https://www.instagram.com/uniformation3dprinter?utm_source=ig_web_button_share_sheet&amp;igsh=ZDNlZDc0MzIxNw==
-Stay Ready To 3D Print Instagram
-www.instagram.com/stayreadyto3dprint
-Check out the NEW AXI Pro here
-https://em-smart.com/?gad_source=1&amp;gad_campaignid=23334198655&amp;gbraid=0AAAABBeSBMzBKNbys7Q5YRsV_Mx_DoqiQ&amp;gclid=CjwKCAiAjojLBhAlEiwAcjhrDmiUXCBi4unFPA7GTY3ovx0MtKBwaBHXN3y40NVDE3SR-j0xSN-WAxoC69wQAvD_BwE
-Thanks for watching! If you're into 3D printing, whether it’s tuning your slicer settings, upgrading your Creality, Bambu Lab, or Elegoo printer, or experimenting with TPU, PLA, PETG, or custom filaments, you’ll feel right at home here.
-Join our Discord server to connect with one of the most active and supportive 3D printing communities online. We share printer mods, filament reviews, print profiles, and behind-the-scenes looks at our latest projects — plus, we run regular giveaways, offer support, and drop early news on upcoming content.
-Stay ready, stay printing — and be sure to check out our latest builds and experiments using today’s top 3D printer brands and materials.
-Join Discord here!  https://discord.gg/E5gPc8C2cs
-🌐 **Facebook Page**  
-📘 https://www.facebook.com/profile.php?id=61565872940311
-👥 **Facebook Group – “Stay Ready To 3D Print”**  
-📘 https://www.facebook.com/share/g/196GC85xxo/?mibextid=wwXIfr  
-📸 **Instagram**  
-https://www.instagram.com/@stayreadyto3dprint
-🎵 **TikTok**  
-https://www.tiktok.com/@stayreadyto3dprint
-🎁 **Patreon** – Get early access &amp; exclusive content  
-https://www.patreon.com/stayreadyfans
-📬 **Business inquiries / sponsorships**  
-Email: stayreadychat@gmail.com</t>
-        </is>
-      </c>
+          <t>PATRICE L. STEWART is live!</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-01-12T13:10:43Z</t>
+          <t>2026-01-06T19:58:45Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>393</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+        <v>0.096692</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>TUNED IN sister,❤ Happy NY, EVEN though the REAL New year is April || HAPPY NEW BEGINNINGS to you and your family Queen P.! || Happy New Year Rodney || 1:23:33 I agree || 💪🏾💪🏾 || Girl! You look so cute! Love your hair!!! Mad I missed the live.  Hope you’re well! || Thank you 🙏🏾 ❤ happy new year! Beautiful and I’ll be on tonight</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Vk2MosCyQdM</t>
+          <t>maZLr_qFnuM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Uniformation 3D Printer Live Giveaway! 1/10/26 11pm CST</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://uniformation3d.com/
-follow on instagram here
-https://www.instagram.com/uniformation3dprinter?utm_source=ig_web_button_share_sheet&amp;igsh=ZDNlZDc0MzIxNw==
-check out the new AXI Pro here
-https://em-smart.com/?gad_source=1&amp;gad_campaignid=23334198655&amp;gbraid=0AAAABBeSBMzBKNbys7Q5YRsV_Mx_DoqiQ&amp;gclid=CjwKCAiAjojLBhAlEiwAcjhrDmiUXCBi4unFPA7GTY3ovx0MtKBwaBHXN3y40NVDE3SR-j0xSN-WAxoC69wQAvD_BwE
-GOOGLE FORM LINK WILL BE POSTED IN THE CHAT! TO ENTER GIVEAWAYS
-Thanks for watching! If you're into 3D printing, whether it’s tuning your slicer settings, upgrading your Creality, Bambu Lab, or Elegoo printer, or experimenting with TPU, PLA, PETG, or custom filaments, you’ll feel right at home here.
-Join our Discord server to connect with one of the most active and supportive 3D printing communities online. We share printer mods, filament reviews, print profiles, and behind-the-scenes looks at our latest projects — plus, we run regular giveaways, offer support, and drop early news on upcoming content.
-Stay ready, stay printing — and be sure to check out our latest builds and experiments using today’s top 3D printer brands and materials.
-Join Discord here!  https://discord.gg/E5gPc8C2cs
-🌐 **Facebook Page**  
-📘 https://www.facebook.com/profile.php?id=61565872940311
-👥 **Facebook Group – “Stay Ready To 3D Print”**  
-📘 https://www.facebook.com/share/g/196GC85xxo/?mibextid=wwXIfr  
-📸 **Instagram**  
-https://www.instagram.com/@stayreadyto3dprint
-🎵 **TikTok**  
-https://www.tiktok.com/@stayreadyto3dprint
-🎁 **Patreon** – Get early access &amp; exclusive content  
-https://www.patreon.com/stayreadyfans
-📬 **Business inquiries / sponsorships**  
-Email: stayreadychat@gmail.com</t>
-        </is>
-      </c>
+          <t>Vision Boards are DEAD! Action Board or Fail in 2026 😱 (Free Workshop TOMORROW) #patricelstewart</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-01-11T18:57:46Z</t>
+          <t>2025-12-27T04:00:49Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>519</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>91</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.145833</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+        <v>0.181118</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Thanks for sharing.  Will you have a workshop for those interested in starting a business? || Never-ending I just went to your website. Thanks again 😊 || 💯</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>P3ik_UAA9u4</t>
+          <t>0P2PYQhmnEU</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Live at CES 2026!</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Check out the all new AXI Pro from EM Smart,  it’s coming soon, so don’t miss out 
-￼www.em-smart.com 
-Thanks for watching! If you're into 3D printing, whether it’s tuning your slicer settings, upgrading your Creality, Bambu Lab, or Elegoo printer, or experimenting with TPU, PLA, PETG, or custom filaments, you’ll feel right at home here.
-Join our Discord server to connect with one of the most active and supportive 3D printing communities online. We share printer mods, filament reviews, print profiles, and behind-the-scenes looks at our latest projects — plus, we run regular giveaways, offer support, and drop early news on upcoming content.
-Stay ready, stay printing — and be sure to check out our latest builds and experiments using today’s top 3D printer brands and materials.
-Join Discord here!  https://discord.gg/E5gPc8C2cs
-🌐 **Facebook Page**  
-📘 https://www.facebook.com/profile.php?id=61565872940311
-👥 **Facebook Group – “Stay Ready To 3D Print”**  
-📘 https://www.facebook.com/share/g/196GC85xxo/?mibextid=wwXIfr  
-📸 **Instagram**  
-https://www.instagram.com/@stayreadyto3dprint
-🎵 **TikTok**  
-https://www.tiktok.com/@stayreadyto3dprint
-🎁 **Patreon** – Get early access &amp; exclusive content  
-https://www.patreon.com/stayreadyfans
-📬 **Business inquiries / sponsorships**  
-Email: stayreadychat@gmail.com</t>
-        </is>
-      </c>
+          <t>See you on Dec.27 @1pm CST!!   #patricelstewart #business  #chicago</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-01-09T23:55:44Z</t>
+          <t>2025-12-23T18:53:17Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>268</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.048276</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+        <v>0.13806</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>💯</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>xzJKWf8-hKQ</t>
+          <t>gwE_NQhSfAE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The Atomform Palette 300 Is Almost Here! #3dprinter #3dprinting #ces2026 #ces</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>The PROFIT &amp; LOSS STATEMENT: all the basics in 5 MINS! #patricelstewart</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Hey! This video provides a clear visual guide to your `profit and loss statement`, a crucial component of your `financial statements`. Understanding this document is vital for effective `accounting` and accurate `business tax preparation`. It's especially important when preparing your annual `tax return`, helping you manage your finances with confidence. 😊</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-01-09T04:52:40Z</t>
+          <t>2025-12-16T00:01:01Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11589</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.03719</v>
+        <v>0.178082</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Show me just ONE shot of it actually printing and I'll place a deposit! Well no? So Atomform, that's how you ruin your business ... || Be patient. Don’t buy it now. Wait till it’s released and full price if you’re unsure. || @stayreadyto3dprintall I want to know is if this is real! Prices are out as far as I know, starting at 999 for the solo machine all the way up to about 1800 for the fully configured combo. But they never showed an actual working machine or even a prototype which seems a bit fishy… || I saw AI and a login menu, so it's not open source? || I’m not sure. I should’ve asked. Dang. || Ive been following this for a while and pretty excited to see it running. || Same
-Here || Can you say "amazing" any fucking more ? I dont see it printing or doing shit. This is a cash grab || Again, I have yet to see this thing run in action. || while I'm subscribing to 'updates' on their website, Imma go ahead and order a few more Bambu printers. They work juss fine. || Great idea lol || An AI assistant that will eventually not allow you to print a thousands of files || Let’s hope not. lol || Is the belt 2mm? It’s dealbreaking. VFAs will be dramatic. || You mean like 10 mm... and yes, I agree with you. My SVO8 has 5.7 mm belts and it is horrible with the VFA's || @treyduval5399I am talking about the teeth. Width of the belt itself is not that important. || @SpectraLzz so you think that going from 2 mm teeth to like 1.5 on the belts is way better VFA? I'm asking this because I'm modding my SVO8 as we speak. || @treyduval5399 Yes. Bambu H series uses 1.5 and is way better than P series which uses 2.0. || @SpectraLzz well how hard is this to do? Would it require replacing motors or stepper drivers or is it just plug and play with a belt and pulleys? || I’ve placed a deposit on it already || @DukeGaGa what does the deposit get you || Nice || @njv.rooyen5353lower backer price || It whould bena lot better when they print something. || I’ll have one soon. So I can show it all. I’m due time || Putting an "AI" button in the menu sounds like a gimmick and is being overused. Can't say if this printer is good or bad without seeing it in action and looking at a finished print. || Yeah I don’t think anyone can form a valid opinion just yet. In theory it’s cool. That’s all. || But if you feel like an AI button is a gimmick then you should prepare yourself because pretty soon. Everything will have AI buttons lol || I need to see how it handles multicolor and I'd be sold. || Same. How much do you think it’ll cost? || @stayreadyto3dprint What I would pay is like $1200. What it probably will be is $1500-$2k lol || 2k for a kick starter scam || @andrewroy9263 $999 for just printer. $1299 with filament box || Kickstarter price anyways. || would love to see it swapping nozzles. || Soon my friend. Lol || Anybody can put a cute box on display, I'd want to see it actually printing and nozzle switching before I believed it was "amazing". || Well, it’s from a reputable company and they’re not gonna tarnish their whole brand name by putting a fake product out that doesn’t work || @stayreadyto3dprint Reputable means having a good reputation. This is their first product; they don't have a reputation yet.
-If you go to their website, you see a computer rendering of the product working, not a video of the actual product working. That suggests the product isn't running yet.  And it's a kickstarter, which means you can send your money and get nothing, not even a box of bricks. || @stayreadyto3dprint reputable my ahh first product they "made" no one has seen it working wasn't even working ces26 because of "technical difficulties"  they're going to take the kick starter money and run || Mova is a huge company. Do some homework before totally knocking them. It’s def not their first product. || So Mova is going to bankrupt their multimillion dollar company over a 3d printer scam? Got it. That makes zero sense. lol || Wow! I have not heard of this company yet. I’m impressed by the nozzle switching tech. || You and me both! || How are you impressed with the nozzle switching tech that no one has seen working or seen the machine printing at all || @Og_paine I guess we will find out whenever a demo occurs lol I am just impressed on the fact they took their ambition and produced a machine ready for CES haha
-But I get your point of view too || So you’ve never seen a concept car and thought it was cool? Or a drawing of something someone was going to build? You gotta see it working to envision the end result? It’s a cool concept is what ppl are saying. Note we wait to see if they release it as they say they are. If they don’t then you don’t lose anything. But Mova is a huge company. Highly doubt they are scamming people just for a few bucks from a printer. Think about it. How dumb that would be for a successful multi million dollar company. || Finally a video! Thanks! Does it look promising? I feel bad not backing the U1. 😢 But looking at it, the swap time will be the same as the H2C as there is only 1 tube going into the tool head. Hopefully it's worth backing. || I think it’s great for a single tool printer. But I do believe multi tool head machines are making single tool printers alot less of a viable option in 2026. Why wouldn’t someone buy a multi tool machine if they could? || @dyops  it pre-stages the next filament right upto end of the ptfe tube inside the chamber. As soon as the current filament retracts passed the pre-staged filament, the next color starts feeding. Don't think the BL machines do that. || Yeah true. || It's Alive!!! been waiting to see a floor model. ;) || Yeah it’s def real! I was a little skeptical myself tbh</t>
+          <t>Love a good visual aid! Hope you’re well Patrice! || Yeanin Leanin!💡 || 🔥🔥🔥🔥</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>_qWzooEmzBo</t>
+          <t>HRzNQQZ3998</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Walk With Me @CES 2026</t>
+          <t>Top 3 Mistakes New Entrepreneurs Make (and How to Avoid Them!)  #patricelstewart</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Check out the em smart AXI Pro laser here https://em-smart.com 
-Thanks for watching! If you're into 3D printing, whether it’s tuning your slicer settings, upgrading your Creality, Bambu Lab, or Elegoo printer, or experimenting with TPU, PLA, PETG, or custom filaments, you’ll feel right at home here.
-Join our Discord server to connect with one of the most active and supportive 3D printing communities online. We share printer mods, filament reviews, print profiles, and behind-the-scenes looks at our latest projects — plus, we run regular giveaways, offer support, and drop early news on upcoming content.
-Stay ready, stay printing — and be sure to check out our latest builds and experiments using today’s top 3D printer brands and materials.
-Join Discord here!  https://discord.gg/E5gPc8C2cs
-🌐 **Facebook Page**  
-📘 https://www.facebook.com/profile.php?id=61565872940311
-👥 **Facebook Group – “Stay Ready To 3D Print”**  
-📘 https://www.facebook.com/share/g/196GC85xxo/?mibextid=wwXIfr  
-📸 **Instagram**  
-https://www.instagram.com/@stayreadyto3dprint
-🎵 **TikTok**  
-https://www.tiktok.com/@stayreadyto3dprint
-🎁 **Patreon** – Get early access &amp; exclusive content  
-https://www.patreon.com/stayreadyfans
-📬 **Business inquiries / sponsorships**  
-Email: stayreadychat@gmail.com</t>
+          <t>Hey! This video provides crucial `entrepreneur advice` by highlighting `common mistakes in business` that often lead to new ventures struggling. It stresses the importance of a clear `vision for business` and the need for `independent thought` to avoid issues that explain `why entrepreneurs fail`. Stay informed to build a stronger foundation for your business! 😊</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-01-08T08:04:57Z</t>
+          <t>2025-12-14T01:00:22Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>414</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>62</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.048077</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+        <v>0.154589</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Very accurate and True ✊🏿✊🏿 || ❤❤❤❤</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>_8WnWYPrRS0</t>
+          <t>UPE_dDeiHDY</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New Printer or another Creality remake? Ender 3 v100 😂</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>The Spending Pattern Nobody Wants to See #patricelstewart  #moneytalk #truth</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Hey! This video offers practical `personal finance` tips, emphasizing `money management` by reviewing your bank statements line by line. This process is crucial for effective `budgeting` and can lead to significant `saving money` by increasing your `financial awareness`. Take control of your finances today! 😊</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-01-07T06:03:49Z</t>
+          <t>2025-12-13T01:15:02Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2204</t>
+          <t>253</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.01225</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>I want more video's, lol || I’m trying lmao. 😅 || Pretty cool man. Yeah, I was wanting to get a scanner. || There are better options out there for less money.</t>
-        </is>
-      </c>
+        <v>0.130435</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>kT19HFqeApc</t>
+          <t>fYJ8PQ9IN-s</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The Most Useful Thing I’ve Done All Year! #3dprinter #3dprinted</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Make Over $150K? Don’t Let These Tax Deductions Slip Away!  #patricelstewart #tax</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Hey! This video breaks down how `income tax` deductions are affected by your adjusted gross income, specifically focusing on `AGI` thresholds. It's crucial for `understanding your deductions` to navigate how these phase-outs impact your `taxable income`. This information is vital for effective `tax planning` to ensure you're well-informed about your financial picture. 😊</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-01-04T23:00:38Z</t>
+          <t>2025-12-10T02:30:39Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7460</t>
+          <t>261</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.017292</v>
+        <v>0.099617</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>I love how it looks kinda OEM next to the actual machine, Very nice 👍🏽 || Same. Thanks || what kind of pens did you use to paint? || They are the Just art from my website. Here’s a link. 
-https://www.stayreadyto3dprint.com/products/72-colors-acrylic-paint-markers-set-with-canvas-bag-dual-tips-with-brush-tip-fine-tip-no-bleed-waterproof-non-toxic-odorless-paint-pens-for-rock-egg-wood-fabric-glass-ceramic-diy?_pos=1&amp;_psq=paint&amp;_ss=e&amp;_v=1.0 || First problem is you use k cups - literally drinking hot plastic 😂 || Taste good to me lol. || What printers || Used the k2 plus and the Bambu x1c for this one. I gotta say the quality from the k2 wasn’t near as good as the x1c this time. || ​@stayreadyto3dprint oh nice i think they both came out good || Thank you !! || The carousel is 100 times better than being forced to randomly remove K-cups until you get the flavor you want. || You just add another box. They’re magnetic. I’d say you can add 3 boxes before it starts looking wild. lol. || I can’t do that awful cluttered look. That’s just me. Plus I only drink one flavor anyways. I may add one more box with another flavor for quest. || That’s significantly worse. I don’t want random flavors. Surprise pumpkin flavored coffee, or decaf, or dark roast when I want light roast would be a terrible surprise. || I loaded mine with one flavor lol. I should have showed random flavors in the video I guess. It’s confusing. If you want more flavors just add another box. They stick together. Although more than 2-3 wouldnt look very good. So if you’re a big flavor drinker this isn’t for you. I’m not. || Only now you can't choose flavor || You just add another box. They’re magnetic. I’d say you can add 3 boxes before it starts looking wild. lol. || @stayreadyto3dprint lol seems counterproductive || I like it. I hate the clutter look of the carousel. That’s just my preference. || bro i am so going to print this tonight for my K-cups, thanks || You can add boxes. They have a place for magnets on the side. But I’d say only add up to 3 or you won’t have any more counter space lol || Sweet || Thanks</t>
+          <t>❤❤❤❤</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UCXS90ukmtQo2kg3Ydf-cj3A</t>
+          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Stay Ready To 3D Print</t>
+          <t>PATRICE L. STEWART</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>vsVbjtoe-g8</t>
+          <t>x9hEVK8HWwQ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Prusa Keeps The Pressure On Competitors with THIS!</t>
+          <t>Tips Tax-Free Up to $25,000?! Avoid IRS Traps  #patricelstewart #taxdeductions</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>The 3D printing market is moving fast right now — and instead of slowing down, Prusa Research is doubling down on meaningful innovation.
-In this video, I break down Prusa’s latest move, including a major new add-on release that pushes the Prusa CORE One platform forward and keeps it competitive as other brands roll out similar ideas. Rather than chasing trends, Prusa continues to refine what actually matters: reliability, expandability, and long-term usability.
-I also share my honest thoughts on the CORE One — where it shines, where it could improve, and how it stacks up in an increasingly crowded field. This isn’t hype or brand loyalty — it’s a real discussion about innovation, pacing, and what keeps a company relevant as the industry accelerates.
-🎁 UPCOMING LIVE GIVEAWAY
-I’m also hosting a LIVE giveaway you won’t want to miss:
-🏆 Prize:
-• Uniformation GK3 Pro Resin Printer
-• 6 bottles of resin
-There will be 4 winners. 1 winner getting the printer and 3 winners getting 2 bottles of resin each!
-🗓 Date: January 10, 2026
-⏰ Time: 9:00 PM CST
-📍 Where: Live right here on my YouTube channel
-How to Enter:
-✅ You must be present live to win
-✅ You must follow Uniformation on Instagram
-https://www.instagram.com/uniformation3dprinter/
-Join our Discord for any questions aboutgiveaways you may have.
-https://mee6.xyz/i/4YMcjZjNO6
-Winners will be selected live on stream, so don’t be late.</t>
+          <t>Hey! This video explains the new `no tax on tips bill`, allowing tips up to $25,000 to be `tax free` for workers. This is great news for `uber driver` and `lyft driver`s, as it directly impacts their `self employment taxes`. Remember to keep your paperwork in order to benefit from this change! 😊</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-01-04T00:38:13Z</t>
+          <t>2025-12-10T01:31:00Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>27443</t>
+          <t>217</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.003753</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>i treyed the MK4S and it was so bad! i sendet it back to Prusa exactly like they told me and better, Prusa aproved it, after inspection the told me shiping damage, -130€ and after 11 weeks in the return progress i still wait to get my money!!! stay away from Prusa!!! || I highly doubt that. They’re one of the best companies out there. I can msg one of my reps to help you but are you sure you’re sharing the whole story here? || @stayreadyto3dprint when they are one of the best, why are they than like that? i even looked up the internet and i am not alone with this kind of support. but i have to say the are better than Nathan Stone. still waiting on my printer 1 year later :D its the Nextruder guy || great take. this is exactly why prusa still matters in the market. they’re not chasing hype features, but building solid platforms that keep evolving. real upgrades, long-term support, and stuff that actually works in practice. you can tell they’re thinking years ahead, not just the next launch || Exactly right. Couldnt agree more. || totally agree. Prusa is top tier, no doubt. The video turned out great and the printer itself is an awesome example of how far 3D printing has come. || Thank you kind sir ! 😊 || I’m personally keen on seeing how the INDX will handle TPU’s on the Core One machines.
-I’m waiting till probably the end of 2026 to either get a Snapmaker U1 or Core One with INDX (or some other brand shows up in 2026 with a new machine)
-Bambu has locked down standard rigid filaments but the H2’s were not deigned with the moving left nozzle to handle flexible cutting out multi colour options on their machines. || I’m def excited for the INDX option for the prusa machines. || Great video 😊 Clearly explained and it all makes sense 👍 You can see that Prusa focuses on honest quality and long term value 💪 That’s why people trust this brand just like I do 🚀 || Thank you. I agree. They are def invested here. They do things that let you know they are listening. And they actually have customer service. Lol || I got the K2 and I am thinking of selling it and buy the core one soon. I understand your point about using the manufacturers slicer but man is the Creality slicer a pain. Curious to know more about why you kick Creality though. For me it is that the K2 wasn't particularly precise or reliable. When it works it's great but when it's clogged it's hell. I've gone through 3 nozzles with this thing. || I can tell you it was about 20% due to machinery. The rest was due to things they did as a brand. Which I’ll be releasing a video about. || Curious to hear more on why you're kicking Creality to the curb. || same || Oh trust me. There’s a video coming soon ! You won’t wanna miss it. I’ll be revealing it all. || LOL, Prusa not putting any pressure on ANY 3D printer manufacturer.  Prusa can't make their old stuff work, let alone the new stuff.  Bondtech stepped in to try and save Josef.  If they can't get this right out of the box, Prusa will be filing for bankruptcy in 2026. || You must not own any of their machines. lol || ​@stayreadyto3dprintNot any more.  Not interested in being Josef's guinea pig cuck.  No amount of toxic gummies will get my money.  IF, when, or ever the INDX hits the consumer market and actually works out of the box, and Josef provides a gummy delete option, I will consider.  However, if the train wreck XL is $5k, what will the INDX be? Only diehard Prusa cucks will buy it. || That’s the cool thing about 3d printing. 10 different people will have 10 different opinions on what brand they like. And none of them are wrong. You gotta use the brand you enjoy most. Whatever brand that may be. These are just MY opinions and preference. That’s all. 
-What brand do you prefer? || Great video 👍 || Ty! || pretty cool stuff, glad the streams are back. oh and its 8 tools for the INDX. either way its going to be an exciting year. || I think so too!!!! Stay tuned for live footage from CES 2026 next week</t>
-        </is>
-      </c>
+        <v>0.07834099999999999</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added Emails Pending sheet to global deduplication
</commit_message>
<xml_diff>
--- a/output/master.xlsx
+++ b/output/master.xlsx
@@ -448,37 +448,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Realest Tax &amp; Business Strategist You Will Ever Meet™️
-I’m Patrice L Stewart—Experienced Entrepreneur &amp; Financial Literacy Advocate 💼
-📊 22 Years in Tax, Accounting, Banking, &amp; Finance industries.
-💡 Knowing Your Numbers is the Key to Business Success! 💡
-I teach Business Owners how to leverage tax laws and loopholes 🏛️ so you can keep more of your hard-earned money 💵 and use strategies the wealthy swear by 💎.
-My Passion: Education &amp; Coaching 🎓
-Join my Online Financial Academy—a monthly Group Coaching Program 📈
-👉 Learn More: plstewart.info/WSWTY
-🚀 Work with me or join an Event/Workshop!
-👉 Book Now: Plstewart.info/help
+          <t xml:space="preserve">**Welcome to Nutri-Tech Solutions (NTS)!** 🌱  
+We’re dedicated to **regenerative agriculture**, helping farmers, agronomists, and home gardeners grow **nutrient-dense food** while restoring soil health. Our channel offers expert insights, **workshops**, and practical training on **organic farming**, **sustainability**, and **crop nutrition**.  
+Learn from **Graeme Sait**, a global leader in **sustainable agriculture**, as he shares innovative strategies to boost yields, enhance **farm management**, and improve soil vitality. Discover practical solutions for **home gardening**, microbial inoculants, and **nutrient-dense food production**.  
+Join our community of **regenerative farmers**, engage in discussions, and stay updated with our latest insights. **Subscribe now** and take your **farming** to the next level! 🌍🌾  
 </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>27100</t>
+          <t>4640</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1294</t>
+          <t>109</t>
         </is>
       </c>
     </row>
@@ -566,47 +560,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>_jxLIKW9dQk</t>
+          <t>oMGRZunNwGM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>We told Blacks to wait your turn! After 1.2 Billion gone #chicago #cityofchicago #politics</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>Gold from the Vaults - Jerry Brunetti - Detoxifying the Rumen &amp; Building Vitality - Ep 10</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t># *Jerry Brunetti: Detoxifying the Rumen &amp; Building Vitality (Gold from the Vault)*
+We have reached the end of Series 4 of our 'How to do it' video series, and as we prepare the next instalment, we are diving into our archives to share more *Gold from the Vault* . In this session, we rejoin the legendary *Jerry Brunetti* for Part 2 of his masterclass on soil and livestock health .
+#NutritionFarming #SoilHealth #LivestockHealth #JerryBrunetti #RumenEcosystem #RegenerativeAg #GraemeSait
+In this episode, Jerry explores the massive metabolic load placed on our animals when we push for production at the expense of biology . He breaks down why high *rumen ammonia* levels (BUN and MUN) are often the precursor to *septicaemic* conditions and immune failure . From the importance of _acetic acid_ (vinegar) in the rumen to the incredible role of _Peyer's patches_ in gut immunity, Jerry connects the dots between soil minerals and the longevity of your herd . If your cows are leaving the herd at an average of 44 months, this video reveals exactly why—and how to fix it .
+*What you'll learn in this episode:*
+🥬 The "energy deficit" trap: Why cranking up cereal starch creates dangerous _D-lactic acid_ .
+🧬 _Manureology_ Revisited: Using your nose to detect metabolic imbalance and *butyric acid* issues .
+💩 The *Ensiling* Secret: Why adding _molasses_ or lactose to your silage creates the perfect microbial fuel .
+📈 The 14% Rule: Why cellulolytic bacteria die off rapidly when rumen pH drops below 6.5 .
+🧪 Gut Integrity: How damaged _villi_ lead to *dysbiosis* and the infiltration of pathogens .
+🐄 Liver Longevity: Understanding how the liver regenerates and why its failure is the final symptom, not the cause .
+👇 *Chapters:*
+00:00 - Introduction - Ammonia &amp; Rumen Issues
+01:33 - Title Sequence
+01:57 - Rumen Acid Production &amp; pH Balancing
+03:53 - Plant Maturity &amp; Forage Quality
+06:17 - Silage Quality, Fortification &amp; Microbe Foods
+09:48 - Growing High Quality Fodder
+11:59 - Balancing Rumen pH
+17:21 - Milk &amp; Pasture Analysis - Refractometer &amp; Brix
+21:30 - Lower Gut Health, Issues &amp; Probiotics
+30:51 - End Credits
+Want to learn more about Nutrition Farming? Check out Graeme's How to do it episode *Getting Started with Nutrition Farming® – 10 Practical Steps to Transform Your Soil and Crop Health - Part 2* …
+https://blog.nutri-tech.com.au/getting-started-with-nutrition-farming-r-10-practical-steps-to-transform-your-soil-and-crop-health-part-2/
+*Nutri-Life BAM™*
+https://nutri-tech.com.au/products/nutri-life-bam
+*Nutri-Gyp™ Natural Gypsum*
+https://nutri-tech.com.au/products/nutri-gyp
+*Sili-Cal (B)™*
+https://nutri-tech.com.au/products/sili-cal-b
+…or try our new NTS FulvX™ Powder for chelation
+https://nutri-tech.com.au/products/nts-fulvx-powder
+*Interested in attending a Certificate in Nutrition Farming course?*
+https://nutri-tech.com.au/pages/courses
+Need assistance? Try out our Soil &amp; Plant Therapy Services
+https://nutri-tech.com.au/pages/soil-plant-therapy
+How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait
+Head to our website to find out more
+https://nutri-tech.com.au/
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+*Follow us on Social Media*
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+Twitter: https://x.com/ntsaustralia</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-01-30T07:07:28Z</t>
+          <t>2026-03-13T05:38:47Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1457</t>
+          <t>490</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.055594</v>
+        <v>0.02449</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -615,59 +659,104 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>I don't blame the migrants for coming here. We left a trail for them to come. I don't hate on my immigrants. My parents are immigrants to this country. I'm a first generation American. I don't hate on any of these people who came here. They had no choice. But we left a trail for them to come. We gave them over a billion dollars to come here. We invited them with free food, free clothing, free rent, free education. &gt;&gt; That's why we're here today. Yeah, &gt;&gt; we can keep talking about whatever head tax and gambling is bad and all this other stuff. We made the gamble. &gt;&gt; We gambled on the migrants and we lost. We put over a billion dollars into into people who've never paid a nickel into the system. &gt;&gt; Meanwhile, Meanwhile, we told the black community, "Wait your turn. [screaming] &gt;&gt; Wait your turn. Yes. &gt;&gt; Sergeant at arms. Sergeant at arms.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Yes a billion dollars...and they STOLE 19 BILLION. || Frfr makes no sense but to cause division still today they are making new free programs for migrants but still no reparation… but black ppl protesting in the streets… I don’t know what to say 😑😑😑 || The left destroys everything they live in a bs reality ! || For President ! || Nobody remembers when everybody was erupting in city hall about them putting migrant hotels in black neighborhoods during Biden. If they could fix it with the migrants, they could of fixed it with the blacks for the last 20 years. || Enjoy the race to the bottom. Instead of solidarity with immigrants, you want to sew division. They're coming for you too you degenerate || And there they go trying to turn us on each other coming from a klan man sounds amazing..never paid a nickel he dosnt know his facts at all do the math and add up how much immigrant paid into the system actual FACTS BILLIONS,  BLACKS HAVE BEEN HERE WAY BEFORE IMMIGRANTS OR DO YOU FORGET "SLAVERY" OR IS THAT NOT IMPORTANT BECAUSE U GUYS ARE TRYING TO ERASE THERE HISTORY.  WHAT A LOOSER || Vote them suckers out! || 0:19 they had no choice to come here? || Ain't that a blip...smh... || I sincerely hope we get pritzker out in 2026 &amp; johnson out in 2027 &amp; most of these liberal Chicago aldermen</t>
-        </is>
-      </c>
+          <t>Um so anyway this blood ammonia levels you start now getting neemic animals you start growing pathogens you lower the immune system. So now we got this high mun bun rin pneumonia issue. The nutritionist comes along, sees your cows look like crap. You're not milking worth the hoot. You know, you've got poor condition. You're not getting cows bred back. And he says, or vet says, you got to put some condition on these animals. These cows have got to have some energy. You got an energy deficit in this herd. All right. So what do you do? He's going to crank up the thermostat and he's going to recommend that you crank up the cereal. So now we come in with another weird substance called starch. Well, here's something that's interesting. If you can see this thing says acetic acid over here. Star starch when it fermentss in the room and produces this thing called dactic acid. When you ferment sugars packed into cellulose, hemiselulose, you produce acetic acid. What's the difference? What is another word for acetic acid? Anybody hear of vinegar? Anybody ever know of your predecessors or some of the old time farmers that used to feed cows vinegar? &gt;&gt; Still do. &gt;&gt; Still do. That's why you feed cows vinegar because they make it. A healthy rin makes vinegar. I'm going to go give you another slide here in a second. [music] &gt;&gt; [music] &gt;&gt; That's what an acetic acid is. And so you get here is another oxymoron. is sort of like the the pH of the urine being high showing acidosis because you don't have any minerals to buffer, so you're using ammonia. How could acetic acid be a good thing for concern about acidosis? Acetic acid has onetenth the acidity that lactic acid has. So an animal that's loaded with lactic acid could actually be buffered by vinegar. The same is true with people who take vinegar to deal with their own acidosis and they get a response. Why? Because the acid that they're neutralizing with the acetic acid is these fermentation acids from eating a lot of sugar and carbohydrates causing all this other acid. So people who take vinegar, the apple cider vinegar with the mother especially in it, &gt;&gt; you'll get better. You'll start feeling alkalized. It's not because of the acid. It's because you've actually alkalized the really really noxious acids with the vinegar. So it's a relative issue. Okay. So anyway, now what you see here is the room pH. See on the top ideal room pH 6.5 to to 7. We got this ammonia thing running rampant because we have poor quality forage. And I can tell you this much unless it's really mature forage. If you've got really high protein forages, chances are they're low in energy. And the converse is usually true. If you have really low energy forages, and I mean energy the way I define it, not necessarily the way the conventional wisdom defines it. You're usually high in NPN. uh coming in forage or pasture or or or serial crops is uh is there a specific time you're sort of talking about of maturity of that plant maturity of the plant of the forage? It depends on how you grow it. We'll talk a little bit about that. But I mean the problem you have growing or harvesting early forges obviously is you got high levels of protein and low effective fiber when it's really young and lush. Now that being said that's always true with conventionally raised forages. And what we find out is if you let those forages just get a little older, if you're doing the right kinds of soil things, you will get the energy and the protein is a better quality protein. So I'm not so worried about the quantity of the nitrogen. I'm concerned about getting amino acid quality protein. Even if it's less, like the dairyman from Washington State, the quality is less. I mean, the quantity is less, [snorts] the quality is higher, and I got more pectants in there. And when you start getting that th that that gap starts to narrow come together where the protein quality and the and the energy quality start running side by side. Now you're not wasting all that energy to get rid of this stuff because what happened here see this this farmer in Washington state. What happened there was because this liver and the kidney and all this stuff was working so hard to get rid of all this ammonia. It was consuming energy out of the cow to get rid of the ammonia. That's why the cows came up in milk after he fed them a poor quality forage because he wasn't poisoning the cows with ammonia and the animals detoxification and elimination organs didn't have to consume energy to get rid of that which he paid for twice. It's pretty logical. You know, the cows are telling you are telling you this stuff and you can smell the ammonia. You don't need a high-tech laboratory to figure out what the hell's going on with a cow. Look at her, smell it. You go into a barn in Pennsylvania this time of the year and I can tell the herds that are getting this right. The ones that are feeding conventionally, the ammonia levels are overwhelming. And that's what's going on. And it's not because of ventilation. It's not because of ventilation. Does that is that refer exactly the same to to the hay all the toes are made. Was that was that u work on your nose is to say the quality of the h? Yes. I mean not to tell everything by your nose but one of the things you use you smell and you s and silage is another good thing. S and soiled hays and forages should have kind of a sweet pickled smell to them. They should not have that butyric acid smell, that really heavy acid smell that when it gets on your clothes, you can't get it off. You know what I'm talking about? That's butyric acid. You don't want that. And you don't want that real real uh vinegary smell either, which is uh you don't want acetic acid production in the silages. You want different kinds of acid productions in the silage. And one of the best ways to do that, and as long as we're talking about that, let's let's so easy to not talk about so many things. There's so much to talk about. So you brought it up and we'll go there right now. When you insile forages, always remember that you're going to take true proteins and break them down into more of these compounds. That's one of the downsides of making hay into silages is that you tend to compromise protein quality because the insulin process, the fermentation process of ensulin tends to break down these proteins and makes more simpler nitrogen compounds. One of the reasons why I like to throw molasses on palage so that I can give the fermentation organisms a lot of sugar to go crazy and cool that thing down really quickly so that we don't get a lot of heat damage and we don't get a lot of fermentation damage. So we throw molasses on that, not a [clears throat] lot. And what that does is that the molasses gives the microbes that are on the leaf surface called the phyosphere. And these are lactic acid organisms that are naturally occurring there and especially yeast organisms. If you really want to kick up the volume, you could throw milk sugar on there. Lactose. Milk sugar is a great thing to throw on silages. That gives you a very fast response because lactose is converted to lactic acid. Now, here's that bad word again, lactic acid. Well, you have lactic acid and you have dlactic acid. Dactic acid is what's going on in the rin, which is killing the rin. Lactic acid is what goes on in fermentation, like when you make sauerkraut and good silage. And also the kind of elactic acid that you find in the small intestine to keep your villi healthy. &gt;&gt; Is this what the inoculates do that we use alongside? &gt;&gt; The inoculants inoculate. They just basically introduce microbes there. But keep in mind microbes need food. So I'm more concerned about the microbes are on I mean I'm not saying not use but to me it's more critical to provide food for the microbes as opposed to putting microbes on silage that has no [clears throat] food. It's like, isn't it more important to try to create a soil that is conducive to earthworms as opposed to inoculating soil that's not doing very well with earthworms? You don't have to inoculate soil with earthworms. You can speed it up with inoculants. You can they some there's some good inoculants out there that still will make an improvement even in addition to adding the fuel that those microbes want to eat. Jerry, if you're growing the herbage in the right soil conditions and harvest at the correct time, can it not produce enough sufficient sugars to do the job? &gt;&gt; Yep. &gt;&gt; So, we're only using bands really, aren't we? &gt;&gt; Yeah. The molasses forages tend to be, you know, obviously compared to grains which have lots of starch and that's another thing you could throw on for you can throw a little starch uh ground up cornmeal. Uh you could throw ground up uh wheat flour on on the on the forages, molasses. What you're trying to do is just give the bugs, you know, an opportunity to really grow well quickly and then get the pH down quickly so that it's cooling off. You don't want to get any heat in that in that bunker and you don't want to get any heat in that bag. And it really does work. I mean, but you're right. uh as the soil starts to increase, as the minerals start to come up in the forages, the pectins and the sugars are naturally produced. Now, sometimes the problem you have is if you're making hay and it's really hot, the plant to protect itself from uh evaporation, transpiration stress will convert more of its uh carbon to make lignen instead of making sugars and pectins because it's trying to save itself from dehydration. So you end up getting more ligant produced and typically that's when you hear the complaints about butter fat test getting low is that you they'll get into the hay mau everybody will complain around the same time because they're all starting to feed third cutting hay you know when it was made in early August you know or second cutting hay when it was made in July or something like that and they'll call and say my butterf is crashing and what's happened is they they're getting into hay that was cut when it was really really hot for a number of days and when that's really hot there's more lignen produced and lignen of course is not fermentable. Now there is one way around the ligman issue or one one help to that is having adequate levels of sulfur in the forge helps to break down lignon more efficiently in the rin. There we are. There's another reason why fertilize with sulfur. See the knee bone is connected to the shin bone. So anyway, I'm just going to go on to this next slide here and see if this Okay. Yeah, this is a good slide for you to finish up with. This is the lactic acid curve and the acetic acid curve all in one. You can see that top line, that's acetic acid. That's your vinegar. Okay, here's your pHes. 7 656 555. All right, look what's going on here. You see what's going on is this is that as the pH starts to drop, and what causes the pH to drop? Starch. Starch causes the pH to drop. As the pH starts to drop, the cellulitic flora which produce acetic acids start to decrease. As they start to decrease, obviously their byproduct, which is acetic acid, starts to wing. And you can see as you get down to the five range, it disappears. Meanwhile, propriionic acid starts to climb. And when you get at six, there's the evil one that shows up. It starts killing the room, lactic acid. And here's the issue. Uh, Professor Richard Zinn at the University of California has said when you get below 65 pH in the rin, every tenth of a point that you drop below 65 in the rin, you start losing these cellulitic bacteria at the rate of 14% an hour. That's a tremendous statistic. 14% an hour below 65. That's why 65 to 7 is your pH range. And that's what you find in the old text. These animals had healthy rumins. You have a healthy room in there, you got longevity in cows. You go to this next range. This next slide is University of Wisconsin slide. Wait a minute. That's fact again. I don't know if that's on there or not. It's not on there. Anyway, there's a there's a slide that I have that shows a 24-hour feeding of a TMR, not a slug feeding, TMR, and it shows every time the cows ate, how the phes of the rin dropped, okay? Up and down, up and down. Well, I looked on that whole graph for 24 hours. I found out in that TMR ration on that Wisconsin herd, 19 out of the 24 hours, the pH was below six. There's no way you can keep a herd around for a long period of time with 19 out of 24 hours of pH below 6. That herd is kaput. There's no way that cow can stand in. So this is what we're trying to emphasize. This is this is the information coming out of the people that know about this stuff, but the feed industry hasn't accommodated to it because the feed industry is not interested in what? Soils. That's why the feed industry is not interested in soils. And I ran into this over there at at Shepherd and I was talking to one guy who's in this neck of the woods and his name is Angelo someone. I can't remember his last name. More paison I see over here than I saw anywhere else in Australia. I don't know why that's the case, but anyway, he said he was Dutch. I didn't believe him, but he told me um a name like Angela, you anyway, his family was born in Holland or some some story. Anyway, he has a dairy herd over here and he said to me, he heard some of this talk. I did an abbreviated version of this over there and he said, "Yeah, I think you're right." He said because some of the herds that I'm working with have got calcium levels and I'll go into this in a little bit here show you how the minerals reflect all this calcium levels on these forages are down to.3 and point4% when we know in order to make energy in a forage you've got to have calcium levels at 1.5 on up. And when you get 1.5% calcium you make energy. And when you get sulfur levels where they're supposed to meet, you make protein. And when you have trace minerals like boron at 40 parts per million, you make energy. So if this is a bunch of bunk that you can't make energy in forages, is that nobody knows what the soil is supposed to do because nobody even cares about the soil. The feed nutritionist basically starts balancing the ration from the point of where the the forage samples show up in front of his computer. And then it's like, well, you know, you can't take bad forage and bandaid it into good forage. You can't do it. You've already lost the window of opportunity to to create that that kind of an ecosystem optimized ecosystem arrangement for that cow to produce milk or meat on low feed costs. Okay. Uh, moving on. So, is everybody with me on this lactic acid curve? You understand why this is got to be in this range and how it's so hard in conventional agriculture to keep it here? Because if you've got these low energy forages and you want to make milk or you want to produce meat on an animal, the only recourse left is grain. That's it. You know, it's either that or you don't have milk, you don't have meat. So that's it's sort of like this you know horns of the lemon. So ultimately if we want to have a room pH here we have to be able to figure out how to produce energy in a forage and that's a soils issue. So &gt;&gt; is bricks test any use at all in testing milk in this sense or not really relevant to &gt;&gt; well the brick yeah well not so much you could use a bricks test to measure solids in milk. I don't use it so much for that. Bricks test, a bricks refratoter. For those of you who don't know who that that is, it's it's a it's a device that measures basically total suspended solids which of which sugars are part of that. They use it in the molasses industry and the honey industry, the antifreeze industry. Um anyway, that this bricks refratoter, a lot of people use that out in the field and it is it is a relative interesting tool. Um, and I'll just go there for a couple minutes because I think a lot of people have some misconceptions about what a refratoter can do for you. Uh, since it is measuring sugar, you'll typically find out that it's a relative any grass if if you let it uh go to the end of the day late in the afternoon before you cut it, you'll find out that your bricks levels simply because of sunshine creating sugar through photosynthesis, the levels of sugar are high. So now if you take the same grass and measure it that way, you'll find out that the bricks levels are consistently high. Now University of Idaho did this research in terms of recommending to dairy farmers in Idaho that if you're going to make hay and this is Holene herds and you're going to cut your alpha alpha, cut it later in the day and you can possibly generate 7 lbs milk per cow per day extra merely by increasing the sugar levels in the hay just by time of cutting. Now that being said is that what you're measuring is the product of photosynthesis which is the production of sugar and all plants do produce sugar. The question is can we increase in that same field the amount of sugar that that plant can produce based on soil fertility and the answer is yes you can and that's what we want to do. So time of day, if you took, for example, if you measured a really biologically tended field early in the morning and took a not so biologically tended field maybe late in the afternoon, you might find that the bricks levels don't show any difference or maybe even the conventional field shows a slight advantage. So it's not a real fair comparison. You got to measure the same time of the day and you got to measure, you know, the same types of, for example, 3 days of rain, for example, 3 days of cloudy weather. those bricks are going to be down and it's going to take a whole another day, day and a half for those bricks to come back up. So, you have to keep that in mind that sunlight, you know, is the primary governor of the bricks levels in a plant. Soil nutrition factors into that, but all the soil nutrition in the world done the right way with 3 days of rain is not going to show you a true reflection of what you've done on that farm. So, it's a reflective tool. Keep that in mind cuz I've got farmers come back saying, "Well, you know, I've tested this field and it was after 3 days of rain and their bricks levels are low and they don't understand why they're not up to 14." It was because it rained. The sun doesn't uh help you out if it's not there. So anyway, so that's to answer your question on that. I'm glad you brought that up and please uh this is this is good stuff because when you bring up these questions, it's really easy to lose drop these these &gt;&gt; marles away. But just one other point in Ardan Anderson's reports he he claims 20 bricks is ideal for milk. I've done a lot of milks around and can &gt;&gt; Yeah, you're talking about the actual and what you're measuring in the milk are because milk is loaded with sugar. &gt;&gt; Okay. And solids. Lots of solids in good milk. And you're right, the the poor quality the milk, the lower the bricks. And if you can get bricks levels in milk like around 20 that tells you that you know those cows are getting nutrient density that's manifesting itself in the milk. That's correct. Right. And and you get some cows that are below 10. Also the phes are even acidic and some not acidic but relatively acidic to other biologically produced milks because what really alkalizes again are the minerals that milk is notoriously rich in calcium, magnesium and potassium. you know, and the fats, the fats are very alkalizing, and that's a whole another thing that people got to understand is that fat is really good for you. So, anyway, we've we've left the rin and now we're down in the lower gut. And so, when you've got this rin that's not functioning properly, now that's an aven intestine for the sake of the slide, but you can see what happened here. You know, perforation of the intestine. And what does that [clears throat] really mean? But when you look at what the villi, the villi are these finger-like projections that stick out of the tube called the small intestine. Obviously, it's there for surface area. It tremendously increases surface area. But maybe the most significant thing about this slide to me is the fact that this is such a a a major demonstration of what a vascular system that the gut is. And you can see the artery goes up here and then it diffuses back into the venus supply. Tremendous exchange going on here of absorption. So when you end up with this kind of a system, a vascular system that's like this, that's very important that this gut stays intact because this gut not only is a site for absorption of necessary nutrients that the blood supply now has to get, but it's also extremely important uh part of the immune system. There's an organ called pyr patches that are located in the villi of the small intestine. So your gut is extremely important to have a healthy immune system. The animal's gut is extremely important. The integrity of the gut is second to none in terms of importance to immunity. And so when you see this starting to go south because of what started in the rin when you start having an unhealthy rin believe me I can tell you that this is what you're looking at is a is a foul gut and absorption of nutrients starts to decrease and the infiltration of pathogens starts to increase. In human medicine we call this disbiosis. And I can tell you right here, right now, if you want to deal with getting well, you've got to correct dispiosis. And most people have some extent of dispiosis or not. In the United States, something like 75 or 80 million Americans are estimated to have candida yeast infections. That's a lot of people and they grow in the villi quite effectively when the acid alkaline balance is all out of whack and then you start feeding the wrong kinds of foods that foster the growth of yeast. And you know, I cut my teeth um in effect tutoring under a real maverick veterinarian in the late '7s by the name of John Whitaker. John Whitaker was a guy that um opened my eyes about blood ura nitrogen levels. He used to write for Acres USA years ago and he was a feed lot specialist actually. He learned about all this stuff from dealing with conventional operations in chickens and feed lots, beef feed lots and dairy feed lots. And the things that I learned from John about he about bun acidosis and the other thing is mcotoxicosis or mold poisoning. See that's the other problem with starch. Starches are great substrates for yeast and mold. And that's why we've got so much yeast infection with people is because we eat so much refined carbohydrate which is the perfect fuel for these pathogens. And animals have it too. So if you get this acid alkaline gut situation really compromised then then on top of everything else you get micotoxins in the the silages or in the stored grains and now you've got these things that are growing amongst the villi just like mold growing on a plant and they're feeding off the blood supply of that animal like a parasite and they're also producing tremendous quantities of micotoxic compounds u which we call micotoxins or um specific Specific names are like aphletox and that's just for one particular mold called aspiggillis flavus but there's a lot of other ones fuceriums and it's a huge huge problem anymore didn't used to be and we feel the main reason why it's a problem is twofold um the problems in the soils we've used a lot of biocides when we start destroying the uh the native flora like the microisy which protect the plant root and I got a slide I think in here somewhere but the the plant root is very much like the root hair is very much like the villi of the small intestine. This villi is coated with lactic acid organisms. They that's their habitat. And when things are right up here in the upper gut, they're right down here in the lower gut. And that villi is coated with these lactic acid organisms which produce really good antibiotic substances like nycin which by the way the pharmaceutical companies are synthesizing to make for an intramary infusion. Nyin produced by bugs, acetyloline, uh lacto peroxidase, uh lactic acid, hydrogen peroxide. These bugs produce tremendous quantities of pathogen growth inhibitors. So that's why fermented foods and humans are so important because it's loaded with all these bugs and all the things that these bugs produce which not only give you the benefits directly but they stimulate your indigenous flora or the animals indigenous flora to keep producing lots more of them. It's a different ecosystem down here than the rin completely different ecosystem but a fantastic one and it's all intact. It's just that's what's amazing about this system. And then you look at this slide here. This is a great slide. Look at the difference of the damaged villi versus the undamaged villi. You see what's going on here? And this could be a human, this could be a cow, this could be, you know, any kind of animal. But when you start getting damages from these toxic overloads from from what starts up in the upper gut, this is what happens. Your surface area decreases. You start getting scar tissue in here. So absorption of a nutrient starts to go down. Feed efficiency starts to drop. Immune systems start to get compromised. Look at the bloom over here on these villi. What a healthy gut looks like. So this is what we want to see in these animals is a gut that looks like that. And that's all starting with, you know, I keep saying it's a soil st. And then ultimately after the liver starts putting up with this crap for, you know, days, weeks, months, you know, [clears throat] you end up with livers that look like that. And I'll guarantee you if you got call cows and you call those cows out for either high sematic cell count or laminitis or reproductive failure, I don't care what it is, you autopsy that cow and I'll guarantee you 95 to 100% of those cows that look like that. what you saw in terms of laminitis or reproductive failure or chronic sematic cell count issues or whatever you saw basically the symptoms of the internal organs finally getting exhausted of having to [clears throat] deal with all this burden that we've been putting on that animal. And so eventually the liver becomes imploded with fat because it can't it can't work anymore. And then you ultimately call animals out. They drop dead sometimes right on site. they just poof, they're gone. Cuz when that shuts down, and what's amazing about the liver, it's so incredibly forgiving. It's one of the few organs that can practically regenerate itself after being almost annihilated. It can regenerate. So, when you've finally done that much damage, and like I said, that slide that I didn't have, but I talked about, it showed 19 out of the 24 hours on the TMR where the spike was like this. And 19 of those 24 hours was under the threshold of 6.0 pH. That's what you get. That's why you call the cows out. That's why they're 44 months of age average calling. That's why it can't happen. And when you think about the cost of cows, you know, it just blows my mind that the feed industry is still trying to find ways to buffer a cow. So, what do you buffer a cow? What do you buffer cows with? Baking soda, right? Okay. Think about this statistic. A cow that's making 60 pounds of milk a day needs to chew her cud 11 hours. It's a lot of cud chewing time, right? In that 11 hours, that cow will produce 3540 gallons of saliva. That's a hell of a large spatoon. 35 to 40 gallons of saliva. And that's equivalent to basically four to five pounds of bicarbonate. &gt;&gt; How much bicarbonate can you feed a cow? Maybe a pound if your sodium levels are allowable for that. Maybe a pound. So what happens to the rest of it? You just can't buffer the cow. So you know and you know and and then the problem you have is this dilemas where you're trying to say okay trying to get this guy to feed some long quality effective fiber hay or even straw, you know, but then that cuts into what? Production. How much are heers going for over here? &gt;&gt; What a replacement heers sell for over here? &gt;&gt; About 1200. &gt;&gt; Anywhere from 900 to,400. Yeah, about the same in the states. So, I don't understand that economics system. I mean, I don't understand how he prices are hanging in there for the last decade around that. They fluctuate like this. Milk prices are like this, you know. Coal cow prices are like this, you know. Heat. [music] [music] [music] Hey, Heat.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>hi9MmOTlWGo</t>
+          <t>yCrAg9vRp2E</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Are you really in business? #business #taxdeductions #taxes #credit #cashflow #income #entrepreneur</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>Gold from the Vaults - Jerry Brunetti - Soil &amp; Livestock Health - The Rumen is an Ecosystem - Ep 9</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>We’ve reached the end of Series 4 of our 'How to do it' video series, so while we prepare the next instalment, we are diving into the archives to share some classic *Gold from the Vault* content. In this session, we revisit the late, great Jerry Brunetti and his profound insights into the inseparable link between soil fertility and animal wellness.
+Jerry Brunetti was a true pioneer who understood that you cannot treat a cow in isolation from the ground she walks upon. In this first part of his legendary presentation, Jerry breaks down the "reductionist" trap of modern agriculture and medicine, explaining why a high-protein diet might actually be poisoning your herd. From "manureology" to the intricacies of the rumen ecosystem, this is a must-watch for any farmer looking to transition from disease management to true wellness care.
+#NutritionFarming #SoilHealth #LivestockHealth #RegenerativeAg #JerryBrunetti #EcoAgriculture #AnimalWellness
+*What you’ll learn in this episode:*
+🥬 Why the *pharmacies* of the future will actually be *farms* .
+🧬 The "funny protein" trap: How high crude protein can lead to ammonia toxicity.
+💩 The science of *manureology* : What a colander and a jet stream can tell you about your herd's health.
+📈 The historical connection between glacial soils and the robust health of the early pioneers.
+🧪 Understanding the *microbial bridge* and the rumen as a fermentation ecosystem.
+👇 *Chapters:*
+00:00 - Soils &amp; Livestock Introduction
+01:39 - Title Sequence
+02:08 - Soil and Stock Health
+05:06 - The current state of play
+07:57 - Milk? Commodity or Medicine?
+10:47 - Dr William Albrect
+11:45 - Fertility: The Great Plains &amp; 40 Million Bison
+13:29 - Herd Health Begins with Digestion
+17:01 - pH &amp; Acidosis
+20:42 - The Rumen as an Ecosystem
+33:57 - End Credits
+Want to learn more about Nutrition Farming? Check out Graeme's How to do it episode *Getting Started with Nutrition Farming® – 10 Practical Steps to Transform Your Soil and Crop Health - Part 2* …
+https://blog.nutri-tech.com.au/getting-started-with-nutrition-farming-r-10-practical-steps-to-transform-your-soil-and-crop-health-part-2/
+*Nutri-Life BAM™*
+https://nutri-tech.com.au/products/nutri-life-bam
+*Nutri-Gyp™ Natural Gypsum*
+https://nutri-tech.com.au/products/nutri-gyp
+*Sili-Cal (B)™*
+https://nutri-tech.com.au/products/sili-cal-b
+…or try our new NTS FulvX™ Powder for chelation
+https://nutri-tech.com.au/products/nts-fulvx-powder
+*Interested in attending a Certificate in Nutrition Farming course?*
+https://nutri-tech.com.au/pages/courses
+Need assistance? Try out our Soil &amp; Plant Therapy Services
+https://nutri-tech.com.au/pages/soil-plant-therapy
+How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait
+Head to our website to find out more
+https://nutri-tech.com.au/
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+*Follow us on Social Media*
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+Twitter: https://x.com/ntsaustralia</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-01-12T19:11:29Z</t>
+          <t>2026-03-06T08:05:39Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>756</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.053266</v>
+        <v>0.034392</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -676,59 +765,117 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Many of you all think just because you are a business or you're a sole proprietor that you don't have to have paperwork and that's not true. You should still have a profit and loss statement that you are providing to us. Every business, if you are a real legitimate business, you should know your numbers and you should have a profit and loss statement at minimum that you are providing to us as well as a balance sheet as well as bank statements to show your transactions. When you are an LLC or a corporation, we are required to get that [music] information from you. Real tax professionals are like myself, someone who was registered as an IRS efile agent. All right? I have a EIN number. I can electronically file your taxes for the last 3 years. So, there are certain documentation and paperwork that the IRS requires me to get from you being a legal legitimate business. All right. Patrice L. Stewart here, the realist tax and business strategist. Follow my page and channel for more tax, credit, and business tips.</t>
+          <t>Well, anyway, um we're going to cover a lot of topics. We're going to cover soils. We're going to cover animal health. We're going to cover soil um forage density. And what I hope to um convey to you folks is that um animal health really I mean often times I get asked to speak on just animal health and uh what typically happens when I do that is I end up starting talking about soils which probably gets people's eyes to get blurry. we're talking about souls for when you really want to know how to treat mastitis or you really want to know how to treat calf scour or ketosis and I will cover those things but I I can't emphasize enough being in this work for nearly three decades now working with all kinds of of farmers from uh mostly which we have as Amish farmers in Pennsylvania um we are a fairly busy dairy state um in Lancaster County alone we are the second largest dairy producing county in the United States only behind county which is a feed lot type of dairy operation in California. We have 2200 dairies in Lancaster County that average about 60 cows. So it's a very busy place with a lot of farms and that's the way we like it. We think we don't care really whether farms are large or small. We like to see lots of farmers. We like to see lots of farms run by families. And so we get a whole variety of challenges because we have a whole variety of soils, whole variety of management issues. But ultimately we try to sew it all together by saying you know certain fundamentals you just can't deviate very far from and um really it becomes as I get older and older which is happening faster and faster um I realize that um the fundamentals really are much much simpler than you really would realize [music] &gt;&gt; [music] &gt;&gt; It's not necessarily something we don't have any magic bullets, but we do see mirrors. Um, and I saw those back in the days when I knew a lot less than I did now. And ultimately, we try to reconcile this thing by bringing on bringing it on home and recognizing that real stock health starts with soil fertility. And I'm going to show you some slides of Malibar Farms, which is a an incredible success story that happened in the 40s and 50s in the United States by Louis Broomfield, who was one of my heroes when I started getting into agriculture in the late 60s and early 70s. He was a Puler surprisewinning author that restored a completely blown out piece of of property in Knox County, Hill Country of Ohio, 1,000 acres of gullied land into into farmland that brought back 15 springs that were exhausted from drought and brought them back so that they could actually use them again for drought. Stories like this are really exciting to me because it's already been done. I'll talk a little bit about Randlay Farms, which was the top herd in in uh in the world for Jersey cows out of New York State by William Keenan. Talk a little bit about Carnation Dairy, which was the top herd in the world, bar none, back in Washington State in the ' 50s, 40s, and 30s. So, those are my teachers. Um, you know, I I think it's a back to the future kind of thing. And that's the great news that we don't have to re relearn all this stuff. It's already been done for us by guys like William Alrech and Dr. Royal Lee and uh uh Dr. Harvey who started the US public health service. I mean there were some tremendous uh farming and health giants that existed back in the early part of the century and there's tons of information that we now can draw upon and put into use. And um I'm fortunate in that I cut my teeth with not just those kinds of people who have since gone on before us but their um proteges. I had learned from them and turn taught people like me so that the torch can be carried on. So anyway, let's uh let's move on with this talk and I always like to bring this quote in there by Fat Sean. that which is lacking in the present world is profound knowledge of the nature of things. And I think that's kind of a really a mantra for me anymore that we recognize that there's this the things that we treat try to understand in a reductionist sense. You know, if you start taking things apart, you take things apart, you take things apart and it's a whole saying of what a specialist is. He he constantly specializes the point there's no consilience between the specialties. You know, you see this particularly in medicine. you know, you talk to specialists that are neurosurgeons that aren't talking to other specialists in the hospital. And as a consequence, there's a great deal of of disease management instead of wellness care. And the same is true on farms. We have aronomists that don't know anything about how a rumin works. And we have dairy nutritionists that don't know how uh the soil food web and soil fertility issues are are are really important to produce the kinds of rubin foods and fuels and proteins that we have to have in order to have sustainable herds. In the United States, our dairy herd populations are lasting 44 months before they're all called out. That's the average age of a dairy cow before they call them out in the United States. 44 months. So, that's not even three lactations. Not even two lactations. So, what's going on here? Is this really is this really progress? You know, I just came from the Sheperton um uh festival over there, which was a conventional uh dairy festival and and uh I should say conference, not festival, but um you know, you hear the same thing as the conventional things all the time, which is how do we become more efficient? How do we get bigger? Um and I feel that I don't size is not the issue in the United States. Cornell University out of New York State has now made the prediction as of recently that we have 105,000 dairy farms left in the United States. In 1960 we had 2 million dairy farms in the United States. So we've lost 95% of that which was in 1960. So the [clears throat] get bigger get out sort of um axiom was followed was it? So now they're saying from here on in from 19 or should 2004 until 2020 which is a mere 16 years away. Thank you. We're talking about going from 105,000 dairy farms down to 16,000. The entire United States, 16,000 dairies. And they're saying that those farms that are milking less than 100 cows will dwindle from 84,000 down to 7,000. And those that are milking more than 500 cows will increase from 2,700 to 3,400. So is this Yeah. &gt;&gt; Okay. For Congress, Jerry? &gt;&gt; Yes. &gt;&gt; Yeah. Yeah, we're going through the same destruction process here, but it's a distorted economic system that's driving it, isn't it? &gt;&gt; Exactly. Yeah. It's all And if it wasn't for Well, and the thing about it is our ancestors uh put the dairy belt together, United States where in the northeastern and upper Midwestern states, the cool season grass areas where you got natural rainfall u and cows did well there without a lot of input. And the new dairy industries are moving into the western states basically relying on commodity purchases which are subsidized by farm bill policies that cause farmers to grow cheap corn, cheap soybeans and run it through feed lot kinds of operations. My feeling about this is is okay I can't do anything about that. I know that. I mean I I realize that the genie's out of the bottom. So in Pennsylvania where we have Amish Menite family farms are not going to get to be 500 cow herds because they can't even if they wanted to. They're just not designed for that. They have 80 acres, you know. So we've got already too many animals from that land producing way too much pot ash and phosphate on the ground. It's ending up in the estuary called the Chesapeake Bay. So what are we going to do? Well, we're trying to take a whole new angle of this thing and say, okay, what is really the cost of production all about? and who's our market and what really is milk. I'm going to talk about that tonight. What is milk? Should it be a commodity or should it be a medicinal substance? And and I'll talk about this medicinal substance factor because in my opinion, being a recovering um individual from a life-threatening illness, I know firsthand that food is medicine and it ought to be medicine. And if it's not medicine, then it's killing you. Either food is healing you or it's killing you. That's the way I look at it. There's no in between. either you're pregnant or you're not pregnant. You know, it's one of those kind of deals. So, either you're getting well or you're getting worse. And uh and I had a window closing on me said either get well or die in 6 months. So, I know that food either heals you or it doesn't. And if [clears throat] it's not healing you, it's not neutral. It's either contributing to health. And that's what to me this is all about. These meetings in in in Australia or these meetings in Pennsylvania are about the future of not just farming but the future of mankind because the farming of the future is going to be about the fact that the pharmacies of the future are going to be farms. And I'll guarantee that's a prophecy that I'd make up. But you can go to the bank with it because in my country, and I guess it's true here, the baby boom generation, which is the single largest population of our country numbers wise, and uh birth rate started in 1946 after the war to 1964. Single largest population is about to hit gray in about three more years. And [clears throat] we spend more on health care uh than any other country in the face of the earth. We have a $1 trillion health care system and a $1.4 trillion agricultural system. And that's not coincidental that they're almost equal. And it's not coincidental to me that when you go to shop for so-called groceries at the grocery store or the supermarket, it's also the same building that houses the pharmacy. Because me the foods are so un unbelievably incapable of sustaining life that you have to rely on pharmaceutical medications to to stay alive. So I I I contend that these meetings are about mankind. These are about society. These are about economics. It's about ecologics. It's about farming. And so [clears throat] I'm here to talk to you about the fact that I think if we start looking at the way our forebears looked at farming which was a health issue. I mean Harvey [clears throat] Wy Dr. Harvey Wy founded the US Public Health Service and he was so convinced that health had everything to do with farming that he pulled soil samples from every single county in the United States back in the early 1900s. He eventually was fired from his task. He started the Food Chemistry Division which became the Food and Drug Administration. Eventually under the USDA started that he was fired from his job under the Taft administration because he was basically trying to contain large powerful interests, pharmaceutical interests that were just starting then. Well, if you think they were powerful in 1912, you can just imagine how powerful they are a century later. So, he knew it. Alrech knew it. How many people have heard of Dr. William Alrech, which is a lot of Okay. Well, Alrech, Albert was a medical student, or at least he started being a medical student. And one of the [clears throat] things that he knew uh that convinced him that soils were the keystone of the health of a civilization in our own country, he actually researched the World War I draft records. And he found out where they had the highest acceptance rates and the highest rejection rates for the doughboys that were going off to World War I. And he found interesting corlaries in that the um the highest rejection rates were in the states of lower Missouri and higher Arkansas, which is the Ozark Mountains, thin rocky soils, not a lot of minerals there. And the highest acceptance rates were in Iowa and Nebraska where the appetiti soils were the calcium phosphate soils, the appetiti soils. They were the rich soils, the calcium phosphate soils. That's where 30 million bison ran from Canada down to Oklahoma and Texas every year recycling nutrients on the Apatiti soils. We had 40 million almost 40 million head about 30 million of them about in that part of the country and the rest of them were scattered through the great plains and as far east as the east coast actually they called them uh forest vines. They were same species but they had adapted to the woodlands and the east coast. So we had this incredible wealth glacial tilt and and that's one of the advantages North America did have over even Australia is we were glaciated and those apotiti soils created a civilization of bison and it ultimately started to create a civilization of of uh Americans that were strong and robust coming from that part of the country. So he knew soils related to because in in World War I in 1917 1918 people didn't haul food in from Florida and California you know there wasn't that kind of a food system back then you ate where you lived whatever you got you got locally so it was a very good correlary today you couldn't do that because in the United States the average distance from uh farm to plate is 1500 miles now every meal you eat in the United States you are buying food that's on the average hauled 1500 miles so that those demographics wouldn't work today. So that's how all this stuff got started was people realize look at the connection between the soil and the health of the people living on those soils and you know was very conclusive. So I think this quote kind of sums that up in that you know we don't look at the obvious now as a animal stock kind of a character I go to this first this is the first place I go when I go to a farm is I look at the cows but I look at the manure and if you're going to deal with health whether it's human health or animal health you've got to look at that which leaves the body because that's the clue food. It's the indication, and I'll say this, an animal or a human is only as healthy as its digestion is. And there's another pandemic we have with people in the United States is god-awful digestion. And look at the prescriptions and over-the-counter drugs. Number one, probably behind aspirins and headache pills are those that deal with bad digestion, including the channel calcium blockers, channel blockers, the um ant acids, all these things that people are taking. isn't because they have excessive stomach secretions. It's because they have deficiencies. 80% of the people anyway, 80% of those that are suffering from reflux have compromised digestion. Livestock have compromised digestion because we aren't looking at the blueprint of what a ruminant is. Aruminant doesn't eat grain. There's only one species of animal that's designed to eat grain is grain, and that's birds. And the reason why birds can eat it and not go through hell eating grain is because they've got an organ called a crop. And that crop is right here. You know, if you pick up chooks at night in the rugery, you can feel the grain that they store in that crop. What is the crop? It's a fermentation vat. But really, it's more of a sprouting vat. What is grain? It's seeds. And seeds have things in them that aren't really good for higher life forms like mammals. And they contain compounds called phytic acid and phitates. Uh they contain enzyme inhibitors. And the way you get rid of these negatives in seed is by doing what seed does best, which is to let it grow. You sprout it. Now you can cook it and that'll destroy the phytic acid and it'll destroy the enzyme inhibitors. That's why you can't feed raw soybeans in the United States to dairy cows to an extent that you cause trison inhibitor problems. Right? Very trison inhibitor. For raw soybeans, you're limited to how many beans you can feed because of the trips inhibitor. Well, it's the same problem they have with all grains. All grains have these enzyme inhibitors. So, when we're starting to realize that we're trying to make milk production or put meat on an animal, we can do it with grain. Clearly, that's proven. There's no doubt about that. But when we start doing that, we recognize, well, what is the price we're paying for that? and we start looking at, you know, the manure on these animals and recognize that there should be a whole science out here called manureology. There's geology, you know, and there's all kinds ofies, but there should be a minurology course out here. And uh you pick up that pie and you look at that pie, you put it in a colander, you know, you put another screen colander on top of that. That's that's a real important thing. put the second colander on top of the first one before you do what I'm telling you to do and hit it with a jet stream because if you don't do that, [clears throat] you'll be really ticked off that I didn't tell you that, you know, and you don't use your spaghetti colander from the kitchen. You have a designated colander, okay? And you take that manure pod, you throw it in that colander, and you look at what is left after you blast it with a high stream of water. Now, if you're feeding grain, there shouldn't be any grain in there, period. If you're not feeding grain, there should be a small amount of digestible fiber from the forages. Maybe a quarter of a cup of broken down fiber. That's all that should be left in that cowpie. Furthermore, that cowpie should have the right consistency. Should not be slimy. It should not have a lot of bubbling going on. That tells you there's acidosis coming out of that animal. It should have a pH. If you have a pH meter, you stick that in that pie. That pH should be around 65 on up. The other thing we do is we look at the urine and we test the urine. The urine should always be slightly acidic around six 265. You never want to see urine get above 7 especially 75 and 8. And the reason for that is because metabolic waste is excreted in the urine. This is true for your own urine. If you want to find out if you're healthy, check your urine first thing in the morning. It should be above six, but it shouldn't be really alkaline either. And the reason for that, if it starts becoming really alkaline, and this is true in the cow because most people think, well, one target because the urine's alkaline. The reason why you don't want to do that is because if the urine is supposed to be acidic because there's metabolic waste leaving the animal and all of a sudden you start seeing the urine of the animals are running at eight. What does that tell you? Well, tells me that the buffering system of that animal is just gone. Which now seems kind of ironic because buffers raise pH. And so if the buffering system is gone, why would the urine pH be alkaline? It should be acidic. Well, here's what happens. And this is very relevant to your own physiology. The blood pH of the cow and the human is about 7.4, slightly alkaline. And that blood pH wants to stay there and it will stay there at all costs at about 7.4. It might go down about 7.35. It might go up about 7.425 or something like that, but it'll stay right about 7.4. It has to do that or there's death. That's your option. 74 or you die. So the body will do everything it can to maintain the blood pH of 74. Well, what maintains a blood pH of 74? Cationic minerals, alkaline minerals, calcium, magnesium, potassium, sodium, some of the trace elements. Those are your buffered minerals. Curiously enough, those are the same cationic minerals we're going to talk about today that buffer the soil and they have to be in the right ratio in the soil as they have to be in the right ratio in the physiology of an animal. The same things are working in a soil are working in the air. Okay, this acid alkaline issue is universal. It's the way nature works. So the alkaline minerals buffer the blood. If we see that the pH of the blood is dropping, we know we've got acidosis issues. But if we see the manure of the pH, pH of the manure, excuse me, dropping, then we know we really have acidosis issues. If we see the urine of the of the animal going up, chances are you'll see that the manure may be going down. And the reason for it again is if the urine pHes are going up, it means that you are deficient in buffering minerals. Okay, so now comes the stupid question. Why did the pH go up if you're deficient in buffering minerals? Well, like I said, the animal will buffer at all costs. There's one other thing it can buffer with, and it's loaded in conventional farming operation feed stuffs, and it's called ammonia. So you could actually test the urine for ammonia and you'll find it there. And that's what's driving the pH because the pH of ammonia runs over 10. See? So the body of that animal will even cannibalize its own tissues. Although with most dairy herds or beef herd operations, it doesn't have to do that because the funny protein that most farmers are growing is so loaded with nonproin nitrogen or nitrate or ura, whatever you want to call it, instead of real protein. There's plenty of raw materials to produce ammonia and I'm going to go into that in a little bit. So what I'm trying to give you is pictures. We're looking at these things ecosystems and what we're looking at here is a rin that is the primary ecosystem. Remember all health starts to begin to get better or begin to fail based on digestion. You're only as healthy as the microfllora in the small intestine. And with a ruminant animal that has a fermentation system that precedes the true stomach, you know, we start out with the true stomach, they start out with a rumin, then they end up with the true stomach, then we all end up with a small intestine. &gt;&gt; This is not coincidental that these systems go from, you know, in a ruminant slightly acid to very acid to very alkaline. That's the way it has to work. And if this manure is telling you otherwise, everything else is going to be screwed up. The band-aids that you're going to have to use on that herd are going to go up in cost because you're going to have to supplement to put out the fires that you created by trying to make milk production from architecturally the wrong food stuffs. And the reason why you're going to do that is because you can't make milk without energy. Energy is the limiting factor in stock. putting on weight, putting on milk. So, if you don't have the energy in the forage, naturally the nutritionist is going to come along and say, you know, obviously your cows are in bad condition. You're not getting them bred back. You know, you're not making the milk you're really wanting to make. So, they turn up the thermostat, which is the BTUs, which comes from cereal. But the problem they have is they don't believe or if they do believe they're not telling anybody that you can actually create energy and forages. So that's what I'm here to tell you is that the real secret to this thing is to do what these other people have done already with the top herds in the world of the Jersey herds and the and the Holene herds and the Gernzy herds. Carnation had top cows in all breeds in the 50s. So and they did it on a high forage ration. So we go from that slide to this slide. And this is this slide could be a whole day. We could actually do a whole day on this this slide, but I promise I won't. So, but I will give you the the the real the creme creme here. This is the rin. This triangle here represents protein. And you see it's split into two sections. We have what we call true protein. What is true protein? Amino acids. methionine, tryptophane, tyrrosine, lysine, amino acids. That's what true protein is. The building blocks of the body are amino acids. Peptides are are groups of those. Then we have this stuff here called nonproin nitrogen, which is not protein, it's nitrogen. Why is it in the protein triangle? Well, go to the very top of that slide. You'll see CP equals N * 6.25. CP stands for crude protein. Crude protein is not, I repeat, crude protein is not a measure of amino acids. Yes, &gt;&gt; good point, J. That's the one they use. What the heck? &gt;&gt; Well, that's what we're going to do. We're going to we're going to do an end round run here and show you how you can take food protein and figure out whether or not you have any true protein in it. Okay, that's that's what we're going to try to do here. And there's some there's some little tricks here because no lab is going to test your amino acid levels of your forage is because it would cost you a bloody fortune to have that done. So, and the reason why they test for crude protein is because all protein without exception on the average, there's that word again. You know what they say about average, you know the definition of averages is you have one foot on dry ice, you have another foot in boiling water and you're comfortable. That's an average. Okay? So when [clears throat] they say averages, always be aware of that word because you what do you mean by averages? So you have all on the average all protein contains 16% nitrogen. It's the only stuff that does contain nitrogen. So if you divide 16 into 100, you come up to 6.25. It's an arbitrary number. It's a starting point. It's not an ending point. So now we've got this thing saying, okay, you've got a 22% protein alpha alpha or a 29% protein alpha alpha. What do you really have? How do you know that's protein? How do you know it's this piece, not that piece? Some of it's And you can see in all in all protein, you're always going to get a little this. Now, here's what happens, and this is what's important to remember. You see the top arrow, the top arrow, 60%. What that says is 60% of true protein solubilizes in the rin to produce ammonia. That's a good thing because what are you feeding now? You're feeding not the cow anymore. You're feeding the cow's basically ecosystem which are microbes. So ammonia becomes the food stuff or the protein for simple life forms called bacteria. Bacteria. And what you got in this room in here, best description I can give it to you, it's like the Serengeti or the savannah. The bacteria are the grazers. They're the herbivores. And then they're prayed on by, and I'll talk about this, the soil food web works the same way. They're prayed on especially by prozzoa, which eat the bacteria. And in the process of bacteria being consumed by other organisms, a lot of energy and a lot of protein is recycled over and over again, increasing the efficiency. And that's exactly what happens in the soil when you have a really healthy soil food web. You recycle the nitrogen. You don't waste it. So what happens here is you've got the Serengeti going on here with the the herbivores, the grazers being the bacteria, which are by the way bacteria are the nitrogen sink of the soil and bacteria are the nitrogen sink of the rin. You want lots of bacteria in that rin because they suck up this stuff. That's why you can feed a cow or a goat or rin I should say ura because they're eating ura and they're synthesizing ura. certain amounts of it. So, but here's the caveat is that with the funny protein, I call this funny protein. The funny protein, 100% of it solubilizes into ammonia compared to 60%. So, needless to say, if you've got a 28% crude protein, I'll guarantee you based on what I can look at the rest of the soil or the forage test, you're going to see this fraction getting much much larger. That means this overflow ammonia gets larger and larger because what has to happen is remember Alrech used to use the axiom all life forms need go foods and grow foods. Grow foods are your proteins or nitrogen. Go foods are your carbons or your energy. So you've got this grow food here. You need go food. Microbes in the rin need go food. There is the wall that the dairy and the beef industry has hit because they're not producing the kinds of go foods or carbohydrates that these microbes that live on this ammonia can populate themselves on. So they come along and they instead of feeding the rin they have to feed the cow by feeding them grain. These organisms are cellulitic organisms, ptoolytic organisms, that is they have a specific substrate that they feed on which are the soluble fibers. So if this level gets up too high because you either fed too much protein or the quality of your protein was too funny, too high in NPN or because you didn't have enough of the right kinds of soluble fibrous energies. Any of those three reasons, you now get this buildup of ammonia which flows through the rin wall. Goes right through the rin wall. Now it's in the bloodstream. alarms start going off and now we got a veterinarian condition called BUN blood ura nitrogen toxic compound and when the blood ura nitrogen levels get to be certain at certain levels you start having all kinds of problems first thing that starts to happen is you don't get cow's bred or if they're bred they won't hold a calf that's the first thing second thing that happens is the kind of stuff that happens in places like western Washington state, high rainfall area, 110 inches of rainfall every year normally. Wouldn't you like to have that here? [laughter] No, you wouldn't. No, you wouldn't. and you go into the Tanuk Valley and it's a dairy area and you go in that area and it's and it's all grass and uh you talk to dairy farmers there and you look at the cows and they're got these rough coats and they're droopy and they're not making great. They're not nobody's having a good time. And you stand there and you look at what's going on. You see the uh the fertigation systems where they're sucking out the the slurry manure and that becomes their fertility program in all these paddics or lays or pastures. What's in slurry manure? What are the primary nutrients in slurry manure? Nitrogen and potassium. The antidote to energy and forage. It's the best way to strip energy out of grasses and leg rooms is dump the nitrogen in the pod ash arm. I'll go into that. All right. So, this is what's going on. Meanwhile, this dairy farmer tells you, "I don't understand this." He said, "I got halage in this this bail over here. It's 27 28% protein." He thinks it's protein. And he said, "And then when I buy hay from the eastern part of Washington State, which is high desert, they get 26 in of rainfall a year and they grow and they have high mineralized soils there and they raise a lot of alalfa there." and he buys a 17% protein alpha alpha hay. The cows come up in milk and he doesn't understand why. And the reason why is because as this ammonia is running around in the bloodstream and the liver knows in its wisdom that it's got to get rid of it. Now see all the blood ultimately gets goes gets a chance to go through the liver. Thank God we've got livers. All the blood gets the chance to go through the liver. And when the liver senses ammonia, what does it do to it? It wants to detoxify it. So, it turns it into a less toxic substance called ura. URA is less toxic than ammonia. They're cousins. Ammonia's NH3 basically and ura's NH2. It's less toxic. Then it sends it back out in the bloodstream and ultimately the kidneys pick up all the blood and the kidneys take the ura and they change it once again into uric acid. and then out the end of the cow goes. Well, assuming you don't have cows dropping dead, which if it gets high enough they will, uh, now the dairy industry in the United States, and I suppose it's possible that's going on here, they have this thing called amuent, milk ura nitrogen. To detect blood ura nitrogen, you have to pull blood tests and usually the vets do that. Now, they've got, you know, you can test right on your own farm for milk nitrogen. In fact, you can test for milk nitrogen now with test kits. In 1996, I was in the UK and I was talking this story. This very same slide was there in front of the people in the UK 1996 and we were talking about this and this one dairyman came up to me later and said, "Man, you hit it right on the head with my farm." I said, "How do you say?" And he said, "Well," he said, "we had calf deaths like you couldn't believe. We just had all our calves were dying. We vaccinated. We had antibiotics on those animals. The vets were just pulling out their hair. And then somebody told me about MUN. And I didn't know what mu meant. And I found out I could buy a kit from the continent to test my milk for mun. And sure enough, his milk was so loaded with this nitrogen substance that it was poisoning his calves, which are not ruminants that cannot deal with it the way a ruminant can. They're monogastrics when they're babies. And so they were dying from nitrate poison. That's what happened. And he didn't. And what did he do? Instead of giving him wonderful whole milk, which is a medicinal substance for calves, it's loaded with all of these enzymes, vitamins, minerals, antibodies, lactic acid organisms, and on and on and on. You know, you had to give them milk</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>❤❤❤❤ || 💪🏾💪🏾 || 💯 || 💪🏾💪🏾 || Yep, please don't wait until you are 3 years in to start generating P&amp;L statements. || Right I see this wayyyy to often with folks || ​@PATRICELSTEWART, this would have saved me a few thousand dollars.</t>
+          <t>Thank you for posting. I never got to meet Jerry in person, but this helps me get to know him in a way now. || Thank you  for sharing || Biofertz represent 🪱🌳☀️🐝</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GK6JhMq6vSQ</t>
+          <t>iktPekYGwzQ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Self Prepared is No Liability #patricelstewart #business #taxdeductions #tax #taxpreparation #taxes</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Regenerative Cattle Management: Doubling Capacity &amp; Reviving the Soil Food Web - How to S4E14</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>*Regenerative Cattle Management: Doubling Capacity &amp; Reviving the Soil Food Web*
+In this inspiring session filmed at the Bolivia Landcare field day, I sit down with Jake Smith, a passionate cattleman managing 8,500 acres around Tenterfield. We dive deep into his remarkable transition from industrial set-stocking to adaptive multi-paddock grazing. 
+#RegenerativeAgriculture #NutritionFarming #MobGrazing #SoilHealth #GraemeSait
+Jake shares the practical steps that allowed him to double his carrying capacity, drastically reduce chemical reliance, and welcome back the ultimate biological indicators: the dung beetles. This is a powerful testament to the fact that when we work with nature, rebuilding the microbial bridge, the farm becomes more profitable, more resilient, and ultimately, produces healthier food for our communities, honouring the soil to soul connection.
+*What you'll learn:*
+🌱 How adaptive mob grazing can naturally suppress weeds like Giant Rat's Tail grass.
+🐄 The simple, low-cost temporary fencing strategies to get started with cell grazing today.
+🪲 Natural alternatives for Buffalo fly control that protect and restore your dung beetle populations.
+🧬 The undeniable link between intense animal impact, soil restoration, and building humus.
+👇 *Chapters:*
+00:00 - Introduction
+01:27 - Title Sequence
+01:57 - Jake Introduction
+03:05 - Holistic Grazing Benefits
+04:28 - Changes in Pasture Species - Blady &amp; Paramatta Grass
+06:02 - Increased Biodiversity &amp; Beneficial Insects
+06:27 - Livestock Health
+07:06 - Nutrition Farming
+07:52 - Dung Beetles &amp; Buffalo Flies
+11:04 - USA Tour &amp; Industry Leaders
+13:37 - Top Recommended Regen Practices
+16:58 - Profitability &amp; Stocking Rates
+17:52 - Wrap Up
+18:03 - End Credits
+Want to learn more about Nutrition Farming? Check out Graeme's two-part article *”Nutrition Farming® – Where Do I Start?* …
+https://blog.nutri-tech.com.au/nutrition-farming-where-do-i-start-part-1/
+*Key Products Mentioned:*
+_Diatomaceous Earth_
+_Boss Bags_
+_Boss Lick (Garlic and Sulphur)_
+These can be sourced from the Kandanga Farm Store in SE QLD.
+https://www.kandangafarmstore.com.au/
+*Nutri-Life BAM™*
+https://nutri-tech.com.au/products/nutri-life-bam
+*Nutri-Gyp™ Natural Gypsum*
+https://nutri-tech.com.au/products/nutri-gyp
+*Sili-Cal (B)™*
+https://nutri-tech.com.au/products/sili-cal-b
+…or try our new NTS FulvX™ Powder for chelation
+https://nutri-tech.com.au/products/nts-fulvx-powder
+*Interested in attending a Certificate in Nutrition Farming course?*
+https://nutri-tech.com.au/pages/courses
+Need assistance? Try out our Soil &amp; Plant Therapy Services
+https://nutri-tech.com.au/pages/soil-plant-therapy
+How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait
+Head to our website to find out more
+https://nutri-tech.com.au/
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+*Follow us on Social Media*
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+Twitter: https://x.com/ntsaustralia</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-01-10T07:31:35Z</t>
+          <t>2026-02-20T07:09:24Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1343</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.108483</v>
+        <v>0.028295</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -737,56 +884,117 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>When you are filing your taxes, you are supposed to receive a full copy of your tax return. All pages, not just the 1040 page, which is two pages. A lot of you all only receive no paperwork or you receive one or two or three pages. An average tax return is about anywhere between 12 to 25 to 30 pages with all of your worksheets, all of your forms, everything. Also, it should not say self-prepared if you are going to a tax professional who says that they can file you professionally and you're paying them to file your taxes. All right? A lot of you all go to people who do your taxes on Turboax and that may be cool with you, but there is a process and there's a difference between someone who is a real tax professional like myself who is an eile agent. We are registered with the IRS. I have an EIN number with the IRS. I also have to have a P10 number. So on the bottom of your paperwork when I give it to you, it has all of my company information because that means I am responsible for the tax return that I filed on your behalf. A lot of people you all go to are doing all of this extra stuff because they have no liability for the tax return. If it says self-prepared, then that means you are responsible for that tax return. Patrice L. Stewart here, the realist tax and business strategist.</t>
+          <t>Welcome everyone. We're here at Bolivia, a little country hall in the middle of nowhere. Um, and we're having a a field day sponsored, wonderfully, generously sponsored by Landare, where we've got a crowd of perhaps 70 people here, uh, learning about all things regenerative. And one of the attendees is a a gentleman who attended my course, how long ago would it be? &gt;&gt; I think it was August last year. It was winter last year anyway. &gt;&gt; Okay. So, his name's Jake Smith. And you know, we talk about young blood and their importance to develop some passion amongst young blood with this whole regenerative approach. And we've got a man who very much has that passion and we thought it'd be a great opportunity to have a bit of a chat with him and let him share his journey, his regenerative journey and what he's found and what he's achieved and some of the strategies that have worked for him. So, thank you for agreeing to talk. &gt;&gt; Thank you, Graeme. Thank you for everything. And thanks to Landare obviously for putting on this event like it's a wonderful wonderful couple of days we've had. &gt;&gt; Yeah, really generous. I mean, I've done land events before, but there's always some kind of charge. This is completely free and all the food's provided and so forth. So, yeah, really good thing. &gt;&gt; So, tell me about yourself. So, Jake Smith, I mean, how much land are we talking? What you farming? &gt;&gt; Um, so we're we operate across um about 4 and a half thousand owned acres of family farm and we probably lease another 4,000 somewhere in that vicinity. &gt;&gt; Thousand. We are a beef operation. Um, solely beef, but I'd actually like to bring in some um some chickens if I could find the right person to run it. Um, just for the clean up behind the the cattle. [music] and we operate all around Tennerfield. So we got country um east, northeast, south, west um all around Tennfield. all different um sorts of soil types and uh they all have their own challenges. But &gt;&gt; so when where when did you begin this regenerative journey? &gt;&gt; Uh well I'm actually a livestock agent by trade auctioneer and um &gt;&gt; I thought you spoke well. &gt;&gt; I actually um I had a client um and he came down from Northern Queensland. His name is Brett Craft and he's um he was a client of mine in Tennerfield and he sort of twigged this little idea in my head. Um before that we were fairly kind of industrial and um &gt;&gt; and I've been very lucky obviously like my old man's in construction so he's given me free reign of the farm. I can do whatever I want to do. Uh and if I fail he doesn't see it cuz he doesn't go down there much. So um that's so I Brett Craft introduced me to this concept of um rotational grazing to start off with and then I got in uh involved with um my grazing uh and then started going to field days and um got involved with RCS and it just really it compounded from there. So, &gt;&gt; and so just describe the changes you've had with this concept of cell grazing of intensive grazing. &gt;&gt; So, we um obviously we used to set stock like everyone does still does in the New England. It's fairly um prevalent. Um the first step that I took was um I mobbed all the cows up. Um after I mean you can have a serious crash if you don't do a lot of research on it first and do the appropriate courses uh and learning material, but I mobbed all the cows up and just started moving them really loosely. Didn't &gt;&gt; how big of mobs? Uh well at the moment we're about 350,000 calves in a mob. Yeah. Um and then sort of three to 500 heers in a mob. Um and same thing 3 to 500 steers in a mob. Okay. &gt;&gt; Um because they're different properties. If if all the properties were together, they'd be much larger, but we're still sort of in still u a building phase. &gt;&gt; U because we've actually compounded our carrying capacity so much just through mobbing cuddle up. even when I didn't really understand what I was doing, I just knew that it was I could feel that it was right. &gt;&gt; Um so we've actually compounded our um carrying capacity probably double I would say. &gt;&gt; Good. &gt;&gt; Um and just just through moving and and I've been doing this for probably &gt;&gt; um loosely for the first two years and then probably pretty well for the last sort of 3 to 5 years, four years. &gt;&gt; Um &gt;&gt; and uh yes. So &gt;&gt; and what kind of changes have you seen? Um well the for starters uh the grass like &gt;&gt; when you mob cattle up when cattle are all um set stocked &gt;&gt; you you tend to get um a monoc culture of the things that you don't want because they as soon as something juicy that they really like pops up there there and they're smashing it straight down to the ground &gt;&gt; and then all of them I mean after a little while it just depletes the root system and then that plant just dies. So you do end up with a monoculture of undesired grasses, which in our case on the eastern full is bladyy grass. &gt;&gt; Um, since I've mobbed the cows up, uh, believe it or not, not only are the bladed grass patches getting smaller, um, but they're actually eating, uh, eating the bladed grass. I mean, some people say, "Oh, you got to have cattle really hungry before you eat the bladed grass." But I actually find that because they're getting so much good grass, they actually I think they eat the bladed grass for a bit of roughage. Yeah. &gt;&gt; So that's really it's an interesting observation. So the country um the country has really benefited. I mean the grass just looks revitalized. There's better species there. We had a massive when I was set stocked um we had an infestation of giant rats tail grass. Um and now uh with some seed application and uh rotational grazing uh there's actually um premier digit and roads plants actually growing and cockia plants growing straight up through the crown of these plants and and they're actually in the middle they're actually drying up and dying and sort of breaking away the rats tail plants um or they're actually dry parameter sorry &gt;&gt; um but yeah that's some of the changes we've seen but just really um fantastic insect populations but good insects I've I mean our neighbors get army worms, all sorts of bad things, but for some reason they mustn't like our fence or something or we must have a really good fence and they just don't come anywhere near us. So &gt;&gt; yeah, &gt;&gt; it's um you see all once you start uh integrating all these systems and cycles together, you start to see something really interesting which I don't fully understand, but obviously that's why I'm here trying to find out a little bit more about &gt;&gt; very special. The the response is is tremendous and you've seen a change in animal health and so forth so yeah. It's um I mean I I don't uh we do supplement our cattle um but I don't rarely rarely get a vet out to see a cow ever anymore. &gt;&gt; Obviously before there was a lot of anti-inflammatories, antibiotics, that sort of thing. I've cut all that out and I've also um cut out most chemicals definitely um Roundup. We don't use any Roundup anymore. I'm pretty sort of against that but um some chemicals we just cannot get away from. We are trying but &gt;&gt; um It's always the process of just pruning them out as you can. &gt;&gt; Yeah. &gt;&gt; Yeah. That's good. &gt;&gt; So the and I feel like so grazing is one half of it and I think um the other half is what you're doing is um this nutrition farming approach actually getting the plants uh healthier through the likes of soil applications but also folure spraying. So I have been following &gt;&gt; I have been on mainly our backgrounding block. I'm a believer in you get the get your best country the engine running and then it pays to do the rest of it. So I'm just trying to focus on our backgrounding block which is our better country. Um and I have been doing soil applications of microbes. Um brewing out different things. Um well this is all after your course that I the 5day course that I did last year. Um &gt;&gt; and uh obviously I mean you see a marked improvement every time you do a soil application for microbes or a folia spray for the plants which feed the microbes. It's uh it's a marked improvement. &gt;&gt; Good. That's good to hear. And you know, little indicators like dung beetles, have you got them back now that you've reduced the chemicals? &gt;&gt; Well, um, so I've spent, uh, I spent a my last probably 5 years of my life trying to kill them accidentally, not meaning to, but just our buffalo fly populations were through the roof. And this year, I just said, um, no more, no more. So, uh, I like a quote from, uh, from Will Harris. Um, well, he talks about, you know, when I was an industrial farmer, all I wanted to do was every time I walked out the door, I was looking for something to kill. But, uh, now he's looking for what he can keep alive. He wants to keep everything alive and let biodiversity and everything happen um, amongst it. So, our dung beetle population since I've stopped uh, we we've gone to a natural method of um, remedying the the the uh, buffalo. &gt;&gt; And what is that method? That' be an interesting thing to share. So we use a thing called dietimmacous earth in a in a product called boss bags um which is uh we actually get it from straight from Kadanga Farmto. They make them up at um Sunshine Coast. &gt;&gt; Fantastic product. Um and we also um use their boss lick which is a um garlic uh well a lys in the garlic and a um sulfur lick but and a base mineral lick also. &gt;&gt; Um good product &gt;&gt; and it's it's been a fantastic product. that I I I suspect next year, we still did have um a few buffalo fly, but I suspect next year when the dung beetle populations build up and breed up, that they'll be burying the dung quicker hopefully in theory than what the what the larae can bury uh can um growing the dung. So, I think next year will be even more of an improvement. So, but I mean they're back in the I hadn't seen it. I remember years ago before we used to treat intensively for um buffalo fly. You you used to be able to not sleep at night in the hut. Like they'd be hitting the hitting the walls of the hut and they'd be poked on the barb wire fences everywhere in the mornings when you went out. For the last 5 years since we've been intensively treating, I haven't seen a dung beetle down there. So something sparked in me and clicked in my mind and I just thought maybe this is what's happening. And um now I mean this year I've seen dung beetles back on that particular property for the first time as I said for four or five years. So which is actually really exciting. &gt;&gt; It's wonderful when you when they come back and forth. And with uh Claudia, my partner is a graze here out of Santo. Um she had exactly the same scenario. There was nothing and they were collecting dung for composting for this market organic market garden that they've got on the farm and there's just and it's exactly it's adapt adapt the approach and slowly they come back and now they're in there in such ridiculous force. Yeah. I mean there's a she let unfortunately the cows got into the house paddic and there's just manure everywhere and the next day the buzz she says you know forget about the crow the reed wobble or whatever that book masses book is let's call it the buzz of the of the of the of the cane beles because it was insane and there was nothing a day later everything has carried in it's just ridiculously intense and so good to see and it's just changing you can see this all changing is all of that tong in that concentrated form when you're sell grazing &gt;&gt; you know it's almost that model is almost like you can't really have too much. It's just how long you leave them there. The more cows the better really. Bigger mobs is is even more effective. &gt;&gt; Bigger mob the better. Yeah. And the smaller area you can concentrate them in and move them on. &gt;&gt; Um we just completed a trip to America um for 5 weeks um farm touring over there and we saw some really cool things. um the likes of we went to Will Harris, Joel Salatin, um Smoke River Ranch in northeast Oklahoma and another one in North Texas um Birdwell Clark Ranch and they're all doing this um sort of um a cross between ultra high density and u adaptive multipatic grazing and um &gt;&gt; so just describe adaptive multip. So adaptive multipatic grazing is um instead of cell cell grazing and having a very prescriptive um move at this time of day have this set paddic they are actually um they have big paddics and they build p they build temporary fences within those paddics. Um so the way that they describe it is that the energy flow of the cattle are moving different ways every time. So they might have the cattle running this way this time and then back across this way this time. So their different seasons and different things determine their paddic sizes um shapes. They always change their shapes. So there's never anything the same and they're never coming back to the same spot at the same time of year ever. Um &gt;&gt; Okay, that's good. I mean one particular example the Burbal Clark ranch they're they're across 14,000 acres in north uh northwest Texas at Henrietta and um they like they it's there is a figure it's like in the last 10 years um each square me or a certain square meter of that um block has been grazed a total of 24 hours in 10 years or so like the figures are there but it's a ridiculous amount so um or little time that is so they uh they do a fantastic job there. And you can see uh Emry Emmery describes um when he bought the ranch that there used to be big planes of nothing like you see in Western New South Wales big planes of just red clay pans, but now I mean they've got Indian grass and things like that. &gt;&gt; It's tremendous when you see it. I mean I saw it on a small scale. I was speaking at a conference in Townsville and for the reef safe group and they show me this little trial they're doing and this is small stuff. Okay, we got this gully that's just weed and crap and really nothing in it. And they just basically, this is the small scale people and people are buying cattle just for this purpose. There might be half a dozen cows and you just basically bring a bail of hay and you fence off just a small area and you got the cow, you got the mob effect in this tiny area and you just move that down the gully and then he show me a year later, two years, three years, four years because this has been an ongoing project and that restoration was just so impressive. I mean you just had this complete transformation of that valley done totally with the animals. &gt;&gt; Yeah. &gt;&gt; Yeah. Such a good concept. &gt;&gt; Animal impact is I believe is the single best thing for landscape recovery. Um &gt;&gt; yeah mixed with a few other things but yeah. &gt;&gt; So what of all the things because we've got a room full of people waiting for us to come back and start the presentation. But what would you consider to be the most effective of the of the regenerative strategies that you've put in place? the most effect I don't know whether there is any most any one thing but probably definitely um is you need to get yourself educated that's one thing courses like yours are obviously paramount um uh but probably the biggest thing for me was um just mobbing the cattle up you don't you can just start moving the cattle and and just watch what happens you will see a marked improvement it's actually ridiculous how much better it is than just set stocking and you will boost your carrying capacity there's no two ways about it. &gt;&gt; And how have you found it from obviously I watch Claudia's situation twice a day she's moving them super labor intensive. How do you manage that? &gt;&gt; We I can't personally do that. We don't really have anyone that works for us. Um and we have farms different places. So I try and move them every sort of 3 days. Okay. &gt;&gt; Um but that will intensify uh especially on a main breeding block. Um &gt;&gt; but it's you'll actually find um you have a lot of fun doing it. &gt;&gt; Yeah, you will. and it's you think it's going to be all a big job, but I mean you can run a a Kiwi Tech fence system or just a Poliwire fence system across a paddic in 10 minutes and that'll be enough area for um you know a couple of hundred cows. So you think it's going to be a lot of hard work, but it's not really. It's actually a lot of fun and just but and I mean then you get to actually &gt;&gt; and they they they get to know that they want to move to the new spot, so it's not that hard to move them around. &gt;&gt; Correct. Yeah. Yeah. &gt;&gt; And you actually get to you can see the difference in the country around behind you like the the dung beetles um a lot of places in America the draw down of the dung is less than 24 hours and there's nothing on the paddic. &gt;&gt; That's like what her place is. It's wonderful. I remember this a couple who grazing a couple thousand acres um in out from Rockampton. Um, and she decided she'd been one to one of the courses and listened to a few things. And so she had this bet with her husband that she could take 200 acres and make as much money as he was making from the other 1,800. He said, "Bring it on, girl." You know, they actually had I think it was a few thousand bet. So she split that 200 into 20 10 acre paddics and she brings 600 head into each paddic for a day. Uh, she planted lina hedges down the in each of those blocks. So those were really good protein source and they eat that tree loosen. But I did the soil test, you know, three years later come back and repeated the soil test and it was this absolute transformation. I mean, it was two and a half times the organic matter and every mineral had changed. It was just like and I said, you know, you cheated. You won your B money, but you cheated. You put some lime on here. Uh you put, you know, these trace minerals or whatever. It even looks like there's some compost. And she said, I I did nothing. I used my animals as my primary fertility tool. And it was such a graphic example of what's possible. &gt;&gt; Yeah. And you don't even realize what's possible until you start doing it. Like &gt;&gt; it's uh we don't even really know what's possible yet. So &gt;&gt; yeah, it might be a good suggestion that people just, you know, get some movable electric and just try it for themselves. It seems believing. &gt;&gt; You can get a you can get a fencing set up, a movable temporary fencing setup for less than a couple of thousand bucks. Like what can you buy for less than a couple of thousand bucks that can create a return on investment like that? &gt;&gt; Yeah. &gt;&gt; I mean it's um &gt;&gt; So your profitability has improved. &gt;&gt; Yeah, definitely. Yeah. I mean, like a lot of farmers, we probably never really we all had off farm jobs. Um, no one had ever really made money off the farm uh for probably 60 years. Um, but now &gt;&gt; something [laughter] thousands of acres of money from the farm. &gt;&gt; But then um since we've purchased another property and um taken on more debt to do that obviously uh but still a lot more profitable. So I mean once your stocking rates um &gt;&gt; improve profitability your profitability improves and I I think through um better grazing management um after doing it for years you don't want to jump straight into a really intensive system but I do believe uh with a really intensive system uh with some tweaks &gt;&gt; uh we we no doubt can triple our stocking rate um compared to in comparison to our set stock system. So &gt;&gt; that's great. Thank you so much for for sharing. At some point, we'll actually have a chat for the podcast as well. There's lots of valuable stuff you can share. But thanks for giving us the time today. &gt;&gt; No worries. Thank you. &gt;&gt; Thank you. [music] [music]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Good morning Beautiful Queen😍...Thanks for the love and information🥂 || Great information! || Thank you for keeping it 💯 || 😊 || Thankyou || You’re welcome 😊 || 💯 || 💪🏾💪🏾 || ❤❤❤ || ❤❤ || ❤️✊🏾 || ❤❤</t>
+          <t>On a hobby farm can chicken tractors be as effective for soil regeneration? || Definitely @christopherburman3340! Chicken Tractors can be a powerful tool for building soil fertility at any scale. || Good on you mate….hopefully more farmers will follow you and make the land better.and the creeks and rivers 👌🏻</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>26JhrkttRwY</t>
+          <t>UHEU6zJBtrE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tax Time let's talk do's and don'ts</t>
+          <t>The Liver Love Smoothie That Extends Your Life - Liver Health Strategies Part 2 - How to S4E13</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Work with Patrice 
-plstewart.info/bookme
-#taxdeductions #business #realestate #chicago #taxes #credit #entrepreneur #tax #taxtips #taxtipsandtricks #taxrefunds #taxreporting #taxtips2026 #w2s #1099 #selfemployed #entrepreneurship #taxwriteoffs #taxwriteoff #taxplanning #taxwithholding #realestateinvesting #1099k #taxhelp #irs #smallbusiness #schedule1 #schedulec #llc #partnership #scorporation #corporate #taxcredits #bigbeautifulbill #bbb #trump #trending #financeeducation #financialfreedom #financialliteracy #finance #mindset</t>
+          <t>In Part 2 of our Liver Health series, Graeme Sait takes us into the kitchen to whip up the ultimate *Liver Love Smoothie* — a powerhouse of glutathione-boosting ingredients. But we don't stop at the liver! We dive deep into the "Second Brain," exploring how *butyrate* , *resistant starch* , and the hidden world of *lectins* dictate your longevity and vitality.
+#LiverHealth #GutHealth #GraemeSait #NutritionFarming #SmoothieRecipe #LeakyGut #ResistantStarch
+*What you’ll learn in this episode:*
+🥬 *The Liver Love Recipe:* How to combine Parsley, Beetroot, Avocado, and Whey Protein for maximum detoxification.
+🧬 *The Power of Butyrate:* Why this short-chain fatty acid is your colon's best friend and a shield against inflammation.
+🍚 *The "Cook &amp; Cool" Secret:* How to turn simple potatoes and rice into life-extending *Resistant Starch* .
+🍅 *The Lectin Lowdown:* Why the Mediterranean diet removes tomato skins and seeds, and how it could solve your joint pain.
+👉 *Don’t forget to like, share, and subscribe* for more Nutrition Farming® insights with Graeme Sait.
+👇 *Chapters:*
+00:00 - Introduction
+00:12 - Title Sequence
+00:42 - Graeme Liver Love Smoothie Recipe
+00:57 - Parsley
+01:13 - Beetroot
+01:52 - Kale
+02:25 - Avocado
+02:59 - Whey Protein Concentrate
+03:18 - Garlic
+04:11 - Curcumin - Curcu-Life
+04:29 - Milk Thistle &amp; Capsicum
+04:44 - Broccoli Sprouts
+04:57 - Water
+05:09 - High Power Blenders
+05:53 - Smoothie Wrap Up
+06:47 - Butarate
+10:45 - Resistant Starch
+13:39 - Leaky Gut
+15:30 - Lectins
+16:05 - The Mediterranean Diet
+17:17 - Pressure Cookers
+17:31 - Wrap Up
+18:15 - End Credits
+Want to learn more about natural health tips?  Check out: Prebiotics, Probiotics &amp; Alcohol: Gut Health Tips You Need to Know - How to S4E2
+https://blog.nutri-tech.com.au/prebiotics-probiotics-alcohol-gut-health-tips-you-need-to-know-how-to-s4e2/
+*Relevant NTS Products Featured in This Episode:*  
+_BioSpark_
+https://www.ntshealth.com.au/products/biospark
+_Curcu-Life_
+https://www.ntshealth.com.au/products/curcu-life
+_Green Defence_
+https://www.ntshealth.com.au/products/green-defence
+_BioBubble™ Probiotic_
+https://www.ntshealth.com.au/products/bio-bubble
+_Nutri-Salt_
+https://www.ntshealth.com.au/products/nutri-salt
+_SweetSure_
+https://www.ntshealth.com.au/products/sweetsure
+*Interested in studying Nutrition Farming?*  
+Certificate in Nutrition Farming courses:  
+https://nutri-tech.com.au/pages/courses  
+Need personalised support?  
+Soil &amp; Plant Therapy Services:  
+https://nutri-tech.com.au/pages/soil-plant-therapy  
+Book a one-hour online consultation with Graeme Sait:  
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
+*Explore more at our website:*  
+https://nutri-tech.com.au/
+Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
+https://nutri-tech.com.au/pages/newsletter  
+*Follow us on Social Media:*  
+Facebook: https://www.facebook.com/NutriTechSolutions/  
+Instagram: https://instagram.com/nutritechsolutionsyandina  
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
+X (Twitter): https://x.com/ntsaustralia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-01-10T01:11:18Z</t>
+          <t>2026-02-06T04:30:31Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -795,7 +1003,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.118421</v>
+        <v>0.019635</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -804,7 +1012,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>I don't know why this still pops up here. Make sure my volume is on. Make sure my volume is up. Good evening. Good evening. Good evening. Good evening. I'm on a few platforms, so I'm just going to allow a minute or two before I get started. Um, tonight I wanted to come on to briefly talk to you about tax updates, especially with these advances right now. Kind of wanted to explain to you all um how these advances work. I know a lot of people are promoting advances and things right now. So, I wanted to actually make sure that you all know the proper process on this and how it all works because you have a lot of people, you know how it is. Every year you get all these hustlers, as I like to call them, you get all the hustlers that's hustling taxes and tax time. And a lot of y'all don't know or get the real information. So, I am also filming on my YouTube channel. As always, YouTube is my number one platform. So, the replay to this video uh will be on my YouTube channel. I will not have this replay on Instagram or on Facebook. I am Patrice L. Stewart on all platforms. The name that you see on on whatever channel you're watching me on is the same name on my YouTube channel. Okay. So, good evening. Good evening. Good evening. It is Thursday night, I believe. Yeah. I don't even remember the days of the week. It's Thursday night. And so, I've been getting a bunch of calls right now around this whole tax advance, right? So, I wanted to share you with you all how this whole tax time season works right now. Okay. Um, and let me just make sure before I say that because I know yesterday, I didn't check today, but as of yesterday, the IRS has not announced the opening filing date for 2026 tax season. So, let me just make sure before I say that that Oh, we got a date. See, things change every single year. So that's why you have to check every single day. So yesterday I checked, we didn't have a date. We actually have a IRS open and filing date. As of right now is Monday, January 26. So I'm glad I decided to check before I said anything. So let's go ahead and get into this update. Um, hello, welcome. My name is Patrice L. Stewart. If you are new here to my page and my channel, better known as the realist tax and business strategist. Um I have over 20 years in the tax accounting banking industry and I am a tax strategist. Okay. Um right now we are in tax season. I want one of the things I want to say is taxes is all year round, right? It's it's only called a season right now because that's the time that majority of you all are filing which is between January and April, right? But just so you know, taxes is all year round. I filed taxes from January to December. The last tax return that I submitted was December 26, okay? A couple of weeks ago. That's why I'm not rushing to file taxes today. Um because I just got through filing the last tax return December 26. So people like me who are real professionals in this industry, uh we file all year. It's it's not seasonal. Taxes does not start um does not stop, excuse me, after April 15th. Right? So, I wanted to put that out there. Taxes is all year round. You can file taxes after April. I have some clients that wait to file their taxes until September, October, November. They want to get their refund closer to the holiday time. All right? So, that's up to you. Just want to put that out there. two, now that we have a IRS date, because I was [clears throat] just getting ready to come on here and say the the IRS is not even open right now, but they have officially now put a opening season date. So, every year, um, the IRS shuts down at the end of the year, usually whatever the last day is of that we filed a tax return. So, this year we were able to file t last year, I'm sorry, we were able to file taxes up until December 26, right? So, the IRS shuts down about a week and then in January they open back up. So, right now you all may be seeing people promoting, "Oh, you can get a cash advance. You can get a cash advance. You can get a cash advance because I've already had four calls today about this cash advance." I wanted to explain that to you all. All right. What is this cash advance and how does it actually work? One, the IRS is not officially open. Okay? They literally just put on here today because I like I said I checked yesterday and they did not have a open seasoning date. Now they have a open seasoning date for 2026 which will be January 26. January 26 is the official day that the IRS actually opens for tax season. Now you all may see people promoting and saying, "Hey, you can get a cash advance. I mean, you can get you can get an advance on your taxes. Let me explain this to you because a lot of people will not explain this to you because again, uh, a lot of them be thirsty to get your money. Real quick, um, I personally don't like to file taxes early January. My office, we're not actually opening until Monday the 12th, and I only file uh, advances for a specific client base, not for everybody. But one with the cash advance, in order for you to apply for a cash advance, you still need all of your forms and documents. Okay? So, the worst thing for you to do is if you have three W2s and you only have one W2 right now and you go and you let somebody prepare your taxes and file for a cash advance, one, the IRS is not open. So, what you're getting, you're doing a pre-agnowledgement advance. Okay? So, there's two different types of acknowledgements. You have a pre-agnowledgement and then you have the post acknowledgement, which means the IRS is actually open. Okay? Right now, any of you all that are working with somebody and you are doing a cash advance today, today is January 8th. All right? You are in a pre-agnowledgement. So that means your taxes are going to be sitting in a uh basically in a waiting pot, okay, till the IRS opens. Now, will they give you that advance? That advance is not through the IRS. That advance is through whatever tax office company that you're using. Their bank is allowing you to offer cash advances. All right? So, I want to explain that cash advances do not come through the IRS. They are not from the IRS. They are actually from whoever you're working with that that office is uh is registered with a bank. That bank is giving you all the cash advance. Okay. But the biggest thing I see when people apply for these cash advances or or give or give me feedback, let me say that because we ask a lot of questions before we push through an advance for somebody. Um, the biggest thing that I've seen that people do is you all go to these offices that are pushing to for you to do these cash advances and you don't have all of your paperwork. Right? That's the biggest first mistake I would say. Do not apply for these cash advances and you are missing paperwork. A lot of you all do not have your W TWS right now. Yes, companies do go online and you have access to your uh portals and W2 information for some of you online, but a lot of employers are still getting your W2s and paperwork together. If you know that you own a home and you file your house, your your mortgage company probably does not have your uh 1098 on there yet, right? If your child goes to school and you need to claim school credit, you probably don't have that school form on there yet. Okay? Most of the time, we are allowed as employers and companies up until January 31st to mail out your W2s, your 1099s, your 1099 KS, your your any form, right? Whether it's investing, whether it's your school form, whether it's your W2s, whether it's 1099s, the companies have up until January 31st to get those mailed out to you. So, the biggest thing that I see is you all are applying for these cash advances with these people that are promoting these things to you, but they're not explaining that to you. You need all of your paperwork before you file for that cash advance. Okay? And again, the official opening date that the IRS will begin processing tax returns officially is January 26. Okay, that's the date. Um, the deadline date this year, and again, deadline is for people who normally owe. All right. They the IRS would like for you to pay by April 15th, but it does not mean that you cannot file taxes after April 15th. You actually have up to three years to file a tax return. Okay? Um if you did not file taxes last year, if you didn't file 2024 taxes, if you haven't filed 2023 taxes, you can still file those. You can still file those electronically. With my office, we can file up to your last three years electronically. So, now that we're in 2026, we're filing 2025 taxes. You have 2024 taxes and 2023 taxes. Any prior years to that would have to be mailed in or uh my office, we have a department that we try to fax in prior year taxes and get them processed through a little bit quicker. Okay. Um but again, you can file taxes after April, you all. Um, all US citizens have the right to do a six-month extension. Okay? So, if you need an extension and you need more time to pay, if you know that you owe and you are not ready to pay that by April 15th, that's where the filing the extension comes in at. All right. Um, and again, all American US cit all US citizens um have the right to file a six-month extension. Okay. Uh, what else did I want to say? What else did I want to say? Tomorrow I am going over the big beautiful bill in my private community and also on the uh YouTube page for members only. So, the big beautiful bill that they um turned into law last year, there are some new updates, all right, for you all. Um, so we'll be going over those in the private community, what school won't teach you. Those of you all who are in the private community, make sure that you sign uh that you join in, that you log in into the Zoom because I will be going live to go over what's in the big beautiful bill and how you can take advantage of some of these tax updates that um the government has set up for you in the big beautiful bill. That's really it. What time is it? I don't have I didn't want to be on here a extra long time. Okay, perfect. 13 minutes I've been on here. So, I will review any questions that you all have now at this time and especially on my YouTube channel. Uh, thank you, Train. What's going on? Happy New Year. Chad, you say, "Can you give us tips on skipping them?" When you say, "Can you give us tips on skipping them?" I don't understand. You need to ask a a better question, Chad. Skipping what? Bid spotter say, "Patrice, I'm just seeing you. [laughter] We're live. Let me listen." Yes, Big Spotter. Go ahead and listen. Take a couple of notes. Like I said, I didn't I'm not going heavy tonight. I just wanted to really bring that up because we do have I had a couple of people call my office today about that whole cash advance thing and I think a lot of times you all get all of these promoters, you know, not knocking anybody, but it is what it is. I mean, I'm I'm a professional in this space. I'm a tax expert. I'm a tax strategist. So, this is my lane. Take it how you want to take it. But we have a you have a lot of people that at this time like to side hustle taxes, right? And they love to promote certain things to you all, give you all these astronomical dollar amounts that you could get. And I'm going just say this like I always say. If it sounds too good to be true, it normally is. Every single week, my office gets calls from you all who have been audited or being audited because you have credits on your tax returns that you should not have. If you normally get back $1,000, $500, whatever you normally get back, and now somebody is telling you, "Oh, I can get you back five to 10 bands, uh, hello." Clearly, they're not doing what you normally do. It's just that simple. So, I don't want to hear that fake weak ass excuse that y'all like to come on here and say, "Oh, well that somebody just put whatever they wanted on my taxes. You was good with it when you was about to get that $5,000, right? You was good with it when you got that five or $10,000. But now that the IRS has audited you, cuz the IRS will give you that money. Let's let's be clear. They will send you that money. People be thinking like, "Oh, well, I got my refund." Yeah, you get that refund and in two to three years you'll be calling my office crying like the rest of these people are, right? And that's what it is. The IRS will give you that money. Let's be clear, right? Sometimes whatever they put on you all's taxes, fraudulent credits and stuff, sometimes it goes through. Yes, it does. But I guarantee you, I bet money on it. Within two to three years, you will be getting a letter saying that you owe this dollar amount, [laughter] saying that you owe this dollar amount. And then you'll be crying talking about, "Oh, the person put on whatever they, you know, put whatever they put on my taxes." Yeah. All right. So, don't come on here with them sad stories lying because you was fine with it. Okay. Just know and understand half of these people that are promoting that stuff, they're not real professionals. Real professionals, we don't even promote stuff like that, right? We're not promoting five, $10,000 refunds. People that promote dollar amounts and numbers usually are hustlers. Hustlers and I like to call them. Real tax professionals don't do that. Real experts don't do that. We don't have to do that. We don't have to do that. It's not a This is not a numbers game, right? This is real. Your finances is real. Your money and your taxes is real. Okay? This is not a game for you to be playing with. And a lot of people who have done it in the last couple of years are seeing that. Everybody going to promote and say, you know, hey, I got the money, but nobody ever comes back on to tell y'all that now they under investigation, right? Uh so that's the reality of it. Um is the big beautiful bill going to help us get a bigger refund? So many people the big beautiful bill will help. Every single one of you all are different individuals. So there's no um you know one sizefits all to taxes. That's what I love to say. Every single person's tax return is different. So is it going to help people who receive tips? Yes, it is. Those of you all who rely on tip jobs, you will be able to have a nice dollar amount that you'll be writing off. seniors. It is helping seniors. Seniors have a whole new tax uh deduction that they've never had before. So again, certain people will benefit from the bill. Certain people won't. Um the standard deduction goes up every single year. That's not nothing new, but the standard deduction has gone up this year. So, some people should see should again I don't know your situation, your paperwork. Also, taxes are based off of what you paid into the system. Okay? So, if you have a W2 and you didn't pay any federal taxes, I'm Let me say this to y'all. Let me get a little closer in the screen when I say this one. Those of you all who pay no federal taxes throughout the whole year and expect the refund, did your mama drop you on your head? Because I really don't understand that. All right. One thing my dad always taught me was either you going to pay taxes throughout the year and you get some money back or you pay or you do not pay taxes and you get your money during the year. All right. But to pay zero in federal taxes, you made a h 100,000 and you paid zero in federal taxes and you expect a tax refund. Why? Does that make any sense to you? Okay, you didn't pay any taxes into the system. So 99.9% of the time you're going to owe. All right. Now, if you have other things like maybe real estate investments, right? Maybe some other things going on that help you with that tax deficit. But those of you all who know that you paid zero in taxes through the whole year and expect a refund, I don't understand your logic behind that. You have none. You don't understand how the system works. Okay? So, I'm I'm on here to tell you that today. If you are a W2 wage earner, you all pay taxes out of your paychecks. Now, if you are someone like me who is a business, I'm a corporation, but I'm also an escorp. I don't pay taxes throughout the year. businesses. We pay our taxes when we file our business taxes at the end of the year, especially service-based businesses like myself. Now, if you are a productbased business or maybe you have a store, a retail location, maybe you sell clothes or maybe you have a grocery store or something like that. A lot of you all pay taxes throughout the year. All right? And this is why I said every single business is different and there's no one-sizefitit all to it when it comes down to taxes. Everybody's situation is different. But I definitely need to put that out there because we have way too many people who pay zero in federal taxes from a W2 that expect the refund. And that just makes no sense to me. I just don't understand why you all think that that you should get that. Especially when you grown grown. You grown. You've been filing taxes for 20 years and you still have that misconception in your head that you should be getting a refund. So maybe you've never gone to a tax professional that knows how to explain this type of stuff to you. And that is the reason why I trademark I'm the realest tax and business strategist because I'm real. I'm honest. I'mma tell you the truth. It ain't no sugar coating over here. We going to get straight to it. I'mma tell you what it is and that's what it is. So, uh, any questions? I'm not going over the big beautiful bill tonight. I'm going over that tomorrow and I'm going over that in the private community. Um, the private community right now for what school won't teach you, it's only $37 a month. So, those of y'all that want to get in class tomorrow night, we'll be on at 6:00, 6:00 to 7:00 p.m. Um, you can get in, you can text me to the phone number and you can get into the private community. It's a membership community that I have and that's where I do all my educating. All of the classes and the workshops that we host are in the in the private community. Um YouTube, do you have any other questions on here? It's been 22 minutes. I I will be on here another eight minutes. Oh, I saw somebody on Instagram. I'm sorry, Instagram. I'm not purposely um ignoring you. I just am not on here much. I really just come on here to let y'all know that I'm live. But I would recommend that you go to my YouTube page and channel. Alan, you say, "Patrice, is it true that Social Security will go untacked in 2026?" Um, it's part of the big beautiful bill. I'mma say that. It is part of the big beautiful bill for Social Security. Um, so that's the most I'm going to say, Allan. It is part of the big beautiful wheel. So people who are on social security, that is something that um that is that will that will be beneficial for you. that is something that will be beneficial for you. But I'm going to go over that in a lot more detail um for you all like I said in class. And then those of you all who are members on my YouTube channel, I do have a membership here on my YouTube channel. So you all also will get access to that as well. And like I said, people who are in tip based industry, you all will be happy. Um, those of you all who are seniors, uh, our seniors will be happy because there is a brand new deduction for our seniors. And it's a couple other things. It's a lot actually. It's a lot, excuse me, that they have added in this big beautiful bill. So, we are going to go over some of those things um tomorrow during the class. And like I said, somebody asked me earlier or inboxed me earlier about the um standard deduction. So, the standard deduction increases every single year. Um every single year. So, it has increased this year. So, a lot of you all should see depend again should I won't say should it could it could be you might see an increase in your tax return you might not it really depends on what your W2s look like right because again everybody pays different amounts in federal taxes those of you all who claim zero all year um you might want to stop doing that because again people who claim zero all year normally you all owe you are welcome Welcome, Alan. Thank you for waiting and being patient cuz I saw your question come in, but I was talking and looking over here at the YouTube uh screen and channel. So, Miss Dos, you said the link won't work, huh? I don't know what's going on. We'll I'll type it in the um I'll type it in the comments. I'll type it in on here. So then that way you could just click it. PL Stewart PL Stewart. But it's that time of the year, so I'll be like back on the back on here doing these live sessions with you all from time to time. [clears throat] Uh they'll be short. Like I say, I give more information in the private community. I have gone into community. We've been on the internet for free for 10 plus years. So now I only focus on people who are serious and people who serious get into the community. Uh, okay, Miss Doss, I just typed it in the comments, so I don't know if it gonna come up right away then. There you go. Oh, and I didn't send it to you. I didn't text you either yet, Miss Dawson. I'm I'mma text it to your phone. I got distracted once we got off the phone. So, I'll send it to your phone cuz I told you I'll text the link to you. Um, okay. I knew YouTube has somebody else. YouTube, y'all always got questions. That's why I love y'all. Uh, how often do we meet in the private community once subscribed? So we meet weekly and then I also put video content up in there as well. So we drop video content and when you join it's it's about 40 different modules in there already for you to watch. So when you join the community it's already 40 different modules in there but that's all from last year. So now I'll be updating um you know more newer information for you. But in the private community, if I don't come on, then we have a guest speaker or somebody else come on. But at minimum, I go live once a month at minimum. But you do we we do normally meet weekly. I do have another coach in there, Chuck Finance. He's in there. So, he does study hall. Um, and then we normally do an interview with a professional to teach you all and educate you all on a different type of topic. So, 2026, we got a lot planned and to roll out. So, the biggest thing that I'm working on for 2026, which I'm really excited about, is my male community. You my YouTube channel is mostly 75% men. And we have 75% men as followers and 25% women. So, I am very big with educating the men, the male. We need the men fully aware, fully financially handsome. If you all remember, I had these shirts, financially sexy for women, financially handsome for men. Um, but this year, 2026, I am completely focused on making more men financially handsome. I am tired [laughter] tired of this whole back and forth 5050 conversation that I see online. Um, a lot of the young guys are driving their girlfriend car, lived in their girlfriend house. So, my goal is to empower more men financially. Um, so I'm really excited about that and especially in the sports and entertainment space. Um, so I definitely have some things that I am working on that we'll be rolling out. Um, and I'm actually going to be hosting a workshop for the male youth. So, if you have a son that's between 13 to 19, within the next 30 days, I will be talking about that. Um, I know it's sports, so I'm trying to figure out and talk to a couple of men on what's the best day to host this in-person workshop, but I am hosting an in-person workshop here in Chicago for the male youth between the ages of 13 to 19. Um, and it's a course. It's a ongoing course. It's not a one-time thing. This first event will be a one time a one day event but moving forward it will be an actual um course a 8 to 12 week course where we are empowering the male youth regarding different financial topics and setting up their retirement account making sure that they understand credit business entrepreneurship um it's a lot geared towards women got everything women empowerment this women empower department that, but I don't really see a lot of information out here for the men and specifically talking to the men. So, I'm meeting with two great fellas this weekend to help me um finalize the curriculum for the course so we can make sure that it's something that the men will, you know, take away from it and get out of it. But yeah, that's that's that's the thing for 2026. I'm I'm real excited to hear about I'm really excited to push this whole program out because this will be nationwide. Y'all will eventually see me traveling from state to state to different locations to talk to the men and the male youth specifically. I'm only focusing on men. It will not be females in these classrooms. It will only be men. So, if you in Chicago and you have a young son that is between 13 and 19, he needs to be in the room. All right? He needs to be in the room so he can learn this. Learn how to get this money, baby. All right? Learn how to get this money cuz once we have the men empowered, once all of our men are back empowered financially, then we can get back get back in equilibrium as a community cuz everything is off whack right now. All right. That's why I said boy my god baby 23 and she talking about her friends friends boyfriends and how are these boys living with girls driving girls cars like nom. I'mma need y'all to get y'all weight up fellas. So we going to focus on that. We're not going to talk about the men. We going to empower the men. So I'm ready. Let's go. Let's roll. Doing that would definitely help provide structure. Exactly. You see another that's the whole point, right? That's the whole point. We we need we need to bring back structure and order. And I'm I've always been a person that's about how do we change things? I'm not a complainer. I'm not on here complaining about nothing. Uh I'm always in how can we fix this, right? What's what can we do? So me being in financial services for the last 23 years, that's what I know that I could do to help out, right? That's what I could do is help share the knowledge and information that I have to the men and also guide you through it. Right? We're helping you set up your investment account. We helping you fix your credit. We helping you start your businesses. Um I got two clients that I helped last year in Florida do they NIL deal. Right? So again, I'm really focusing on the male youth and especially the ones that are in sports and entertainment. Um because I feel like we have a huge need there. If we have 30 boys in a room, the reality is one of them is going to the league. The other 29 is not. Right? So in my mind, y'all setting these kids up for failure because what are we doing if you only teaching them to do football and basketball and you know in a room of 30 kids only one is going to the league the other 29 what are we doing? Right? So in my mind I'm like this this is whack. [laughter] We need to fix this. That's a problem. Right? So, for me, that's that's one of the things I'm going to do. And it's a it's an untapped market. I have literally talked to about 50 different coaches, mentors, teachers, educators, men that work with the male youth already. And I literally asked that question, do you have a financial literacy program for these young boys? And they, every single one of them, right hand to God, every single one of them said no. Every single one. 50 coaches. And that's just in Chicago or the South Suburbs. 50. Every single one said, "No, we do not have a financial literacy program." Baby, how? Why? Okay. Well, here I am. Let's get it going. Let's start it. So, if you are a male or know a male and you got friends that's coaches and all that, tap in. get with me cuz I will be moving around. I'mma start in Chicago, but the goal is to definitely at some point this year, travel to other states, travel to other cities, get in the room with you all, get in the room with these young men. Um, and teach them cuz it's it's time. It's overtime. Exactly. [laughter] I like that. Uh see another you say we need more trays and less dough boys. Exactly. Exactly. Exactly. We need way more trades and less dough boys. And college and and all of that is not for everybody. You know what I'm saying? Every young man doesn't want to go to college. But we also have trades. We don't talk about that enough. And we actually have a lack of men, specifically black men in the trades. I have a friend that uh he runs the program for the trucking, no for for the electrical um apprenticeship for com. And he said the last what probably four [snorts] years it's like no black men in there. Like all Hispanic. It's like I think he said the last class that they did it was one black man in there. That's crazy. You know, some of these classes have 50 to 75 people in them and we only and you only got one black man to learn electrical to learn electrical trade. That's crazy to me. Crazy. So, we need to start having these conversations. And on that football field, in that basketball field, there's like a hundred other positions, right? I just said only one of them go into the league. Everybody can't be a quarterback. Everybody can't be the line running back or whatever these, right? It's it's so many other positions within that same industry. But why are we not talking to these young men about that? Right? Why are we not talking about that? Why are we not empowering them to do more? cuz I have seen so many grown men who were once young boys trying to go to the league and once they don't make it to the league they depressed and then their life is over. They don't do nothing else. They don't do nothing else with themselves. That's horrible. So that's why I said when I reached out to those men and asked them about if they have a financial literacy program for their um you know mentees and and all 50 of them said no. I knew then that that was a need that that was a need that needs to be serviced. So I'm excited to to service it. Let's get in the room and change some lives. What's Dawson see another? I'm still learning. I don't know sports too well. I got a I still I'm still learning a lot since I'm about to be talking to these kids. I've been studying and learning some stuff. But what's at Dawson? Is that a location or a school? I saw somebody say something about their sons. Dedra, you said, "Love that for the boys. Our young men need this. I have two sons. I hope they will be able to participate. So that's what I really need to find out like if I wanted to host a workshop within the next 30 days like it would is a Saturday. Okay? Cuz I know a lot of you all I don't have kids so I don't know when y'all are practicing. Are y'all practicing? Are they practicing on Saturdays? You know, uh Sunday everybody sitting there watching football. So I don't want to do a Sunday. But I need to find out from these coaches that I'll be reaching back out to this year as far as like what's the best day to do that? If I did an hour workshop once a week, every you know once a week for an hour to two hours, what would be the best day to host that? Right? So that's that's been my biggest question now is like what would be the best day to provide that service to them. And I do actually have a fullfledged 501c3. So I will be on here at some point asking y'all for donations and donors because again we need to get this information to the kids and the youth. Um, but yeah, 2026 we rolling. So, Dedra, I'll be posting more about it. I'm getting ready to sit down with two fellas this weekend that I'm meeting on Sunday. Um, so probably on Monday, I'll be talking more about an actual date, but the goal is to have our first one day event within the next 30 days at minimum. within the next 30 days. And I'm open to it could be the evening, it could be, you know, a weekend. I just don't know what's what is the best what's a good day to do this for those of you all that are in sports and entertainment. So, Dedra, if you got two sons, then let me know that. Give me that feedback. What day will they be available to meet for one or two hours to learn this information? And the program is called financially handsome because again we are changing it's raining like casting dogs right now. Jeez. We are changing the mindset of the youth. Changing the mindset of the youth. Okay. You say Dawson is the tech school on 39th and state. Okay, let me write that down. Somebody gave me the le the um somebody gave me the information to Leo, the principal at Leo High School on 79th Street. So, 39th in State Dawson. I'mma write that down. Dawson Tech. Thank you. C Nether. Yeah, they gave me Leo High School infor</t>
+          <t>So, let's look at our little uh recipe. And we're going to what we're going to do is make we're going to blend it and we're going to drink it hopefully. Uh and we're going to make oursel it's called Graham's Liver Love Smoothie. So, we're going to begin with two large sprigs of parsley. Now, of course, you've heard me talk about parsley previously. I'm going to put more than two. I'm going to put this much in there. Slightly more than two. So we've put that into our into our blender. Uh parsley the story of course uh one of the most powerful kidney supporting herbs um but also a source of glutathione and hence we're using it in this blend but at the same time we're going to be supporting uh kidney health. One of the most powerful tools to boost kidney health. Uh a mediumsized beetroot which we'll cut up now. There it is. Okay. So, I'll just take the bit of the rough stuff off and throw it over the edge. And we'll cut up our beetroot and put the beetroot into the mix. Wonderful food. Of course, this is antyanins, this wonderful purple pigment. And we're even going to go one step further with this model. We're going to put in as our beetroot. We're going to put in some beetroot leaves. And who would have thought that the beetroot leaves have almost as much nutrition as the beetroot? Apart from folic acid, they actually have as just as much. You can see that purple color. And we're going to put some of that in there. Then we're going to put out three kale leaves. This is the kale that was produced during my little garden segment. If you recall, we showed you how with kale on his broad fork. Uh how quickly you can put a garden in. And this is the wonderful kale that that came from that. I'll cut that up a little bit. We got quite a lot into this. This is quite a big I might have overdone it, but we'll see. Um, so we've got our beetroot, our kale, we've got our avocado coming up. Thank you. We'll scoop out the avocado goodies. of course this wonderful range of fats in avocado that was kind of unparalleled but a very good source of glutathione and of course it was demonized the fat and in and avocado at one point and then we realized oh my goodness it's one of the best fats you can possibly eat and it's something you never get sick of I mean I eat avocado every day and I've never yet got sick of it now whey protein concentrate we're talking about so we'll just undo this and we'll put a tablespoon of that is how much we've got for this a heap tablespoon of whey protein. We'll put that into the mix. Quite a quite a heap tablespoon. We're going to put our bruised garlic. So, let's open our garlic, our Australian garlic, our wonderful Australian garlic. And let's get ourselves a couple of cloves. And of course, we got to quickly peel them and bruise them. And how am I going to bruise them? I'm going to bang them with this honey jar. That's done the job. That's one bruised clove. I'll just get a second one. Big cloves. These lovely Australian garlic. I'm hoping I produce something similar this year myself. Bun crop to grow. I love it. Give it a bruise. That's good. Bruise garlet. Leave it sitting there for a few seconds. Get all It's going to get well and surely oxidized in a moment. Um, now where are we at? We're talking about whey protein, a calcul of course. How much curcul is it? A heaped teaspoon. So here's our calcul. It's combination of turmeric and pepper. And we're going to put a decent heap teaspoon in there. Then we've got milk thistle, which we don't have, but we do have our little bit of capsicum for the capsicum. this jalapeno and we'll hope that it's not going to be too hot but I won't put too much in there in case it it really burns us up. That might do us. This is a touch of capsic as we mentioned the substance that activates glutathione. The broccoli sprouts we don't have but and we don't have the milk thistle tablets or milk thistle powder. Um, so you can imagine that you put those in there. And then we're going to add our bit of water, a glass of water. Hopefully that's enough. It might not be. And we'll get this show on the road. And we'll just make ourselves a smoothie. Now, let's see if we can get this going. What we'll do is we'll just add ourselves a little more water. Thank you. Add a little more water cuz she's a bit too thick. That's better. Now, of course, the idea of making a green smoothie is you need to have one of these high power. This one's many years old. I've made many smoothies in it life. Um, this is Vitamix from the US. This blend from Germany. Now, you need these two horsepower blenders to do it as quickly as you can because you don't want it to go on forever and you want it to be genuinely micronized. So, let's just finish it off. &gt;&gt; Okay. Okay. So, let's have ourselves a really thick. We could have made it a little thinner than this, but let's see what it tastes like. You'd make it a little more runny. We put another half glass of water in there. But let's taste. Yeah, I reckon we should have put a bit of It's actually pretty nice. Um, yeah, I have a taste. &gt;&gt; Yeah, &gt;&gt; you could have put a bit of fruit in there if we wanted to sweeten it up a little more, but that's that's pretty palatable. You can almost taste it, feel it going to work on the liver. Thank you. So, that's how you make a liver love smoothie. and we'll move on and talk about a few other things relative to how you can live a longer just clean my mouth off longer happier healthy life. We're going to talk about a gut health understand how important your gut health is. We've talked about the need for probiotics but we're going to talk about something called buteryrate at this point and why is it important? It's really important because bowel cancer is the fourth major cause of premature death and fiber is hugely important as you as you all know. Now let's talk about the dynamics of how this thing works. So we have this thin layer of epithelial cells that are interconnected. These cells are connected by structures that are called kite junctures and that keeps the gut contents whatever you've eaten from entering entering uh moving through into your blood system. holds everything in there basically. So these epithelial cells exude this mucous material. It's called the mucous layer and that's really protective. It protects against microbial pathogens against enzymes, acids and food associated toxins. Now when we move down to the colon which is part of what we're going to talk about here um in the they're called colonosytes these same epithelial cells and they have to be energized because they got this really important protective function and what they use to derive their energies. In the top half of your gut it's glucose that gives the cells the energies the epithelial cells their energy to do this really important protective role. But in the bottom half, there's these things called shortchain fatty acids. And they come from certain types of fiber in the colon. And that's really important because the colon's replacing its every four days, the cells are. And the most important by far of those short- chain fatty acids is called butyric acid or butyrate. Now, let's look at the roles of butyric acid or butyrate. Butyrate is anti-inflammatory. Um, so this is huge for people with bowel issues, things like irritable bowel or that very painful condition called colitis. Um, massively important IBS and colitis. Um, that you're producing good amounts of this anti-inflammatory called butyric acid. It increases mucosal secretion when that reduces the pathogenic bacteria that can grow uh and and it also produces some antimicrobial peptides. So, it's got quite protective in that context. Um, it's an immune enhancer, butyric acid. It activates anti-inflammatory immune cells in the colons. Again, really important for things like irritable bowel syndrome. It sponsors glutathione production. We've just talked about how important that was. High levels of butyrate produce high levels of glutathione, which gives you even more protection from some of those inflammatory bowel diseases and bowel cancer. It combats type 2 diabetes. Several people papers have demonstrated that butyrate or butyric acid increases the production of hormones that improve blood sugar balance. So you know one in three of us have got poor blood sugar balance which makes us pre-diabetic and the experts are telling us that diabetes is becoming plague. So that sounds like a good thing to look at. But what's fascinating is its role in terms of cancer. that can specifically target can cancerous cells in the colon and reduce their energy and eventually initiate what's called apoptosis which is cell death. So there's a very famous p paper by Anna Han and some of her colleagues in the cancer journal called enco target and she demonstrated that butyrate this is quite unique because it's not a common thing in nature but butyrate can seek out the cancer cells and then it shuts down their capacity to utilize butyrate as an energy source. So it shuts down the capacity of this thing to to take itself in which is kind of like not a very common thing and uh that then reduces their energy and and eventually leads to their demise. So it's unique where a substance actually shuts down the capacity for its own utilization. That makes it quite a special substance. So how can we spike the production of butyric acid this very very protective thing in our bowel? One of the most powerful uh is to bring some resistant starch into our diets. Uh basically resistant starch also has a major impact on insulin sensitivity and a study published in the journal of nutrition by Kevin K. Mackey uh showed a 33 to 50% improvement in insulin sensitivity in just four weeks by eating 15 to 30 grams of resistant starch a day. And I'll explain what that is shortly and you'll understand that it's not a hard thing to do. It's actually thought to be resistant starch, a major tool to avoid chronic disease and improve life quality. So, what's ideal? 25 to 30 grams a day. What do Australians eat? Six grams a day. What do Americans and Europeans eat? 5 grams a day of resistant starch. What do the Chinese have? 15 grams. Still not where you need to be, the 25, but 15 grams. And they've got much less obesity. You've all seen it. And they have far fewer digestive issues. So fairly good argument for bringing in some resistant starch. So how do you do it? It's called the cook and cool concept. If you cook potatoes and then you store them in the fridge for a minimum of 12 hours, that high starch since potatoes aren't actually particularly good because they spike sugar more than table sugar. You know, the GI of potatoes is 95. Pure white table sugar is 70. So potatoes are not good from that perspective. Sweet potatoes, no problem. They've got the fiber component. They break down much more slowly and they've got a GI of just of 35. So sweet potatoes, you can eat what you like, but potatoes do spike blood sugar, spike insulin production, speed cell division, and shorten your life, basically. So, is there a better way to eat them? Yeah, there is. Uh, you have potato salads. Now, you say, "Oh, you I can cool it down, then I can slice it up and have it for chips." No. uh as soon as you've warmed it up again, you've changed the resistant starch back to that super blood sugar spiking form of uh refined carbohydrates or or carbohydrates that spike blood sugar very quickly. So, potato salad, you leave it cold. Um preferably don't fill it with mayonnaise, a good dressing, pumpkin seed oil if you've ever had it. It is incredible. And of course, it's jam-packed with zinc, balsamic vinegar, and a lot of black pepper, you know, and put that on your potato salad. It's beautiful. Now, that cook and cool concept can extend to things like rice and pasta. This rice salads, part of the Mediterranean diet, which is noted for its longevity. And of course, the Japanese got it right with the wonderful thing called sushi because not only is it based upon white rice, um, but it's wrapped in that beautiful all 74 minerals, including very high levels of iodine, that kelp uh jacket that's wrapped around the sushi. And then they put things like wonderful things like avocado and high omega-3 salmon. And really it becomes a very very healthy diet that could be part of your 25 grams uh of resistant starch on a daily basis. So let's just talk back on that uh on that layer u because the epithelial layer because when we talked about those strong junctures which are the barriers between the epithelial cells and without butyrate without butyric acid they can become weakened but there are some other players that perhaps we should think about and try and avoid. Uh antibiotics kill the organisms that produce butyrate. So that can be really counterproductive for gut health and and and le make you more likely to suffer from this leaky gut where things from your gut go into your blood system and there are a whole bunch of side effects that come with that. Uh non-steroidal anti-inflammatory drugs like a ibuprofen are major place because they shut down the protein messages that govern the interchange of gut cells because every four days you're supposed to have new ones and there's a message that's shut down by ibuprofen so you don't replace them and so they get tired and weak. The old cells become weak and that weakens the junctures to create intestinal permeability which is also called leaky gut. So what are the symptoms of leaky gut? Tick the boxes. Tiredness after eating. This is why people hate the afterdinner presentation uh when you're giving seminars because that's the point where people because there's a lot of energy anyway involved in digestion but if you've got leaky gut you get really tired and you see the people uh droop off. I try and keep things entertaining enough so that doesn't happen and thankfully it's quite rare but it does happen occasionally. You're going to have things like sore joy. You're going to have things like eczema skin conditions. You're going to have poor immunity, headaches, brain fog, memory loss, anxiety and depression, ADHD, multiple autoimmune diseases. All can be linked to this condition called leaky gut. So that's just a little thing and we want to we want to keep our butyric acid up. So the resistant starch is really important in that context. And finally, we're going to talk about something called lectins. Now, you may have heard of them. There's a guy called Dr. Steven Gundry who's everywhere at the moment, who's sort of an expert talking about how lectins can be linked to leaky gut, to heart disease, to autoimmune diseases, and the very important neurodeeneration. He's seen a 90% of his autoimmune patients improve just by removing these things called lectins from their diet. So, what what contains high lectins? Well, the nightshade family. So that's potatoes, capsicums, eggplants, and of course the big one which is tomatoes, uh beans, pulses, whole grains, and so forth are all part of the lectin story. So just continuing the lectin story. So you might have all heard about the Mediterranean diet and it's linked to enhanced longevity, but you might have wondered perhaps why do they go to such great lengths to remove the tomato skins, uh to remove the seeds when they make the tomato sauces and so forth. And that's where the lectins are. The lectins are in the skin. They're in the seeds at high quite rate. So, so what the Italian dishes do is that they utilize tomatoes as lycopine and some other wonderful benefits including high vitamin C, but they remove the negatives, the seeds and the skin. So basically in beans, they soak them for 24 hours on the Mediterranean diet uh to remove the lectins and they change the water every four hours when you're soaking them. So it's a few changes over 24 hours, six or seven changes cuz you can't do it when you're sleeping. Now part of the sourdough story is that the so process removes the lectins. Um so basically when we're talking chili peppers, capsicums, eggplants, at least remove their seeds and ideally remove their skin. And one other really cool tool um to reduce lectin content of any food is to use a pressure cooker. It's become, you know, a real tool in trade and it's fairly popular amongst amongst the Steven Gundry and his strategies to reduce your lectin content and reduce your inflammation. And I think it's worth many people visiting that idea. I was in Rockampton uh with a couple on a farm where they grow loose and a few other things. And the the the farmer himself was telling me that he was so crippled that he couldn't even pull things out of the fridge without dropping things um with just this arthritic kind of condition. And someone suggested why don't you just try cutting out the night change, cut out the tomatoes. He's a very big tomato eater and it took about five to six weeks and his pain disappeared. So, it's probably something worth trying if you've got inflammatory conditions because tomatoes that night family can on some people have quite a strong appeal and it may well be linked and probably is linked to that lectin component. So, I hope there's something of value for you there. Thanks for watching. [music]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -812,135 +1020,320 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>geilOn3K8ks</t>
+          <t>HrRSKP7YE5Y</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART is live!</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Liver Strategies - Turmeric, Garlic &amp; Broccoli Sprouts Heal Liver Damage - How to S4E12</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Welcome back to another episode of the *How To Do It* series 🌿🧠
+Where Graeme explores one of the most essential — yet often overlooked — organs in the human body: the *liver* .
+*#LiverHealth #Detox #Nutrition #HowToDoIt #Glutathione #HealthTips #Wellness*
+While heart disease dominates many health conversations, this episode explains why the liver may be the primary organ of survival, responsible for detoxification, antioxidant production, metabolic balance, and long-term vitality. Research suggests that *one in fourteen people* may already be living with undiagnosed liver fibrosis — a condition that often progresses silently until serious damage has occurred.
+*So, how do we protect the liver before it reaches that point?*
+Graeme introduces the idea of *“learning to love your liver”* through practical, evidence-based nutritional strategies that support the body’s natural detoxification and repair systems. A key focus is placed on *glutathione* , the body’s master detox molecule, and the nutrients that support its production.
+*In this episode, you’ll learn:*
+🍊 Why *vitamin C* supports *glutathione* and antioxidant defences
+🧪 The role of *selenium* in liver protection
+💊 The benefits of *turmeric* , *milk thistle* , and *alpha-lipoic acid*
+🥦 How *broccoli sprouts* supply sulforaphane
+🧄 Why *garlic-derived allicin* stands out medicinally
+Graeme also outlines a simple liver-supporting *green smoothie recipe* designed to reduce oxidative stress and support detoxification.
+Your liver works tirelessly every day. This episode shows you how to work with it 💚
+👉 *Don’t forget to like, share, and subscribe* for more Nutrition Farming® insights with Graeme Sait.
+👇 *Chapters:*
+00:00 - Introduction
+01:28 - Title Sequence
+01:58 - Liver Fibrosis
+02:53 - Sulphur Compounds: Glutathione - Glutamine, Cystein &amp; Glycine
+04:14 - Vitamin C
+06:05 - Whey Protein Concentrate
+07:05 - Turmeric - Curcumin &amp; Pepperine
+07:51 - Milk Thistle Extract
+08:27 - Selenium
+09:26 - Alpha Lipoic Acid
+10:49 - Sulphurafane
+12:34 - Garlic - Alicin
+16:17 - Smoothie Wrap Up
+16:30 - End Credits
+Want to learn more about natural health tips?  Check out: Prebiotics, Probiotics &amp; Alcohol: Gut Health Tips You Need to Know - How to S4E2
+https://blog.nutri-tech.com.au/prebiotics-probiotics-alcohol-gut-health-tips-you-need-to-know-how-to-s4e2/
+*Relevant NTS Products Featured in This Episode:*  
+_BioSpark_
+https://www.ntshealth.com.au/products/biospark
+_Curcu-Life_
+https://www.ntshealth.com.au/products/curcu-life
+_Green Defence_
+https://www.ntshealth.com.au/products/green-defence
+_BioBubble™ Probiotic_
+https://www.ntshealth.com.au/products/bio-bubble
+_MagSorb™ Magnesium Spray_
+https://www.ntshealth.com.au/products/magsorb
+_Nutri-Salt_
+https://www.ntshealth.com.au/products/nutri-salt
+_SweetSure_
+https://www.ntshealth.com.au/products/sweetsure
+*Interested in studying Nutrition Farming?*  
+Certificate in Nutrition Farming courses:  
+https://nutri-tech.com.au/pages/courses  
+Need personalised support?  
+Soil &amp; Plant Therapy Services:  
+https://nutri-tech.com.au/pages/soil-plant-therapy  
+Book a one-hour online consultation with Graeme Sait:  
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
+*Explore more at our website:*  
+https://nutri-tech.com.au/
+Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
+https://nutri-tech.com.au/pages/newsletter  
+*Follow us on Social Media:*  
+Facebook: https://www.facebook.com/NutriTechSolutions/  
+Instagram: https://instagram.com/nutritechsolutionsyandina  
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
+X (Twitter): https://x.com/ntsaustralia</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-01-06T19:58:45Z</t>
+          <t>2026-01-23T04:30:09Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>868</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.096692</v>
+        <v>0.028802</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>TUNED IN sister,❤ Happy NY, EVEN though the REAL New year is April || HAPPY NEW BEGINNINGS to you and your family Queen P.! || Happy New Year Rodney || 1:23:33 I agree || 💪🏾💪🏾 || Girl! You look so cute! Love your hair!!! Mad I missed the live.  Hope you’re well! || Thank you 🙏🏾 ❤ happy new year! Beautiful and I’ll be on tonight</t>
+          <t>Oh poo - video finished before Graeme could make the smoothie! || It was a too long for one episode, so you will have to come back for Part 2! || OK.... Where is part 2?</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>maZLr_qFnuM</t>
+          <t>XVTBG1xVe4Q</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Vision Boards are DEAD! Action Board or Fail in 2026 😱 (Free Workshop TOMORROW) #patricelstewart</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>Cancer Strategies: How to Build a Body That Protects Itself - How to S4E11</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>In this *How To Do It* episode, Graeme Sait explores *#CancerStrategies*, *#ImmuneHealth* and *#MetabolicHealth* — sharing calm, biology-first insights into nutrition, minerals and lifestyle choices that help the body build real resilience 🌱🧬
+Filmed high on the ridge at Nutrition Farms as the sun sets 🌄, this is a thoughtful, grounded conversation about a subject most of us would rather avoid — and yet one that touches so many lives.
+Rather than fear, hype or miracle claims, Graeme gently reframes the discussion around *how the body is designed to protect, repair and restore itself* when given the right conditions. It’s about understanding biology — not fighting it.
+Throughout the episode, themes of *metabolism* , *inflammation* , *immune strength* and *detoxification* are woven together as parts of a beautifully connected system. Small, consistent choices around food quality, mineral sufficiency and gut health can profoundly influence how well that system performs.
+There’s a strong emphasis on working *with* the body 🤝 — reducing unnecessary stressors, supporting natural clean-up processes, and creating an internal environment where healing is more likely to occur.
+This episode isn’t about quick fixes. It’s about *informed choices*, *long-term thinking*, and reclaiming a sense of agency over your health.
+Whether your focus is prevention, recovery, or simply living with greater awareness, this is a calm, empowering conversation that brings health back to first principles — biology, balance, and common sense 🌿
+👨‍🌾 *Stay tuned* for more practical, science-driven insights in future episodes of the *How to Do It* series.
+👉 *Don’t forget to like, share, and subscribe* for more Nutrition Farming® insights with Graeme Sait.
+👇 *Chapters:*
+00:00 - Introduction
+01:09 - Title Sequence
+01:39 - Sugar &amp; Insulin
+03:01 - Sulforaphane
+03:59 - Omega-3 &amp; Cod liver Oil
+04:53 - Naltrexone
+05:52 - Plant-Based Diets
+06:42 - Boosting the Immune System
+07:22 - High Dose Vitamin C
+07:55 - B Vitamins
+08:39 - Selenium
+09:40 - Glutathione &amp; Whey Protein Concentrate
+10:00 - Zinc &amp; Immunity
+11:03 - Magnesium &amp; Relaxation
+11:37 - Bone Broth
+13:26 - Herbal Teas - Soursop &amp; Herb Robert
+14:46 - Autophagy &amp; Time Restricted Eating
+16:18 - Summary
+16:32 - End Credits
+Want to learn more about natural methods to deal with cancer?  
+Check out Gold from the Vaults - Episode 7 - Jerry Brunetti - Food as Medicine: Natural Cancer Treatments Part 1  
+https://blog.nutri-tech.com.au/gold-from-the-vaults-episode-7-jerry-brunetti/
+*Relevant NTS Products Featured in This Episode:*  
+_BioBubble™ Probiotic_
+https://www.ntshealth.com.au/products/bio-bubble
+_MagSorb™ Magnesium Spray_
+https://www.ntshealth.com.au/products/magsorb
+_Nutri-Salt_
+https://www.ntshealth.com.au/products/nutri-salt
+_SweetSure_
+https://www.ntshealth.com.au/products/sweetsure
+_BioSpark_
+https://www.ntshealth.com.au/products/biospark
+_Curcu-Life_
+https://www.ntshealth.com.au/products/curcu-life
+_Green Defence_
+https://www.ntshealth.com.au/products/green-defence
+*Interested in studying Nutrition Farming?*  
+Certificate in Nutrition Farming courses:  
+https://nutri-tech.com.au/pages/courses  
+Need personalised support?  
+Soil &amp; Plant Therapy Services:  
+https://nutri-tech.com.au/pages/soil-plant-therapy  
+Book a one-hour online consultation with Graeme Sait:  
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
+*Explore more at our website:*  
+https://nutri-tech.com.au/
+Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
+https://nutri-tech.com.au/pages/newsletter  
+*Follow us on Social Media:*  
+Facebook: https://www.facebook.com/NutriTechSolutions/  
+Instagram: https://instagram.com/nutritechsolutionsyandina  
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
+X (Twitter): https://x.com/ntsaustralia</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-12-27T04:00:49Z</t>
+          <t>2026-01-09T04:32:57Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>519</t>
+          <t>1114</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.181118</v>
+        <v>0.044883</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Thanks for sharing.  Will you have a workshop for those interested in starting a business? || Never-ending I just went to your website. Thanks again 😊 || 💯</t>
+          <t>Can you recommend a specific cod liver oil without a guaranteed analysis? || I have reached out to Graeme for his specific recommendation. From my research Rosita's is a highly recommend natural source,
+https://www.amazon.com.au/Rosita-EVCLO-Softgel/dp/B09B7BGZDD || @NutriTechSolutionsNTS Thank you so much :). I'm a banana farmer in Hawaii. Are you guys still doing online consults? || Great one again - thank you and I found the sound good || Thanks @markhiggins3054! || Really appreciate the content, but please.......please....address the sound quality issue. || Thanks, we are glad you appreciate the content! Can you explain the sound quality issue? as it sounds fine on my devices. || The voice sounds muffled</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0P2PYQhmnEU</t>
+          <t>jl2LucE_jhc</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>See you on Dec.27 @1pm CST!!   #patricelstewart #business  #chicago</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>Visual Soil Assessment: Simple Tests Every Farmer Needs - How to S4E10</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>In this episode of *How To Do It* , we explore *visual soil assessment* , soil structure, biology, and practical field tests that reveal true soil health — straight from the paddock.
+#soilhealth, #regenerativeagriculture, #visualsoilassessment, #soilbiology, #soilstructure, #organicmatter, #earthworms, #microbiallife, #nutritionfarming, #regenerativefarming, #agronomy, #farmingeducation, #soilcarbon, #soilresilience, #soilaggregation, #sustainablefarming, #howtodoit, #nutritechsolutions, #graemesait, #biologicalfarming
+Joining me today is Marco, Head Agronomist at Nutri-Tech Solutions, as we return to the farm where his agronomy journey began. Together, we walk through a *practical, hands-on approach* to understanding soil health using visual soil assessment techniques.
+Rather than relying solely on chemistry, we dig into the *physical foundations* of soil performance — texture, structure, porosity, colour, aggregation, and earthworm activity. You’ll see how compost, humic substances, mulch, and biological management dramatically change soil outcomes, even over short distances.
+Marco demonstrates simple field tests, including the ribbon test, soil texture jar test, slaking test, and earthworm counts — revealing how biology drives aggregation, water infiltration, oxygen movement, and nutrient efficiency.
+This episode highlights why soil structure is the gateway to productivity, resilience, and water-holding capacity — and why biology-first management delivers compounding returns over time.
+👇 *Chapters:*
+00:00 - Introduction - Brewing
+01:27 - Title Sequence
+01:57 - Soil Texture
+05:52 - Soil Structure
+10:31 - Soil Porosity
+12:43 - Earthworm Counts
+13:57 - Slaking Test
+15:36 - General Biodiversity
+16:15 - Why is Soil Structure so important?
+18:31 - The Importance of Mulch &amp; Microbial Foods
+20:09 - End Credits
+Visual Soil Assessment Guide: https://cdn.shopify.com/s/files/1/1213/7046/files/Visual_Soil_Assessment_VSA_Workshop.pdf?v=1766715528
+For a deeper dive into the principles behind aggregation, biology, and soil resilience, this article pairs perfectly with today’s episode: Gas Exchange – How to Maximise your Money Maker - https://blog.nutri-tech.com.au/gas-exchange/
+*Humate Granules*
+https://nutri-tech.com.au/products/humate-granules
+*Life Force® Gold Pellets*
+https://nutri-tech.com.au/products/life-force-gold-pellets
+*Brewstar 200™*
+https://nutri-tech.com.au/products/brewstar-200
+*SeaChange® Liquid Kelp*
+https://nutri-tech.com.au/products/seachange-liquid-kelp
+*FulvX™*
+https://nutri-tech.com.au/products/fulvx
+*Interested in studying Nutrition Farming?*  
+Certificate in Nutrition Farming courses:  
+https://nutri-tech.com.au/pages/courses  
+Need personalised support?  
+Soil &amp; Plant Therapy Services:  
+https://nutri-tech.com.au/pages/soil-plant-therapy  
+Book a one-hour online consultation with Graeme Sait:  
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
+Explore more at our website:  
+https://nutri-tech.com.au/
+Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
+https://nutri-tech.com.au/pages/newsletter  
+*Follow us on Social Media:*  
+Facebook: https://www.facebook.com/NutriTechSolutions/  
+Instagram: https://instagram.com/nutritechsolutionsyandina  
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
+X (Twitter): https://x.com/ntsaustralia</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-12-23T18:53:17Z</t>
+          <t>2025-12-26T04:30:37Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>1426</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -950,284 +1343,554 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.13806</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>💯</t>
-        </is>
-      </c>
+        <v>0.025245</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>gwE_NQhSfAE</t>
+          <t>mGeeAsi5p0g</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The PROFIT &amp; LOSS STATEMENT: all the basics in 5 MINS! #patricelstewart</t>
+          <t>Expert Nursery Owner Spills REAL Secrets on Farming! Pt2 - How to S4E9</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hey! This video provides a clear visual guide to your `profit and loss statement`, a crucial component of your `financial statements`. Understanding this document is vital for effective `accounting` and accurate `business tax preparation`. It's especially important when preparing your annual `tax return`, helping you manage your finances with confidence. 😊</t>
+          <t>Welcome back to another inspiring episode of the *How To Do It* series.
+This week, we’re visiting the Sunshine Coast’s remarkable _Eumundi Palms Nursery_ — a commercial nursery proving that *biological farming,* *chemical-free growing,* and *plant resilience* can outperform conventional systems while using significantly less water.
+#howtodoit, #biologicalfarming, #chemicalfreefarming, #regenerativeagriculture, #commercialnursery, #cocopeat, #trichoderma, #plantresilience, #beneficialmicrobes, #sustainablehorticulture
+In this episode, Graeme is joined by _Phil,_ founder of Eumundi Palms, to explore how a curiosity — growing a palm in a palm — led to the adoption of pure coconut fibre as a potting medium and the rapid transition away from systemic fungicides.
+We unpack how coco peat’s moisture-retentive structure creates the perfect environment for beneficial biology, particularly _Trichoderma,_ which thrives in fibrous media and provides both disease suppression and strong root stimulation. The result? Healthier plants, reduced water use, and the ability to access premium chemical-free export markets.
+The conversation then turns to *cell wall strength* and true plant resilience. Silica, calcium, and boron play a central role in strengthening plant architecture, improving stress tolerance, and reducing pest and disease pressure. You’ll also hear how advanced biological tools like _BAM_ and _MAD (Micro-Amino Drive)_ improve nutrient uptake efficiency and overall plant vitality.
+Beyond the agronomy, Phil shares the human side of Nutrition Farming — protecting staff health, building a committed long-term team, and involving the next generation in a business they’re proud to inherit.
+Whether you’re a grower, nursery operator, agronomist, or passionate home gardener, this episode offers practical insights into how *biology replaces chemistry* when we work with nature, not against it.
+👇 *Chapters:*
+00:00 - Introduction  
+01:16 - Title Sequence  
+01:46 - Coco Coir, Trichoderma &amp; Moisture Retention  
+04:09 - Cell Strength: Silica, Calcium &amp; Boron  
+06:02 - Beneficial Anaerobic Microbes &amp; Micro Amino Drive  
+08:04 - Export Markets  
+08:56 - Industry Adoption of Nutrition Farming &amp; Family  
+12:21 - Practical Application of Nutrition Farming  
+14:38 - The Importance of pH  
+15:28 - Walk &amp; Talk: Healthy &amp; Resilient Palms  
+21:52 - End Credits  
+Want to learn more about the role of silica and calcium in building resilient plants?  
+Check out Graeme’s article on the NTS blog:  
+_Sili-Cal (B)™ — a unique combination of three synergistic, cell-strengthening elements_  
+https://blog.nutri-tech.com.au/
+*Visit Eumundi Palms:*  
+https://eumundipalms.com.au/
+*Relevant NTS Products Featured in This Episode:*  
+_Sili-Cal (B)™_  
+https://nutri-tech.com.au/products/sili-cal-b  
+_Tri-Kelp™_  
+https://nutri-tech.com.au/products/tri-kelp  
+_Nutri-Life BAM™_  
+https://nutri-tech.com.au/products/nutri-life-bam  
+_NTS FulvX™ Powder_  
+https://nutri-tech.com.au/products/nts-fulvx-powder  
+_Nutri-Stim Triacontanol™_  
+https://nutri-tech.com.au/products/nutri-stim-triacontanol  
+*Interested in studying Nutrition Farming?*  
+Certificate in Nutrition Farming courses:  
+https://nutri-tech.com.au/pages/courses  
+Need personalised support?  
+Soil &amp; Plant Therapy Services:  
+https://nutri-tech.com.au/pages/soil-plant-therapy  
+Book a one-hour online consultation with Graeme Sait:  
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
+Explore more at our website:  
+https://nutri-tech.com.au/
+Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
+https://nutri-tech.com.au/pages/newsletter  
+*Follow us on Social Media:*  
+Facebook: https://www.facebook.com/NutriTechSolutions/  
+Instagram: https://instagram.com/nutritechsolutionsyandina  
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
+X (Twitter): https://x.com/ntsaustralia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025-12-16T00:01:01Z</t>
+          <t>2025-12-12T04:30:38Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>853</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.178082</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Love a good visual aid! Hope you’re well Patrice! || Yeanin Leanin!💡 || 🔥🔥🔥🔥</t>
-        </is>
-      </c>
+        <v>0.024619</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HRzNQQZ3998</t>
+          <t>b9rRVtnn5x8</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Top 3 Mistakes New Entrepreneurs Make (and How to Avoid Them!)  #patricelstewart</t>
+          <t>Farming Secrets From a Real Plant Nursery! Eumundi Palms Interview Pt1 - How to S4E8</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hey! This video provides crucial `entrepreneur advice` by highlighting `common mistakes in business` that often lead to new ventures struggling. It stresses the importance of a clear `vision for business` and the need for `independent thought` to avoid issues that explain `why entrepreneurs fail`. Stay informed to build a stronger foundation for your business! 😊</t>
+          <t>Welcome back to another inspiring episode of the *How To Do It* series.
+This week, we’re visiting the Sunshine Coast’s remarkable *Eumundi Palms Nursery* — a thriving family business committed to growing stronger, healthier plants without relying on chemical crutches. 🌿✨
+#chemicalfree #biologicalgrowing #plantresilience #regenerativehorticulture #healthyplants #organicnursery #plantpropagation #pottingmix #beneficialmicrobes #nurseryproduction 
+In Part 1 of this interview, owner *Philip Redhead* shares how he transformed a modest nursery into one of Queensland’s standout examples of sustainable plant production. As we walk through the lush rows of ornamentals and palms, Philip explains the turning points, challenges, and practical strategies that shaped this transformation. 🌴💬
+A major theme of this episode is the choice to step away from conventional, chemical-heavy growing systems. Philip explains how repeated chemical use often weakens plants over time, while healthier soils and beneficial biology build plants that truly *thrive* once they leave the nursery. The improvements in resilience, strength, and long-term performance are unmistakable. 🌱💪
+We explore propagation techniques, potting mix improvements, natural disease management, and efficient systems that support the nursery through busy seasons. Philip also shares the emotional rewards of nursery life — watching roots develop strongly, reusing returned pots, and nurturing plants destined to enrich gardens for decades. 🪴😊
+You’ll also get an honest look at the challenges of running a family nursery: staffing shortages, rising demand, and the constant effort to maintain quality under pressure. Through it all, Philip’s commitment to integrity, plant health, and sustainable practices shines brightly. 🌏💚
+Whether you’re a grower, home gardener, landscaper, or simply someone who loves hearing real stories of people doing things better, this episode is full of practical insights and fresh inspiration.
+*Stay tuned for Part 2* , where we dive deeper into biological strategies, advanced growing techniques, and the powerful philosophy behind Eumundi Palms’ long-term success.
+Thanks for watching — enjoy the episode! 🙌🌿
+👇 *Chapters:*
+00:00 - Introduction
+01:33 - Title Sequence
+02:03 - Phil's Backstory
+04:12 - Plant Fundamentals for Health - Silica &amp; Tsunami
+05:57 - Pest &amp; Disease Management
+07:09 - Foliar &amp; Fertigated Nutrition - Uptake Efficiency
+08:52 - Silica, Calcium &amp; Boron - Benefits Continued
+11:47 - Pseudomonas Florescence - Silica Solubilisation &amp; Other Benefits
+14:32 - Plant Nursery Priorities - Insects
+15:47 - Ecological Priorities - Power &amp; Recyclable Pots
+17:11 - End Credits
+Want to learn more about Nutrition Farming? Check out Graeme's article on *”Sili-Cal (B)™ a unique combination of three synergistic, cell-strengthening elements* …
+https://blog.nutri-tech.com.au/sili-cal-b-a-unique-combination-of-three-cell-strengthening-elements-2/
+*Check out Eumundi Palms' website below*
+https://eumundipalms.com.au/
+*Sili-Cal (B)™*
+https://nutri-tech.com.au/products/sili-cal-b
+*Tri-Kelp™*
+https://nutri-tech.com.au/products/tri-kelp
+*Nutri-Life BAM™*
+https://nutri-tech.com.au/products/nutri-life-bam
+*NTS FulvX™ Powder*
+https://nutri-tech.com.au/products/nts-fulvx-powder
+*Nutri-Stim Triacontanol™*
+https://nutri-tech.com.au/products/nutri-stim-triacontanol
+*Interested in attending a Certificate in Nutrition Farming course?*
+https://nutri-tech.com.au/pages/courses
+Need assistance? Try out our Soil &amp; Plant Therapy Services
+https://nutri-tech.com.au/pages/soil-plant-therapy
+How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait
+Head to our website to find out more
+https://nutri-tech.com.au/
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+*Follow us on Social Media*
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+X (Twitter): https://x.com/ntsaustralia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025-12-14T01:00:22Z</t>
+          <t>2025-11-28T04:30:26Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>1105</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.154589</v>
+        <v>0.034389</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Very accurate and True ✊🏿✊🏿 || ❤❤❤❤</t>
+          <t>Wow got a lot out of this! I nearly skipped it! Thank you both for sharing with us your time and knowledge it is greatly appreciated! We can’t wait to do the course next week!! || At the 11:45 time period Graeme introduces the silica solubilizing microbe Pseudomonas Florescens and goes on to talk about ice formations created by microbes. The particular species identified is another of the Pseudomonas family…..Syringae. Check out the shift from liquid to solid when Syringae is added to cold water and the phase shifts from liquid to solid.
+https://www.youtube.com/shorts/DiDNVSHm-cA || Awesome, thanks for sharing this Brad!
+For some reason the link opens with studio. hopefully this link works better...
+https://www.youtube.com/shorts/DiDNVSHm-cA || Interesting Tsunami has rice husks. I want to try the sheoak (casaurina) brew from another episode but it seems the sheoak does not contain much Si so I am planning to add rice husks. Any idea if that would lift the Si in the final brew? || Thanks for the question! Tsunami is based on rice husks, though the active component is relatively complex extraction. 
+Yes, She oak (Casuarina) has been a common ingredient for BD508 in Australia, though there isn't a lot of research on it's actual silica content. Rice husks have been studied more widely and are a very good source of bioavailable silica, with it making up about 15–20% of the husk dry weight. So including it in a well managed brew would certainly deliver more available Silica.
+There are other pH factors to be mindful of but ashes from these plant materials can be another highly concentrated source of Silica, for reference Rice Husk ashes can range from 74–98% SiO₂. || ​@NutriTechSolutionsNTS I asked AI for info on rice husks and yes it seems making the Si is a headache for DIY people. And I suspect that the process of making AI in rice husks plant available will increase the pH which I want to avoid because it then becomes incompatible with most other fertilisers || Seems to me that combining the BD508 with a little potassium silicate could be an easy compromise || Thanks for posting, interesting that you want 800ppm Si on the tissue test, will try get up to that. || Can SilicaB be used on all plants from stone fruit trees, citrus trees and vegetables. || Thanks or the question! Yes, Ideally this would always be based on a soil test, but you can use Sili-Cal B on all crops, the importance of these nutrients are foundational to any healthy crop.
+https://nutri-tech.com.au/products/sili-cal-b?_pos=1&amp;_psq=sili&amp;_ss=e&amp;_v=1.0 || ​@NutriTechSolutionsNTSthank you.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>UPE_dDeiHDY</t>
+          <t>-r6y2epf7jQ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The Spending Pattern Nobody Wants to See #patricelstewart  #moneytalk #truth</t>
+          <t>Can You Really Change Your Mood in 2 Minutes? Human Health Tips! - How to S4E7</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hey! This video offers practical `personal finance` tips, emphasizing `money management` by reviewing your bank statements line by line. This process is crucial for effective `budgeting` and can lead to significant `saving money` by increasing your `financial awareness`. Take control of your finances today! 😊</t>
+          <t>* Two-Minute Tips for #StressRelief and #HealthyLiving *
+In this uplifting episode, Graeme shares four simple, fast and transformative strategies to help you reduce stress and cultivate greater calm in your daily life. These ideas are *micro-habits* with *macro-benefits* , designed for busy people who need practical tools for immediate change. 🌿
+#stressrelief #wellnesshabits #mentalhealthtips #EFTtapping #mindfulness #breathingexercises #reduceanxiety #balanceexercise #brainhealth #lowstressliving #healthylifestyle
+We begin with the *Emotional Freedom Technique (EFT).* This combination of intention, affirmation and tapping on key acupuncture points may sound -too good to be true-, yet a growing body of research shows that EFT can quickly ease anxiety, emotional tension and accumulated stress. Graeme demonstrates each tapping point, guiding you through a sequence that takes just two minutes and can deliver surprising relief. ✨
+The episode then explores the importance of *living in the present moment.* Drawing from Lao Tzu and echoed by modern thinkers like Eckhart Tolle, Graeme explains why living in the past creates depression, living in the future creates anxiety, and why only the present moment contains genuine peace. You’ll learn a simple technique: stop once an hour and take *three slow, deep breaths.* This short practice interrupts racing thoughts, supports the lymphatic system and gradually retrains your nervous system toward calm. 🌬️
+You’ll also discover the fascinating *two-minute balance challenge* from Chinese health master Zhong Li Ba Ren. Standing on one leg with your eyes closed challenges your neurological balance and provides a quick window into your biological age. The practice is associated with benefits for blood pressure, blood sugar, spinal mobility and long-term brain function. Whether or not you fully accept the bold claims, it is a fun and revealing daily test of stability and mind–body connection. 🧠💫
+Finally, Graeme presents the simplest tip of all: *reduce your screen time.* Constant exposure to media-driven negativity can drain joy and increase stress. Swapping some screen time for music, uplifting reading, creativity or meaningful connection can dramatically improve wellbeing.
+These ten *two-minute tips* are practical, powerful and accessible for everyone. Try them consistently for two weeks and observe the shift in clarity, calm and resilience. 💚
+👇 *Chapters:*
+00:00 - Introduction - Human Health Exercises
+01:32 - Title Sequence
+02:02 - Emotional Freedom Technique - Tapping
+05:47 - Living in the Moment - Meditation
+11:01 - Being Proactive - Mindset, Love or Fear
+16:14 - The Golden Cockerel - Balance
+23:30 - End Credits
+If you want to learn more about Human Health strategies. Check out Graeme's interview article with the late great Jerry Brunetti…
+https://blog.nutri-tech.com.au/jerry-brunetti-interview-part-1-2/
+Bio-Bubble
+https://www.ntshealth.com.au/products/bio-bubble
+Nutri-Salt
+https://www.ntshealth.com.au/products/nutri-salt
+SweetSure
+https://www.ntshealth.com.au/products/sweetsure
+BioSpark
+https://www.ntshealth.com.au/products/biospark
+Curcu-Life
+https://www.ntshealth.com.au/products/curcu-life
+Green Defence
+https://www.ntshealth.com.au/products/green-defence
+Head to our website to find out more
+https://nutri-tech.com.au/
+Interested in attending a Certificate in Nutrition Farming course?
+https://nutri-tech.com.au/pages/courses
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+Follow us on Social Media
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+X (Twitter): https://x.com/ntsaustralia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-12-13T01:15:02Z</t>
+          <t>2025-11-14T04:30:01Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>920</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.130435</v>
-      </c>
-      <c r="M11" t="inlineStr"/>
+        <v>0.030435</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Absolutely well said yet again. 
+Loved your course a few weeks ago - life changing.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>fYJ8PQ9IN-s</t>
+          <t>JKGkOqX-pOw</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Make Over $150K? Don’t Let These Tax Deductions Slip Away!  #patricelstewart #tax</t>
+          <t>The Future of Farming - 10 Practical Steps to get Started - Part 2 - How to S4E6</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hey! This video breaks down how `income tax` deductions are affected by your adjusted gross income, specifically focusing on `AGI` thresholds. It's crucial for `understanding your deductions` to navigate how these phase-outs impact your `taxable income`. This information is vital for effective `tax planning` to ensure you're well-informed about your financial picture. 😊</t>
+          <t>In this powerful follow-up episode, *Graeme Sait* continues his step-by-step guide to launching your *regenerative journey* with practical demonstrations, tools, and insights that empower both *farmers and consultants* to get real results — in the field and in life.
+#NutritionFarming #GraemeSait #SoilHealth #RegenerativeAgriculture #BAM #MicrobialBrewing #HealthySoilHealthyYou #SustainableFarming #FarmersHealth
+🔥 *Highlights from this episode:*
+🌿 *1️⃣ Brewing Living Fertilisers*
+Discover how to create your own *on-farm biological inputs.* Graeme demonstrates the *three-in-one brewer* for producing *aerobic* , *anaerobic* , and *extract* brews — including *vermicompost extracts* , *Bacillus subtilis* , *Trichoderma* , and *Azotobacter.* These living brews boost soil life, crop resilience, and productivity while slashing input costs.
+💧 *2️⃣ The Simplicity of BAM*
+Learn about *BAM – Beneficial Anaerobic Microbes* — a microbial inoculum that can be brewed on-farm with *molasses and water.* With a two-year shelf life and remarkable versatility, BAM is now *used in over 55 countries* as a foundation of biological success.
+🔬 *3️⃣ Tools for Precision Nutrition*
+Graeme explains how to measure and manage your results using:
+• The *Brix meter* for monitoring sugars and plant vitality.
+• *pH strips* to track potassium movement between leaves.
+• Simple nutrient mobility checks to detect deficiencies early.
+These practical tools help you make smarter, faster nutrient decisions.
+💚 *4️⃣ Fear-Based vs Love-Based Farming*
+Graeme shares a heartfelt message about mindset — contrasting the *fear-driven chemical model* with the *love-based regenerative approach* that nurtures *soil life, human health,* and *planetary wellbeing.* Every farming choice, he says, is either *fear or love in action.*
+🌼 *5️⃣ Natural Disease Protection*
+A simple recipe for *powdery mildew control* — combining *BAM and milk powder* , optionally enhanced with *manganese* — delivers a sustainable, cost-effective disease solution that strengthens plants naturally.
+🌾 *6️⃣ Farmer Wellbeing and Self-Care*
+Graeme closes with tips for *managing stress, supporting magnesium and B6 levels,* and embracing *autophagy* through intermittent fasting — reminding us that *healthy soil and healthy farmers are inseparable*.
+✨ *Practical, inspiring, and deeply transformative,* this episode reconnects the roots of *Nutrition Farming®* with the heart of *personal wellbeing.*
+👇 *Chapters:*
+00:00 Introduction - Brewing
+00:59 Title Sequence
+01:29 Brewing your own Living Fertilisers
+02:55 Checking Your Progress
+08:08 Being Proactive - Mindset, Love or Fear
+11:12 Taking care of your Health
+17:06 End Credits
+Want to learn more about Nutrition Farming? Check out Graeme's article *”Ten Tips for Microbe Brewing - DIY Living Fertilisers* …
+https://blog.nutri-tech.com.au/10-tips-for-microbe-brewing/
+*Nutri-Life BAM™*
+https://nutri-tech.com.au/products/nutri-life-bam
+*NTS FulvX™ Powder*
+https://nutri-tech.com.au/products/nts-fulvx-powder
+*Tri-Kelp™*
+https://nutri-tech.com.au/products/tri-kelp
+*Nutri-Stim Triacontanol™*
+https://nutri-tech.com.au/products/nutri-stim-triacontanol
+*Cal-Tech™*
+https://nutri-tech.com.au/products/cal-tech
+*Sili-Cal (B)™*
+https://nutri-tech.com.au/products/sili-cal-b
+*Interested in attending a Certificate in Nutrition Farming course?*
+https://nutri-tech.com.au/pages/courses
+Need assistance? Try out our Soil &amp; Plant Therapy Services
+https://nutri-tech.com.au/pages/soil-plant-therapy
+How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait
+Head to our website to find out more
+https://nutri-tech.com.au/
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+*Follow us on Social Media*
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+X (Twitter): https://x.com/ntsaustralia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-12-10T02:30:39Z</t>
+          <t>2025-10-31T04:30:15Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>261</t>
+          <t>1430</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.099617</v>
+        <v>0.037762</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>❤❤❤❤</t>
+          <t>Unreal series! So much important information, thanks || Is there some kind of instructional manual or video instruction on how to brew and use the brewer and products for specific applications. || Make your own compost, way cheaper.
+Just google compost extraction || ​@666bruvhave been making my own. Always nice to find other recipes. || ​@johnharris7244don't waste your money on bug in a jug || Thanks for the question @johnharris7244!
+I have created a playlist below containing all the videos we have produced to date on brewing microbes. Most of these weren't filmed using the new 3 in 1 Brewer, but they can easily be adapted to do so. We plan to produce more videos featuring this unit in the future. 
+https://www.youtube.com/playlist?list=PLXReS_QZvjWAB7kPDqcqPTEiQ41VuD4cT || Thanks for the comment! They all help with the algorithm to further highlight our videos featuring "Bug in a Jug".
+I suggest you look deeper into the different classes of microbes in relation to their association with plants and other microbes. Compost is an incredible tool, but it still has many limitations when it comes to culturing the complete range of beneficial microbes. 
+Obligate Symbionts (Plant-Reliant Microbes)The microbes that form the most intimate, beneficial plant partnerships generally do not survive standard composting. 
+Arbuscular Mycorrhizal Fungi (AMF): They are obligate symbionts, meaning they must be connected to a living root to reproduce and thrive. The high temperatures of the active composting phase will typically destroy their delicate spores and hyphae.
+Symbiotic Nitrogen-Fixing Bacteria (Rhizobium): While they can survive in soil, they are highly specific. For effective inoculation, you must use specialized, host-specific inoculants (e.g., coating legume seeds) rather than relying on a general compost mix. || Is there much difference between EM and BAM? || Great question,  I brewed up some EM1 a couple of weeks ago and it has very distinctive sweet aroma , yesterday I opened up a container of BAM and it smells very similar and that was my exact thought. || Thanks for the question @howardroe7515!
+Yes, there are some differences between EM (Effective Microorganisms) and BAM (Beneficial Anaerobic Microbes), although they share similar foundational concepts. Both products are designed to enhance soil health and plant growth through the use of beneficial microorganisms, but they have distinct compositions and applications:
+EM (Effective Microorganisms): Developed by Professor Teruo Higa, EM is a blend of various beneficial microorganisms, including lactic acid bacteria, yeast, and photosynthetic bacteria. It is widely used in agriculture to improve soil health, composting, and plant growth.
+BAM (Beneficial Anaerobic Microbes): BAM is based on the original EM formula but includes additional microbial varieties. It contains over 80 different microbe varieties, including lactobacillus, purple non-sulphur bacteria (PNSB), fermenting fungi, yeast, and actinomycetes. BAM is designed to perform similar functions to EM but with a broader spectrum of microorganisms. || ​@NutriTechSolutionsNTSdoes that make BAM a good foliage spray option. || Yes, BAM is a great all rounder, it's certainly helpful via foliar, though it's most effective in the soil, especially for recovering anaerobic soils.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UC_15lYbMxpZXv5OEVY5rN2w</t>
+          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PATRICE L. STEWART</t>
+          <t>NutriTechSolutions</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>x9hEVK8HWwQ</t>
+          <t>6JQ7quA88xo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Tips Tax-Free Up to $25,000?! Avoid IRS Traps  #patricelstewart #taxdeductions</t>
+          <t>The Future of Farming - 10 Practical Steps to get Started - Part 1 - How to S4E5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Hey! This video explains the new `no tax on tips bill`, allowing tips up to $25,000 to be `tax free` for workers. This is great news for `uber driver` and `lyft driver`s, as it directly impacts their `self employment taxes`. Remember to keep your paperwork in order to benefit from this change! 😊</t>
+          <t>Welcome to *Episode 5 of Series 4* of the *“How to Do It”* video series. In this special instalment, we take a short break from our *Human Health* focus to explore the practical heart of *Nutrition Farming ®*  — how to actually get started.
+After four seasons and over sixty episodes, many viewers have shared a common challenge: *“Where do I begin?”*  In this inspiring session, Graeme Sait cuts through the information overload and lays out a *10-step action plan* designed to move you from learning to doing.
+*Take away the guesswork.* Learn why *tissue testing* and *soil testing* are essential, how to interpret results, and how to avoid wasting money on unnecessary inputs.
+*Measure your microbial workforce.* Discover how tools like the *Microbiometer ®* can reveal soil vitality by measuring *total microbial biomass* and the critical *fungal-to-bacterial ratio.* Graeme explains why rebuilding the fungal component is central to creating well-structured, living soil.
+👉 *From there, you’ll explore:*
+• The importance of *humic and fulvic acid* in boosting nutrient uptake and soil structure.
+• Why *FulvX™* , a new humic-fulvic combination, offers the best of both worlds.
+• The role of *mycorrhizal fungi* and *Trichoderma* in extending root systems, enhancing nutrient delivery, and protecting crops from *root-knot nematodes.*
+• The game-changing potential of *foliar nutrition* — particularly *foliar urea* and *calcium-boron* combinations — to dramatically lift plant performance while reducing input costs.
+• And finally, the extraordinary natural plant growth compound *Triacontanol* , described as the *most powerful plant growth promoter ever researched.*
+💡This practical, down-to-earth guide provides the perfect foundation for farmers and gardeners ready to turn theory into results. Whether you adopt one step or all ten, the key message is clear: *action transforms everything*.
+🎥 *Join Graeme Sait as he reignites the movement from awareness to implementation — the essence of Nutrition Farming ®.*
+#NutritionFarming #SoilHealth #HowToDoIt #GraemeSait #FulvicAcid #HumicAcid #Microbiometer #MycorrhizalFungi #Triacontanol #FoliarFeeding #SustainableFarming #RegenerativeAgriculture #SoilMicrobes #PlantNutrition #CalciumBoron #FulvX #Trichoderma #SoilTesting #TissueTesting #MicrobialBiomass #ActionNotTalk
+👇 *Chapters:*
+00:00 - Introduction
+01:35 - Title Sequence
+02:05 - Plant Tissue Testing
+02:55 - Soil Testing &amp; Dealing with Deficiencies
+04:54 - Testing Microbial Activity - MicroBiometer
+08:51 - Humates
+10:35 - Experimentation &amp; Microbial Inoculums
+12:15 - Foliar Nutrition, Urea, Calcium &amp; Triacontanol
+Want to learn more about Nutrition Farming? Check out Graeme's article *”Ten Tips for Microbe Brewing - DIY Living Fertilisers* …
+https://blog.nutri-tech.com.au/10-tips-for-microbe-brewing/
+*Nutri-Life BAM™*
+https://nutri-tech.com.au/products/nutri-life-bam
+*NTS FulvX™ Powder*
+https://nutri-tech.com.au/products/nts-fulvx-powder
+*Tri-Kelp™*
+https://nutri-tech.com.au/products/tri-kelp
+*Nutri-Stim Triacontanol™*
+https://nutri-tech.com.au/products/nutri-stim-triacontanol
+*Cal-Tech™*
+https://nutri-tech.com.au/products/cal-tech
+*Sili-Cal (B)™*
+https://nutri-tech.com.au/products/sili-cal-b
+*Interested in attending a Certificate in Nutrition Farming course?*
+https://nutri-tech.com.au/pages/courses
+Need assistance? Try out our Soil &amp; Plant Therapy Services
+https://nutri-tech.com.au/pages/soil-plant-therapy
+How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
+https://nutri-tech.com.au/pages/consultations-with-graeme-sait
+Head to our website to find out more
+https://nutri-tech.com.au/
+Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
+https://nutri-tech.com.au/pages/newsletter
+*Follow us on Social Media*
+Facebook: https://www.facebook.com/NutriTechSolutions/
+Instagram: https://instagram.com/nutritechsolutionsyandina
+LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
+X (Twitter): https://x.com/ntsaustralia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025-12-10T01:31:00Z</t>
+          <t>2025-10-17T04:30:03Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>2628</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>59</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.07834099999999999</v>
-      </c>
-      <c r="M13" t="inlineStr"/>
+        <v>0.023592</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Excellent episode, Thanks very much || Question about the foliar calcium, if we use chelated calcium nitrate, on the one hand, good for foliar calcium but I'm trying to avoid nitrate applications for the reason mentioned in the foliar urea section of the vid.  Do you have any idea how impactful foliar calnitrate is upon plant energy in this context, assuming here the plant absorbs it in leaves and then needs to convert it to amino which will take lots of energy. Any alternatives to foliar chelated calcium nitrate? || Thanks for the great question @davidspghill!
+This really depends on the required outcome. If this specifically to deal with a calcium deficiency, a chelated form of Calcium Nitrate is still one of the most practical methods we would recommend, due to it's high availability, solubility and ease of application. An average crop requires 10-12 times more nitrogen than calcium, so this is still just a fraction of the overall N required. The remaining N could be applied via foliar urea applications throughout the season.
+Otherwise you could opt for micronised lime, it has a much lower effective foliar uptake rate, but due to the lower cost per kilogram it still works out at a similar cost per hectare. It does require slightly more specialised spray equipment due to the insoluble particles and the need for constant agitation during application, but it is certainly another practical option. It would also allow for the inclusion of chelated urea in the same application.
+It's true that nitrate requires around 8 times more energy for foliar uptake than urea, but this is just one aspect. If you have a severe calcium deficiency the increased energy production due to it's alleviation will easily counteract the additional energy required to utilise the nitrate.
+I hope that helps!</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refreshed niche generation with new adjacent high-ticket niches
</commit_message>
<xml_diff>
--- a/output/master.xlsx
+++ b/output/master.xlsx
@@ -448,31 +448,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Welcome to Nutri-Tech Solutions (NTS)!** 🌱  
-We’re dedicated to **regenerative agriculture**, helping farmers, agronomists, and home gardeners grow **nutrient-dense food** while restoring soil health. Our channel offers expert insights, **workshops**, and practical training on **organic farming**, **sustainability**, and **crop nutrition**.  
-Learn from **Graeme Sait**, a global leader in **sustainable agriculture**, as he shares innovative strategies to boost yields, enhance **farm management**, and improve soil vitality. Discover practical solutions for **home gardening**, microbial inoculants, and **nutrient-dense food production**.  
-Join our community of **regenerative farmers**, engage in discussions, and stay updated with our latest insights. **Subscribe now** and take your **farming** to the next level! 🌍🌾  
+          <t xml:space="preserve">Welcome to the official YouTube channel of EJS Golf, hosted by me, Coach Erik Schjolberg, top rated golf coach in the golf mecca of Scottsdale, AZ. With over 25 years of experience as a Professional Golf Coach, I’ve had the privilege to work with PGA Tour Players, college athletes, high-level developing juniors, and golf enthusiasts who are willing to commit to progress and weekend warriors that want to get better for that day or tournament.
+Are you tired of hitting fat golf shots, topping, not having the shaft lean you want, etc.?   There are root causes to these that have to be fixed to become the ball striking machine anyone can become.   Improve your game from the very first lesson.  Every golfer should get better from their very first lesson. My feedback-driven approach to practice, demanding only 15 minutes of commitment per day, guarantees results.
+Coach Erik Schjolberg
+EJSGolf.com
+Scottsdale Golf Lessons
+Online Golf Lessons
+(480) 861-9370
 </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4640</t>
+          <t>7290</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>935</t>
         </is>
       </c>
     </row>
@@ -560,88 +563,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>oMGRZunNwGM</t>
+          <t>lrMjPBep7x0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Gold from the Vaults - Jerry Brunetti - Detoxifying the Rumen &amp; Building Vitality - Ep 10</t>
+          <t>The Trail Knee Drill That Moves Low Point Forward</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t># *Jerry Brunetti: Detoxifying the Rumen &amp; Building Vitality (Gold from the Vault)*
-We have reached the end of Series 4 of our 'How to do it' video series, and as we prepare the next instalment, we are diving into our archives to share more *Gold from the Vault* . In this session, we rejoin the legendary *Jerry Brunetti* for Part 2 of his masterclass on soil and livestock health .
-#NutritionFarming #SoilHealth #LivestockHealth #JerryBrunetti #RumenEcosystem #RegenerativeAg #GraemeSait
-In this episode, Jerry explores the massive metabolic load placed on our animals when we push for production at the expense of biology . He breaks down why high *rumen ammonia* levels (BUN and MUN) are often the precursor to *septicaemic* conditions and immune failure . From the importance of _acetic acid_ (vinegar) in the rumen to the incredible role of _Peyer's patches_ in gut immunity, Jerry connects the dots between soil minerals and the longevity of your herd . If your cows are leaving the herd at an average of 44 months, this video reveals exactly why—and how to fix it .
-*What you'll learn in this episode:*
-🥬 The "energy deficit" trap: Why cranking up cereal starch creates dangerous _D-lactic acid_ .
-🧬 _Manureology_ Revisited: Using your nose to detect metabolic imbalance and *butyric acid* issues .
-💩 The *Ensiling* Secret: Why adding _molasses_ or lactose to your silage creates the perfect microbial fuel .
-📈 The 14% Rule: Why cellulolytic bacteria die off rapidly when rumen pH drops below 6.5 .
-🧪 Gut Integrity: How damaged _villi_ lead to *dysbiosis* and the infiltration of pathogens .
-🐄 Liver Longevity: Understanding how the liver regenerates and why its failure is the final symptom, not the cause .
-👇 *Chapters:*
-00:00 - Introduction - Ammonia &amp; Rumen Issues
-01:33 - Title Sequence
-01:57 - Rumen Acid Production &amp; pH Balancing
-03:53 - Plant Maturity &amp; Forage Quality
-06:17 - Silage Quality, Fortification &amp; Microbe Foods
-09:48 - Growing High Quality Fodder
-11:59 - Balancing Rumen pH
-17:21 - Milk &amp; Pasture Analysis - Refractometer &amp; Brix
-21:30 - Lower Gut Health, Issues &amp; Probiotics
-30:51 - End Credits
-Want to learn more about Nutrition Farming? Check out Graeme's How to do it episode *Getting Started with Nutrition Farming® – 10 Practical Steps to Transform Your Soil and Crop Health - Part 2* …
-https://blog.nutri-tech.com.au/getting-started-with-nutrition-farming-r-10-practical-steps-to-transform-your-soil-and-crop-health-part-2/
-*Nutri-Life BAM™*
-https://nutri-tech.com.au/products/nutri-life-bam
-*Nutri-Gyp™ Natural Gypsum*
-https://nutri-tech.com.au/products/nutri-gyp
-*Sili-Cal (B)™*
-https://nutri-tech.com.au/products/sili-cal-b
-…or try our new NTS FulvX™ Powder for chelation
-https://nutri-tech.com.au/products/nts-fulvx-powder
-*Interested in attending a Certificate in Nutrition Farming course?*
-https://nutri-tech.com.au/pages/courses
-Need assistance? Try out our Soil &amp; Plant Therapy Services
-https://nutri-tech.com.au/pages/soil-plant-therapy
-How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait
-Head to our website to find out more
-https://nutri-tech.com.au/
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-*Follow us on Social Media*
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-Twitter: https://x.com/ntsaustralia</t>
+          <t>Get my free 16 Drills guide: EJSGolf.com/my-drills
+Coach Erik Schjolberg breaks down the one constraint drill that fixes low point, eliminates flipping, early extension and creates ball-first contact on every iron. If your divots start behind the ball or you catch it thin, your trail knee is stalling and your pressure never transfers. This aim-stick gate drill physically forces the trail knee to drive toward the target, clearing the pelvis and shifting the low point 2–4 inches ahead of the ball.
+You will learn: 
+✅ (1) How to set up the alignment-stick gate for your trail knee. 
+✅(2) Why trail knee stall kills compression and creates early extension. ✅(3) How to feel the pressure shift from trail foot to lead foot by P6.
+✅ (4) Measurable checkpoints using divot position, strike spray, and TrackMan data (low point, shaft lean, dynamic loft).
+This is The Science of Better Golf—data-driven, constraint-led instruction that produces day-one improvement. No swing thoughts. No guessing. Just a physical gate that makes your body move correctly.
+Get my free 16 Drills guide: EJSGolf.com/my-drills
+Book a lesson in Scottsdale: EJSGolf.com
+Coach Erik Schjolberg
+The Science of Better Golf
+EJSGolf.com
+Scottsdale Golf Lessons
+Online Golf Lessons  
+#golfswingmechanics #golfswinganalysis #golfimpact #golfpower #golfdistance #EJSGolf #Titleist #Linksoul</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-13T05:38:47Z</t>
+          <t>2026-03-23T21:36:51Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>490</t>
+          <t>1223</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -650,7 +621,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.02449</v>
+        <v>0.012265</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -659,7 +630,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Um so anyway this blood ammonia levels you start now getting neemic animals you start growing pathogens you lower the immune system. So now we got this high mun bun rin pneumonia issue. The nutritionist comes along, sees your cows look like crap. You're not milking worth the hoot. You know, you've got poor condition. You're not getting cows bred back. And he says, or vet says, you got to put some condition on these animals. These cows have got to have some energy. You got an energy deficit in this herd. All right. So what do you do? He's going to crank up the thermostat and he's going to recommend that you crank up the cereal. So now we come in with another weird substance called starch. Well, here's something that's interesting. If you can see this thing says acetic acid over here. Star starch when it fermentss in the room and produces this thing called dactic acid. When you ferment sugars packed into cellulose, hemiselulose, you produce acetic acid. What's the difference? What is another word for acetic acid? Anybody hear of vinegar? Anybody ever know of your predecessors or some of the old time farmers that used to feed cows vinegar? &gt;&gt; Still do. &gt;&gt; Still do. That's why you feed cows vinegar because they make it. A healthy rin makes vinegar. I'm going to go give you another slide here in a second. [music] &gt;&gt; [music] &gt;&gt; That's what an acetic acid is. And so you get here is another oxymoron. is sort of like the the pH of the urine being high showing acidosis because you don't have any minerals to buffer, so you're using ammonia. How could acetic acid be a good thing for concern about acidosis? Acetic acid has onetenth the acidity that lactic acid has. So an animal that's loaded with lactic acid could actually be buffered by vinegar. The same is true with people who take vinegar to deal with their own acidosis and they get a response. Why? Because the acid that they're neutralizing with the acetic acid is these fermentation acids from eating a lot of sugar and carbohydrates causing all this other acid. So people who take vinegar, the apple cider vinegar with the mother especially in it, &gt;&gt; you'll get better. You'll start feeling alkalized. It's not because of the acid. It's because you've actually alkalized the really really noxious acids with the vinegar. So it's a relative issue. Okay. So anyway, now what you see here is the room pH. See on the top ideal room pH 6.5 to to 7. We got this ammonia thing running rampant because we have poor quality forage. And I can tell you this much unless it's really mature forage. If you've got really high protein forages, chances are they're low in energy. And the converse is usually true. If you have really low energy forages, and I mean energy the way I define it, not necessarily the way the conventional wisdom defines it. You're usually high in NPN. uh coming in forage or pasture or or or serial crops is uh is there a specific time you're sort of talking about of maturity of that plant maturity of the plant of the forage? It depends on how you grow it. We'll talk a little bit about that. But I mean the problem you have growing or harvesting early forges obviously is you got high levels of protein and low effective fiber when it's really young and lush. Now that being said that's always true with conventionally raised forages. And what we find out is if you let those forages just get a little older, if you're doing the right kinds of soil things, you will get the energy and the protein is a better quality protein. So I'm not so worried about the quantity of the nitrogen. I'm concerned about getting amino acid quality protein. Even if it's less, like the dairyman from Washington State, the quality is less. I mean, the quantity is less, [snorts] the quality is higher, and I got more pectants in there. And when you start getting that th that that gap starts to narrow come together where the protein quality and the and the energy quality start running side by side. Now you're not wasting all that energy to get rid of this stuff because what happened here see this this farmer in Washington state. What happened there was because this liver and the kidney and all this stuff was working so hard to get rid of all this ammonia. It was consuming energy out of the cow to get rid of the ammonia. That's why the cows came up in milk after he fed them a poor quality forage because he wasn't poisoning the cows with ammonia and the animals detoxification and elimination organs didn't have to consume energy to get rid of that which he paid for twice. It's pretty logical. You know, the cows are telling you are telling you this stuff and you can smell the ammonia. You don't need a high-tech laboratory to figure out what the hell's going on with a cow. Look at her, smell it. You go into a barn in Pennsylvania this time of the year and I can tell the herds that are getting this right. The ones that are feeding conventionally, the ammonia levels are overwhelming. And that's what's going on. And it's not because of ventilation. It's not because of ventilation. Does that is that refer exactly the same to to the hay all the toes are made. Was that was that u work on your nose is to say the quality of the h? Yes. I mean not to tell everything by your nose but one of the things you use you smell and you s and silage is another good thing. S and soiled hays and forages should have kind of a sweet pickled smell to them. They should not have that butyric acid smell, that really heavy acid smell that when it gets on your clothes, you can't get it off. You know what I'm talking about? That's butyric acid. You don't want that. And you don't want that real real uh vinegary smell either, which is uh you don't want acetic acid production in the silages. You want different kinds of acid productions in the silage. And one of the best ways to do that, and as long as we're talking about that, let's let's so easy to not talk about so many things. There's so much to talk about. So you brought it up and we'll go there right now. When you insile forages, always remember that you're going to take true proteins and break them down into more of these compounds. That's one of the downsides of making hay into silages is that you tend to compromise protein quality because the insulin process, the fermentation process of ensulin tends to break down these proteins and makes more simpler nitrogen compounds. One of the reasons why I like to throw molasses on palage so that I can give the fermentation organisms a lot of sugar to go crazy and cool that thing down really quickly so that we don't get a lot of heat damage and we don't get a lot of fermentation damage. So we throw molasses on that, not a [clears throat] lot. And what that does is that the molasses gives the microbes that are on the leaf surface called the phyosphere. And these are lactic acid organisms that are naturally occurring there and especially yeast organisms. If you really want to kick up the volume, you could throw milk sugar on there. Lactose. Milk sugar is a great thing to throw on silages. That gives you a very fast response because lactose is converted to lactic acid. Now, here's that bad word again, lactic acid. Well, you have lactic acid and you have dlactic acid. Dactic acid is what's going on in the rin, which is killing the rin. Lactic acid is what goes on in fermentation, like when you make sauerkraut and good silage. And also the kind of elactic acid that you find in the small intestine to keep your villi healthy. &gt;&gt; Is this what the inoculates do that we use alongside? &gt;&gt; The inoculants inoculate. They just basically introduce microbes there. But keep in mind microbes need food. So I'm more concerned about the microbes are on I mean I'm not saying not use but to me it's more critical to provide food for the microbes as opposed to putting microbes on silage that has no [clears throat] food. It's like, isn't it more important to try to create a soil that is conducive to earthworms as opposed to inoculating soil that's not doing very well with earthworms? You don't have to inoculate soil with earthworms. You can speed it up with inoculants. You can they some there's some good inoculants out there that still will make an improvement even in addition to adding the fuel that those microbes want to eat. Jerry, if you're growing the herbage in the right soil conditions and harvest at the correct time, can it not produce enough sufficient sugars to do the job? &gt;&gt; Yep. &gt;&gt; So, we're only using bands really, aren't we? &gt;&gt; Yeah. The molasses forages tend to be, you know, obviously compared to grains which have lots of starch and that's another thing you could throw on for you can throw a little starch uh ground up cornmeal. Uh you could throw ground up uh wheat flour on on the on the forages, molasses. What you're trying to do is just give the bugs, you know, an opportunity to really grow well quickly and then get the pH down quickly so that it's cooling off. You don't want to get any heat in that in that bunker and you don't want to get any heat in that bag. And it really does work. I mean, but you're right. uh as the soil starts to increase, as the minerals start to come up in the forages, the pectins and the sugars are naturally produced. Now, sometimes the problem you have is if you're making hay and it's really hot, the plant to protect itself from uh evaporation, transpiration stress will convert more of its uh carbon to make lignen instead of making sugars and pectins because it's trying to save itself from dehydration. So you end up getting more ligant produced and typically that's when you hear the complaints about butter fat test getting low is that you they'll get into the hay mau everybody will complain around the same time because they're all starting to feed third cutting hay you know when it was made in early August you know or second cutting hay when it was made in July or something like that and they'll call and say my butterf is crashing and what's happened is they they're getting into hay that was cut when it was really really hot for a number of days and when that's really hot there's more lignen produced and lignen of course is not fermentable. Now there is one way around the ligman issue or one one help to that is having adequate levels of sulfur in the forge helps to break down lignon more efficiently in the rin. There we are. There's another reason why fertilize with sulfur. See the knee bone is connected to the shin bone. So anyway, I'm just going to go on to this next slide here and see if this Okay. Yeah, this is a good slide for you to finish up with. This is the lactic acid curve and the acetic acid curve all in one. You can see that top line, that's acetic acid. That's your vinegar. Okay, here's your pHes. 7 656 555. All right, look what's going on here. You see what's going on is this is that as the pH starts to drop, and what causes the pH to drop? Starch. Starch causes the pH to drop. As the pH starts to drop, the cellulitic flora which produce acetic acids start to decrease. As they start to decrease, obviously their byproduct, which is acetic acid, starts to wing. And you can see as you get down to the five range, it disappears. Meanwhile, propriionic acid starts to climb. And when you get at six, there's the evil one that shows up. It starts killing the room, lactic acid. And here's the issue. Uh, Professor Richard Zinn at the University of California has said when you get below 65 pH in the rin, every tenth of a point that you drop below 65 in the rin, you start losing these cellulitic bacteria at the rate of 14% an hour. That's a tremendous statistic. 14% an hour below 65. That's why 65 to 7 is your pH range. And that's what you find in the old text. These animals had healthy rumins. You have a healthy room in there, you got longevity in cows. You go to this next range. This next slide is University of Wisconsin slide. Wait a minute. That's fact again. I don't know if that's on there or not. It's not on there. Anyway, there's a there's a slide that I have that shows a 24-hour feeding of a TMR, not a slug feeding, TMR, and it shows every time the cows ate, how the phes of the rin dropped, okay? Up and down, up and down. Well, I looked on that whole graph for 24 hours. I found out in that TMR ration on that Wisconsin herd, 19 out of the 24 hours, the pH was below six. There's no way you can keep a herd around for a long period of time with 19 out of 24 hours of pH below 6. That herd is kaput. There's no way that cow can stand in. So this is what we're trying to emphasize. This is this is the information coming out of the people that know about this stuff, but the feed industry hasn't accommodated to it because the feed industry is not interested in what? Soils. That's why the feed industry is not interested in soils. And I ran into this over there at at Shepherd and I was talking to one guy who's in this neck of the woods and his name is Angelo someone. I can't remember his last name. More paison I see over here than I saw anywhere else in Australia. I don't know why that's the case, but anyway, he said he was Dutch. I didn't believe him, but he told me um a name like Angela, you anyway, his family was born in Holland or some some story. Anyway, he has a dairy herd over here and he said to me, he heard some of this talk. I did an abbreviated version of this over there and he said, "Yeah, I think you're right." He said because some of the herds that I'm working with have got calcium levels and I'll go into this in a little bit here show you how the minerals reflect all this calcium levels on these forages are down to.3 and point4% when we know in order to make energy in a forage you've got to have calcium levels at 1.5 on up. And when you get 1.5% calcium you make energy. And when you get sulfur levels where they're supposed to meet, you make protein. And when you have trace minerals like boron at 40 parts per million, you make energy. So if this is a bunch of bunk that you can't make energy in forages, is that nobody knows what the soil is supposed to do because nobody even cares about the soil. The feed nutritionist basically starts balancing the ration from the point of where the the forage samples show up in front of his computer. And then it's like, well, you know, you can't take bad forage and bandaid it into good forage. You can't do it. You've already lost the window of opportunity to to create that that kind of an ecosystem optimized ecosystem arrangement for that cow to produce milk or meat on low feed costs. Okay. Uh, moving on. So, is everybody with me on this lactic acid curve? You understand why this is got to be in this range and how it's so hard in conventional agriculture to keep it here? Because if you've got these low energy forages and you want to make milk or you want to produce meat on an animal, the only recourse left is grain. That's it. You know, it's either that or you don't have milk, you don't have meat. So that's it's sort of like this you know horns of the lemon. So ultimately if we want to have a room pH here we have to be able to figure out how to produce energy in a forage and that's a soils issue. So &gt;&gt; is bricks test any use at all in testing milk in this sense or not really relevant to &gt;&gt; well the brick yeah well not so much you could use a bricks test to measure solids in milk. I don't use it so much for that. Bricks test, a bricks refratoter. For those of you who don't know who that that is, it's it's a it's a device that measures basically total suspended solids which of which sugars are part of that. They use it in the molasses industry and the honey industry, the antifreeze industry. Um anyway, that this bricks refratoter, a lot of people use that out in the field and it is it is a relative interesting tool. Um, and I'll just go there for a couple minutes because I think a lot of people have some misconceptions about what a refratoter can do for you. Uh, since it is measuring sugar, you'll typically find out that it's a relative any grass if if you let it uh go to the end of the day late in the afternoon before you cut it, you'll find out that your bricks levels simply because of sunshine creating sugar through photosynthesis, the levels of sugar are high. So now if you take the same grass and measure it that way, you'll find out that the bricks levels are consistently high. Now University of Idaho did this research in terms of recommending to dairy farmers in Idaho that if you're going to make hay and this is Holene herds and you're going to cut your alpha alpha, cut it later in the day and you can possibly generate 7 lbs milk per cow per day extra merely by increasing the sugar levels in the hay just by time of cutting. Now that being said is that what you're measuring is the product of photosynthesis which is the production of sugar and all plants do produce sugar. The question is can we increase in that same field the amount of sugar that that plant can produce based on soil fertility and the answer is yes you can and that's what we want to do. So time of day, if you took, for example, if you measured a really biologically tended field early in the morning and took a not so biologically tended field maybe late in the afternoon, you might find that the bricks levels don't show any difference or maybe even the conventional field shows a slight advantage. So it's not a real fair comparison. You got to measure the same time of the day and you got to measure, you know, the same types of, for example, 3 days of rain, for example, 3 days of cloudy weather. those bricks are going to be down and it's going to take a whole another day, day and a half for those bricks to come back up. So, you have to keep that in mind that sunlight, you know, is the primary governor of the bricks levels in a plant. Soil nutrition factors into that, but all the soil nutrition in the world done the right way with 3 days of rain is not going to show you a true reflection of what you've done on that farm. So, it's a reflective tool. Keep that in mind cuz I've got farmers come back saying, "Well, you know, I've tested this field and it was after 3 days of rain and their bricks levels are low and they don't understand why they're not up to 14." It was because it rained. The sun doesn't uh help you out if it's not there. So anyway, so that's to answer your question on that. I'm glad you brought that up and please uh this is this is good stuff because when you bring up these questions, it's really easy to lose drop these these &gt;&gt; marles away. But just one other point in Ardan Anderson's reports he he claims 20 bricks is ideal for milk. I've done a lot of milks around and can &gt;&gt; Yeah, you're talking about the actual and what you're measuring in the milk are because milk is loaded with sugar. &gt;&gt; Okay. And solids. Lots of solids in good milk. And you're right, the the poor quality the milk, the lower the bricks. And if you can get bricks levels in milk like around 20 that tells you that you know those cows are getting nutrient density that's manifesting itself in the milk. That's correct. Right. And and you get some cows that are below 10. Also the phes are even acidic and some not acidic but relatively acidic to other biologically produced milks because what really alkalizes again are the minerals that milk is notoriously rich in calcium, magnesium and potassium. you know, and the fats, the fats are very alkalizing, and that's a whole another thing that people got to understand is that fat is really good for you. So, anyway, we've we've left the rin and now we're down in the lower gut. And so, when you've got this rin that's not functioning properly, now that's an aven intestine for the sake of the slide, but you can see what happened here. You know, perforation of the intestine. And what does that [clears throat] really mean? But when you look at what the villi, the villi are these finger-like projections that stick out of the tube called the small intestine. Obviously, it's there for surface area. It tremendously increases surface area. But maybe the most significant thing about this slide to me is the fact that this is such a a a major demonstration of what a vascular system that the gut is. And you can see the artery goes up here and then it diffuses back into the venus supply. Tremendous exchange going on here of absorption. So when you end up with this kind of a system, a vascular system that's like this, that's very important that this gut stays intact because this gut not only is a site for absorption of necessary nutrients that the blood supply now has to get, but it's also extremely important uh part of the immune system. There's an organ called pyr patches that are located in the villi of the small intestine. So your gut is extremely important to have a healthy immune system. The animal's gut is extremely important. The integrity of the gut is second to none in terms of importance to immunity. And so when you see this starting to go south because of what started in the rin when you start having an unhealthy rin believe me I can tell you that this is what you're looking at is a is a foul gut and absorption of nutrients starts to decrease and the infiltration of pathogens starts to increase. In human medicine we call this disbiosis. And I can tell you right here, right now, if you want to deal with getting well, you've got to correct dispiosis. And most people have some extent of dispiosis or not. In the United States, something like 75 or 80 million Americans are estimated to have candida yeast infections. That's a lot of people and they grow in the villi quite effectively when the acid alkaline balance is all out of whack and then you start feeding the wrong kinds of foods that foster the growth of yeast. And you know, I cut my teeth um in effect tutoring under a real maverick veterinarian in the late '7s by the name of John Whitaker. John Whitaker was a guy that um opened my eyes about blood ura nitrogen levels. He used to write for Acres USA years ago and he was a feed lot specialist actually. He learned about all this stuff from dealing with conventional operations in chickens and feed lots, beef feed lots and dairy feed lots. And the things that I learned from John about he about bun acidosis and the other thing is mcotoxicosis or mold poisoning. See that's the other problem with starch. Starches are great substrates for yeast and mold. And that's why we've got so much yeast infection with people is because we eat so much refined carbohydrate which is the perfect fuel for these pathogens. And animals have it too. So if you get this acid alkaline gut situation really compromised then then on top of everything else you get micotoxins in the the silages or in the stored grains and now you've got these things that are growing amongst the villi just like mold growing on a plant and they're feeding off the blood supply of that animal like a parasite and they're also producing tremendous quantities of micotoxic compounds u which we call micotoxins or um specific Specific names are like aphletox and that's just for one particular mold called aspiggillis flavus but there's a lot of other ones fuceriums and it's a huge huge problem anymore didn't used to be and we feel the main reason why it's a problem is twofold um the problems in the soils we've used a lot of biocides when we start destroying the uh the native flora like the microisy which protect the plant root and I got a slide I think in here somewhere but the the plant root is very much like the root hair is very much like the villi of the small intestine. This villi is coated with lactic acid organisms. They that's their habitat. And when things are right up here in the upper gut, they're right down here in the lower gut. And that villi is coated with these lactic acid organisms which produce really good antibiotic substances like nycin which by the way the pharmaceutical companies are synthesizing to make for an intramary infusion. Nyin produced by bugs, acetyloline, uh lacto peroxidase, uh lactic acid, hydrogen peroxide. These bugs produce tremendous quantities of pathogen growth inhibitors. So that's why fermented foods and humans are so important because it's loaded with all these bugs and all the things that these bugs produce which not only give you the benefits directly but they stimulate your indigenous flora or the animals indigenous flora to keep producing lots more of them. It's a different ecosystem down here than the rin completely different ecosystem but a fantastic one and it's all intact. It's just that's what's amazing about this system. And then you look at this slide here. This is a great slide. Look at the difference of the damaged villi versus the undamaged villi. You see what's going on here? And this could be a human, this could be a cow, this could be, you know, any kind of animal. But when you start getting damages from these toxic overloads from from what starts up in the upper gut, this is what happens. Your surface area decreases. You start getting scar tissue in here. So absorption of a nutrient starts to go down. Feed efficiency starts to drop. Immune systems start to get compromised. Look at the bloom over here on these villi. What a healthy gut looks like. So this is what we want to see in these animals is a gut that looks like that. And that's all starting with, you know, I keep saying it's a soil st. And then ultimately after the liver starts putting up with this crap for, you know, days, weeks, months, you know, [clears throat] you end up with livers that look like that. And I'll guarantee you if you got call cows and you call those cows out for either high sematic cell count or laminitis or reproductive failure, I don't care what it is, you autopsy that cow and I'll guarantee you 95 to 100% of those cows that look like that. what you saw in terms of laminitis or reproductive failure or chronic sematic cell count issues or whatever you saw basically the symptoms of the internal organs finally getting exhausted of having to [clears throat] deal with all this burden that we've been putting on that animal. And so eventually the liver becomes imploded with fat because it can't it can't work anymore. And then you ultimately call animals out. They drop dead sometimes right on site. they just poof, they're gone. Cuz when that shuts down, and what's amazing about the liver, it's so incredibly forgiving. It's one of the few organs that can practically regenerate itself after being almost annihilated. It can regenerate. So, when you've finally done that much damage, and like I said, that slide that I didn't have, but I talked about, it showed 19 out of the 24 hours on the TMR where the spike was like this. And 19 of those 24 hours was under the threshold of 6.0 pH. That's what you get. That's why you call the cows out. That's why they're 44 months of age average calling. That's why it can't happen. And when you think about the cost of cows, you know, it just blows my mind that the feed industry is still trying to find ways to buffer a cow. So, what do you buffer a cow? What do you buffer cows with? Baking soda, right? Okay. Think about this statistic. A cow that's making 60 pounds of milk a day needs to chew her cud 11 hours. It's a lot of cud chewing time, right? In that 11 hours, that cow will produce 3540 gallons of saliva. That's a hell of a large spatoon. 35 to 40 gallons of saliva. And that's equivalent to basically four to five pounds of bicarbonate. &gt;&gt; How much bicarbonate can you feed a cow? Maybe a pound if your sodium levels are allowable for that. Maybe a pound. So what happens to the rest of it? You just can't buffer the cow. So you know and you know and and then the problem you have is this dilemas where you're trying to say okay trying to get this guy to feed some long quality effective fiber hay or even straw, you know, but then that cuts into what? Production. How much are heers going for over here? &gt;&gt; What a replacement heers sell for over here? &gt;&gt; About 1200. &gt;&gt; Anywhere from 900 to,400. Yeah, about the same in the states. So, I don't understand that economics system. I mean, I don't understand how he prices are hanging in there for the last decade around that. They fluctuate like this. Milk prices are like this, you know. Coal cow prices are like this, you know. Heat. [music] [music] [music] Hey, Heat.</t>
+          <t>Hi friends, golfers. This is part two for those of you that hate seeing in the video your knee going out like this on the down swing. So you're swinging it goes here. First we covered relationship between heel toe on the way we're moving back using an alignment stick and the weight down how we're pushing here. We're going to cover just working on that trail knee. So real simple drill. Okay. So you set up an aim stick here. Shove it in the ground. Whatever you have to do. And I just all you're going to do is put it in front of your knee. And I want you to feel the difference in this move. Okay. Some of you that are older will remember Tom Wargo from the senior tour and he had every shot like this and I want you to look at my back foot down. I want you kind of doing this for a while feeling like this lead knee is staying inside or the trail knee is staying inside the lead. Okay. But this is going to give you the reinforcement here so that when I go up and I come down my left side start pushing down. Look how that knee works more like this. See it's in. And it also helps me. Now the lead leg is pushing back and I get that nice push back. Okay. So real real let me show you how how to do it. Just, you know, get it about an inch away or so. And we don't want to go fast because we want to learn to do the move um and feel really feel it. Okay. So if I'm here, make sure I'm on the left side. Boom. So see that just stays in here. Boom. Leave leg straighten. Work on this line stick. You'll you'll get really good at where you start hitting and then you can go full after you've recreated these steels and learned how your feet move on the ground and understand those ground reaction forces. Thanks again for watching this part two. Eric Schs golf sign</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -667,96 +638,62 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>yCrAg9vRp2E</t>
+          <t>OJWTDx0nNy4</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Gold from the Vaults - Jerry Brunetti - Soil &amp; Livestock Health - The Rumen is an Ecosystem - Ep 9</t>
+          <t>Why You’re Not Compressing the Golf Ball — And How to Fix it with my Pressure Shift Drill!</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>We’ve reached the end of Series 4 of our 'How to do it' video series, so while we prepare the next instalment, we are diving into the archives to share some classic *Gold from the Vault* content. In this session, we revisit the late, great Jerry Brunetti and his profound insights into the inseparable link between soil fertility and animal wellness.
-Jerry Brunetti was a true pioneer who understood that you cannot treat a cow in isolation from the ground she walks upon. In this first part of his legendary presentation, Jerry breaks down the "reductionist" trap of modern agriculture and medicine, explaining why a high-protein diet might actually be poisoning your herd. From "manureology" to the intricacies of the rumen ecosystem, this is a must-watch for any farmer looking to transition from disease management to true wellness care.
-#NutritionFarming #SoilHealth #LivestockHealth #RegenerativeAg #JerryBrunetti #EcoAgriculture #AnimalWellness
-*What you’ll learn in this episode:*
-🥬 Why the *pharmacies* of the future will actually be *farms* .
-🧬 The "funny protein" trap: How high crude protein can lead to ammonia toxicity.
-💩 The science of *manureology* : What a colander and a jet stream can tell you about your herd's health.
-📈 The historical connection between glacial soils and the robust health of the early pioneers.
-🧪 Understanding the *microbial bridge* and the rumen as a fermentation ecosystem.
-👇 *Chapters:*
-00:00 - Soils &amp; Livestock Introduction
-01:39 - Title Sequence
-02:08 - Soil and Stock Health
-05:06 - The current state of play
-07:57 - Milk? Commodity or Medicine?
-10:47 - Dr William Albrect
-11:45 - Fertility: The Great Plains &amp; 40 Million Bison
-13:29 - Herd Health Begins with Digestion
-17:01 - pH &amp; Acidosis
-20:42 - The Rumen as an Ecosystem
-33:57 - End Credits
-Want to learn more about Nutrition Farming? Check out Graeme's How to do it episode *Getting Started with Nutrition Farming® – 10 Practical Steps to Transform Your Soil and Crop Health - Part 2* …
-https://blog.nutri-tech.com.au/getting-started-with-nutrition-farming-r-10-practical-steps-to-transform-your-soil-and-crop-health-part-2/
-*Nutri-Life BAM™*
-https://nutri-tech.com.au/products/nutri-life-bam
-*Nutri-Gyp™ Natural Gypsum*
-https://nutri-tech.com.au/products/nutri-gyp
-*Sili-Cal (B)™*
-https://nutri-tech.com.au/products/sili-cal-b
-…or try our new NTS FulvX™ Powder for chelation
-https://nutri-tech.com.au/products/nts-fulvx-powder
-*Interested in attending a Certificate in Nutrition Farming course?*
-https://nutri-tech.com.au/pages/courses
-Need assistance? Try out our Soil &amp; Plant Therapy Services
-https://nutri-tech.com.au/pages/soil-plant-therapy
-How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait
-Head to our website to find out more
-https://nutri-tech.com.au/
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-*Follow us on Social Media*
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-Twitter: https://x.com/ntsaustralia</t>
+          <t>Most golfers are trying to compress the golf ball while staying stuck on their trail side. That does not work.
+In this video, I break down why pressure shift is one of the biggest missing pieces in the golf swing and why so many golfers never get to their lead side in time. That is why they hang back, lose shaft lean, lose rotation, and struggle to compress the golf ball.
+I go through the truth about pressure shift, why the old 80/20 advice got misread, and the exact drills I use in lessons to get golfers moving more like elite players. If you want better strike, more compression, and more distance, this is where it starts.
+Work on these drills and let me know what you feel.
+Get my free drills guide here:
+EJSGolf.com/my-drills
+Coach Erik Schjolberg
+The Science of Better Golf
+EJSGolf.com
+Scottsdale Golf Lessons
+Online Golf Lessons  
+#SGL #golfswing #EJSGolfAcademy #CoachErik #golftechnique #golftips #golfdrills #golflessons #stopcasting #stopscooping #shaftlean #onlinegolflessons  #ScottsdaleGolfLessons #golfswingmechanics #golfswinganalysis #golfimpact #golfpower #golfdistance #ejsgolf  #Titleist #Linksoul</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-06T08:05:39Z</t>
+          <t>2026-03-13T23:56:22Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>756</t>
+          <t>123</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.034392</v>
+        <v>0.00813</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -765,117 +702,65 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Well, anyway, um we're going to cover a lot of topics. We're going to cover soils. We're going to cover animal health. We're going to cover soil um forage density. And what I hope to um convey to you folks is that um animal health really I mean often times I get asked to speak on just animal health and uh what typically happens when I do that is I end up starting talking about soils which probably gets people's eyes to get blurry. we're talking about souls for when you really want to know how to treat mastitis or you really want to know how to treat calf scour or ketosis and I will cover those things but I I can't emphasize enough being in this work for nearly three decades now working with all kinds of of farmers from uh mostly which we have as Amish farmers in Pennsylvania um we are a fairly busy dairy state um in Lancaster County alone we are the second largest dairy producing county in the United States only behind county which is a feed lot type of dairy operation in California. We have 2200 dairies in Lancaster County that average about 60 cows. So it's a very busy place with a lot of farms and that's the way we like it. We think we don't care really whether farms are large or small. We like to see lots of farmers. We like to see lots of farms run by families. And so we get a whole variety of challenges because we have a whole variety of soils, whole variety of management issues. But ultimately we try to sew it all together by saying you know certain fundamentals you just can't deviate very far from and um really it becomes as I get older and older which is happening faster and faster um I realize that um the fundamentals really are much much simpler than you really would realize [music] &gt;&gt; [music] &gt;&gt; It's not necessarily something we don't have any magic bullets, but we do see mirrors. Um, and I saw those back in the days when I knew a lot less than I did now. And ultimately, we try to reconcile this thing by bringing on bringing it on home and recognizing that real stock health starts with soil fertility. And I'm going to show you some slides of Malibar Farms, which is a an incredible success story that happened in the 40s and 50s in the United States by Louis Broomfield, who was one of my heroes when I started getting into agriculture in the late 60s and early 70s. He was a Puler surprisewinning author that restored a completely blown out piece of of property in Knox County, Hill Country of Ohio, 1,000 acres of gullied land into into farmland that brought back 15 springs that were exhausted from drought and brought them back so that they could actually use them again for drought. Stories like this are really exciting to me because it's already been done. I'll talk a little bit about Randlay Farms, which was the top herd in in uh in the world for Jersey cows out of New York State by William Keenan. Talk a little bit about Carnation Dairy, which was the top herd in the world, bar none, back in Washington State in the ' 50s, 40s, and 30s. So, those are my teachers. Um, you know, I I think it's a back to the future kind of thing. And that's the great news that we don't have to re relearn all this stuff. It's already been done for us by guys like William Alrech and Dr. Royal Lee and uh uh Dr. Harvey who started the US public health service. I mean there were some tremendous uh farming and health giants that existed back in the early part of the century and there's tons of information that we now can draw upon and put into use. And um I'm fortunate in that I cut my teeth with not just those kinds of people who have since gone on before us but their um proteges. I had learned from them and turn taught people like me so that the torch can be carried on. So anyway, let's uh let's move on with this talk and I always like to bring this quote in there by Fat Sean. that which is lacking in the present world is profound knowledge of the nature of things. And I think that's kind of a really a mantra for me anymore that we recognize that there's this the things that we treat try to understand in a reductionist sense. You know, if you start taking things apart, you take things apart, you take things apart and it's a whole saying of what a specialist is. He he constantly specializes the point there's no consilience between the specialties. You know, you see this particularly in medicine. you know, you talk to specialists that are neurosurgeons that aren't talking to other specialists in the hospital. And as a consequence, there's a great deal of of disease management instead of wellness care. And the same is true on farms. We have aronomists that don't know anything about how a rumin works. And we have dairy nutritionists that don't know how uh the soil food web and soil fertility issues are are are really important to produce the kinds of rubin foods and fuels and proteins that we have to have in order to have sustainable herds. In the United States, our dairy herd populations are lasting 44 months before they're all called out. That's the average age of a dairy cow before they call them out in the United States. 44 months. So, that's not even three lactations. Not even two lactations. So, what's going on here? Is this really is this really progress? You know, I just came from the Sheperton um uh festival over there, which was a conventional uh dairy festival and and uh I should say conference, not festival, but um you know, you hear the same thing as the conventional things all the time, which is how do we become more efficient? How do we get bigger? Um and I feel that I don't size is not the issue in the United States. Cornell University out of New York State has now made the prediction as of recently that we have 105,000 dairy farms left in the United States. In 1960 we had 2 million dairy farms in the United States. So we've lost 95% of that which was in 1960. So the [clears throat] get bigger get out sort of um axiom was followed was it? So now they're saying from here on in from 19 or should 2004 until 2020 which is a mere 16 years away. Thank you. We're talking about going from 105,000 dairy farms down to 16,000. The entire United States, 16,000 dairies. And they're saying that those farms that are milking less than 100 cows will dwindle from 84,000 down to 7,000. And those that are milking more than 500 cows will increase from 2,700 to 3,400. So is this Yeah. &gt;&gt; Okay. For Congress, Jerry? &gt;&gt; Yes. &gt;&gt; Yeah. Yeah, we're going through the same destruction process here, but it's a distorted economic system that's driving it, isn't it? &gt;&gt; Exactly. Yeah. It's all And if it wasn't for Well, and the thing about it is our ancestors uh put the dairy belt together, United States where in the northeastern and upper Midwestern states, the cool season grass areas where you got natural rainfall u and cows did well there without a lot of input. And the new dairy industries are moving into the western states basically relying on commodity purchases which are subsidized by farm bill policies that cause farmers to grow cheap corn, cheap soybeans and run it through feed lot kinds of operations. My feeling about this is is okay I can't do anything about that. I know that. I mean I I realize that the genie's out of the bottom. So in Pennsylvania where we have Amish Menite family farms are not going to get to be 500 cow herds because they can't even if they wanted to. They're just not designed for that. They have 80 acres, you know. So we've got already too many animals from that land producing way too much pot ash and phosphate on the ground. It's ending up in the estuary called the Chesapeake Bay. So what are we going to do? Well, we're trying to take a whole new angle of this thing and say, okay, what is really the cost of production all about? and who's our market and what really is milk. I'm going to talk about that tonight. What is milk? Should it be a commodity or should it be a medicinal substance? And and I'll talk about this medicinal substance factor because in my opinion, being a recovering um individual from a life-threatening illness, I know firsthand that food is medicine and it ought to be medicine. And if it's not medicine, then it's killing you. Either food is healing you or it's killing you. That's the way I look at it. There's no in between. either you're pregnant or you're not pregnant. You know, it's one of those kind of deals. So, either you're getting well or you're getting worse. And uh and I had a window closing on me said either get well or die in 6 months. So, I know that food either heals you or it doesn't. And if [clears throat] it's not healing you, it's not neutral. It's either contributing to health. And that's what to me this is all about. These meetings in in in Australia or these meetings in Pennsylvania are about the future of not just farming but the future of mankind because the farming of the future is going to be about the fact that the pharmacies of the future are going to be farms. And I'll guarantee that's a prophecy that I'd make up. But you can go to the bank with it because in my country, and I guess it's true here, the baby boom generation, which is the single largest population of our country numbers wise, and uh birth rate started in 1946 after the war to 1964. Single largest population is about to hit gray in about three more years. And [clears throat] we spend more on health care uh than any other country in the face of the earth. We have a $1 trillion health care system and a $1.4 trillion agricultural system. And that's not coincidental that they're almost equal. And it's not coincidental to me that when you go to shop for so-called groceries at the grocery store or the supermarket, it's also the same building that houses the pharmacy. Because me the foods are so un unbelievably incapable of sustaining life that you have to rely on pharmaceutical medications to to stay alive. So I I I contend that these meetings are about mankind. These are about society. These are about economics. It's about ecologics. It's about farming. And so [clears throat] I'm here to talk to you about the fact that I think if we start looking at the way our forebears looked at farming which was a health issue. I mean Harvey [clears throat] Wy Dr. Harvey Wy founded the US Public Health Service and he was so convinced that health had everything to do with farming that he pulled soil samples from every single county in the United States back in the early 1900s. He eventually was fired from his task. He started the Food Chemistry Division which became the Food and Drug Administration. Eventually under the USDA started that he was fired from his job under the Taft administration because he was basically trying to contain large powerful interests, pharmaceutical interests that were just starting then. Well, if you think they were powerful in 1912, you can just imagine how powerful they are a century later. So, he knew it. Alrech knew it. How many people have heard of Dr. William Alrech, which is a lot of Okay. Well, Alrech, Albert was a medical student, or at least he started being a medical student. And one of the [clears throat] things that he knew uh that convinced him that soils were the keystone of the health of a civilization in our own country, he actually researched the World War I draft records. And he found out where they had the highest acceptance rates and the highest rejection rates for the doughboys that were going off to World War I. And he found interesting corlaries in that the um the highest rejection rates were in the states of lower Missouri and higher Arkansas, which is the Ozark Mountains, thin rocky soils, not a lot of minerals there. And the highest acceptance rates were in Iowa and Nebraska where the appetiti soils were the calcium phosphate soils, the appetiti soils. They were the rich soils, the calcium phosphate soils. That's where 30 million bison ran from Canada down to Oklahoma and Texas every year recycling nutrients on the Apatiti soils. We had 40 million almost 40 million head about 30 million of them about in that part of the country and the rest of them were scattered through the great plains and as far east as the east coast actually they called them uh forest vines. They were same species but they had adapted to the woodlands and the east coast. So we had this incredible wealth glacial tilt and and that's one of the advantages North America did have over even Australia is we were glaciated and those apotiti soils created a civilization of bison and it ultimately started to create a civilization of of uh Americans that were strong and robust coming from that part of the country. So he knew soils related to because in in World War I in 1917 1918 people didn't haul food in from Florida and California you know there wasn't that kind of a food system back then you ate where you lived whatever you got you got locally so it was a very good correlary today you couldn't do that because in the United States the average distance from uh farm to plate is 1500 miles now every meal you eat in the United States you are buying food that's on the average hauled 1500 miles so that those demographics wouldn't work today. So that's how all this stuff got started was people realize look at the connection between the soil and the health of the people living on those soils and you know was very conclusive. So I think this quote kind of sums that up in that you know we don't look at the obvious now as a animal stock kind of a character I go to this first this is the first place I go when I go to a farm is I look at the cows but I look at the manure and if you're going to deal with health whether it's human health or animal health you've got to look at that which leaves the body because that's the clue food. It's the indication, and I'll say this, an animal or a human is only as healthy as its digestion is. And there's another pandemic we have with people in the United States is god-awful digestion. And look at the prescriptions and over-the-counter drugs. Number one, probably behind aspirins and headache pills are those that deal with bad digestion, including the channel calcium blockers, channel blockers, the um ant acids, all these things that people are taking. isn't because they have excessive stomach secretions. It's because they have deficiencies. 80% of the people anyway, 80% of those that are suffering from reflux have compromised digestion. Livestock have compromised digestion because we aren't looking at the blueprint of what a ruminant is. Aruminant doesn't eat grain. There's only one species of animal that's designed to eat grain is grain, and that's birds. And the reason why birds can eat it and not go through hell eating grain is because they've got an organ called a crop. And that crop is right here. You know, if you pick up chooks at night in the rugery, you can feel the grain that they store in that crop. What is the crop? It's a fermentation vat. But really, it's more of a sprouting vat. What is grain? It's seeds. And seeds have things in them that aren't really good for higher life forms like mammals. And they contain compounds called phytic acid and phitates. Uh they contain enzyme inhibitors. And the way you get rid of these negatives in seed is by doing what seed does best, which is to let it grow. You sprout it. Now you can cook it and that'll destroy the phytic acid and it'll destroy the enzyme inhibitors. That's why you can't feed raw soybeans in the United States to dairy cows to an extent that you cause trison inhibitor problems. Right? Very trison inhibitor. For raw soybeans, you're limited to how many beans you can feed because of the trips inhibitor. Well, it's the same problem they have with all grains. All grains have these enzyme inhibitors. So, when we're starting to realize that we're trying to make milk production or put meat on an animal, we can do it with grain. Clearly, that's proven. There's no doubt about that. But when we start doing that, we recognize, well, what is the price we're paying for that? and we start looking at, you know, the manure on these animals and recognize that there should be a whole science out here called manureology. There's geology, you know, and there's all kinds ofies, but there should be a minurology course out here. And uh you pick up that pie and you look at that pie, you put it in a colander, you know, you put another screen colander on top of that. That's that's a real important thing. put the second colander on top of the first one before you do what I'm telling you to do and hit it with a jet stream because if you don't do that, [clears throat] you'll be really ticked off that I didn't tell you that, you know, and you don't use your spaghetti colander from the kitchen. You have a designated colander, okay? And you take that manure pod, you throw it in that colander, and you look at what is left after you blast it with a high stream of water. Now, if you're feeding grain, there shouldn't be any grain in there, period. If you're not feeding grain, there should be a small amount of digestible fiber from the forages. Maybe a quarter of a cup of broken down fiber. That's all that should be left in that cowpie. Furthermore, that cowpie should have the right consistency. Should not be slimy. It should not have a lot of bubbling going on. That tells you there's acidosis coming out of that animal. It should have a pH. If you have a pH meter, you stick that in that pie. That pH should be around 65 on up. The other thing we do is we look at the urine and we test the urine. The urine should always be slightly acidic around six 265. You never want to see urine get above 7 especially 75 and 8. And the reason for that is because metabolic waste is excreted in the urine. This is true for your own urine. If you want to find out if you're healthy, check your urine first thing in the morning. It should be above six, but it shouldn't be really alkaline either. And the reason for that, if it starts becoming really alkaline, and this is true in the cow because most people think, well, one target because the urine's alkaline. The reason why you don't want to do that is because if the urine is supposed to be acidic because there's metabolic waste leaving the animal and all of a sudden you start seeing the urine of the animals are running at eight. What does that tell you? Well, tells me that the buffering system of that animal is just gone. Which now seems kind of ironic because buffers raise pH. And so if the buffering system is gone, why would the urine pH be alkaline? It should be acidic. Well, here's what happens. And this is very relevant to your own physiology. The blood pH of the cow and the human is about 7.4, slightly alkaline. And that blood pH wants to stay there and it will stay there at all costs at about 7.4. It might go down about 7.35. It might go up about 7.425 or something like that, but it'll stay right about 7.4. It has to do that or there's death. That's your option. 74 or you die. So the body will do everything it can to maintain the blood pH of 74. Well, what maintains a blood pH of 74? Cationic minerals, alkaline minerals, calcium, magnesium, potassium, sodium, some of the trace elements. Those are your buffered minerals. Curiously enough, those are the same cationic minerals we're going to talk about today that buffer the soil and they have to be in the right ratio in the soil as they have to be in the right ratio in the physiology of an animal. The same things are working in a soil are working in the air. Okay, this acid alkaline issue is universal. It's the way nature works. So the alkaline minerals buffer the blood. If we see that the pH of the blood is dropping, we know we've got acidosis issues. But if we see the manure of the pH, pH of the manure, excuse me, dropping, then we know we really have acidosis issues. If we see the urine of the of the animal going up, chances are you'll see that the manure may be going down. And the reason for it again is if the urine pHes are going up, it means that you are deficient in buffering minerals. Okay, so now comes the stupid question. Why did the pH go up if you're deficient in buffering minerals? Well, like I said, the animal will buffer at all costs. There's one other thing it can buffer with, and it's loaded in conventional farming operation feed stuffs, and it's called ammonia. So you could actually test the urine for ammonia and you'll find it there. And that's what's driving the pH because the pH of ammonia runs over 10. See? So the body of that animal will even cannibalize its own tissues. Although with most dairy herds or beef herd operations, it doesn't have to do that because the funny protein that most farmers are growing is so loaded with nonproin nitrogen or nitrate or ura, whatever you want to call it, instead of real protein. There's plenty of raw materials to produce ammonia and I'm going to go into that in a little bit. So what I'm trying to give you is pictures. We're looking at these things ecosystems and what we're looking at here is a rin that is the primary ecosystem. Remember all health starts to begin to get better or begin to fail based on digestion. You're only as healthy as the microfllora in the small intestine. And with a ruminant animal that has a fermentation system that precedes the true stomach, you know, we start out with the true stomach, they start out with a rumin, then they end up with the true stomach, then we all end up with a small intestine. &gt;&gt; This is not coincidental that these systems go from, you know, in a ruminant slightly acid to very acid to very alkaline. That's the way it has to work. And if this manure is telling you otherwise, everything else is going to be screwed up. The band-aids that you're going to have to use on that herd are going to go up in cost because you're going to have to supplement to put out the fires that you created by trying to make milk production from architecturally the wrong food stuffs. And the reason why you're going to do that is because you can't make milk without energy. Energy is the limiting factor in stock. putting on weight, putting on milk. So, if you don't have the energy in the forage, naturally the nutritionist is going to come along and say, you know, obviously your cows are in bad condition. You're not getting them bred back. You know, you're not making the milk you're really wanting to make. So, they turn up the thermostat, which is the BTUs, which comes from cereal. But the problem they have is they don't believe or if they do believe they're not telling anybody that you can actually create energy and forages. So that's what I'm here to tell you is that the real secret to this thing is to do what these other people have done already with the top herds in the world of the Jersey herds and the and the Holene herds and the Gernzy herds. Carnation had top cows in all breeds in the 50s. So and they did it on a high forage ration. So we go from that slide to this slide. And this is this slide could be a whole day. We could actually do a whole day on this this slide, but I promise I won't. So, but I will give you the the the real the creme creme here. This is the rin. This triangle here represents protein. And you see it's split into two sections. We have what we call true protein. What is true protein? Amino acids. methionine, tryptophane, tyrrosine, lysine, amino acids. That's what true protein is. The building blocks of the body are amino acids. Peptides are are groups of those. Then we have this stuff here called nonproin nitrogen, which is not protein, it's nitrogen. Why is it in the protein triangle? Well, go to the very top of that slide. You'll see CP equals N * 6.25. CP stands for crude protein. Crude protein is not, I repeat, crude protein is not a measure of amino acids. Yes, &gt;&gt; good point, J. That's the one they use. What the heck? &gt;&gt; Well, that's what we're going to do. We're going to we're going to do an end round run here and show you how you can take food protein and figure out whether or not you have any true protein in it. Okay, that's that's what we're going to try to do here. And there's some there's some little tricks here because no lab is going to test your amino acid levels of your forage is because it would cost you a bloody fortune to have that done. So, and the reason why they test for crude protein is because all protein without exception on the average, there's that word again. You know what they say about average, you know the definition of averages is you have one foot on dry ice, you have another foot in boiling water and you're comfortable. That's an average. Okay? So when [clears throat] they say averages, always be aware of that word because you what do you mean by averages? So you have all on the average all protein contains 16% nitrogen. It's the only stuff that does contain nitrogen. So if you divide 16 into 100, you come up to 6.25. It's an arbitrary number. It's a starting point. It's not an ending point. So now we've got this thing saying, okay, you've got a 22% protein alpha alpha or a 29% protein alpha alpha. What do you really have? How do you know that's protein? How do you know it's this piece, not that piece? Some of it's And you can see in all in all protein, you're always going to get a little this. Now, here's what happens, and this is what's important to remember. You see the top arrow, the top arrow, 60%. What that says is 60% of true protein solubilizes in the rin to produce ammonia. That's a good thing because what are you feeding now? You're feeding not the cow anymore. You're feeding the cow's basically ecosystem which are microbes. So ammonia becomes the food stuff or the protein for simple life forms called bacteria. Bacteria. And what you got in this room in here, best description I can give it to you, it's like the Serengeti or the savannah. The bacteria are the grazers. They're the herbivores. And then they're prayed on by, and I'll talk about this, the soil food web works the same way. They're prayed on especially by prozzoa, which eat the bacteria. And in the process of bacteria being consumed by other organisms, a lot of energy and a lot of protein is recycled over and over again, increasing the efficiency. And that's exactly what happens in the soil when you have a really healthy soil food web. You recycle the nitrogen. You don't waste it. So what happens here is you've got the Serengeti going on here with the the herbivores, the grazers being the bacteria, which are by the way bacteria are the nitrogen sink of the soil and bacteria are the nitrogen sink of the rin. You want lots of bacteria in that rin because they suck up this stuff. That's why you can feed a cow or a goat or rin I should say ura because they're eating ura and they're synthesizing ura. certain amounts of it. So, but here's the caveat is that with the funny protein, I call this funny protein. The funny protein, 100% of it solubilizes into ammonia compared to 60%. So, needless to say, if you've got a 28% crude protein, I'll guarantee you based on what I can look at the rest of the soil or the forage test, you're going to see this fraction getting much much larger. That means this overflow ammonia gets larger and larger because what has to happen is remember Alrech used to use the axiom all life forms need go foods and grow foods. Grow foods are your proteins or nitrogen. Go foods are your carbons or your energy. So you've got this grow food here. You need go food. Microbes in the rin need go food. There is the wall that the dairy and the beef industry has hit because they're not producing the kinds of go foods or carbohydrates that these microbes that live on this ammonia can populate themselves on. So they come along and they instead of feeding the rin they have to feed the cow by feeding them grain. These organisms are cellulitic organisms, ptoolytic organisms, that is they have a specific substrate that they feed on which are the soluble fibers. So if this level gets up too high because you either fed too much protein or the quality of your protein was too funny, too high in NPN or because you didn't have enough of the right kinds of soluble fibrous energies. Any of those three reasons, you now get this buildup of ammonia which flows through the rin wall. Goes right through the rin wall. Now it's in the bloodstream. alarms start going off and now we got a veterinarian condition called BUN blood ura nitrogen toxic compound and when the blood ura nitrogen levels get to be certain at certain levels you start having all kinds of problems first thing that starts to happen is you don't get cow's bred or if they're bred they won't hold a calf that's the first thing second thing that happens is the kind of stuff that happens in places like western Washington state, high rainfall area, 110 inches of rainfall every year normally. Wouldn't you like to have that here? [laughter] No, you wouldn't. No, you wouldn't. and you go into the Tanuk Valley and it's a dairy area and you go in that area and it's and it's all grass and uh you talk to dairy farmers there and you look at the cows and they're got these rough coats and they're droopy and they're not making great. They're not nobody's having a good time. And you stand there and you look at what's going on. You see the uh the fertigation systems where they're sucking out the the slurry manure and that becomes their fertility program in all these paddics or lays or pastures. What's in slurry manure? What are the primary nutrients in slurry manure? Nitrogen and potassium. The antidote to energy and forage. It's the best way to strip energy out of grasses and leg rooms is dump the nitrogen in the pod ash arm. I'll go into that. All right. So, this is what's going on. Meanwhile, this dairy farmer tells you, "I don't understand this." He said, "I got halage in this this bail over here. It's 27 28% protein." He thinks it's protein. And he said, "And then when I buy hay from the eastern part of Washington State, which is high desert, they get 26 in of rainfall a year and they grow and they have high mineralized soils there and they raise a lot of alalfa there." and he buys a 17% protein alpha alpha hay. The cows come up in milk and he doesn't understand why. And the reason why is because as this ammonia is running around in the bloodstream and the liver knows in its wisdom that it's got to get rid of it. Now see all the blood ultimately gets goes gets a chance to go through the liver. Thank God we've got livers. All the blood gets the chance to go through the liver. And when the liver senses ammonia, what does it do to it? It wants to detoxify it. So, it turns it into a less toxic substance called ura. URA is less toxic than ammonia. They're cousins. Ammonia's NH3 basically and ura's NH2. It's less toxic. Then it sends it back out in the bloodstream and ultimately the kidneys pick up all the blood and the kidneys take the ura and they change it once again into uric acid. and then out the end of the cow goes. Well, assuming you don't have cows dropping dead, which if it gets high enough they will, uh, now the dairy industry in the United States, and I suppose it's possible that's going on here, they have this thing called amuent, milk ura nitrogen. To detect blood ura nitrogen, you have to pull blood tests and usually the vets do that. Now, they've got, you know, you can test right on your own farm for milk nitrogen. In fact, you can test for milk nitrogen now with test kits. In 1996, I was in the UK and I was talking this story. This very same slide was there in front of the people in the UK 1996 and we were talking about this and this one dairyman came up to me later and said, "Man, you hit it right on the head with my farm." I said, "How do you say?" And he said, "Well," he said, "we had calf deaths like you couldn't believe. We just had all our calves were dying. We vaccinated. We had antibiotics on those animals. The vets were just pulling out their hair. And then somebody told me about MUN. And I didn't know what mu meant. And I found out I could buy a kit from the continent to test my milk for mun. And sure enough, his milk was so loaded with this nitrogen substance that it was poisoning his calves, which are not ruminants that cannot deal with it the way a ruminant can. They're monogastrics when they're babies. And so they were dying from nitrate poison. That's what happened. And he didn't. And what did he do? Instead of giving him wonderful whole milk, which is a medicinal substance for calves, it's loaded with all of these enzymes, vitamins, minerals, antibodies, lactic acid organisms, and on and on and on. You know, you had to give them milk</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Thank you for posting. I never got to meet Jerry in person, but this helps me get to know him in a way now. || Thank you  for sharing || Biofertz represent 🪱🌳☀️🐝</t>
-        </is>
-      </c>
+          <t>Hi. Are you not getting pressure to your lead side? Are you stuck back something like this? Not getting the compression you want, not getting the shaft you want? I got great drills for you today. And we're going to be talking about pressure shift. getting like the tour pros who are like this at impacting 80 to 90% to their lead foot. What I see in my lessons is 80 and 90% on their back foot back here in transition and maybe 60% by the time they're at impact. Hi, I'm Eric Short with EJS Golf. Stick with me today. I got great drills for you today to get you to start to compress the ball, hitting it further and compressing it. Like I said, shaftling and rotation, they all go together, folks. All of them go together. So, welcome in to my bay here at Scottsdale, Arizona, McCormack Ranch. So, let's talk a bit about exactly what goes on in the golf swing and where these misconceptions have gone wrong. So, as I grew up, we heard about this 8020 shift. The problem was is the 8020 shift is happening all the way through to here. The shift should only happen to about here. Okay? Good players are only shifting pressure to right here. From here forward, there's no more shift going into this trail foot. It's starting to go over to this side. So, we're reentering back into the middle by this point. Okay? So, everything is going towards the lead side. Most golfers just continue to load, load, load, load, load, load, load, load, load. That's why this low and slow advice that we've heard in the past was so bad because what would what would that cause? It caused everybody to just to keep loading into this trail side. I'd rather see some speed to cause some breaking forces. Now, what's a breaking force? It's a force in this back leg that's going to stop me from going into it and get me to start going this way. Now, a key concept to understand about this is force precedes motion. Okay. Now, what happens is is lay viewers, they view video and they go, "Okay, I see this golfer moving." Now, the problem is is since force proceeds motion, they've been pushing way before you see them moving. Okay? So you have to assume if you see somebody moving this way, it happened way before since the force had to push there. It's not instantaneous. I go, "Okay, I'm here. Here it happens. I have to start pushing." So for a golfer to load here, they're starting to push right away to get over there. It doesn't happen at the top. And that's where everything's gotten confused. Okay? It's a way earlier move. So I want you to think about the maximum load is just to right here. And then we want to make sure we're getting into our lead foot massively by impact. Okay, so let's get into how we're gonna do this. And I'm not going to make this super long video where we get way into details because I have other ones where we can talk a ton about ground reaction forces and stuff like that, but I I want to get more into a couple of drills that are really kind of just going to help you with this. Okay? And this is one of my favorite ones to um feel this. I call the heel to heel toe stomp drill. Okay. So, how you're going to set up is this. This heel is going to be up. This toe is going to be up. So, lead toe up and the heel up on the back foot. Now, the way we start our back swing is this stops down with a lot of pressure and force. And then almost immediately we're pushing down into this lead foot. Okay? So, I go boom. So this is up boom boom. So you go it's working backwards. Okay. So I go heel to toe heel. So I'm towing this and then I slam this heel down here so I can get back into this heel over this lead foot. Okay. So heel is up on this lead foot and I'm kind of feeling the toe up a little bit in my shoe here. So I slam this down and I'm going slow here. And now I'm in the toe over here on my lead foot. Now I'm right away I'm picking that up and I'm picking that foot up and I'm now I'm slamming this heel down which is moving me over into this lead side. Okay, that's the heel toe stop and we can hit with this. Okay, so I start with my heel up and feel kind of the toe slam down. Boom. Boom. And you can already see just with me doing that. I wasn't even trying and the speed generation was just really incredible. Okay, so toe heel up feel kind of toes up and sometimes I think it's good just start this way. Boom boom boom. And I want to feel some speed with it. Okay. So, I'm quickly boom, boom. And the key is getting this back down quickly because if I'm slamming this down, I need to get back over to this lead side. So, I want to slam this front side down quickly as possible because this toe is coming up, which raises this heel up and boom. And then I can slam that down and gain a lot of speed. And you can hit with this. It's a great drill to hit with. Great. And and I want you just to focus on what the body is doing. Don't worry so much about the shot. Okay? But if I'm just here, I'm going here. Boom. I just absolutely ripped that thing. Okay. And I felt like I didn't even swing at it. Okay. So, heel toe stomp for that one. All right. Now, next one we're going to do is we're going to do kind of a a couple step step drills. And you can find a bunch of these on my uh on my YouTube page where you're at right now. So, and this is just getting the feeling of getting to that lead side and our body working in two ways at the same time. Because what it is like if when you're on your back foot here, it's like throwing a ball like this. You would never throw a baseball. If you were throwing a baseball, you would everything would be like this. Everything is forward in in in life that we do in any sport. We would never be like this that we do in golf from our back foot. Okay? So, I want you just get your feet together. Club goes like this. And when this club starts going back, we're going to step forward and go. Okay. So, what is this doing? This is moving our body in two ways at the same time. Okay. So, I'm going here and I step and go. All right. Now, this is another drill we can hit with. Now, I just want you to time this out. I want you to see how big your step is so that we get the step correct. I don't want you hitting it from way off the back. And I'm going to show you how we can do this. Again, I'm just going to test. My step is about right to here. Okay. Another great feeling again. Okay, now I'm going to show you one more version of this step drill that baseball players seem to love. I didn't play baseball growing up uh much. I obviously can swing a bat, but we're just going to go tap tap. Okay, so I'll show it from this end, too. So, if I start here, feet apart, tap tap. So, the key is here. I want to get this back here, but then I want to get this tapped right away. Now, the key is I don't want this center staying back and just like stepping this way. I want the center going with me like that. Okay? So, it'll be like this. Forward, step, boom. You're going to notice these are powerful moves that help you start compressing the golf ball and give you that feeling down to this rotation and down here like this, down here that you've been wanting for a long time. I hear it in my lessons all the time. It's what I change in lessons all the time. So, go through these drills, work on them, give me some feedback down below. Let me know what you think after doing some of these drills. Also, check out my drills guide, which are going to hit a whole host of other um issues that you have. My ejsgolf.com/my-drills. You'll see a link down below. But thanks for watching ejsgolf.com. And uh thanks for watching. Again, Eric Schwberg, the science of better golf.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>iktPekYGwzQ</t>
+          <t>6IIsc4TL71g</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Regenerative Cattle Management: Doubling Capacity &amp; Reviving the Soil Food Web - How to S4E14</t>
+          <t>🏌️‍♂️ Stop Pulling FIRST in TRANSITION and Start Rotating Through Impact with Shaft Lean an #shorts</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>*Regenerative Cattle Management: Doubling Capacity &amp; Reviving the Soil Food Web*
-In this inspiring session filmed at the Bolivia Landcare field day, I sit down with Jake Smith, a passionate cattleman managing 8,500 acres around Tenterfield. We dive deep into his remarkable transition from industrial set-stocking to adaptive multi-paddock grazing. 
-#RegenerativeAgriculture #NutritionFarming #MobGrazing #SoilHealth #GraemeSait
-Jake shares the practical steps that allowed him to double his carrying capacity, drastically reduce chemical reliance, and welcome back the ultimate biological indicators: the dung beetles. This is a powerful testament to the fact that when we work with nature, rebuilding the microbial bridge, the farm becomes more profitable, more resilient, and ultimately, produces healthier food for our communities, honouring the soil to soul connection.
-*What you'll learn:*
-🌱 How adaptive mob grazing can naturally suppress weeds like Giant Rat's Tail grass.
-🐄 The simple, low-cost temporary fencing strategies to get started with cell grazing today.
-🪲 Natural alternatives for Buffalo fly control that protect and restore your dung beetle populations.
-🧬 The undeniable link between intense animal impact, soil restoration, and building humus.
-👇 *Chapters:*
-00:00 - Introduction
-01:27 - Title Sequence
-01:57 - Jake Introduction
-03:05 - Holistic Grazing Benefits
-04:28 - Changes in Pasture Species - Blady &amp; Paramatta Grass
-06:02 - Increased Biodiversity &amp; Beneficial Insects
-06:27 - Livestock Health
-07:06 - Nutrition Farming
-07:52 - Dung Beetles &amp; Buffalo Flies
-11:04 - USA Tour &amp; Industry Leaders
-13:37 - Top Recommended Regen Practices
-16:58 - Profitability &amp; Stocking Rates
-17:52 - Wrap Up
-18:03 - End Credits
-Want to learn more about Nutrition Farming? Check out Graeme's two-part article *”Nutrition Farming® – Where Do I Start?* …
-https://blog.nutri-tech.com.au/nutrition-farming-where-do-i-start-part-1/
-*Key Products Mentioned:*
-_Diatomaceous Earth_
-_Boss Bags_
-_Boss Lick (Garlic and Sulphur)_
-These can be sourced from the Kandanga Farm Store in SE QLD.
-https://www.kandangafarmstore.com.au/
-*Nutri-Life BAM™*
-https://nutri-tech.com.au/products/nutri-life-bam
-*Nutri-Gyp™ Natural Gypsum*
-https://nutri-tech.com.au/products/nutri-gyp
-*Sili-Cal (B)™*
-https://nutri-tech.com.au/products/sili-cal-b
-…or try our new NTS FulvX™ Powder for chelation
-https://nutri-tech.com.au/products/nts-fulvx-powder
-*Interested in attending a Certificate in Nutrition Farming course?*
-https://nutri-tech.com.au/pages/courses
-Need assistance? Try out our Soil &amp; Plant Therapy Services
-https://nutri-tech.com.au/pages/soil-plant-therapy
-How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait
-Head to our website to find out more
-https://nutri-tech.com.au/
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-*Follow us on Social Media*
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-Twitter: https://x.com/ntsaustralia</t>
+          <t>🏌️♂️ Stop Pulling FIRST in TRANSITION and Start Rotating Through Impact with Shaft Lean and Compression 🧨
+⛳️ If your impact looks stuck, cramped, or stalled, this is one of my favorite fixes. I put an alignment stick under the trail armpit to teach the body what real delivery feels like. The goal is not to yank the handle down. The goal is to get to the lead side, push the pelvis back, and keep the trail arm connected long enough for the body to rotate through. This is how you start to become a ball striking machine nailing your low points.
+Try it slowly first, then tell me what changed in your strike.
+Coach Erik Schjolberg
+Scottsdale Golf Lessons
+Online Golf Lessons
+#golf #golfswing #golfdrill #impact #ballstriking #rotation #alignmentstick #golfcoach #ejsgolf #thescienceofbettergolf #golfinstruction #compressitgolfball #lowpointcontrol #scottsdalegolflessons #golftips</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-20T07:09:24Z</t>
+          <t>2026-03-09T18:04:37Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1343</t>
+          <t>1213</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.028295</v>
+        <v>0.012366</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -884,117 +769,58 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Welcome everyone. We're here at Bolivia, a little country hall in the middle of nowhere. Um, and we're having a a field day sponsored, wonderfully, generously sponsored by Landare, where we've got a crowd of perhaps 70 people here, uh, learning about all things regenerative. And one of the attendees is a a gentleman who attended my course, how long ago would it be? &gt;&gt; I think it was August last year. It was winter last year anyway. &gt;&gt; Okay. So, his name's Jake Smith. And you know, we talk about young blood and their importance to develop some passion amongst young blood with this whole regenerative approach. And we've got a man who very much has that passion and we thought it'd be a great opportunity to have a bit of a chat with him and let him share his journey, his regenerative journey and what he's found and what he's achieved and some of the strategies that have worked for him. So, thank you for agreeing to talk. &gt;&gt; Thank you, Graeme. Thank you for everything. And thanks to Landare obviously for putting on this event like it's a wonderful wonderful couple of days we've had. &gt;&gt; Yeah, really generous. I mean, I've done land events before, but there's always some kind of charge. This is completely free and all the food's provided and so forth. So, yeah, really good thing. &gt;&gt; So, tell me about yourself. So, Jake Smith, I mean, how much land are we talking? What you farming? &gt;&gt; Um, so we're we operate across um about 4 and a half thousand owned acres of family farm and we probably lease another 4,000 somewhere in that vicinity. &gt;&gt; Thousand. We are a beef operation. Um, solely beef, but I'd actually like to bring in some um some chickens if I could find the right person to run it. Um, just for the clean up behind the the cattle. [music] and we operate all around Tennerfield. So we got country um east, northeast, south, west um all around Tennfield. all different um sorts of soil types and uh they all have their own challenges. But &gt;&gt; so when where when did you begin this regenerative journey? &gt;&gt; Uh well I'm actually a livestock agent by trade auctioneer and um &gt;&gt; I thought you spoke well. &gt;&gt; I actually um I had a client um and he came down from Northern Queensland. His name is Brett Craft and he's um he was a client of mine in Tennerfield and he sort of twigged this little idea in my head. Um before that we were fairly kind of industrial and um &gt;&gt; and I've been very lucky obviously like my old man's in construction so he's given me free reign of the farm. I can do whatever I want to do. Uh and if I fail he doesn't see it cuz he doesn't go down there much. So um that's so I Brett Craft introduced me to this concept of um rotational grazing to start off with and then I got in uh involved with um my grazing uh and then started going to field days and um got involved with RCS and it just really it compounded from there. So, &gt;&gt; and so just describe the changes you've had with this concept of cell grazing of intensive grazing. &gt;&gt; So, we um obviously we used to set stock like everyone does still does in the New England. It's fairly um prevalent. Um the first step that I took was um I mobbed all the cows up. Um after I mean you can have a serious crash if you don't do a lot of research on it first and do the appropriate courses uh and learning material, but I mobbed all the cows up and just started moving them really loosely. Didn't &gt;&gt; how big of mobs? Uh well at the moment we're about 350,000 calves in a mob. Yeah. Um and then sort of three to 500 heers in a mob. Um and same thing 3 to 500 steers in a mob. Okay. &gt;&gt; Um because they're different properties. If if all the properties were together, they'd be much larger, but we're still sort of in still u a building phase. &gt;&gt; U because we've actually compounded our carrying capacity so much just through mobbing cuddle up. even when I didn't really understand what I was doing, I just knew that it was I could feel that it was right. &gt;&gt; Um so we've actually compounded our um carrying capacity probably double I would say. &gt;&gt; Good. &gt;&gt; Um and just just through moving and and I've been doing this for probably &gt;&gt; um loosely for the first two years and then probably pretty well for the last sort of 3 to 5 years, four years. &gt;&gt; Um &gt;&gt; and uh yes. So &gt;&gt; and what kind of changes have you seen? Um well the for starters uh the grass like &gt;&gt; when you mob cattle up when cattle are all um set stocked &gt;&gt; you you tend to get um a monoc culture of the things that you don't want because they as soon as something juicy that they really like pops up there there and they're smashing it straight down to the ground &gt;&gt; and then all of them I mean after a little while it just depletes the root system and then that plant just dies. So you do end up with a monoculture of undesired grasses, which in our case on the eastern full is bladyy grass. &gt;&gt; Um, since I've mobbed the cows up, uh, believe it or not, not only are the bladed grass patches getting smaller, um, but they're actually eating, uh, eating the bladed grass. I mean, some people say, "Oh, you got to have cattle really hungry before you eat the bladed grass." But I actually find that because they're getting so much good grass, they actually I think they eat the bladed grass for a bit of roughage. Yeah. &gt;&gt; So that's really it's an interesting observation. So the country um the country has really benefited. I mean the grass just looks revitalized. There's better species there. We had a massive when I was set stocked um we had an infestation of giant rats tail grass. Um and now uh with some seed application and uh rotational grazing uh there's actually um premier digit and roads plants actually growing and cockia plants growing straight up through the crown of these plants and and they're actually in the middle they're actually drying up and dying and sort of breaking away the rats tail plants um or they're actually dry parameter sorry &gt;&gt; um but yeah that's some of the changes we've seen but just really um fantastic insect populations but good insects I've I mean our neighbors get army worms, all sorts of bad things, but for some reason they mustn't like our fence or something or we must have a really good fence and they just don't come anywhere near us. So &gt;&gt; yeah, &gt;&gt; it's um you see all once you start uh integrating all these systems and cycles together, you start to see something really interesting which I don't fully understand, but obviously that's why I'm here trying to find out a little bit more about &gt;&gt; very special. The the response is is tremendous and you've seen a change in animal health and so forth so yeah. It's um I mean I I don't uh we do supplement our cattle um but I don't rarely rarely get a vet out to see a cow ever anymore. &gt;&gt; Obviously before there was a lot of anti-inflammatories, antibiotics, that sort of thing. I've cut all that out and I've also um cut out most chemicals definitely um Roundup. We don't use any Roundup anymore. I'm pretty sort of against that but um some chemicals we just cannot get away from. We are trying but &gt;&gt; um It's always the process of just pruning them out as you can. &gt;&gt; Yeah. &gt;&gt; Yeah. That's good. &gt;&gt; So the and I feel like so grazing is one half of it and I think um the other half is what you're doing is um this nutrition farming approach actually getting the plants uh healthier through the likes of soil applications but also folure spraying. So I have been following &gt;&gt; I have been on mainly our backgrounding block. I'm a believer in you get the get your best country the engine running and then it pays to do the rest of it. So I'm just trying to focus on our backgrounding block which is our better country. Um and I have been doing soil applications of microbes. Um brewing out different things. Um well this is all after your course that I the 5day course that I did last year. Um &gt;&gt; and uh obviously I mean you see a marked improvement every time you do a soil application for microbes or a folia spray for the plants which feed the microbes. It's uh it's a marked improvement. &gt;&gt; Good. That's good to hear. And you know, little indicators like dung beetles, have you got them back now that you've reduced the chemicals? &gt;&gt; Well, um, so I've spent, uh, I spent a my last probably 5 years of my life trying to kill them accidentally, not meaning to, but just our buffalo fly populations were through the roof. And this year, I just said, um, no more, no more. So, uh, I like a quote from, uh, from Will Harris. Um, well, he talks about, you know, when I was an industrial farmer, all I wanted to do was every time I walked out the door, I was looking for something to kill. But, uh, now he's looking for what he can keep alive. He wants to keep everything alive and let biodiversity and everything happen um, amongst it. So, our dung beetle population since I've stopped uh, we we've gone to a natural method of um, remedying the the the uh, buffalo. &gt;&gt; And what is that method? That' be an interesting thing to share. So we use a thing called dietimmacous earth in a in a product called boss bags um which is uh we actually get it from straight from Kadanga Farmto. They make them up at um Sunshine Coast. &gt;&gt; Fantastic product. Um and we also um use their boss lick which is a um garlic uh well a lys in the garlic and a um sulfur lick but and a base mineral lick also. &gt;&gt; Um good product &gt;&gt; and it's it's been a fantastic product. that I I I suspect next year, we still did have um a few buffalo fly, but I suspect next year when the dung beetle populations build up and breed up, that they'll be burying the dung quicker hopefully in theory than what the what the larae can bury uh can um growing the dung. So, I think next year will be even more of an improvement. So, but I mean they're back in the I hadn't seen it. I remember years ago before we used to treat intensively for um buffalo fly. You you used to be able to not sleep at night in the hut. Like they'd be hitting the hitting the walls of the hut and they'd be poked on the barb wire fences everywhere in the mornings when you went out. For the last 5 years since we've been intensively treating, I haven't seen a dung beetle down there. So something sparked in me and clicked in my mind and I just thought maybe this is what's happening. And um now I mean this year I've seen dung beetles back on that particular property for the first time as I said for four or five years. So which is actually really exciting. &gt;&gt; It's wonderful when you when they come back and forth. And with uh Claudia, my partner is a graze here out of Santo. Um she had exactly the same scenario. There was nothing and they were collecting dung for composting for this market organic market garden that they've got on the farm and there's just and it's exactly it's adapt adapt the approach and slowly they come back and now they're in there in such ridiculous force. Yeah. I mean there's a she let unfortunately the cows got into the house paddic and there's just manure everywhere and the next day the buzz she says you know forget about the crow the reed wobble or whatever that book masses book is let's call it the buzz of the of the of the of the cane beles because it was insane and there was nothing a day later everything has carried in it's just ridiculously intense and so good to see and it's just changing you can see this all changing is all of that tong in that concentrated form when you're sell grazing &gt;&gt; you know it's almost that model is almost like you can't really have too much. It's just how long you leave them there. The more cows the better really. Bigger mobs is is even more effective. &gt;&gt; Bigger mob the better. Yeah. And the smaller area you can concentrate them in and move them on. &gt;&gt; Um we just completed a trip to America um for 5 weeks um farm touring over there and we saw some really cool things. um the likes of we went to Will Harris, Joel Salatin, um Smoke River Ranch in northeast Oklahoma and another one in North Texas um Birdwell Clark Ranch and they're all doing this um sort of um a cross between ultra high density and u adaptive multipatic grazing and um &gt;&gt; so just describe adaptive multip. So adaptive multipatic grazing is um instead of cell cell grazing and having a very prescriptive um move at this time of day have this set paddic they are actually um they have big paddics and they build p they build temporary fences within those paddics. Um so the way that they describe it is that the energy flow of the cattle are moving different ways every time. So they might have the cattle running this way this time and then back across this way this time. So their different seasons and different things determine their paddic sizes um shapes. They always change their shapes. So there's never anything the same and they're never coming back to the same spot at the same time of year ever. Um &gt;&gt; Okay, that's good. I mean one particular example the Burbal Clark ranch they're they're across 14,000 acres in north uh northwest Texas at Henrietta and um they like they it's there is a figure it's like in the last 10 years um each square me or a certain square meter of that um block has been grazed a total of 24 hours in 10 years or so like the figures are there but it's a ridiculous amount so um or little time that is so they uh they do a fantastic job there. And you can see uh Emry Emmery describes um when he bought the ranch that there used to be big planes of nothing like you see in Western New South Wales big planes of just red clay pans, but now I mean they've got Indian grass and things like that. &gt;&gt; It's tremendous when you see it. I mean I saw it on a small scale. I was speaking at a conference in Townsville and for the reef safe group and they show me this little trial they're doing and this is small stuff. Okay, we got this gully that's just weed and crap and really nothing in it. And they just basically, this is the small scale people and people are buying cattle just for this purpose. There might be half a dozen cows and you just basically bring a bail of hay and you fence off just a small area and you got the cow, you got the mob effect in this tiny area and you just move that down the gully and then he show me a year later, two years, three years, four years because this has been an ongoing project and that restoration was just so impressive. I mean you just had this complete transformation of that valley done totally with the animals. &gt;&gt; Yeah. &gt;&gt; Yeah. Such a good concept. &gt;&gt; Animal impact is I believe is the single best thing for landscape recovery. Um &gt;&gt; yeah mixed with a few other things but yeah. &gt;&gt; So what of all the things because we've got a room full of people waiting for us to come back and start the presentation. But what would you consider to be the most effective of the of the regenerative strategies that you've put in place? the most effect I don't know whether there is any most any one thing but probably definitely um is you need to get yourself educated that's one thing courses like yours are obviously paramount um uh but probably the biggest thing for me was um just mobbing the cattle up you don't you can just start moving the cattle and and just watch what happens you will see a marked improvement it's actually ridiculous how much better it is than just set stocking and you will boost your carrying capacity there's no two ways about it. &gt;&gt; And how have you found it from obviously I watch Claudia's situation twice a day she's moving them super labor intensive. How do you manage that? &gt;&gt; We I can't personally do that. We don't really have anyone that works for us. Um and we have farms different places. So I try and move them every sort of 3 days. Okay. &gt;&gt; Um but that will intensify uh especially on a main breeding block. Um &gt;&gt; but it's you'll actually find um you have a lot of fun doing it. &gt;&gt; Yeah, you will. and it's you think it's going to be all a big job, but I mean you can run a a Kiwi Tech fence system or just a Poliwire fence system across a paddic in 10 minutes and that'll be enough area for um you know a couple of hundred cows. So you think it's going to be a lot of hard work, but it's not really. It's actually a lot of fun and just but and I mean then you get to actually &gt;&gt; and they they they get to know that they want to move to the new spot, so it's not that hard to move them around. &gt;&gt; Correct. Yeah. Yeah. &gt;&gt; And you actually get to you can see the difference in the country around behind you like the the dung beetles um a lot of places in America the draw down of the dung is less than 24 hours and there's nothing on the paddic. &gt;&gt; That's like what her place is. It's wonderful. I remember this a couple who grazing a couple thousand acres um in out from Rockampton. Um, and she decided she'd been one to one of the courses and listened to a few things. And so she had this bet with her husband that she could take 200 acres and make as much money as he was making from the other 1,800. He said, "Bring it on, girl." You know, they actually had I think it was a few thousand bet. So she split that 200 into 20 10 acre paddics and she brings 600 head into each paddic for a day. Uh, she planted lina hedges down the in each of those blocks. So those were really good protein source and they eat that tree loosen. But I did the soil test, you know, three years later come back and repeated the soil test and it was this absolute transformation. I mean, it was two and a half times the organic matter and every mineral had changed. It was just like and I said, you know, you cheated. You won your B money, but you cheated. You put some lime on here. Uh you put, you know, these trace minerals or whatever. It even looks like there's some compost. And she said, I I did nothing. I used my animals as my primary fertility tool. And it was such a graphic example of what's possible. &gt;&gt; Yeah. And you don't even realize what's possible until you start doing it. Like &gt;&gt; it's uh we don't even really know what's possible yet. So &gt;&gt; yeah, it might be a good suggestion that people just, you know, get some movable electric and just try it for themselves. It seems believing. &gt;&gt; You can get a you can get a fencing set up, a movable temporary fencing setup for less than a couple of thousand bucks. Like what can you buy for less than a couple of thousand bucks that can create a return on investment like that? &gt;&gt; Yeah. &gt;&gt; I mean it's um &gt;&gt; So your profitability has improved. &gt;&gt; Yeah, definitely. Yeah. I mean, like a lot of farmers, we probably never really we all had off farm jobs. Um, no one had ever really made money off the farm uh for probably 60 years. Um, but now &gt;&gt; something [laughter] thousands of acres of money from the farm. &gt;&gt; But then um since we've purchased another property and um taken on more debt to do that obviously uh but still a lot more profitable. So I mean once your stocking rates um &gt;&gt; improve profitability your profitability improves and I I think through um better grazing management um after doing it for years you don't want to jump straight into a really intensive system but I do believe uh with a really intensive system uh with some tweaks &gt;&gt; uh we we no doubt can triple our stocking rate um compared to in comparison to our set stock system. So &gt;&gt; that's great. Thank you so much for for sharing. At some point, we'll actually have a chat for the podcast as well. There's lots of valuable stuff you can share. But thanks for giving us the time today. &gt;&gt; No worries. Thank you. &gt;&gt; Thank you. [music] [music]</t>
+          <t>Are you tired of having to look like this at impact? Okay, maybe not even hips rotate like that. You're more like this. I see it every day in lessons. Okay, I'm going to show you one of the great fixes I have for it. So, you take a lining stick. We're going to put it under our trail armpit. Okay? And then you're just going to take every like normal. Now, when you look from this end, you should see kind of that these these are nearly the same. It doesn't have to be exact, but kind of the same angle as the uh the um club. So, what we're going to do is we're going to swing up to here like left arm parallel. You see how it gets on my arm here. Okay. So, I want to make sure though when I start down, I'm on my left side here. This is still on my arm. Now, what I want to do first is get since I'm on my left side, the lower body goes out of the way. And I see how I'm keeping this on me. As I'm rotating, rotating, it's still on me. Still on me. And it's barely off. But look where I'm at. So, yes. Is this an extreme version of it? Yes. Right there. But yeah. So, left side, push back. Keep it on. Keep it on. Keep it on. So, look at that. Okay. Incredible. So, it's just a little aim strike drill under your pit. Do that a bunch of times in slow mo to get the feel and try to pick up what are you doing different. And you're going to notice it's some body movements, not this big pull down. Okay. Thanks for watching. Eric Silver, EJS Golf and the science of bettergolf.com. Leave a comment down below after you've tried this and let me know how it went. Thank you.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>On a hobby farm can chicken tractors be as effective for soil regeneration? || Definitely @christopherburman3340! Chicken Tractors can be a powerful tool for building soil fertility at any scale. || Good on you mate….hopefully more farmers will follow you and make the land better.and the creeks and rivers 👌🏻</t>
+          <t>This performance is really helpful I did not expect it to be this good.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>UHEU6zJBtrE</t>
+          <t>-zXcHbCKESA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>The Liver Love Smoothie That Extends Your Life - Liver Health Strategies Part 2 - How to S4E13</t>
+          <t>⛳️  Most Golfers Hit Behind It. This T Drill Fixes That. 🎯 #shorts</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>In Part 2 of our Liver Health series, Graeme Sait takes us into the kitchen to whip up the ultimate *Liver Love Smoothie* — a powerhouse of glutathione-boosting ingredients. But we don't stop at the liver! We dive deep into the "Second Brain," exploring how *butyrate* , *resistant starch* , and the hidden world of *lectins* dictate your longevity and vitality.
-#LiverHealth #GutHealth #GraemeSait #NutritionFarming #SmoothieRecipe #LeakyGut #ResistantStarch
-*What you’ll learn in this episode:*
-🥬 *The Liver Love Recipe:* How to combine Parsley, Beetroot, Avocado, and Whey Protein for maximum detoxification.
-🧬 *The Power of Butyrate:* Why this short-chain fatty acid is your colon's best friend and a shield against inflammation.
-🍚 *The "Cook &amp; Cool" Secret:* How to turn simple potatoes and rice into life-extending *Resistant Starch* .
-🍅 *The Lectin Lowdown:* Why the Mediterranean diet removes tomato skins and seeds, and how it could solve your joint pain.
-👉 *Don’t forget to like, share, and subscribe* for more Nutrition Farming® insights with Graeme Sait.
-👇 *Chapters:*
-00:00 - Introduction
-00:12 - Title Sequence
-00:42 - Graeme Liver Love Smoothie Recipe
-00:57 - Parsley
-01:13 - Beetroot
-01:52 - Kale
-02:25 - Avocado
-02:59 - Whey Protein Concentrate
-03:18 - Garlic
-04:11 - Curcumin - Curcu-Life
-04:29 - Milk Thistle &amp; Capsicum
-04:44 - Broccoli Sprouts
-04:57 - Water
-05:09 - High Power Blenders
-05:53 - Smoothie Wrap Up
-06:47 - Butarate
-10:45 - Resistant Starch
-13:39 - Leaky Gut
-15:30 - Lectins
-16:05 - The Mediterranean Diet
-17:17 - Pressure Cookers
-17:31 - Wrap Up
-18:15 - End Credits
-Want to learn more about natural health tips?  Check out: Prebiotics, Probiotics &amp; Alcohol: Gut Health Tips You Need to Know - How to S4E2
-https://blog.nutri-tech.com.au/prebiotics-probiotics-alcohol-gut-health-tips-you-need-to-know-how-to-s4e2/
-*Relevant NTS Products Featured in This Episode:*  
-_BioSpark_
-https://www.ntshealth.com.au/products/biospark
-_Curcu-Life_
-https://www.ntshealth.com.au/products/curcu-life
-_Green Defence_
-https://www.ntshealth.com.au/products/green-defence
-_BioBubble™ Probiotic_
-https://www.ntshealth.com.au/products/bio-bubble
-_Nutri-Salt_
-https://www.ntshealth.com.au/products/nutri-salt
-_SweetSure_
-https://www.ntshealth.com.au/products/sweetsure
-*Interested in studying Nutrition Farming?*  
-Certificate in Nutrition Farming courses:  
-https://nutri-tech.com.au/pages/courses  
-Need personalised support?  
-Soil &amp; Plant Therapy Services:  
-https://nutri-tech.com.au/pages/soil-plant-therapy  
-Book a one-hour online consultation with Graeme Sait:  
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
-*Explore more at our website:*  
-https://nutri-tech.com.au/
-Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
-https://nutri-tech.com.au/pages/newsletter  
-*Follow us on Social Media:*  
-Facebook: https://www.facebook.com/NutriTechSolutions/  
-Instagram: https://instagram.com/nutritechsolutionsyandina  
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>⛳️  Most Golfers Hit Behind It. This T Drill Fixes That. 🎯
+If your contact is inconsistent, stop chasing random swing thoughts and start training low point.
+This T drill is one of the fastest ways and simplest ways to teach golfers how to move the strike forward, compress the ball, and finally get ball first then turf. I set the tee about 4 inches in front of the ball and the goal is simple: take it out with a short swing.  Be super aggressive towards the tee.  Crush it if you must! 💪
+That is how you start to build a ball-striking machine. 💥. Let's do it!
+playbettergolf #scottsdalegolflessons #ejsgolf #simturf #onform</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-06T04:30:31Z</t>
+          <t>2026-03-08T18:03:31Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>769</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1003,7 +829,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.019635</v>
+        <v>0.007802</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1012,7 +838,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>So, let's look at our little uh recipe. And we're going to what we're going to do is make we're going to blend it and we're going to drink it hopefully. Uh and we're going to make oursel it's called Graham's Liver Love Smoothie. So, we're going to begin with two large sprigs of parsley. Now, of course, you've heard me talk about parsley previously. I'm going to put more than two. I'm going to put this much in there. Slightly more than two. So we've put that into our into our blender. Uh parsley the story of course uh one of the most powerful kidney supporting herbs um but also a source of glutathione and hence we're using it in this blend but at the same time we're going to be supporting uh kidney health. One of the most powerful tools to boost kidney health. Uh a mediumsized beetroot which we'll cut up now. There it is. Okay. So, I'll just take the bit of the rough stuff off and throw it over the edge. And we'll cut up our beetroot and put the beetroot into the mix. Wonderful food. Of course, this is antyanins, this wonderful purple pigment. And we're even going to go one step further with this model. We're going to put in as our beetroot. We're going to put in some beetroot leaves. And who would have thought that the beetroot leaves have almost as much nutrition as the beetroot? Apart from folic acid, they actually have as just as much. You can see that purple color. And we're going to put some of that in there. Then we're going to put out three kale leaves. This is the kale that was produced during my little garden segment. If you recall, we showed you how with kale on his broad fork. Uh how quickly you can put a garden in. And this is the wonderful kale that that came from that. I'll cut that up a little bit. We got quite a lot into this. This is quite a big I might have overdone it, but we'll see. Um, so we've got our beetroot, our kale, we've got our avocado coming up. Thank you. We'll scoop out the avocado goodies. of course this wonderful range of fats in avocado that was kind of unparalleled but a very good source of glutathione and of course it was demonized the fat and in and avocado at one point and then we realized oh my goodness it's one of the best fats you can possibly eat and it's something you never get sick of I mean I eat avocado every day and I've never yet got sick of it now whey protein concentrate we're talking about so we'll just undo this and we'll put a tablespoon of that is how much we've got for this a heap tablespoon of whey protein. We'll put that into the mix. Quite a quite a heap tablespoon. We're going to put our bruised garlic. So, let's open our garlic, our Australian garlic, our wonderful Australian garlic. And let's get ourselves a couple of cloves. And of course, we got to quickly peel them and bruise them. And how am I going to bruise them? I'm going to bang them with this honey jar. That's done the job. That's one bruised clove. I'll just get a second one. Big cloves. These lovely Australian garlic. I'm hoping I produce something similar this year myself. Bun crop to grow. I love it. Give it a bruise. That's good. Bruise garlet. Leave it sitting there for a few seconds. Get all It's going to get well and surely oxidized in a moment. Um, now where are we at? We're talking about whey protein, a calcul of course. How much curcul is it? A heaped teaspoon. So here's our calcul. It's combination of turmeric and pepper. And we're going to put a decent heap teaspoon in there. Then we've got milk thistle, which we don't have, but we do have our little bit of capsicum for the capsicum. this jalapeno and we'll hope that it's not going to be too hot but I won't put too much in there in case it it really burns us up. That might do us. This is a touch of capsic as we mentioned the substance that activates glutathione. The broccoli sprouts we don't have but and we don't have the milk thistle tablets or milk thistle powder. Um, so you can imagine that you put those in there. And then we're going to add our bit of water, a glass of water. Hopefully that's enough. It might not be. And we'll get this show on the road. And we'll just make ourselves a smoothie. Now, let's see if we can get this going. What we'll do is we'll just add ourselves a little more water. Thank you. Add a little more water cuz she's a bit too thick. That's better. Now, of course, the idea of making a green smoothie is you need to have one of these high power. This one's many years old. I've made many smoothies in it life. Um, this is Vitamix from the US. This blend from Germany. Now, you need these two horsepower blenders to do it as quickly as you can because you don't want it to go on forever and you want it to be genuinely micronized. So, let's just finish it off. &gt;&gt; Okay. Okay. So, let's have ourselves a really thick. We could have made it a little thinner than this, but let's see what it tastes like. You'd make it a little more runny. We put another half glass of water in there. But let's taste. Yeah, I reckon we should have put a bit of It's actually pretty nice. Um, yeah, I have a taste. &gt;&gt; Yeah, &gt;&gt; you could have put a bit of fruit in there if we wanted to sweeten it up a little more, but that's that's pretty palatable. You can almost taste it, feel it going to work on the liver. Thank you. So, that's how you make a liver love smoothie. and we'll move on and talk about a few other things relative to how you can live a longer just clean my mouth off longer happier healthy life. We're going to talk about a gut health understand how important your gut health is. We've talked about the need for probiotics but we're going to talk about something called buteryrate at this point and why is it important? It's really important because bowel cancer is the fourth major cause of premature death and fiber is hugely important as you as you all know. Now let's talk about the dynamics of how this thing works. So we have this thin layer of epithelial cells that are interconnected. These cells are connected by structures that are called kite junctures and that keeps the gut contents whatever you've eaten from entering entering uh moving through into your blood system. holds everything in there basically. So these epithelial cells exude this mucous material. It's called the mucous layer and that's really protective. It protects against microbial pathogens against enzymes, acids and food associated toxins. Now when we move down to the colon which is part of what we're going to talk about here um in the they're called colonosytes these same epithelial cells and they have to be energized because they got this really important protective function and what they use to derive their energies. In the top half of your gut it's glucose that gives the cells the energies the epithelial cells their energy to do this really important protective role. But in the bottom half, there's these things called shortchain fatty acids. And they come from certain types of fiber in the colon. And that's really important because the colon's replacing its every four days, the cells are. And the most important by far of those short- chain fatty acids is called butyric acid or butyrate. Now, let's look at the roles of butyric acid or butyrate. Butyrate is anti-inflammatory. Um, so this is huge for people with bowel issues, things like irritable bowel or that very painful condition called colitis. Um, massively important IBS and colitis. Um, that you're producing good amounts of this anti-inflammatory called butyric acid. It increases mucosal secretion when that reduces the pathogenic bacteria that can grow uh and and it also produces some antimicrobial peptides. So, it's got quite protective in that context. Um, it's an immune enhancer, butyric acid. It activates anti-inflammatory immune cells in the colons. Again, really important for things like irritable bowel syndrome. It sponsors glutathione production. We've just talked about how important that was. High levels of butyrate produce high levels of glutathione, which gives you even more protection from some of those inflammatory bowel diseases and bowel cancer. It combats type 2 diabetes. Several people papers have demonstrated that butyrate or butyric acid increases the production of hormones that improve blood sugar balance. So you know one in three of us have got poor blood sugar balance which makes us pre-diabetic and the experts are telling us that diabetes is becoming plague. So that sounds like a good thing to look at. But what's fascinating is its role in terms of cancer. that can specifically target can cancerous cells in the colon and reduce their energy and eventually initiate what's called apoptosis which is cell death. So there's a very famous p paper by Anna Han and some of her colleagues in the cancer journal called enco target and she demonstrated that butyrate this is quite unique because it's not a common thing in nature but butyrate can seek out the cancer cells and then it shuts down their capacity to utilize butyrate as an energy source. So it shuts down the capacity of this thing to to take itself in which is kind of like not a very common thing and uh that then reduces their energy and and eventually leads to their demise. So it's unique where a substance actually shuts down the capacity for its own utilization. That makes it quite a special substance. So how can we spike the production of butyric acid this very very protective thing in our bowel? One of the most powerful uh is to bring some resistant starch into our diets. Uh basically resistant starch also has a major impact on insulin sensitivity and a study published in the journal of nutrition by Kevin K. Mackey uh showed a 33 to 50% improvement in insulin sensitivity in just four weeks by eating 15 to 30 grams of resistant starch a day. And I'll explain what that is shortly and you'll understand that it's not a hard thing to do. It's actually thought to be resistant starch, a major tool to avoid chronic disease and improve life quality. So, what's ideal? 25 to 30 grams a day. What do Australians eat? Six grams a day. What do Americans and Europeans eat? 5 grams a day of resistant starch. What do the Chinese have? 15 grams. Still not where you need to be, the 25, but 15 grams. And they've got much less obesity. You've all seen it. And they have far fewer digestive issues. So fairly good argument for bringing in some resistant starch. So how do you do it? It's called the cook and cool concept. If you cook potatoes and then you store them in the fridge for a minimum of 12 hours, that high starch since potatoes aren't actually particularly good because they spike sugar more than table sugar. You know, the GI of potatoes is 95. Pure white table sugar is 70. So potatoes are not good from that perspective. Sweet potatoes, no problem. They've got the fiber component. They break down much more slowly and they've got a GI of just of 35. So sweet potatoes, you can eat what you like, but potatoes do spike blood sugar, spike insulin production, speed cell division, and shorten your life, basically. So, is there a better way to eat them? Yeah, there is. Uh, you have potato salads. Now, you say, "Oh, you I can cool it down, then I can slice it up and have it for chips." No. uh as soon as you've warmed it up again, you've changed the resistant starch back to that super blood sugar spiking form of uh refined carbohydrates or or carbohydrates that spike blood sugar very quickly. So, potato salad, you leave it cold. Um preferably don't fill it with mayonnaise, a good dressing, pumpkin seed oil if you've ever had it. It is incredible. And of course, it's jam-packed with zinc, balsamic vinegar, and a lot of black pepper, you know, and put that on your potato salad. It's beautiful. Now, that cook and cool concept can extend to things like rice and pasta. This rice salads, part of the Mediterranean diet, which is noted for its longevity. And of course, the Japanese got it right with the wonderful thing called sushi because not only is it based upon white rice, um, but it's wrapped in that beautiful all 74 minerals, including very high levels of iodine, that kelp uh jacket that's wrapped around the sushi. And then they put things like wonderful things like avocado and high omega-3 salmon. And really it becomes a very very healthy diet that could be part of your 25 grams uh of resistant starch on a daily basis. So let's just talk back on that uh on that layer u because the epithelial layer because when we talked about those strong junctures which are the barriers between the epithelial cells and without butyrate without butyric acid they can become weakened but there are some other players that perhaps we should think about and try and avoid. Uh antibiotics kill the organisms that produce butyrate. So that can be really counterproductive for gut health and and and le make you more likely to suffer from this leaky gut where things from your gut go into your blood system and there are a whole bunch of side effects that come with that. Uh non-steroidal anti-inflammatory drugs like a ibuprofen are major place because they shut down the protein messages that govern the interchange of gut cells because every four days you're supposed to have new ones and there's a message that's shut down by ibuprofen so you don't replace them and so they get tired and weak. The old cells become weak and that weakens the junctures to create intestinal permeability which is also called leaky gut. So what are the symptoms of leaky gut? Tick the boxes. Tiredness after eating. This is why people hate the afterdinner presentation uh when you're giving seminars because that's the point where people because there's a lot of energy anyway involved in digestion but if you've got leaky gut you get really tired and you see the people uh droop off. I try and keep things entertaining enough so that doesn't happen and thankfully it's quite rare but it does happen occasionally. You're going to have things like sore joy. You're going to have things like eczema skin conditions. You're going to have poor immunity, headaches, brain fog, memory loss, anxiety and depression, ADHD, multiple autoimmune diseases. All can be linked to this condition called leaky gut. So that's just a little thing and we want to we want to keep our butyric acid up. So the resistant starch is really important in that context. And finally, we're going to talk about something called lectins. Now, you may have heard of them. There's a guy called Dr. Steven Gundry who's everywhere at the moment, who's sort of an expert talking about how lectins can be linked to leaky gut, to heart disease, to autoimmune diseases, and the very important neurodeeneration. He's seen a 90% of his autoimmune patients improve just by removing these things called lectins from their diet. So, what what contains high lectins? Well, the nightshade family. So that's potatoes, capsicums, eggplants, and of course the big one which is tomatoes, uh beans, pulses, whole grains, and so forth are all part of the lectin story. So just continuing the lectin story. So you might have all heard about the Mediterranean diet and it's linked to enhanced longevity, but you might have wondered perhaps why do they go to such great lengths to remove the tomato skins, uh to remove the seeds when they make the tomato sauces and so forth. And that's where the lectins are. The lectins are in the skin. They're in the seeds at high quite rate. So, so what the Italian dishes do is that they utilize tomatoes as lycopine and some other wonderful benefits including high vitamin C, but they remove the negatives, the seeds and the skin. So basically in beans, they soak them for 24 hours on the Mediterranean diet uh to remove the lectins and they change the water every four hours when you're soaking them. So it's a few changes over 24 hours, six or seven changes cuz you can't do it when you're sleeping. Now part of the sourdough story is that the so process removes the lectins. Um so basically when we're talking chili peppers, capsicums, eggplants, at least remove their seeds and ideally remove their skin. And one other really cool tool um to reduce lectin content of any food is to use a pressure cooker. It's become, you know, a real tool in trade and it's fairly popular amongst amongst the Steven Gundry and his strategies to reduce your lectin content and reduce your inflammation. And I think it's worth many people visiting that idea. I was in Rockampton uh with a couple on a farm where they grow loose and a few other things. And the the the farmer himself was telling me that he was so crippled that he couldn't even pull things out of the fridge without dropping things um with just this arthritic kind of condition. And someone suggested why don't you just try cutting out the night change, cut out the tomatoes. He's a very big tomato eater and it took about five to six weeks and his pain disappeared. So, it's probably something worth trying if you've got inflammatory conditions because tomatoes that night family can on some people have quite a strong appeal and it may well be linked and probably is linked to that lectin component. So, I hope there's something of value for you there. Thanks for watching. [music]</t>
+          <t>This is the T drill to work on low point. Okay, so got a T here. We're going to lie it down on its side. Now, just so you see it here, it's going to be about four inches in front of the ball like right here. We're going to do it two different ways. We're going to start off heels together, toes apart. You can do toes apart or together if you want. We're going to do both here. So, I'm going heels together, toes kind of apart. And I just want to feel how do I take that tee out with a real short swing here. Okay, that's the main goal. How do I do this? Okay, so wasn't perfect connection on that. That's okay, though. Accomplished what I wanted. I got to the tea. Got my low point well forward. Now we're going to just do it with feet apart. Try the same thing. Okay, real short swing again. And our goal here is to take this PE out, which obviously I did. And how how do I know? Another way to check is my low point was 5.4A inches in front was my lowest point. Okay, so I really got forward. Most golfers have behind. Unfortunately, they're behind with their low point. We need to make sure we get in front so we're compressing this ball, getting the right spin, right distance. All right, thanks for watching.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1020,325 +846,172 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HrRSKP7YE5Y</t>
+          <t>fPv9OkVg_Xg</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Liver Strategies - Turmeric, Garlic &amp; Broccoli Sprouts Heal Liver Damage - How to S4E12</t>
+          <t>⛳️. Swing Plane Perfector: Fix Low Point AND Swing Path at the Same Time 🧨 #shorts</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Welcome back to another episode of the *How To Do It* series 🌿🧠
-Where Graeme explores one of the most essential — yet often overlooked — organs in the human body: the *liver* .
-*#LiverHealth #Detox #Nutrition #HowToDoIt #Glutathione #HealthTips #Wellness*
-While heart disease dominates many health conversations, this episode explains why the liver may be the primary organ of survival, responsible for detoxification, antioxidant production, metabolic balance, and long-term vitality. Research suggests that *one in fourteen people* may already be living with undiagnosed liver fibrosis — a condition that often progresses silently until serious damage has occurred.
-*So, how do we protect the liver before it reaches that point?*
-Graeme introduces the idea of *“learning to love your liver”* through practical, evidence-based nutritional strategies that support the body’s natural detoxification and repair systems. A key focus is placed on *glutathione* , the body’s master detox molecule, and the nutrients that support its production.
-*In this episode, you’ll learn:*
-🍊 Why *vitamin C* supports *glutathione* and antioxidant defences
-🧪 The role of *selenium* in liver protection
-💊 The benefits of *turmeric* , *milk thistle* , and *alpha-lipoic acid*
-🥦 How *broccoli sprouts* supply sulforaphane
-🧄 Why *garlic-derived allicin* stands out medicinally
-Graeme also outlines a simple liver-supporting *green smoothie recipe* designed to reduce oxidative stress and support detoxification.
-Your liver works tirelessly every day. This episode shows you how to work with it 💚
-👉 *Don’t forget to like, share, and subscribe* for more Nutrition Farming® insights with Graeme Sait.
-👇 *Chapters:*
-00:00 - Introduction
-01:28 - Title Sequence
-01:58 - Liver Fibrosis
-02:53 - Sulphur Compounds: Glutathione - Glutamine, Cystein &amp; Glycine
-04:14 - Vitamin C
-06:05 - Whey Protein Concentrate
-07:05 - Turmeric - Curcumin &amp; Pepperine
-07:51 - Milk Thistle Extract
-08:27 - Selenium
-09:26 - Alpha Lipoic Acid
-10:49 - Sulphurafane
-12:34 - Garlic - Alicin
-16:17 - Smoothie Wrap Up
-16:30 - End Credits
-Want to learn more about natural health tips?  Check out: Prebiotics, Probiotics &amp; Alcohol: Gut Health Tips You Need to Know - How to S4E2
-https://blog.nutri-tech.com.au/prebiotics-probiotics-alcohol-gut-health-tips-you-need-to-know-how-to-s4e2/
-*Relevant NTS Products Featured in This Episode:*  
-_BioSpark_
-https://www.ntshealth.com.au/products/biospark
-_Curcu-Life_
-https://www.ntshealth.com.au/products/curcu-life
-_Green Defence_
-https://www.ntshealth.com.au/products/green-defence
-_BioBubble™ Probiotic_
-https://www.ntshealth.com.au/products/bio-bubble
-_MagSorb™ Magnesium Spray_
-https://www.ntshealth.com.au/products/magsorb
-_Nutri-Salt_
-https://www.ntshealth.com.au/products/nutri-salt
-_SweetSure_
-https://www.ntshealth.com.au/products/sweetsure
-*Interested in studying Nutrition Farming?*  
-Certificate in Nutrition Farming courses:  
-https://nutri-tech.com.au/pages/courses  
-Need personalised support?  
-Soil &amp; Plant Therapy Services:  
-https://nutri-tech.com.au/pages/soil-plant-therapy  
-Book a one-hour online consultation with Graeme Sait:  
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
-*Explore more at our website:*  
-https://nutri-tech.com.au/
-Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
-https://nutri-tech.com.au/pages/newsletter  
-*Follow us on Social Media:*  
-Facebook: https://www.facebook.com/NutriTechSolutions/  
-Instagram: https://instagram.com/nutritechsolutionsyandina  
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>⛳️. Swing Plane Perfector: Fix Low Point AND Swing Path at the Same Time 🧨
+🏌️ Most golfers I see have one major problem — their low point is behind the golf ball. That means no compression, no forward shaft lean, and no consistency. In this video, I show you a different way to use the Swing Plane Perfector that I haven't seen anyone else teach — fixing your low point AND your swing path at the same time. Kill two birds with one stone.
+This is how I train golfers at EJS Golf in Scottsdale, Arizona — using real cause-and-effect coaching, not band-aids.
+🔗 Get a Swing Plane Perfector with a discount code: EJSGolf.com/gear
+🔗 Grab my free drills guide: EJSGolf.com/my-drills
+🔗 Learn more about The Science of Better Golf: EJSGolf.com
+🔗 Read the blog: EJSGolf.com/blog
+📍 In-person lessons: McCormick Ranch Golf Club, Scottsdale, AZ
+🌐 Online coaching available worldwide
+#golf #golfswing #golftips #golflesson #ballstriking #swingplaneperfector #lowpoint #ejsgolf</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-01-23T04:30:09Z</t>
+          <t>2026-03-02T19:03:59Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>868</t>
+          <t>949</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.028802</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Oh poo - video finished before Graeme could make the smoothie! || It was a too long for one episode, so you will have to come back for Part 2! || OK.... Where is part 2?</t>
-        </is>
-      </c>
+        <v>0.001054</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>XVTBG1xVe4Q</t>
+          <t>69zdsNCQG30</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cancer Strategies: How to Build a Body That Protects Itself - How to S4E11</t>
+          <t>🔥 Stop Flipping the Club! This Simple Drill Forces Body Rotation Through Impact ⛳ #shorts</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>In this *How To Do It* episode, Graeme Sait explores *#CancerStrategies*, *#ImmuneHealth* and *#MetabolicHealth* — sharing calm, biology-first insights into nutrition, minerals and lifestyle choices that help the body build real resilience 🌱🧬
-Filmed high on the ridge at Nutrition Farms as the sun sets 🌄, this is a thoughtful, grounded conversation about a subject most of us would rather avoid — and yet one that touches so many lives.
-Rather than fear, hype or miracle claims, Graeme gently reframes the discussion around *how the body is designed to protect, repair and restore itself* when given the right conditions. It’s about understanding biology — not fighting it.
-Throughout the episode, themes of *metabolism* , *inflammation* , *immune strength* and *detoxification* are woven together as parts of a beautifully connected system. Small, consistent choices around food quality, mineral sufficiency and gut health can profoundly influence how well that system performs.
-There’s a strong emphasis on working *with* the body 🤝 — reducing unnecessary stressors, supporting natural clean-up processes, and creating an internal environment where healing is more likely to occur.
-This episode isn’t about quick fixes. It’s about *informed choices*, *long-term thinking*, and reclaiming a sense of agency over your health.
-Whether your focus is prevention, recovery, or simply living with greater awareness, this is a calm, empowering conversation that brings health back to first principles — biology, balance, and common sense 🌿
-👨‍🌾 *Stay tuned* for more practical, science-driven insights in future episodes of the *How to Do It* series.
-👉 *Don’t forget to like, share, and subscribe* for more Nutrition Farming® insights with Graeme Sait.
-👇 *Chapters:*
-00:00 - Introduction
-01:09 - Title Sequence
-01:39 - Sugar &amp; Insulin
-03:01 - Sulforaphane
-03:59 - Omega-3 &amp; Cod liver Oil
-04:53 - Naltrexone
-05:52 - Plant-Based Diets
-06:42 - Boosting the Immune System
-07:22 - High Dose Vitamin C
-07:55 - B Vitamins
-08:39 - Selenium
-09:40 - Glutathione &amp; Whey Protein Concentrate
-10:00 - Zinc &amp; Immunity
-11:03 - Magnesium &amp; Relaxation
-11:37 - Bone Broth
-13:26 - Herbal Teas - Soursop &amp; Herb Robert
-14:46 - Autophagy &amp; Time Restricted Eating
-16:18 - Summary
-16:32 - End Credits
-Want to learn more about natural methods to deal with cancer?  
-Check out Gold from the Vaults - Episode 7 - Jerry Brunetti - Food as Medicine: Natural Cancer Treatments Part 1  
-https://blog.nutri-tech.com.au/gold-from-the-vaults-episode-7-jerry-brunetti/
-*Relevant NTS Products Featured in This Episode:*  
-_BioBubble™ Probiotic_
-https://www.ntshealth.com.au/products/bio-bubble
-_MagSorb™ Magnesium Spray_
-https://www.ntshealth.com.au/products/magsorb
-_Nutri-Salt_
-https://www.ntshealth.com.au/products/nutri-salt
-_SweetSure_
-https://www.ntshealth.com.au/products/sweetsure
-_BioSpark_
-https://www.ntshealth.com.au/products/biospark
-_Curcu-Life_
-https://www.ntshealth.com.au/products/curcu-life
-_Green Defence_
-https://www.ntshealth.com.au/products/green-defence
-*Interested in studying Nutrition Farming?*  
-Certificate in Nutrition Farming courses:  
-https://nutri-tech.com.au/pages/courses  
-Need personalised support?  
-Soil &amp; Plant Therapy Services:  
-https://nutri-tech.com.au/pages/soil-plant-therapy  
-Book a one-hour online consultation with Graeme Sait:  
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
-*Explore more at our website:*  
-https://nutri-tech.com.au/
-Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
-https://nutri-tech.com.au/pages/newsletter  
-*Follow us on Social Media:*  
-Facebook: https://www.facebook.com/NutriTechSolutions/  
-Instagram: https://instagram.com/nutritechsolutionsyandina  
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>🔥 Stop Flipping the Club! This Simple Drill Forces Body Rotation Through Impact ⛳
+🏌🏿♂️ Are you all arms through impact? If you're flipping the club and never rotating through the ball, this drill is for you.
+HI. I'm coach Erik Schjolberg, founder of EJS Golf in Scottsdale, Arizona. In this video, I show you a simple silicon band drill that forces your body to rotate through impact instead of relying on your hands and the small muscles. When you rotate correctly, you move your low point forward, deliver the club with forward shaft lean, and produce controllable spin with a predictable launch angle. This is how you become a great chipper.
+This is not a swing thought. This is a constraint that makes your body do the right thing. You should feel improvement on the first rep 💥
+Get my FREE DRILLS guide at EJSGolf.com/my-drills
+🏌️ Work with me in person in Scottsdale, AZ at McCormick Ranch Golf Club or online:
+👉 https://EJSGolf.com
+👉 Learn more about me: https://EJSGolf.com/about
+👉 Get my drills guide: https://EJSGolf.com/my-drills
+👉 Read the blog: https://EJSGolf.com/blog
+#GolfDrill #BodyRotation #StopFlipping #BallStriking #ForwardShaftLean #LowPointControl #GolfInstruction #ScottsdaleGolf #EJSGolf #TheScienceOfBetterGolf #GolfTips</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-01-09T04:32:57Z</t>
+          <t>2026-02-26T16:32:05Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>548</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.044883</v>
+        <v>0.009124</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Can you recommend a specific cod liver oil without a guaranteed analysis? || I have reached out to Graeme for his specific recommendation. From my research Rosita's is a highly recommend natural source,
-https://www.amazon.com.au/Rosita-EVCLO-Softgel/dp/B09B7BGZDD || @NutriTechSolutionsNTS Thank you so much :). I'm a banana farmer in Hawaii. Are you guys still doing online consults? || Great one again - thank you and I found the sound good || Thanks @markhiggins3054! || Really appreciate the content, but please.......please....address the sound quality issue. || Thanks, we are glad you appreciate the content! Can you explain the sound quality issue? as it sounds fine on my devices. || The voice sounds muffled</t>
+          <t>The content is amazing I will come back to watch it again. || Get my FREE DRILLS guide at EJSGolf.com/my-drills</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>jl2LucE_jhc</t>
+          <t>bRzUXlu5ILA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Visual Soil Assessment: Simple Tests Every Farmer Needs - How to S4E10</t>
+          <t>INSTANT Low Point Fix (Yoga Wedge Drill) | Stop Chunking Irons + Compress It</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>In this episode of *How To Do It* , we explore *visual soil assessment* , soil structure, biology, and practical field tests that reveal true soil health — straight from the paddock.
-#soilhealth, #regenerativeagriculture, #visualsoilassessment, #soilbiology, #soilstructure, #organicmatter, #earthworms, #microbiallife, #nutritionfarming, #regenerativefarming, #agronomy, #farmingeducation, #soilcarbon, #soilresilience, #soilaggregation, #sustainablefarming, #howtodoit, #nutritechsolutions, #graemesait, #biologicalfarming
-Joining me today is Marco, Head Agronomist at Nutri-Tech Solutions, as we return to the farm where his agronomy journey began. Together, we walk through a *practical, hands-on approach* to understanding soil health using visual soil assessment techniques.
-Rather than relying solely on chemistry, we dig into the *physical foundations* of soil performance — texture, structure, porosity, colour, aggregation, and earthworm activity. You’ll see how compost, humic substances, mulch, and biological management dramatically change soil outcomes, even over short distances.
-Marco demonstrates simple field tests, including the ribbon test, soil texture jar test, slaking test, and earthworm counts — revealing how biology drives aggregation, water infiltration, oxygen movement, and nutrient efficiency.
-This episode highlights why soil structure is the gateway to productivity, resilience, and water-holding capacity — and why biology-first management delivers compounding returns over time.
-👇 *Chapters:*
-00:00 - Introduction - Brewing
-01:27 - Title Sequence
-01:57 - Soil Texture
-05:52 - Soil Structure
-10:31 - Soil Porosity
-12:43 - Earthworm Counts
-13:57 - Slaking Test
-15:36 - General Biodiversity
-16:15 - Why is Soil Structure so important?
-18:31 - The Importance of Mulch &amp; Microbial Foods
-20:09 - End Credits
-Visual Soil Assessment Guide: https://cdn.shopify.com/s/files/1/1213/7046/files/Visual_Soil_Assessment_VSA_Workshop.pdf?v=1766715528
-For a deeper dive into the principles behind aggregation, biology, and soil resilience, this article pairs perfectly with today’s episode: Gas Exchange – How to Maximise your Money Maker - https://blog.nutri-tech.com.au/gas-exchange/
-*Humate Granules*
-https://nutri-tech.com.au/products/humate-granules
-*Life Force® Gold Pellets*
-https://nutri-tech.com.au/products/life-force-gold-pellets
-*Brewstar 200™*
-https://nutri-tech.com.au/products/brewstar-200
-*SeaChange® Liquid Kelp*
-https://nutri-tech.com.au/products/seachange-liquid-kelp
-*FulvX™*
-https://nutri-tech.com.au/products/fulvx
-*Interested in studying Nutrition Farming?*  
-Certificate in Nutrition Farming courses:  
-https://nutri-tech.com.au/pages/courses  
-Need personalised support?  
-Soil &amp; Plant Therapy Services:  
-https://nutri-tech.com.au/pages/soil-plant-therapy  
-Book a one-hour online consultation with Graeme Sait:  
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
-Explore more at our website:  
-https://nutri-tech.com.au/
-Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
-https://nutri-tech.com.au/pages/newsletter  
-*Follow us on Social Media:*  
-Facebook: https://www.facebook.com/NutriTechSolutions/  
-Instagram: https://instagram.com/nutritechsolutionsyandina  
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>Most golfers don’t need another “swing tip.” They need low point control. In this video I show you my favorite cheap training aid: a simple foam yoga wedge that trains a descending angle of attack and a low point in front of the ball—exactly how you create compression and stop hitting behind it.
+How to use it: place the wedge just ahead of the ball, make small swings, rotate through impact, and finish without flipping/scooping. I like the feel of my trail wrist staying extended in the finish because it confirms my body delivered the strike instead of my hands saving it.
+Want my full drill library and practice plan? Get my FREE Drills Guide at EJSGolf.com/my-drills.
+Coach Erik Schjolberg
+The Science of Better Golf
+#golf #golftips #golfdrills #ballstriking #compression #ironplay #lowpoint #impact #scottsdalegolf #ejsgolf</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-12-26T04:30:37Z</t>
+          <t>2026-02-17T17:13:16Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1426</t>
+          <t>148</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1347,102 +1020,61 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.025245</v>
+        <v>0</v>
       </c>
       <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>mGeeAsi5p0g</t>
+          <t>qVSu1aAhowo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Expert Nursery Owner Spills REAL Secrets on Farming! Pt2 - How to S4E9</t>
+          <t>Stop Chunking | Blading Chips and add Spin Today:   Simple Techniques that Anyone Can Do!</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Welcome back to another inspiring episode of the *How To Do It* series.
-This week, we’re visiting the Sunshine Coast’s remarkable _Eumundi Palms Nursery_ — a commercial nursery proving that *biological farming,* *chemical-free growing,* and *plant resilience* can outperform conventional systems while using significantly less water.
-#howtodoit, #biologicalfarming, #chemicalfreefarming, #regenerativeagriculture, #commercialnursery, #cocopeat, #trichoderma, #plantresilience, #beneficialmicrobes, #sustainablehorticulture
-In this episode, Graeme is joined by _Phil,_ founder of Eumundi Palms, to explore how a curiosity — growing a palm in a palm — led to the adoption of pure coconut fibre as a potting medium and the rapid transition away from systemic fungicides.
-We unpack how coco peat’s moisture-retentive structure creates the perfect environment for beneficial biology, particularly _Trichoderma,_ which thrives in fibrous media and provides both disease suppression and strong root stimulation. The result? Healthier plants, reduced water use, and the ability to access premium chemical-free export markets.
-The conversation then turns to *cell wall strength* and true plant resilience. Silica, calcium, and boron play a central role in strengthening plant architecture, improving stress tolerance, and reducing pest and disease pressure. You’ll also hear how advanced biological tools like _BAM_ and _MAD (Micro-Amino Drive)_ improve nutrient uptake efficiency and overall plant vitality.
-Beyond the agronomy, Phil shares the human side of Nutrition Farming — protecting staff health, building a committed long-term team, and involving the next generation in a business they’re proud to inherit.
-Whether you’re a grower, nursery operator, agronomist, or passionate home gardener, this episode offers practical insights into how *biology replaces chemistry* when we work with nature, not against it.
-👇 *Chapters:*
-00:00 - Introduction  
-01:16 - Title Sequence  
-01:46 - Coco Coir, Trichoderma &amp; Moisture Retention  
-04:09 - Cell Strength: Silica, Calcium &amp; Boron  
-06:02 - Beneficial Anaerobic Microbes &amp; Micro Amino Drive  
-08:04 - Export Markets  
-08:56 - Industry Adoption of Nutrition Farming &amp; Family  
-12:21 - Practical Application of Nutrition Farming  
-14:38 - The Importance of pH  
-15:28 - Walk &amp; Talk: Healthy &amp; Resilient Palms  
-21:52 - End Credits  
-Want to learn more about the role of silica and calcium in building resilient plants?  
-Check out Graeme’s article on the NTS blog:  
-_Sili-Cal (B)™ — a unique combination of three synergistic, cell-strengthening elements_  
-https://blog.nutri-tech.com.au/
-*Visit Eumundi Palms:*  
-https://eumundipalms.com.au/
-*Relevant NTS Products Featured in This Episode:*  
-_Sili-Cal (B)™_  
-https://nutri-tech.com.au/products/sili-cal-b  
-_Tri-Kelp™_  
-https://nutri-tech.com.au/products/tri-kelp  
-_Nutri-Life BAM™_  
-https://nutri-tech.com.au/products/nutri-life-bam  
-_NTS FulvX™ Powder_  
-https://nutri-tech.com.au/products/nts-fulvx-powder  
-_Nutri-Stim Triacontanol™_  
-https://nutri-tech.com.au/products/nutri-stim-triacontanol  
-*Interested in studying Nutrition Farming?*  
-Certificate in Nutrition Farming courses:  
-https://nutri-tech.com.au/pages/courses  
-Need personalised support?  
-Soil &amp; Plant Therapy Services:  
-https://nutri-tech.com.au/pages/soil-plant-therapy  
-Book a one-hour online consultation with Graeme Sait:  
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait  
-Explore more at our website:  
-https://nutri-tech.com.au/
-Sign up for our Newsletter and receive a *free digital copy of Graeme’s book:*  
-https://nutri-tech.com.au/pages/newsletter  
-*Follow us on Social Media:*  
-Facebook: https://www.facebook.com/NutriTechSolutions/  
-Instagram: https://instagram.com/nutritechsolutionsyandina  
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions  
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>If your chips feel random—one checks, one releases, one gets bladed—that’s not “touch.” That’s missing impact conditions. In this video I walk you through my chipping procedures that make the strike measurable and repeatable: ball first, turf second, with a PREDICTABLE amount of spin so you can actually trust what happens when it lands.
+Here’s the foundation. I build a stock chip shot that covers roughly 85–90% of what you’ll face around the green. Feet closer together, shoulders level (most golfers “get left” by shoving left and popping the lead shoulder up—don’t do that), lead foot flared to make rotation easier, and a descending strike. Then I show you the #1 DEADLY SIN that wrecks contact:
+I show you how I create spin without getting wristy or feel like you have to drive the ball into the ground.  With a wide, pivot-driven swing,  I can change distance by changing pivot speed—not by flipping my hands. I also teach the “float” action: the club head doesn’t dive down immediately. Finish matters too. I hold the finish because it tells the truth—face the target, handle pointing back at you, club face staying semi - open unless you’re intentionally running it.
+If you want this measured with TrackMan (dynamic loft + attack angle = the spin/launch window you’re actually delivering), book a session with me and I’ll build your stock chip around your clubs and your matchups.
+To find out how to book a lesson with me in Scottsdale, AZ at McCormick Ranch or online, go to my website, EJSGolf.com.  
+If you want me to cover the “runner” version (how I intentionally close the face to launch lower and release), comment “RUNNER” and I’ll film it for you.
+YouTube tags (comma-separated)
+Coach Erik Schjolberg
+The Science of Better Golf
+EJSGolf.com
+Scottsdale Golf Lessons
+Online Golf Lessons  
+#Golf #Chipping #ShortGame #BallStriking #EJSGolf</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025-12-12T04:30:38Z</t>
+          <t>2026-01-30T20:29:34Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>853</t>
+          <t>261</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1451,446 +1083,252 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.024619</v>
+        <v>0.003831</v>
       </c>
       <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>b9rRVtnn5x8</t>
+          <t>B5wDtzaY4MI</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Farming Secrets From a Real Plant Nursery! Eumundi Palms Interview Pt1 - How to S4E8</t>
+          <t>Stop Flipping: Split-Hand HOCKEY DRILL to FIX Casting and GAIN Compression, Rotation and Shaft Lean!</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Welcome back to another inspiring episode of the *How To Do It* series.
-This week, we’re visiting the Sunshine Coast’s remarkable *Eumundi Palms Nursery* — a thriving family business committed to growing stronger, healthier plants without relying on chemical crutches. 🌿✨
-#chemicalfree #biologicalgrowing #plantresilience #regenerativehorticulture #healthyplants #organicnursery #plantpropagation #pottingmix #beneficialmicrobes #nurseryproduction 
-In Part 1 of this interview, owner *Philip Redhead* shares how he transformed a modest nursery into one of Queensland’s standout examples of sustainable plant production. As we walk through the lush rows of ornamentals and palms, Philip explains the turning points, challenges, and practical strategies that shaped this transformation. 🌴💬
-A major theme of this episode is the choice to step away from conventional, chemical-heavy growing systems. Philip explains how repeated chemical use often weakens plants over time, while healthier soils and beneficial biology build plants that truly *thrive* once they leave the nursery. The improvements in resilience, strength, and long-term performance are unmistakable. 🌱💪
-We explore propagation techniques, potting mix improvements, natural disease management, and efficient systems that support the nursery through busy seasons. Philip also shares the emotional rewards of nursery life — watching roots develop strongly, reusing returned pots, and nurturing plants destined to enrich gardens for decades. 🪴😊
-You’ll also get an honest look at the challenges of running a family nursery: staffing shortages, rising demand, and the constant effort to maintain quality under pressure. Through it all, Philip’s commitment to integrity, plant health, and sustainable practices shines brightly. 🌏💚
-Whether you’re a grower, home gardener, landscaper, or simply someone who loves hearing real stories of people doing things better, this episode is full of practical insights and fresh inspiration.
-*Stay tuned for Part 2* , where we dive deeper into biological strategies, advanced growing techniques, and the powerful philosophy behind Eumundi Palms’ long-term success.
-Thanks for watching — enjoy the episode! 🙌🌿
-👇 *Chapters:*
-00:00 - Introduction
-01:33 - Title Sequence
-02:03 - Phil's Backstory
-04:12 - Plant Fundamentals for Health - Silica &amp; Tsunami
-05:57 - Pest &amp; Disease Management
-07:09 - Foliar &amp; Fertigated Nutrition - Uptake Efficiency
-08:52 - Silica, Calcium &amp; Boron - Benefits Continued
-11:47 - Pseudomonas Florescence - Silica Solubilisation &amp; Other Benefits
-14:32 - Plant Nursery Priorities - Insects
-15:47 - Ecological Priorities - Power &amp; Recyclable Pots
-17:11 - End Credits
-Want to learn more about Nutrition Farming? Check out Graeme's article on *”Sili-Cal (B)™ a unique combination of three synergistic, cell-strengthening elements* …
-https://blog.nutri-tech.com.au/sili-cal-b-a-unique-combination-of-three-cell-strengthening-elements-2/
-*Check out Eumundi Palms' website below*
-https://eumundipalms.com.au/
-*Sili-Cal (B)™*
-https://nutri-tech.com.au/products/sili-cal-b
-*Tri-Kelp™*
-https://nutri-tech.com.au/products/tri-kelp
-*Nutri-Life BAM™*
-https://nutri-tech.com.au/products/nutri-life-bam
-*NTS FulvX™ Powder*
-https://nutri-tech.com.au/products/nts-fulvx-powder
-*Nutri-Stim Triacontanol™*
-https://nutri-tech.com.au/products/nutri-stim-triacontanol
-*Interested in attending a Certificate in Nutrition Farming course?*
-https://nutri-tech.com.au/pages/courses
-Need assistance? Try out our Soil &amp; Plant Therapy Services
-https://nutri-tech.com.au/pages/soil-plant-therapy
-How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait
-Head to our website to find out more
-https://nutri-tech.com.au/
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-*Follow us on Social Media*
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>If you’re tired of flipping at impact with negative shaft lean—hands behind the ball, club head passing early, and zero compression—this is the drill I go to. It’s a hockey-style split-hand grip that forces the correct sequencing: rotation delivers the strike, not a last-second hand throw. The goal is simple and non-negotiable: ball first contact, then turf, with real shaft lean and a stable club face.
+Here’s the key: split your hands on the grip, rehearse without a ball first, then hit small shots. If your body tries to “save it” by casting, you’ll feel it immediately. When you do it right, your hands work left through rotation while the club head stays out in front of your chest longer—exactly what clean ball strikers do.
+Want the full breakdown on why you cast (and how to fix your impact fast)? Watch more on my YouTube channel and grab my free drills guide here: EJSGolf.com/my-drills
+If you want me to diagnose your swing and give you the fastest fix for your impact, send me your swing video for a FREE analysis.
+Coach Erik Schjolberg
+The Science of Better Golf
+EJSGolf.com
+Scottsdale Golf Lessons
+Online Golf Lessons  
+#SGL #golfswing #EJSGolfAcademy #CoachErik #golftechnique #ejsgolf #golf #golfgear #shallow #Rotation #shaftlean</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025-11-28T04:30:26Z</t>
+          <t>2026-01-26T00:05:44Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1105</t>
+          <t>956</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.034389</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Wow got a lot out of this! I nearly skipped it! Thank you both for sharing with us your time and knowledge it is greatly appreciated! We can’t wait to do the course next week!! || At the 11:45 time period Graeme introduces the silica solubilizing microbe Pseudomonas Florescens and goes on to talk about ice formations created by microbes. The particular species identified is another of the Pseudomonas family…..Syringae. Check out the shift from liquid to solid when Syringae is added to cold water and the phase shifts from liquid to solid.
-https://www.youtube.com/shorts/DiDNVSHm-cA || Awesome, thanks for sharing this Brad!
-For some reason the link opens with studio. hopefully this link works better...
-https://www.youtube.com/shorts/DiDNVSHm-cA || Interesting Tsunami has rice husks. I want to try the sheoak (casaurina) brew from another episode but it seems the sheoak does not contain much Si so I am planning to add rice husks. Any idea if that would lift the Si in the final brew? || Thanks for the question! Tsunami is based on rice husks, though the active component is relatively complex extraction. 
-Yes, She oak (Casuarina) has been a common ingredient for BD508 in Australia, though there isn't a lot of research on it's actual silica content. Rice husks have been studied more widely and are a very good source of bioavailable silica, with it making up about 15–20% of the husk dry weight. So including it in a well managed brew would certainly deliver more available Silica.
-There are other pH factors to be mindful of but ashes from these plant materials can be another highly concentrated source of Silica, for reference Rice Husk ashes can range from 74–98% SiO₂. || ​@NutriTechSolutionsNTS I asked AI for info on rice husks and yes it seems making the Si is a headache for DIY people. And I suspect that the process of making AI in rice husks plant available will increase the pH which I want to avoid because it then becomes incompatible with most other fertilisers || Seems to me that combining the BD508 with a little potassium silicate could be an easy compromise || Thanks for posting, interesting that you want 800ppm Si on the tissue test, will try get up to that. || Can SilicaB be used on all plants from stone fruit trees, citrus trees and vegetables. || Thanks or the question! Yes, Ideally this would always be based on a soil test, but you can use Sili-Cal B on all crops, the importance of these nutrients are foundational to any healthy crop.
-https://nutri-tech.com.au/products/sili-cal-b?_pos=1&amp;_psq=sili&amp;_ss=e&amp;_v=1.0 || ​@NutriTechSolutionsNTSthank you.</t>
-        </is>
-      </c>
+        <v>0.018828</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-r6y2epf7jQ</t>
+          <t>C7EvmfEoZNU</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Can You Really Change Your Mood in 2 Minutes? Human Health Tips! - How to S4E7</t>
+          <t>How to Gain Speed, Distance, Shaft Lean and More in your Golf Swing with these 2 Drills</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>* Two-Minute Tips for #StressRelief and #HealthyLiving *
-In this uplifting episode, Graeme shares four simple, fast and transformative strategies to help you reduce stress and cultivate greater calm in your daily life. These ideas are *micro-habits* with *macro-benefits* , designed for busy people who need practical tools for immediate change. 🌿
-#stressrelief #wellnesshabits #mentalhealthtips #EFTtapping #mindfulness #breathingexercises #reduceanxiety #balanceexercise #brainhealth #lowstressliving #healthylifestyle
-We begin with the *Emotional Freedom Technique (EFT).* This combination of intention, affirmation and tapping on key acupuncture points may sound -too good to be true-, yet a growing body of research shows that EFT can quickly ease anxiety, emotional tension and accumulated stress. Graeme demonstrates each tapping point, guiding you through a sequence that takes just two minutes and can deliver surprising relief. ✨
-The episode then explores the importance of *living in the present moment.* Drawing from Lao Tzu and echoed by modern thinkers like Eckhart Tolle, Graeme explains why living in the past creates depression, living in the future creates anxiety, and why only the present moment contains genuine peace. You’ll learn a simple technique: stop once an hour and take *three slow, deep breaths.* This short practice interrupts racing thoughts, supports the lymphatic system and gradually retrains your nervous system toward calm. 🌬️
-You’ll also discover the fascinating *two-minute balance challenge* from Chinese health master Zhong Li Ba Ren. Standing on one leg with your eyes closed challenges your neurological balance and provides a quick window into your biological age. The practice is associated with benefits for blood pressure, blood sugar, spinal mobility and long-term brain function. Whether or not you fully accept the bold claims, it is a fun and revealing daily test of stability and mind–body connection. 🧠💫
-Finally, Graeme presents the simplest tip of all: *reduce your screen time.* Constant exposure to media-driven negativity can drain joy and increase stress. Swapping some screen time for music, uplifting reading, creativity or meaningful connection can dramatically improve wellbeing.
-These ten *two-minute tips* are practical, powerful and accessible for everyone. Try them consistently for two weeks and observe the shift in clarity, calm and resilience. 💚
-👇 *Chapters:*
-00:00 - Introduction - Human Health Exercises
-01:32 - Title Sequence
-02:02 - Emotional Freedom Technique - Tapping
-05:47 - Living in the Moment - Meditation
-11:01 - Being Proactive - Mindset, Love or Fear
-16:14 - The Golden Cockerel - Balance
-23:30 - End Credits
-If you want to learn more about Human Health strategies. Check out Graeme's interview article with the late great Jerry Brunetti…
-https://blog.nutri-tech.com.au/jerry-brunetti-interview-part-1-2/
-Bio-Bubble
-https://www.ntshealth.com.au/products/bio-bubble
-Nutri-Salt
-https://www.ntshealth.com.au/products/nutri-salt
-SweetSure
-https://www.ntshealth.com.au/products/sweetsure
-BioSpark
-https://www.ntshealth.com.au/products/biospark
-Curcu-Life
-https://www.ntshealth.com.au/products/curcu-life
-Green Defence
-https://www.ntshealth.com.au/products/green-defence
-Head to our website to find out more
-https://nutri-tech.com.au/
-Interested in attending a Certificate in Nutrition Farming course?
-https://nutri-tech.com.au/pages/courses
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-Follow us on Social Media
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>Most golfers don’t need a swing rebuild to hit it farther and compress the ball. They need better impact conditions—more forward shaft lean, better low point control, and a body that actually supports speed instead of stalling so the hands can “catch up.” In this video I show two simple drills you can do with what you already own: a golf club and an alignment stick (or training club).
+Drill #1 fixes the most common speed killer I see: the “pull-down gap” where the arms separate, the club gets yanked down, and the body has to stall to survive impact. I use an under-the-armpit connection constraint so you stop ripping from the top and learn how to rotate through with structure. If you can keep your lead arm connected longer, your sequencing improves and your impact starts looking like a ball striker—hands forward, club head delivered with intention, and compression you can actually feel.
+Drill #2 is my favorite speed producer before a round: swing as fast as you can and STOP in a controlled “impact checkpoint.” If you can’t stop it, your body isn’t supporting your speed—period. When you learn to stop it, your body organizes itself automatically: you clear space, you get the hands forward, and you find the kind of impact position golfers chase for years by thinking about ten different swing thoughts. I’m not interested in thoughts. I’m interested in measurable outcomes.
+Coach Erik Schjolberg
+The Science of Better Golf
+EJSGolf.com
+Scottsdale Golf Lessons
+Online Golf Lessons  
+#GolfDrills #ShaftLean #GolfSpeed #Compression #BallStriking #IncreaseDistance #ImpactPosition</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-11-14T04:30:01Z</t>
+          <t>2026-01-25T07:09:14Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>920</t>
+          <t>110</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.030435</v>
+        <v>0.054545</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Absolutely well said yet again. 
-Loved your course a few weeks ago - life changing.</t>
+          <t>1 MORE is LESS Skill applications being accepted || Thanks for the comment!</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JKGkOqX-pOw</t>
+          <t>QigOaULFjv8</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The Future of Farming - 10 Practical Steps to get Started - Part 2 - How to S4E6</t>
+          <t>Nail the Jump Move for Perfect Golf Rotation! #shorts</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>In this powerful follow-up episode, *Graeme Sait* continues his step-by-step guide to launching your *regenerative journey* with practical demonstrations, tools, and insights that empower both *farmers and consultants* to get real results — in the field and in life.
-#NutritionFarming #GraemeSait #SoilHealth #RegenerativeAgriculture #BAM #MicrobialBrewing #HealthySoilHealthyYou #SustainableFarming #FarmersHealth
-🔥 *Highlights from this episode:*
-🌿 *1️⃣ Brewing Living Fertilisers*
-Discover how to create your own *on-farm biological inputs.* Graeme demonstrates the *three-in-one brewer* for producing *aerobic* , *anaerobic* , and *extract* brews — including *vermicompost extracts* , *Bacillus subtilis* , *Trichoderma* , and *Azotobacter.* These living brews boost soil life, crop resilience, and productivity while slashing input costs.
-💧 *2️⃣ The Simplicity of BAM*
-Learn about *BAM – Beneficial Anaerobic Microbes* — a microbial inoculum that can be brewed on-farm with *molasses and water.* With a two-year shelf life and remarkable versatility, BAM is now *used in over 55 countries* as a foundation of biological success.
-🔬 *3️⃣ Tools for Precision Nutrition*
-Graeme explains how to measure and manage your results using:
-• The *Brix meter* for monitoring sugars and plant vitality.
-• *pH strips* to track potassium movement between leaves.
-• Simple nutrient mobility checks to detect deficiencies early.
-These practical tools help you make smarter, faster nutrient decisions.
-💚 *4️⃣ Fear-Based vs Love-Based Farming*
-Graeme shares a heartfelt message about mindset — contrasting the *fear-driven chemical model* with the *love-based regenerative approach* that nurtures *soil life, human health,* and *planetary wellbeing.* Every farming choice, he says, is either *fear or love in action.*
-🌼 *5️⃣ Natural Disease Protection*
-A simple recipe for *powdery mildew control* — combining *BAM and milk powder* , optionally enhanced with *manganese* — delivers a sustainable, cost-effective disease solution that strengthens plants naturally.
-🌾 *6️⃣ Farmer Wellbeing and Self-Care*
-Graeme closes with tips for *managing stress, supporting magnesium and B6 levels,* and embracing *autophagy* through intermittent fasting — reminding us that *healthy soil and healthy farmers are inseparable*.
-✨ *Practical, inspiring, and deeply transformative,* this episode reconnects the roots of *Nutrition Farming®* with the heart of *personal wellbeing.*
-👇 *Chapters:*
-00:00 Introduction - Brewing
-00:59 Title Sequence
-01:29 Brewing your own Living Fertilisers
-02:55 Checking Your Progress
-08:08 Being Proactive - Mindset, Love or Fear
-11:12 Taking care of your Health
-17:06 End Credits
-Want to learn more about Nutrition Farming? Check out Graeme's article *”Ten Tips for Microbe Brewing - DIY Living Fertilisers* …
-https://blog.nutri-tech.com.au/10-tips-for-microbe-brewing/
-*Nutri-Life BAM™*
-https://nutri-tech.com.au/products/nutri-life-bam
-*NTS FulvX™ Powder*
-https://nutri-tech.com.au/products/nts-fulvx-powder
-*Tri-Kelp™*
-https://nutri-tech.com.au/products/tri-kelp
-*Nutri-Stim Triacontanol™*
-https://nutri-tech.com.au/products/nutri-stim-triacontanol
-*Cal-Tech™*
-https://nutri-tech.com.au/products/cal-tech
-*Sili-Cal (B)™*
-https://nutri-tech.com.au/products/sili-cal-b
-*Interested in attending a Certificate in Nutrition Farming course?*
-https://nutri-tech.com.au/pages/courses
-Need assistance? Try out our Soil &amp; Plant Therapy Services
-https://nutri-tech.com.au/pages/soil-plant-therapy
-How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait
-Head to our website to find out more
-https://nutri-tech.com.au/
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-*Follow us on Social Media*
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>🏌🏿♂️Nail the Jump Move for Perfect Golf Rotation!
+🏃♂️ Ready to elevate your golf game? The jump move is your key to crushing rotation, shaft lean, power, speed, compresion andd reducing early extension! ⛳ Feel the difference with my jump drill! 🙌 Let's go!
+Coach Erik Schjolberg
+EJS Golf
+The Science of Better Golf
+Scottsdale Golf Lesson
+Online Golf Lessons
+ #Golf #SwingTips #JumpMove #Golfers #Training</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-10-31T04:30:15Z</t>
+          <t>2026-01-11T18:03:28Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1430</t>
+          <t>1083</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.037762</v>
+        <v>0.003693</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Unreal series! So much important information, thanks || Is there some kind of instructional manual or video instruction on how to brew and use the brewer and products for specific applications. || Make your own compost, way cheaper.
-Just google compost extraction || ​@666bruvhave been making my own. Always nice to find other recipes. || ​@johnharris7244don't waste your money on bug in a jug || Thanks for the question @johnharris7244!
-I have created a playlist below containing all the videos we have produced to date on brewing microbes. Most of these weren't filmed using the new 3 in 1 Brewer, but they can easily be adapted to do so. We plan to produce more videos featuring this unit in the future. 
-https://www.youtube.com/playlist?list=PLXReS_QZvjWAB7kPDqcqPTEiQ41VuD4cT || Thanks for the comment! They all help with the algorithm to further highlight our videos featuring "Bug in a Jug".
-I suggest you look deeper into the different classes of microbes in relation to their association with plants and other microbes. Compost is an incredible tool, but it still has many limitations when it comes to culturing the complete range of beneficial microbes. 
-Obligate Symbionts (Plant-Reliant Microbes)The microbes that form the most intimate, beneficial plant partnerships generally do not survive standard composting. 
-Arbuscular Mycorrhizal Fungi (AMF): They are obligate symbionts, meaning they must be connected to a living root to reproduce and thrive. The high temperatures of the active composting phase will typically destroy their delicate spores and hyphae.
-Symbiotic Nitrogen-Fixing Bacteria (Rhizobium): While they can survive in soil, they are highly specific. For effective inoculation, you must use specialized, host-specific inoculants (e.g., coating legume seeds) rather than relying on a general compost mix. || Is there much difference between EM and BAM? || Great question,  I brewed up some EM1 a couple of weeks ago and it has very distinctive sweet aroma , yesterday I opened up a container of BAM and it smells very similar and that was my exact thought. || Thanks for the question @howardroe7515!
-Yes, there are some differences between EM (Effective Microorganisms) and BAM (Beneficial Anaerobic Microbes), although they share similar foundational concepts. Both products are designed to enhance soil health and plant growth through the use of beneficial microorganisms, but they have distinct compositions and applications:
-EM (Effective Microorganisms): Developed by Professor Teruo Higa, EM is a blend of various beneficial microorganisms, including lactic acid bacteria, yeast, and photosynthetic bacteria. It is widely used in agriculture to improve soil health, composting, and plant growth.
-BAM (Beneficial Anaerobic Microbes): BAM is based on the original EM formula but includes additional microbial varieties. It contains over 80 different microbe varieties, including lactobacillus, purple non-sulphur bacteria (PNSB), fermenting fungi, yeast, and actinomycetes. BAM is designed to perform similar functions to EM but with a broader spectrum of microorganisms. || ​@NutriTechSolutionsNTSdoes that make BAM a good foliage spray option. || Yes, BAM is a great all rounder, it's certainly helpful via foliar, though it's most effective in the soil, especially for recovering anaerobic soils.</t>
+          <t>Get my FREE DRILLS guide at EJSGolf.com/my-drills</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UCCUQcYl9nqmztVGjuTbzCOQ</t>
+          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NutriTechSolutions</t>
+          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>6JQ7quA88xo</t>
+          <t>PJNm8Wq2wJY</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The Future of Farming - 10 Practical Steps to get Started - Part 1 - How to S4E5</t>
+          <t>🏌🏿‍♂️Nail the Jump Move for Perfect Golf Rotation!</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Welcome to *Episode 5 of Series 4* of the *“How to Do It”* video series. In this special instalment, we take a short break from our *Human Health* focus to explore the practical heart of *Nutrition Farming ®*  — how to actually get started.
-After four seasons and over sixty episodes, many viewers have shared a common challenge: *“Where do I begin?”*  In this inspiring session, Graeme Sait cuts through the information overload and lays out a *10-step action plan* designed to move you from learning to doing.
-*Take away the guesswork.* Learn why *tissue testing* and *soil testing* are essential, how to interpret results, and how to avoid wasting money on unnecessary inputs.
-*Measure your microbial workforce.* Discover how tools like the *Microbiometer ®* can reveal soil vitality by measuring *total microbial biomass* and the critical *fungal-to-bacterial ratio.* Graeme explains why rebuilding the fungal component is central to creating well-structured, living soil.
-👉 *From there, you’ll explore:*
-• The importance of *humic and fulvic acid* in boosting nutrient uptake and soil structure.
-• Why *FulvX™* , a new humic-fulvic combination, offers the best of both worlds.
-• The role of *mycorrhizal fungi* and *Trichoderma* in extending root systems, enhancing nutrient delivery, and protecting crops from *root-knot nematodes.*
-• The game-changing potential of *foliar nutrition* — particularly *foliar urea* and *calcium-boron* combinations — to dramatically lift plant performance while reducing input costs.
-• And finally, the extraordinary natural plant growth compound *Triacontanol* , described as the *most powerful plant growth promoter ever researched.*
-💡This practical, down-to-earth guide provides the perfect foundation for farmers and gardeners ready to turn theory into results. Whether you adopt one step or all ten, the key message is clear: *action transforms everything*.
-🎥 *Join Graeme Sait as he reignites the movement from awareness to implementation — the essence of Nutrition Farming ®.*
-#NutritionFarming #SoilHealth #HowToDoIt #GraemeSait #FulvicAcid #HumicAcid #Microbiometer #MycorrhizalFungi #Triacontanol #FoliarFeeding #SustainableFarming #RegenerativeAgriculture #SoilMicrobes #PlantNutrition #CalciumBoron #FulvX #Trichoderma #SoilTesting #TissueTesting #MicrobialBiomass #ActionNotTalk
-👇 *Chapters:*
-00:00 - Introduction
-01:35 - Title Sequence
-02:05 - Plant Tissue Testing
-02:55 - Soil Testing &amp; Dealing with Deficiencies
-04:54 - Testing Microbial Activity - MicroBiometer
-08:51 - Humates
-10:35 - Experimentation &amp; Microbial Inoculums
-12:15 - Foliar Nutrition, Urea, Calcium &amp; Triacontanol
-Want to learn more about Nutrition Farming? Check out Graeme's article *”Ten Tips for Microbe Brewing - DIY Living Fertilisers* …
-https://blog.nutri-tech.com.au/10-tips-for-microbe-brewing/
-*Nutri-Life BAM™*
-https://nutri-tech.com.au/products/nutri-life-bam
-*NTS FulvX™ Powder*
-https://nutri-tech.com.au/products/nts-fulvx-powder
-*Tri-Kelp™*
-https://nutri-tech.com.au/products/tri-kelp
-*Nutri-Stim Triacontanol™*
-https://nutri-tech.com.au/products/nutri-stim-triacontanol
-*Cal-Tech™*
-https://nutri-tech.com.au/products/cal-tech
-*Sili-Cal (B)™*
-https://nutri-tech.com.au/products/sili-cal-b
-*Interested in attending a Certificate in Nutrition Farming course?*
-https://nutri-tech.com.au/pages/courses
-Need assistance? Try out our Soil &amp; Plant Therapy Services
-https://nutri-tech.com.au/pages/soil-plant-therapy
-How about a one-hour Online Consultation with Graeme Sait? Book an online consultation today…
-https://nutri-tech.com.au/pages/consultations-with-graeme-sait
-Head to our website to find out more
-https://nutri-tech.com.au/
-Sign up for our Newsletter &amp; Receive a free digital copy of Graeme's book
-https://nutri-tech.com.au/pages/newsletter
-*Follow us on Social Media*
-Facebook: https://www.facebook.com/NutriTechSolutions/
-Instagram: https://instagram.com/nutritechsolutionsyandina
-LinkedIn: https://www.linkedin.com/company/nutri-tech-solutions
-X (Twitter): https://x.com/ntsaustralia</t>
+          <t>🏌🏿‍♂️Nail the Jump Move for Perfect Golf Rotation!
+🏃‍♂️ Ready to elevate your golf game? The jump move is your key to crushing rotation, shaft lean, power, speed, compresion andd reducing early extension! ⛳ Feel the difference with my jump drill! 🙌 Let's go!
+Coach Erik Schjolberg
+EJS Golf
+The Science of Better Golf
+Scottsdale Golf Lesson
+Online Golf Lessons
+ #Golf #SwingTips #JumpMove #Golfers #Training</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025-10-17T04:30:03Z</t>
+          <t>2026-01-11T17:57:28Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2628</t>
+          <t>718</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.023592</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Excellent episode, Thanks very much || Question about the foliar calcium, if we use chelated calcium nitrate, on the one hand, good for foliar calcium but I'm trying to avoid nitrate applications for the reason mentioned in the foliar urea section of the vid.  Do you have any idea how impactful foliar calnitrate is upon plant energy in this context, assuming here the plant absorbs it in leaves and then needs to convert it to amino which will take lots of energy. Any alternatives to foliar chelated calcium nitrate? || Thanks for the great question @davidspghill!
-This really depends on the required outcome. If this specifically to deal with a calcium deficiency, a chelated form of Calcium Nitrate is still one of the most practical methods we would recommend, due to it's high availability, solubility and ease of application. An average crop requires 10-12 times more nitrogen than calcium, so this is still just a fraction of the overall N required. The remaining N could be applied via foliar urea applications throughout the season.
-Otherwise you could opt for micronised lime, it has a much lower effective foliar uptake rate, but due to the lower cost per kilogram it still works out at a similar cost per hectare. It does require slightly more specialised spray equipment due to the insoluble particles and the need for constant agitation during application, but it is certainly another practical option. It would also allow for the inclusion of chelated urea in the same application.
-It's true that nitrate requires around 8 times more energy for foliar uptake than urea, but this is just one aspect. If you have a severe calcium deficiency the increased energy production due to it's alleviation will easily counteract the additional energy required to utilise the nitrate.
-I hope that helps!</t>
-        </is>
-      </c>
+        <v>0.008357</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update niche prompt: add 100 coach-based ecosystems, remove old skill-based niches
</commit_message>
<xml_diff>
--- a/output/master.xlsx
+++ b/output/master.xlsx
@@ -448,34 +448,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Welcome to the official YouTube channel of EJS Golf, hosted by me, Coach Erik Schjolberg, top rated golf coach in the golf mecca of Scottsdale, AZ. With over 25 years of experience as a Professional Golf Coach, I’ve had the privilege to work with PGA Tour Players, college athletes, high-level developing juniors, and golf enthusiasts who are willing to commit to progress and weekend warriors that want to get better for that day or tournament.
-Are you tired of hitting fat golf shots, topping, not having the shaft lean you want, etc.?   There are root causes to these that have to be fixed to become the ball striking machine anyone can become.   Improve your game from the very first lesson.  Every golfer should get better from their very first lesson. My feedback-driven approach to practice, demanding only 15 minutes of commitment per day, guarantees results.
-Coach Erik Schjolberg
-EJSGolf.com
-Scottsdale Golf Lessons
-Online Golf Lessons
-(480) 861-9370
+          <t xml:space="preserve">Feeling stuck with what to paint… or unsure how to begin? You’re in the right place.
+I’m Joy Fahey, and I share simple, easy-to-follow abstract painting tutorials to help you start painting with confidence — even if you haven’t painted in years.
+Here you’ll learn how to:
+find ideas for your paintings
+start on canvas without overthinking
+use colour, shape, and intuition in a simple way
+This is a calm, supportive space where you can relax, explore, and enjoy the process — without pressure or perfection.
+If you’d like gentle guidance, creative inspiration, and practical ways to get started…
+subscribe and paint along with me.
 </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7290</t>
+          <t>11000</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>935</t>
+          <t>236</t>
         </is>
       </c>
     </row>
@@ -563,65 +565,88 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>lrMjPBep7x0</t>
+          <t>vNmu9SFgkn0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The Trail Knee Drill That Moves Low Point Forward</t>
+          <t>Start HERE - If You Don't Know What or How to Paint an Acrylic Abstract Painting</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Get my free 16 Drills guide: EJSGolf.com/my-drills
-Coach Erik Schjolberg breaks down the one constraint drill that fixes low point, eliminates flipping, early extension and creates ball-first contact on every iron. If your divots start behind the ball or you catch it thin, your trail knee is stalling and your pressure never transfers. This aim-stick gate drill physically forces the trail knee to drive toward the target, clearing the pelvis and shifting the low point 2–4 inches ahead of the ball.
-You will learn: 
-✅ (1) How to set up the alignment-stick gate for your trail knee. 
-✅(2) Why trail knee stall kills compression and creates early extension. ✅(3) How to feel the pressure shift from trail foot to lead foot by P6.
-✅ (4) Measurable checkpoints using divot position, strike spray, and TrackMan data (low point, shaft lean, dynamic loft).
-This is The Science of Better Golf—data-driven, constraint-led instruction that produces day-one improvement. No swing thoughts. No guessing. Just a physical gate that makes your body move correctly.
-Get my free 16 Drills guide: EJSGolf.com/my-drills
-Book a lesson in Scottsdale: EJSGolf.com
-Coach Erik Schjolberg
-The Science of Better Golf
-EJSGolf.com
-Scottsdale Golf Lessons
-Online Golf Lessons  
-#golfswingmechanics #golfswinganalysis #golfimpact #golfpower #golfdistance #EJSGolf #Titleist #Linksoul</t>
+          <t>⭐Join the Wait list for 'The Free Taster Course' The Simple Way to Paint Abstracts.
+ - https://www.joyfaheyclasses.com/free-taster-a-simple-way-to-paint-abstracts-with-confidence
+_______________________________________________________________________
+If you’ve ever sat in front of a blank canvas wondering What or How to Paint an Acrylic Abstract Painting… you’re not alone.
+In this video, I’ll show you a simple, relaxing way to start a canvas painting for beginners, even if you feel stuck, uninspired, or lacking confidence. This easy abstract painting method helps you move past overthinking and just begin.
+Whether you’re:
+starting painting again after a break
+a beginner learning how to paint on canvas
+or simply looking for fresh painting ideas
+this step-by-step approach will give you a gentle, creative starting point.
+We’ll explore:
+how to find ideas for your painting
+how to turn simple shapes into a composition
+how to start painting on canvas with confidence
+and how to enjoy the process without pressure
+This is about making painting simple, intuitive, and enjoyable,  no complicated techniques, just a calm and encouraging way to begin.
+I share simple, easy-to-follow abstract painting tutorials to help you feel confident, find ideas, and start paintings you'll enjoy without overthinking. Great for beginners and more experienced art lovers alike. 
+Subscribe to paint along with me and enjoy the process.
+_______________________________________________________________________
+Want more step-by-step support and painting ideas? 
+🎨 Learn more about the Heart &amp; Soul Art Academy - to Start Your Free Month click
+https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout
+✨ Free Abstract Painting Tutorial -
+https://www.joyfaheyclasses.com/offers/zKznsbqH/checkout
+💝 Get a Solid Foundation  from start to finish in your abstracts paintings with "The Complete Abstract Painting Course" for just $27 Click - https://joyfahey.com/the-complete-abstract-art-painting-course/ 
+⭐Learn More about my 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+#AbstractAcrylicPaintingforBeginners #AcrylicAbstractArtTutorials. 
+#paintingforbeginners #intuitiveart #artinspiration
+#howtopaint</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-23T21:36:51Z</t>
+          <t>2026-03-28T11:01:08Z</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1223</t>
+          <t>859</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>72</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.012265</v>
+        <v>0.088475</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -630,70 +655,100 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Hi friends, golfers. This is part two for those of you that hate seeing in the video your knee going out like this on the down swing. So you're swinging it goes here. First we covered relationship between heel toe on the way we're moving back using an alignment stick and the weight down how we're pushing here. We're going to cover just working on that trail knee. So real simple drill. Okay. So you set up an aim stick here. Shove it in the ground. Whatever you have to do. And I just all you're going to do is put it in front of your knee. And I want you to feel the difference in this move. Okay. Some of you that are older will remember Tom Wargo from the senior tour and he had every shot like this and I want you to look at my back foot down. I want you kind of doing this for a while feeling like this lead knee is staying inside or the trail knee is staying inside the lead. Okay. But this is going to give you the reinforcement here so that when I go up and I come down my left side start pushing down. Look how that knee works more like this. See it's in. And it also helps me. Now the lead leg is pushing back and I get that nice push back. Okay. So real real let me show you how how to do it. Just, you know, get it about an inch away or so. And we don't want to go fast because we want to learn to do the move um and feel really feel it. Okay. So if I'm here, make sure I'm on the left side. Boom. So see that just stays in here. Boom. Leave leg straighten. Work on this line stick. You'll you'll get really good at where you start hitting and then you can go full after you've recreated these steels and learned how your feet move on the ground and understand those ground reaction forces. Thanks again for watching this part two. Eric Schs golf sign</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+          <t>Hello and welcome to my channel. I'm Joy Fay and in this video today we're going to talk about a question that I'm asked regularly and that is what paint and my answer usually is well what inspires you to paint. What is it that you want to paint and then show you which is the key point of how to paint it? That's what we're going to cover in this video today. Just before we start, I'm just showing you these two paintings which which I got to last week in the video and over the week they've arrived here. Now, how did I go from there to here and that's what I'm going to show you. I've actually got another canvas the same size. So, I want to complete the series. So, um I'm going to sort of follow that theme. So for you, if you've got a sketchbook at hand, that would be great. Um because I'll take you step by step through the process. So you can go from your uh sketches on your um in your book, your sketchbook onto a canvas if you want to or onto another piece of paper. So you get the whole feel of the process of developing a painting. You know, they don't happen overnight. It takes time. You know, these have still got a lot that that needs to be done. Um, but I've got the the main part of it now. Um, and I'd love to share that with you of how you get to that stage where you feel really great and satisfied with your painting. So, let's dive in, start with our sketchbook and go from there. Now, when we say what inspires us to paint, we can look at it in two different ways. We can go and have a look at all the wonderful um things around us. We can look um you know in wonderful art books. We can look around our house. We can go outside. Um you know we can do so many different things to get inspiration. And obviously Pinterest is another one that's wonderful to look at. But your free drawing is something to really explore. You will have seen a lot of different things on YouTube probably talking about free drawing. But you know whether you like drawing circles or whether you like drawing squares or triangles, what you want to do is to feel what's good for you. You really want to make it mean something to you if you like. It's the outside in versus the inside out. We want to have a look what's going on inside. So you're very authentic with what you're doing. For me, I enjoy doing my um abstract figures. It's all about relationships to me. But that's where I am. How you approach it will be very different for you and you can approach it in so many different ways. And you know that's the beauty of it really. So um explore your drawing and once you you find these shapes that you like then start outlining them. So you you make them more uh you know stronger. You can do all kinds of things with them. Then um you know like I'm doing here outline some of them transfer that onto canvas and then you can be painting them or transfer it onto paper even paint into them. Do lots of different kind of experiments um to move into actually feeling confident about yourself and how you're expressing yourself on your um on your paintings on your paper and canvas. These are the drawings that I've done and I'm going to translate this onto my canvas uh which I'll show you. And I've got a brand new canvas here which is really exciting. So I'm looking forward to um getting um on with this. I'm going to be using a sponge and also a scraper. So here are the colors I'm going to be using. I've got a yellow ocra. I've got cadium orange, a Mars red, phthalo blue, and black and white. And I might drop in a little bit of the daylow orange because it's lovely. And I've got some uh magenta, which again just adds some extra uh pop to to a painting. And I've got them over here um in my palette ready to go. So, I'm putting the first um layers down just to get rid of the white and um activate the canvas and get it started. So, I'm going to do some layers with some okra and orange and uh see from there. So, now I have added some u molding paste for some extra texture. I could have done some more layers of paint. Uh but actually I thought, well, let's try this for a change. And um just any molding paste um would work on this. And uh let's see when it's dried and I put the painting the paint on. You know, you'll get some of these nice ridges that are in the in the paste coming through. So I've drawn my picture now onto the uh canvas and I've started now you know adding uh the colors that I want. And obviously these are first layers and it will slowly bring uh you know slowly build up as as you go. And I love all this because you you know you're creating um extra textures and a real kind of great foundation for your painting. And remember, you know, whatever you do, if you're not happy with it, you can &gt;&gt; [clears throat] &gt;&gt; um, you know, always paint over it. But it's really great to have these layers underneath um as you go because um it builds depth and it gives you something to play with and to work into. And you can see here on these close-ups, I've scraped into it, so I'm getting that color from underneath. And you can see I'm getting this texture from the molding paste. And it starts to have, you know, some body in it and some substance and energy. And, you know, that's what we're looking for. And you can really be brave and courageous with this cuz they're your first layers. You're building it up. You're getting connected to the painting. And it really starts then coming together and gives you such a great feeling. So, while I'm carrying on with the painting, I've got something really interesting to tell you about. Well, I'm very excited to tell you about my new free taster course, A Simple Way to Paint Abstracts with Confidence, which I'm launching very soon. And um I've just opened the weight list. So, if this is something that you feel you would really enjoy and get the benefit from, and if you love abstract painting, but you know, sometimes feel unsure of how to start or find yourself not finishing what you begin, then you're not alone. There's a lot of people who start many paintings and don't finish them. So, you might have tried different approaches, followed many different videos, or experimented, but still feel like you're guessing rather than painting with clarity and confidence. And this free taste course is here to gently change that. So, you can join the weight list and you'll be the first to experience a calmer, more confident way to approach your abstract painting. What you'll find inside is a simple way to start an abstract painting without overthinking. How to keep going even when you feel, you know, unsure and uncertain and a gentle process to help you finish your paintings in a way that feels right for you. And when you join, you'll also receive a free inspirational painting prompts guide. And this is um about making paintings feel easier and more natural and finally uh finishing what you start. So it's coming very soon. So if you join the wait list today uh you'll be one of the first to get access to this great free course. So I've put the link below. Click that link and you will get your free um your your free inspirational uh painting prompts guide. and I will keep you in the loop of when we're launching the actual course which is going to be very soon. Okay. Well, hopefully see you there. So, now coming back to the painting, I'm going to now start really bringing it together and increasing the layers and going through um you know the next uh interesting process. It's such a nice feeling to see your um lovely drawings, your free drawings that you did, you know, come to life on a on a painting. Let yourself just go with the flow and respond to what you see and uh you know, really enjoy it. Feel the freedom of it and, you know, have the courage to really explore all the different possibilities. So, we're at this stage now, and it's really beginning to take um shape. I'm getting um really now to refine it. I'm thinking of making some changes. I think I might put another orange circle in here, but I'm not sure. So, I'm going to sleep on it and see how I feel tomorrow. But you can see how you know slowly but surely this is over a couple of days how this um s you know suddenly comes to life and you can start you know getting different effects and building the layers and getting the feel of the painting and I'm getting a very interesting dynamic from it myself and um be interesting to know what you think um what what's it telling you? Perhaps you could write me in the comments what you feel the energies coming from this painting. And also um you know if you've enjoyed this whole tutorial uh please like and subscribe. Even if you're on the television, you can do that. I know a lot of you watch the YouTube videos on TV like I do, but you can still like and subscribe and that would be fantastic. So, I'm going to leave it for a little while and come back to it tomorrow and continue working on it and see, you know, how I'm going to finish uh the painting. And here we are. [laughter] I did put that circle in. I feel that it balanced it and added some other detail. And remember, you know, all the details come at the end and you need to give yourself a bit of time just to evaluate so you feel um good about it and you know to find where you feel it's right to finish. So here are the three together as the series and they tell an interesting story. I wonder what story it tells you. I'd be interested to hear. And uh I hope you've enjoyed watching this tutorial and don't forget to join our wait list for the new taster course coming up. And um enjoy doing your own series and I'll see you soon.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>So many good ideas. Subscribed... and look forward to learning more.😊 Ann, in Florida SUV solo camper || Thank you for subscribing, Ann! Welcome to the channel! 🎨✨ || You have several things going on in you painting that I like - complementary colours, dark vs light, round shapes vs squares&amp;rectangles. || Thank you so much, I'm glad you enjoyed those elements! 🎨✨</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>OJWTDx0nNy4</t>
+          <t>fcbP4AY5Jyo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Why You’re Not Compressing the Golf Ball — And How to Fix it with my Pressure Shift Drill!</t>
+          <t>How to Prepare and Paint Over a Canvas - Easy Acrylic Painting</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Most golfers are trying to compress the golf ball while staying stuck on their trail side. That does not work.
-In this video, I break down why pressure shift is one of the biggest missing pieces in the golf swing and why so many golfers never get to their lead side in time. That is why they hang back, lose shaft lean, lose rotation, and struggle to compress the golf ball.
-I go through the truth about pressure shift, why the old 80/20 advice got misread, and the exact drills I use in lessons to get golfers moving more like elite players. If you want better strike, more compression, and more distance, this is where it starts.
-Work on these drills and let me know what you feel.
-Get my free drills guide here:
-EJSGolf.com/my-drills
-Coach Erik Schjolberg
-The Science of Better Golf
-EJSGolf.com
-Scottsdale Golf Lessons
-Online Golf Lessons  
-#SGL #golfswing #EJSGolfAcademy #CoachErik #golftechnique #golftips #golfdrills #golflessons #stopcasting #stopscooping #shaftlean #onlinegolflessons  #ScottsdaleGolfLessons #golfswingmechanics #golfswinganalysis #golfimpact #golfpower #golfdistance #ejsgolf  #Titleist #Linksoul</t>
+          <t>⭐Join the Wait list for 'The Free Taster Course' The Simple Way to Paint Abstracts.
+ - https://www.joyfaheyclasses.com/free-taster-a-simple-way-to-paint-abstracts-with-confidence
+_______________________________________________________________________
+Have an old canvas you don’t know what to do with?
+In this video, I’ll show you how to paint over a canvas using acrylics, turning something you might have given up on into a fresh, expressive painting.
+This is a simple and freeing approach to abstract painting for beginners, especially if you feel stuck or unsure what to paint. Instead of starting from scratch, you’ll learn how to reuse a canvas, build layers, and let your intuition guide the process.
+Whether you’re:
+wondering what to paint
+looking for easy acrylic painting ideas
+or wanting to start painting again with confidence this method will help you begin without pressure.
+I’ll guide you step-by-step through:
+how to paint over an existing canvas
+how to create new shapes and layers
+how to use colour in a simple, intuitive way
+and how to let go of perfection and enjoy the process
+This is about making painting easy, relaxed, and enjoyable — no rules, just a gentle way to get started again.
+I share simple, easy-to-follow abstract painting tutorials to help you feel confident, find ideas, and start paintings you'll enjoy without overthinking. Great for beginners and more experienced art lovers alike. 
+Subscribe to paint along with me and enjoy the process.
+_______________________________________________________________________
+Want more step-by-step support and painting ideas? 
+🎨 Learn more about the Heart &amp; Soul Art Academy - to Start Your Free Month click
+https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout
+✨ Free Abstract Painting Tutorial -
+https://www.joyfaheyclasses.com/offers/zKznsbqH/checkout
+💝 Get a Solid Foundation  from start to finish in your abstracts paintings with "The Complete Abstract Painting Course" for just $27 Click - https://joyfahey.com/the-complete-abstract-art-painting-course/ 
+⭐Learn More about my 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+#AbstractAcrylicPaintingforBeginners #AcrylicAbstractArtTutorials. 
+#paintingforbeginners #intuitiveart #artinspiration
+#howtopaint</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-13T23:56:22Z</t>
+          <t>2026-03-26T17:00:57Z</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>858</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.00813</v>
+        <v>0.089744</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -702,65 +757,105 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Hi. Are you not getting pressure to your lead side? Are you stuck back something like this? Not getting the compression you want, not getting the shaft you want? I got great drills for you today. And we're going to be talking about pressure shift. getting like the tour pros who are like this at impacting 80 to 90% to their lead foot. What I see in my lessons is 80 and 90% on their back foot back here in transition and maybe 60% by the time they're at impact. Hi, I'm Eric Short with EJS Golf. Stick with me today. I got great drills for you today to get you to start to compress the ball, hitting it further and compressing it. Like I said, shaftling and rotation, they all go together, folks. All of them go together. So, welcome in to my bay here at Scottsdale, Arizona, McCormack Ranch. So, let's talk a bit about exactly what goes on in the golf swing and where these misconceptions have gone wrong. So, as I grew up, we heard about this 8020 shift. The problem was is the 8020 shift is happening all the way through to here. The shift should only happen to about here. Okay? Good players are only shifting pressure to right here. From here forward, there's no more shift going into this trail foot. It's starting to go over to this side. So, we're reentering back into the middle by this point. Okay? So, everything is going towards the lead side. Most golfers just continue to load, load, load, load, load, load, load, load, load. That's why this low and slow advice that we've heard in the past was so bad because what would what would that cause? It caused everybody to just to keep loading into this trail side. I'd rather see some speed to cause some breaking forces. Now, what's a breaking force? It's a force in this back leg that's going to stop me from going into it and get me to start going this way. Now, a key concept to understand about this is force precedes motion. Okay. Now, what happens is is lay viewers, they view video and they go, "Okay, I see this golfer moving." Now, the problem is is since force proceeds motion, they've been pushing way before you see them moving. Okay? So you have to assume if you see somebody moving this way, it happened way before since the force had to push there. It's not instantaneous. I go, "Okay, I'm here. Here it happens. I have to start pushing." So for a golfer to load here, they're starting to push right away to get over there. It doesn't happen at the top. And that's where everything's gotten confused. Okay? It's a way earlier move. So I want you to think about the maximum load is just to right here. And then we want to make sure we're getting into our lead foot massively by impact. Okay, so let's get into how we're gonna do this. And I'm not going to make this super long video where we get way into details because I have other ones where we can talk a ton about ground reaction forces and stuff like that, but I I want to get more into a couple of drills that are really kind of just going to help you with this. Okay? And this is one of my favorite ones to um feel this. I call the heel to heel toe stomp drill. Okay. So, how you're going to set up is this. This heel is going to be up. This toe is going to be up. So, lead toe up and the heel up on the back foot. Now, the way we start our back swing is this stops down with a lot of pressure and force. And then almost immediately we're pushing down into this lead foot. Okay? So, I go boom. So this is up boom boom. So you go it's working backwards. Okay. So I go heel to toe heel. So I'm towing this and then I slam this heel down here so I can get back into this heel over this lead foot. Okay. So heel is up on this lead foot and I'm kind of feeling the toe up a little bit in my shoe here. So I slam this down and I'm going slow here. And now I'm in the toe over here on my lead foot. Now I'm right away I'm picking that up and I'm picking that foot up and I'm now I'm slamming this heel down which is moving me over into this lead side. Okay, that's the heel toe stop and we can hit with this. Okay, so I start with my heel up and feel kind of the toe slam down. Boom. Boom. And you can already see just with me doing that. I wasn't even trying and the speed generation was just really incredible. Okay, so toe heel up feel kind of toes up and sometimes I think it's good just start this way. Boom boom boom. And I want to feel some speed with it. Okay. So, I'm quickly boom, boom. And the key is getting this back down quickly because if I'm slamming this down, I need to get back over to this lead side. So, I want to slam this front side down quickly as possible because this toe is coming up, which raises this heel up and boom. And then I can slam that down and gain a lot of speed. And you can hit with this. It's a great drill to hit with. Great. And and I want you just to focus on what the body is doing. Don't worry so much about the shot. Okay? But if I'm just here, I'm going here. Boom. I just absolutely ripped that thing. Okay. And I felt like I didn't even swing at it. Okay. So, heel toe stomp for that one. All right. Now, next one we're going to do is we're going to do kind of a a couple step step drills. And you can find a bunch of these on my uh on my YouTube page where you're at right now. So, and this is just getting the feeling of getting to that lead side and our body working in two ways at the same time. Because what it is like if when you're on your back foot here, it's like throwing a ball like this. You would never throw a baseball. If you were throwing a baseball, you would everything would be like this. Everything is forward in in in life that we do in any sport. We would never be like this that we do in golf from our back foot. Okay? So, I want you just get your feet together. Club goes like this. And when this club starts going back, we're going to step forward and go. Okay. So, what is this doing? This is moving our body in two ways at the same time. Okay. So, I'm going here and I step and go. All right. Now, this is another drill we can hit with. Now, I just want you to time this out. I want you to see how big your step is so that we get the step correct. I don't want you hitting it from way off the back. And I'm going to show you how we can do this. Again, I'm just going to test. My step is about right to here. Okay. Another great feeling again. Okay, now I'm going to show you one more version of this step drill that baseball players seem to love. I didn't play baseball growing up uh much. I obviously can swing a bat, but we're just going to go tap tap. Okay, so I'll show it from this end, too. So, if I start here, feet apart, tap tap. So, the key is here. I want to get this back here, but then I want to get this tapped right away. Now, the key is I don't want this center staying back and just like stepping this way. I want the center going with me like that. Okay? So, it'll be like this. Forward, step, boom. You're going to notice these are powerful moves that help you start compressing the golf ball and give you that feeling down to this rotation and down here like this, down here that you've been wanting for a long time. I hear it in my lessons all the time. It's what I change in lessons all the time. So, go through these drills, work on them, give me some feedback down below. Let me know what you think after doing some of these drills. Also, check out my drills guide, which are going to hit a whole host of other um issues that you have. My ejsgolf.com/my-drills. You'll see a link down below. But thanks for watching ejsgolf.com. And uh thanks for watching. Again, Eric Schwberg, the science of better golf.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>I thought today it might be interesting to kind of hang out in my studio. I've been looking at these two um old pictures which I've been hanging around for ages and I wanted to do something with them. I've given them a coat of gesso, which if you don't know, that's like a white primer, which kind of can, you know, really prepares the canvas for painting on and especially um, you know, if you want to paint over something, it gives you a nice foundation. So, just before we start, I'm just going to show you my palette. I've got a wet palette here. This is here. And this is just a little box that I put um some damp rag in underneath and then my pallet paper on the top and it keeps the acrylics from drying out too quickly. In actual fact, this palette has lasted already a week. So, it really does uh make a difference to you uh not wasting any of your acrylic paint. I've got a whole collection of um different brushes from thin ones to thick ones. I've got some pallet knives and a sponge, a roller. I sort of tend to have everything around me to use if that comes across that I want to do. [laughter] You know, have everything ready. So if the feeling moves you into it, then you've got the things there to to do. Now, let me come on to the actual picture. I hope you're going to be able to see it. All right. Here. Now, you know, most of you know, if you've seen any of my videos, I like to do some free drawing on the top. Um, how relevant it is to actually the picture, it it doesn't really matter. It just gets you in the zone. um connects you up and you know you can respond and feel where it wants to go. Now this is very much about um the process of really intuitive painting and allowing yourself to uh bring that up inside you. We don't know what might happen. It's unexpected and that's the exciting thing about it. whatever might happen, how it will evolve and that's all part of the wonderful process. And honestly, there's no right or wrong. You know, I get so many questions and comments about, you know, people saying, "I don't know what I'm doing. I don't know if it's right or wrong." Whatever you do is right for you. And if you allow yourself without overthinking it or thinking at all actually, then something inside you will come and be creative. So that's where we're heading. So when I'm looking at this, that's exactly what I'm doing. I'm just allowing a movement to um occur just to see where I might go with it. And you know, [snorts] I might enjoy some shapes with it. I might see how I feel about where those shapes are, but you know, you're never going to see this under the painting. And it's kind of very loose. Now, if you feel as if you can't loosen up here, go to your non-dominant hand because that's not in control. [laughter] So, you could You can do your shapes with that. It's an interesting little exercise to do anyway, but if you find yourself thinking, swap over and try it with the other hand and you know, your marks will be a little bit different. So, I'm going to go back to here. [snorts] So, that's my free drawing. Lovely scribbles and things. Now, some of them I might pick up in the painting, but some of them I probably won't. Now, I'm hoping that you'll be able to see this. Okay, it's quite difficult to get the Where are we? The the the angle right so you can see me painting on an easel. When it's on the table, it's a bit easier. Okay. So, I'm actually going to start with the sponge um and just dive in and see what happens. I'm going to go with I've got some uh pink and some day glow on here. And oh, that's lovely. So, I love using a sponge. It gives you a great covering and you can blend your colors together and it's very quick to, you know, get a really good foundation and uh easy to do. Uh the colors that I'm using I'll put in the description below. But you know you feel free to use the colors that you know you feel drawn to and um you know you can just enjoy this whole process. Um you know I use a sponge a lot and it's very freeing and easy to do particularly you know when you're first starting off. It's a It's a great a great thing to have and feel in the zone with. Okay. Well, that's the first layer of that one. Nice, you know, loose. Just giving me that feeling of moving into it and, you know, using some different colors. I'm not using a massive palette. I keep the the paints, you know, so they will harmonize. If you saw the the um video from last week, you'll know what I'm talking about is that we harmonize the colors by using a little bit of all of them in each in in each um color difference. So, I'm going to let that dry. And while that's drying, I'm going to move on to the next one. So, I'm going to do the same thing on this. I'm going to come and draw on it and then start the um the actual painting. So, I've speeded this up again because you've already seen this process with the other video. And are you enjoying this? Um, is it helpful for you? And if it is, it would be great if you would like and subscribe so you don't miss out on any of the other videos that I do. So you can see here I'm using a rag and um just making some different things with texture which is slightly different to I did last time and you know again just really enjoying the process and having fun with that creativity. Okay, well we've done the two first layers of both of the paintings and uh I'm going to come back to it when they're all dry. Okay. So, now the fun begins. I've got some charcoal and I'm going to uh draw into the paintings now. Um, obviously I did the drawing before, but now we're kind of getting into the body of it and I'm going to see what happens. So, let's go. Um, I love doing these uh drawings on top of a um a painting. You can do it in charcoal or paint or whatever you know feels right for you and whatever shapes that you like. And then just allowing yourself to you can go within the shapes or not. Use them as a guide or not. But you know like a little bit like we did underneath when we first started off. It just kind of keeps you um you know loose and in the zone. And you can see here I'm using my uh roller. This this is a wonderful way of uh blending colors together and getting you know spreading the color across the painting. You know it becomes a really kind of playful experiment rather than um trying to make something perfect. You know we're not looking for perfection. We're looking for, you know, what's going on inside as our our intuitive feeling about something. And if you're interested in exploring this more and going a little bit deeper, I've got something very special to share with you. So, I'm very excited to uh tell you about the new free taster course, a simple way to paint abstracts with confidence that I'm uh just launching. And if you would like to come on the wait list for this so you'd be the first to know about it when I do launch it, that would be fantastic. Um, and so you know, if you love painting abstracts, but sometimes you feel a bit unsure about how to start or find yourself not finishing uh what you begin like a lot of us, then you're not alone. Inside the um free taster, you will find um a simple way uh to start an abstract painting without overthinking, how to keep going even when you feel unsure, and a gentle process to help you finish your painting in a way that feels right to you. And uh when you join the uh list, the weight list, you will have a free inspirational paintings prompts guide um which is really helpful. It's about making paintings feel easier and more natural and finally finishing what you start. So it's coming soon. I'll put the link in the uh description below. So sign up and I will look forward to seeing you there. &gt;&gt; [clears throat] &gt;&gt; So coming back to the painting, you can see it's you know slowly developing and um you know it's creating a really great uh second layer to continue working on which obviously I will do and um you know see again where it would where it would take me. It's an ongoing process. You know it doesn't happen [clears throat] overnight. It can take a while. maybe, you know, a few days or a week I might leave it and then come back to it, but it's certainly been been enjoyable to um share this with you and go through this process. So, there's been quite a transformation on these pictures and if you're still here, thank you so much. Um I hope you've enjoyed this whole process. So, this was the first one. But obviously I still got a lot to do to it and um it's but it's full of color and energy which I'm really loving. And then I did a little bit more um on this one. Um you know I didn't want you to be here all day like me. Um but I've had a lovely time um working on them both. This is very different with I kind of structured some shapes differently. And I think that's the point is that you're free to do whatever takes you with any of the paintings. You know, give yourself permission to explore and discover new things. [snorts] So, if you've got any um comments, uh do ask me any questions. If there are any subjects that you'd like me to cover, I'm more than happy to do that. So, I'm going to leave these now. I'll come back to them. It's been great to spend this studio day with you and um please go away and have some fun with your own painting. Go from your sketchbook to a canvas. Have the courage [laughter] and I look forward to seeing you in the next video. Okay, all the best. Lots of love. Bye for now. [music]</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Thanks, Joy, I signed up for the Complimentary Taster &amp; downloaded the prompt guide🥰🙏🏽  I Trust that You're doing well, and am sending You Hugs from Canada🤗🧡 || Thank you for signing up, Great! And for the warm hugs all the way from Canada! 🤗🎨 || @JoyFaheyArtist ☺🌹 || Thanks Joy. Love your colors. ❤ Which tool did you use to scratch marks on the canvas? || Thanks for your comment I used the end of my brush and a pallet knife 🗡️🎨😊 || Fantastic Joy, thank you. When you said there is no right or wrong it made my week!
+(I'm self teaching, only about 8 months in).
+Your art is beautiful! || Thank you so much, I'm glad I could make your week! Happy painting! ❤️🎨</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6IIsc4TL71g</t>
+          <t>pfdcetb_C1U</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>🏌️‍♂️ Stop Pulling FIRST in TRANSITION and Start Rotating Through Impact with Shaft Lean an #shorts</t>
+          <t>Too Many Colours Ruining Your Abstract Painting? Try This”</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>🏌️♂️ Stop Pulling FIRST in TRANSITION and Start Rotating Through Impact with Shaft Lean and Compression 🧨
-⛳️ If your impact looks stuck, cramped, or stalled, this is one of my favorite fixes. I put an alignment stick under the trail armpit to teach the body what real delivery feels like. The goal is not to yank the handle down. The goal is to get to the lead side, push the pelvis back, and keep the trail arm connected long enough for the body to rotate through. This is how you start to become a ball striking machine nailing your low points.
-Try it slowly first, then tell me what changed in your strike.
-Coach Erik Schjolberg
-Scottsdale Golf Lessons
-Online Golf Lessons
-#golf #golfswing #golfdrill #impact #ballstriking #rotation #alignmentstick #golfcoach #ejsgolf #thescienceofbettergolf #golfinstruction #compressitgolfball #lowpointcontrol #scottsdalegolflessons #golftips</t>
+          <t>⭐Try the Heart &amp; Soul Art Academy FREE for a month - https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout
+_______________________________________________________________________
+What happens when you limit your colours to just three?
+In this abstract painting demonstration I explore the power of a limited colour palette and show how using only three colours can create harmony, simplify decision-making, and lead to surprising results.
+In this video I work with a simple palette and allow the painting to develop intuitively, showing how colour mixing, layering and experimentation can open up new creative possibilities.
+Working with fewer colours can help you:
+• create natural colour harmony
+• simplify your painting process
+• gain confidence in colour mixing
+• develop a more intuitive painting style
+This approach is perfect for artists who sometimes feel overwhelmed by too many colour choices.
+🎨 In this video you'll see:
+• how to start a painting with a limited palette
+• how colours mix and interact naturally
+• how simple colour choices can create depth and balance
+• how intuition plays a role in the creative process
+If you enjoy thoughtful, intuitive painting and exploring colour in a relaxed way, this video will give you new ideas to try in your own work.
+The 3 different colour pallets
+1️⃣ Ultramarine + Burnt Sienna + White
+This palette gives beautiful moody neutrals and soft blues, perfect for rivers, skies, misty  abstract landscapes.
+2️⃣ Magenta + Yellow Ochre + Blue
+Very interesting palette - produces unexpected greens, warm pinks and glowing neutrals.
+3️⃣ Rose  Magenta + Yellow Ochre + Primary Blue
+A classic limited palette that can create almost every colour which I use in this painting demonstration
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Gaudi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#paintingdemo #limitedpalette #abstractpainting #acrylicpainting
+#artprocess#AbstractAcrylicPainting. #AcrylicAbstractArtTutorials. #IntuitiveAbstractart.
+About - Abstract Painting in Acrylics tutorials and demonstration</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-09T18:04:37Z</t>
+          <t>2026-03-08T16:32:29Z</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1213</t>
+          <t>1253</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>159</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.012366</v>
+        <v>0.140463</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -769,67 +864,96 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Are you tired of having to look like this at impact? Okay, maybe not even hips rotate like that. You're more like this. I see it every day in lessons. Okay, I'm going to show you one of the great fixes I have for it. So, you take a lining stick. We're going to put it under our trail armpit. Okay? And then you're just going to take every like normal. Now, when you look from this end, you should see kind of that these these are nearly the same. It doesn't have to be exact, but kind of the same angle as the uh the um club. So, what we're going to do is we're going to swing up to here like left arm parallel. You see how it gets on my arm here. Okay. So, I want to make sure though when I start down, I'm on my left side here. This is still on my arm. Now, what I want to do first is get since I'm on my left side, the lower body goes out of the way. And I see how I'm keeping this on me. As I'm rotating, rotating, it's still on me. Still on me. And it's barely off. But look where I'm at. So, yes. Is this an extreme version of it? Yes. Right there. But yeah. So, left side, push back. Keep it on. Keep it on. Keep it on. So, look at that. Okay. Incredible. So, it's just a little aim strike drill under your pit. Do that a bunch of times in slow mo to get the feel and try to pick up what are you doing different. And you're going to notice it's some body movements, not this big pull down. Okay. Thanks for watching. Eric Silver, EJS Golf and the science of bettergolf.com. Leave a comment down below after you've tried this and let me know how it went. Thank you.</t>
+          <t>So today we're going to do something a bit different. I'm I've been inspired this week by some of the prompts that I've been doing in my um Heart and Soul Art Academy course. And one of them was um very much about how you feel about color. And that got me to thinking that um it would be interesting to have a look at different combinations of a limited palette. Now, I don't know if you're like me, but if somebody says, you know, do a limited palette, we tend to dive in to the same colors that we're familiar with, and it stops us kind of experimenting with other combinations. So today I'm going to show you some really beautiful different combinations that you might not have seen before. And I think you'll find it um inspiring and beautiful to see how your painting could come together with this kind of combination. So, let's dive in, have a look, and um hopefully you'll be able to experiment yourself using some of these color combinations. So, first of all, I'm going to show you three different um combinations. The first one is uh ultramarine blue, burnt sienna, and white. The second one is magenta, a yellow ocra, and ultramarine blue. And the third one is a magenta rose, a primary blue, and yellow ocra. Now, who would have thought of putting those together? The one that we're going to focus on today is this last one is the rose, primary blue, and yellow ocra. Now, I was playing around with this earlier so I could show you. And this is what I've done. Couple of things here to uh interest you. I've used a little bit of white as well, by the way. So, I put those colors up here, and then I'm mixing them. First of all, I mixed the primary blue and the magenta together. um and did it in different strengths cuz I really want you to experiment because the color combinations are so amazing. I could fill up two pages of this very easily, but I I wanted to just give you a small example of what you can get from these three colors and and white and how you probably wouldn't have even thought about putting yellow ocra with magenta together. I certainly it wasn't sort of top of my list but then when I started experimenting I thought wow this is really really beautiful. So we've got kind of these violets purples here we've got these peachy pinks here and then we've got these beautiful subtle greens here from the okra and the blue and I could go on and on and on. So that's we're going to do a picture using this kind of uh this combination. Now when I was practicing this and going through it, playing seeing what was what, every time I wanted to clean the brush, instead of cleaning the brush, I started to put together a painting which was sort of accidental really. I haven't finished it as you can see. But what I noticed was because I was just getting rid of the paint on my brush, I wasn't thinking about what I was doing. I was just kind of thinking, "Oh, this would be nice here and this would be nice here." And one of the most interesting things is when you do a palette like this, everything harmonizes because you're using those colors in the combination. So it holds together. And that's something that is, you know, you can think about for any of the paintings that you do that if you if you mixing those colors on your palette together, even if it's only a little, it harmonizes the whole picture. There's a lovely continuity in it. [snorts] and this sort of, you know, okay, it's just playing. That's what that's the whole purpose of the exercise is to play and see. But I've now I'm going to do a little bit of drawing and then use these colors on the painting. But if I carry on with this, I'll probably land up with quite an interesting little play painting with these beautiful colors. So, I wanted to uh show you that. Um, so let's get cracking with the uh picture uh using the colors. So I put them here on my palette and um we'll uh make a start. I'm using different things. I've got a sponge I might use. I've got some flat brushes. Uh I've got a roller. I've got a thicker brush somewhere. Uh where is it? There it is. And um I'll see how I go, you know, as we go. I'll I'll discover. So, you know, always when I start, and you will have seen this in many of the videos that I've done, and it's kind of one of the things that I'm passionate about, you could say. First of all, having an intention or having a prompt or having a question. So the question that I was doing within my course at the heart and soul was um what colors do I feel and what colors what colors do I feel and what shapes come to me and I had this kind of nice feeling to be able to have that intention. So, if you were just to take a breath before you started, [snorts] just kind of center yourself, take a breath. You're here at your art table, sitting down, standing up on an easel or wherever, and this is your special time. So, let's make the best of it. So, concentrate, take a deep breath, let yourself relax into it. What is your intention? Well, my intention here for this is to explore these beautiful new combinations of colors in a very um heartfelt way. That's how I'm feeling because I want to share it with you. So, you can take something away and go and have a wonderful experience with it. So when I feel that I just have kind of very soft um very soft drawing. There's nothing specific. It's just to relax me to get into into a zone where I can begin to paint. you know, you're never going to see this, but it's helping me um, you know, connect to the paper, connect to myself, connect to how I'm feeling, and hopefully connect to you [laughter] if you don't think I'm completely crackers, but it's a wonderful way to begin because you you get yourself into the right space. So, having having done that, um my feeling is to maybe cover this with a sponge with some of those colors just to give me um a start. So, I'm going to go with a little bit of the pink just to begin with. And again, I'm I'm just feeling into it. I'm not doing anything, you know, drastic. Um, loving that very pale, beautiful pink. Let's do a little bit more. And it's it's just covering the white paper up, which, you know, I know a lot of people don't like starting with white because what do you do with it? [laughter] Well, this this kind of helps you get started in a very easy, free, gentle way. Gets you connected to the paper. and starts you on this journey and you know to discover what these colors might do. Add a little bit of blue in here. And obviously the pink and the blue are going to go into those violets. But it just kind of starts me off with something um I can then respond to um as I move forward. So you can see it's kind of developing [snorts] in an interesting way and I'm just enjoying the flow that I'm getting from doing this with it and it's building up a layer. Um I'm using some watercolor paper. Um and I've obviously you can see I've taped it down. Um and it's in my sketchbook. So, uh, you know, it's part of, you know, my my time to see what I really enjoy, what I love doing. Now, you might decide not to start like that. You might start going straight in with some shapes and color, but for me, it's lovely to get a a base color to uh to begin with and let myself respond to it in a way that feels authentic to me. And I feel that that's important. Authenticity is a is an important aspect of this. But in order to be authentic, you you need to develop your confidence. And building your confidence in this way is is a great way to get to you. You know what you will do will be unique to you and it makes the enjoyment of painting so lovely. And you know when I work within my my my lovely membership group, my heart and soul, you know, we're doing interesting prompts like this all the time. And then it's wonderful to see how different everybody's paintings are and how how everybody responds to it. It's fascinating. So, we've got a nice first layer with um those colors. I'm going to let it dry and then I'm going to come back to it. So, now it's dry. I'm going to uh dive in with um some of these colors now. and mix and have some fun as we go. So when I, you know, when I feel about it, this has just given me um a really nice beginning. And I I love this combination of the uh lilac. And you can see we can have that color. Really, it's beautiful. I'm going to start off with some of that. And I'm going to kind of just play. I haven't got a a plan. I've got my intention. I'm going to see how it feels as I go and add these lovely colors. Um again, as we go, see what kind of takes me into um you know, differences and feel of it. You know, when you're doing this kind of thing, just playing, I want you to really kind of feel that you're you're having fun with it. It's not um it might turn out to be beautiful, but the the point of the exercise is to see all the beautiful colors that you can make as you as you experiment and see what happens. &gt;&gt; [snorts] &gt;&gt; Now I haven't got any black on here and it might be such that I put some black in later but I can get quite a dark gray. If you see this color now this is quite a dark gray. So maybe you know lovely bluey gray. Maybe this will be enough for our lights and our darks possibly. and to come down here. Now I am conscious even though I'm playing of of getting balance and um you know thinking about composition in a in a in a very loose way because you know you want the painting to have those lights and darks, those differences. You want the painting to have a focal point and you want it to, you know, pop. And as we go, we learn how that that will, you know, materialize. So, you know, at the moment, obviously, it's just the first layer and it's it's kind of interesting how those colors all blend, but you can see how they all work together. I'm just going to change brushes now to go um into the pink itself, which I love. And I'm going to put this in here. Um you know, it might not stay that way, but look how lovely it is when it goes over the blue. And this magenta is transparent, so I'm going to get what's underneath a little, which is lovely. And again, if I put it over here, I'll get a lovely tone of it. Can you see how beautiful that looks? Um, if I put it over across here, you know, it'll be more pure because I've got a lighter background. Um, and that's the interesting thing about using um transparent um colors as opposed to opaque colors. So, I like that. Um, and then I might just go right into this blue again and make that a little bit darker. Put a little bit of the ocra in it. So, it goes with quite sort of greeny, but it will work because I'm adding the colors that are already in the painting. It's not going to it's not going to clash with anything. See, that's kind of quite interesting, isn't it? the color there. How that's working. Let's come up here with some of that. Let's make it a bit more um yellow and put a little bit of uh let's put a little bit of white in it. Let's see what happens with that. Yeah, that's interesting, too. So, because we can combine all these colors together, we get these lovely differences, but they all are in harmony with each other. That's lovely, isn't it? Let's pop some over here just for balance. And you know, you can do these paintings really quite quickly um to, you know, see where they go to. Let's add a little bit of blue into that. So, we go a bit of a darker green, but uh it can go olive green if we add some white. Now, let's see what this is. That's lovely. That's quite a teal color. And um blends lovely. I love that color. Can you see how free I'm being? I'm not worrying about it. I'm just exploring what these colors might do. and slowly but surely it will come together with a bit of luck and a following wind. Um, another thing that I love doing is when I've got colors over like I did with that, in fact, I'm going to do it on here, is to take the excess paint off and rub it off on here. Then I'm not wasting the paint and clogging up the drains with lots of acrylic. Okay. So, we've got a nice basis happening. I'd like to go a little bit orangey. So, I'm going to use pink and the okra together. That's going to a little bit of white. That's going to give me this lovely color here. And it's obviously complimentary to the green, so that works really well. See how it all kind of blends together and gives a beautiful um effect. I'm going to use a little bit more of that down here. And maybe pop a bit of yellow in here, you know, to make it interesting. &gt;&gt; [laughter] [gasps] &gt;&gt; That's what we're looking for. We're looking for interest and you know how it will come together. I think I'm going to go very light blue over here. So, I've speeded this up a little bit because um it's a long video. Um I hope you're still with me. And if you are enjoying the video, it would be wonderful if you would um like and subscribe to my channel. You know, it's all free. [laughter] And um it really helps me share this to more people. And even if you're watching it on the television, you can you can do that. I watch most of my videos on the on the um television because it's a nice big screen and you can really see what's going on. But it would be great if you would uh like and uh subscribe. So you can see I'm making some progress on on the painting. you know, adding this lighter color, using my roller. You know, you you're free to experiment with whatever. Don't let anything hold you back. You know, this is your wonderful time in your zone uh enjoying the process. And you know, another thing that's so interesting about doing these little paintings that parts of them you might really love and parts of them you might not be so keen on. And you can always cut the bits out that you like and turn them into little cards. And I do that quite often. And um you know, it doesn't have to just sit in your sketchbook and do nothing. You can turn them into little cards which you can give people as as gifts. And um you know, it makes it all worthwhile. So you can see here I'm I'm I'm making some darker um color to emphasize the light. And again, it helps with the uh composition and those differences between lights and darks. That blue against the pinky peachy color is is lovely. So, you can see how this is coming together. And um I hope you've enjoyed the process and that you'll actually experiment this for yourself. Okay, I think we're done on this bit. I might draw into it, but what a lovely color combination. So, I'm going to take the tape off and let's see what it looks like once we've taken that off. So, there we are. I'll turn it round so you can see it from the way that I've painted it. It's come together really nicely. It's kind of got a sort of a little bit of a landscapy feel to it, hasn't it? And then, you know, when you look at the um the colors that we started with, it's beautiful to see how that can come together in um in a little painting. And you know, it was fun also to, as I showed you before, to have a little play piece. And all of the things we can do things with, you know, I could use that as collage. I could experiment with it on the top with some drawing. So, a lot of different things that you can do and [snorts] um you know, enjoy yourself and and have some fun with it. Now, I've been mentioning to you, you know, over the video about the Heart and Soul Art Academy. If you want to have a little look at it, um if you click the link below in the description, it describes everything that we do in there. So, you would have an idea of um all the things that go on in the academy. And it's wonderful. You can have the first month for free and then it's only $10 a month for the membership, which is fantastic because there are over I think there's 15 u master classes and the heart and soul course and the artist diary. There's loads of things going on. So go and check it out because it might be something that you know would be of interest to you. and and we do, you know, all the kinds of different things that we do from techniques and skills, learning all about color mixing and composition and intuitive painting, landscape, abstract landscapes, all kinds of things. So, I hope you've enjoyed and um you'll experiment with these different colors. So, do leave me a comment, tell me what you feel about these lovely colors. Be great to hear. And if you've enjoyed the process, um, that's great. So, I look forward to seeing you next time with something new and interesting to inspire you with your painting. So, lots of love and take care. See you soon. Bye for now.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>This performance is really helpful I did not expect it to be this good.</t>
+          <t>Thank you so very much for your wonderful tutorial sessions!  I am a new comer to abstract art making. I love seeing all of the different styles of painting. You have really inspired me to try it out! I really don’t think I have any artistic talents whatsoever, but I am still going to give it a good try 🤞 I really enjoy the way you teach. You take it slow and you explain things wonderfully. I am older so I like to take my time to learn all of the things I would need to know for the best possible experience. 
+Wish me luck because I will definitely need it. 
+My best to you,
+Judy || Welcome to the world of  abstract art, Judy! I am so happy I could inspire you to give it a try. Most importantly have fun! 🎨✨ || Can you let me know which Rose Magenta you use. I have scoured the Internet and can find Permanent Rose, Magenta, or Quin Magenta. |Are any of these close? Love your videos. || I used Amsterdam Rose 385. Different makes have different names however any pink/rose magenta will work well. 😊🎨🖌️ || Thank you for a very informative also visual tutorial, I will definitely be trying with different combinations ❤ || I can't wait to see what combinations you come up with! ❤️🎨 || High quality paint is expensive (Golden being my favorite) and my grandparents got married during the depression…. I don’t waste anything and always wipe the extra paint off my brush onto a paper or canvas- I call those my serendipity paintings. Sometimes they’re important starts for abstract work, and sometimes they just start filling in the canvas weave and I paint over them. || That's great! 🖌️🎨 || Your tutorial has given me inspiration to test this rose magenta as my primay red. It is not a colour that comes naturally to me, but your colour mixes was wonderful! || I’m so glad the magenta inspired you to try something new! 🎨✨ || I was stuck in a colour groove. So I went back to primary  colours, thinking about Picasso. || Going back to basics with primaries is such a great way to break through a rut! 🎨✨ || Tack Joy! jag verkligen njuter av att titta på dina videon och höra din vägledning i måleriet. Jag har gått genom din gratiskurs och bara den gav mig så många anledningar till att öva målningen så jag kan fortsätta med det ett bra tag till. Har sett att du har nu en kurs  Heart &amp; Soul Art Academy och Complete Abstract Painting Course
+och vet inte vilket jag ska välja och fortsätta måla med dig || Thanks for your commitment I'm happy you enjoy my videos. If you join the Heart and Soul Academy the Abstract course is in there too.! Plus you can have the first month for free. It would be great to welcome you there😊🎨 || @JoyFaheyArtist Tack så mycket för svaret. || Thank you for making this video. I find it very, very helpful. || Thanks so much 🙏 I'm so glad you found the tips helpful for your paintings! 😊🎨</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>-zXcHbCKESA</t>
+          <t>DC1Yrx9KPeo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>⛳️  Most Golfers Hit Behind It. This T Drill Fixes That. 🎯 #shorts</t>
+          <t>Turning a Loose Watercolour Into a Finished Abstract</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>⛳️  Most Golfers Hit Behind It. This T Drill Fixes That. 🎯
-If your contact is inconsistent, stop chasing random swing thoughts and start training low point.
-This T drill is one of the fastest ways and simplest ways to teach golfers how to move the strike forward, compress the ball, and finally get ball first then turf. I set the tee about 4 inches in front of the ball and the goal is simple: take it out with a short swing.  Be super aggressive towards the tee.  Crush it if you must! 💪
-That is how you start to build a ball-striking machine. 💥. Let's do it!
-playbettergolf #scottsdalegolflessons #ejsgolf #simturf #onform</t>
+          <t>⭐Go to https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout 
+To see what the Heart &amp; Soul Art Academy is all about! 
+_______________________________________________________________________
+In this video I show how I take a loose watercolour abstract painting and finish it using acrylic layers, adding depth, structure and clarity while keeping the freshness of the first marks.
+If you’ve ever wondered how to finish an abstract painting without overworking it, this step-by-step demonstration shows the whole process — from soft watercolour beginnings through to stronger acrylic shapes and colour harmony.
+You’ll see how to:
+• layer acrylic over watercolour
+• add depth and structure to an abstract painting
+• repeat colour to unify a composition
+• know when a painting is finished
+This is Part 2 of the series where we move from playful beginnings into a more resolved abstract painting.
+If you missed Part 1 Here's the Link - https://youtu.be/p8Qfzzpq2pM?si=H6nGfNTe-cEbCV9V
+And if you’d like ongoing support, deeper demonstrations and a gentle, encouraging community, check out the Heart &amp; Soul Academy. Try it out for a whole month for FREE and then it's only $10 per month! Amazing! Go to - https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout 
+Thank you for watching, and enjoy the process 🌿
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Gaudi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#AbstractPainting #AcrylicPainting #WatercolourPainting #PaintingProcess #AbstractPaintingTutorial #HowToMakeAcrylicPaintingsOnCanvas
+About - Abstract Painting in Acrylics tutorials and demonstration</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-08T18:03:31Z</t>
+          <t>2026-02-28T17:17:53Z</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>769</t>
+          <t>784</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>91</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.007802</v>
+        <v>0.131378</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -838,486 +962,682 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>This is the T drill to work on low point. Okay, so got a T here. We're going to lie it down on its side. Now, just so you see it here, it's going to be about four inches in front of the ball like right here. We're going to do it two different ways. We're going to start off heels together, toes apart. You can do toes apart or together if you want. We're going to do both here. So, I'm going heels together, toes kind of apart. And I just want to feel how do I take that tee out with a real short swing here. Okay, that's the main goal. How do I do this? Okay, so wasn't perfect connection on that. That's okay, though. Accomplished what I wanted. I got to the tea. Got my low point well forward. Now we're going to just do it with feet apart. Try the same thing. Okay, real short swing again. And our goal here is to take this PE out, which obviously I did. And how how do I know? Another way to check is my low point was 5.4A inches in front was my lowest point. Okay, so I really got forward. Most golfers have behind. Unfortunately, they're behind with their low point. We need to make sure we get in front so we're compressing this ball, getting the right spin, right distance. All right, thanks for watching.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>In last week's video, uh, we started with how to start a painting, which was great fun. And thank you so much. I've had such a brilliant response from it. It's wonderful. So many thanks for all your likes and your comments and your subscriptions. Tremendous. So, this week we're going to carry on with it. And I was promising that I was going to do some um acrylic over the top, which is what we're going to do. We actually started it if you obviously if you've seen it, we did it in watercolor and then did some pastels with it which was um you know an interesting process. So this week we're going to do some more to it. And I feel that you know it's important because we can start a painting often and then wonder what to do next. So this is the what to do next bit. So without further ado, let's get started. I've got my acrylic paints ready and uh we're going to have a play with the painting and it was this one. We'll start with this one first and if we've got time I'll go on to the second one. So, this was all done as as you know this was all done in watercolor and I did a little bit of pastel over the top of it. So, now we're going to see what happens if we put some acrylic over it. It's a wonderful thing when you're painting to experiment, to really connect with something creative inside you. And for me, this is what painting is all about. It helps me focus. It helps me balance myself up and, you know, get into that zone and all the cares of the world go away when I'm painting. So, I hope the same thing happens to you. Why don't you let me know in the comments? Tell me what happens to you when you start painting. Does it did you get into that zone? Do you feel like you're in your own world, in your own bubble? So, it would be great to hear, but let's get on with the painting. So, I've put my uh palette together here uh with the colors obviously that I've used. Um, I've got some different greens, olive green, vidian green, got some lovely teal, lemon yellow, um, some orange, and um, so that's where we're going to start. I've got a collection of different tools that I might use. I've got a flat brush. I've got one that's a little bit bigger, which is fun. I've got a couple of pallet knives, and I've got a a little roller. So, you know, dependent on what we might do. Um, I've got those at hand. So, I'm going to really, um, I'm going to start off with the flat brush. And, you know, looking at this, um, I I think it'd be nice to have a little bit of, uh, texture on it. So, um, when I'm looking at the colors, I'm I'm kind of going to go near the color. If it's not the same, it doesn't matter. But I feel that, you know, it would be nice to um do some uh texture on it. So, I speeded up the video a little because otherwise we'll be here all afternoon. And um you know, you can actually sort of see what I'm doing just watching um you know, layering this um acrylic on to give it some nice effects and um really just to strengthen the picture up, which is you know what the intention is, which is fantastic. And um you know, at the end you'll see what I actually do with this picture, which is quite amazing. So, you'll have to stick around [laughter] to um to see um what happens, which is great. So, you know, I hope that you know, this is inspiring you to really um explore different ways of painting. You know, starting with the watercolor, using some pastels, going with acrylic. There's so many different ways that you can do this. You don't have to just do it one way. And I think this is one of the challenges that um you know a lot of people tend to get into is that they try and you know do something over and over and over again um and then wonder why they're not getting anything different. So um I really when I started off the um heart and soul art academy um it's really to help and encourage um members to explore different mediums different approaches to see you know what really fits with you what do you resonate with and I think that's so important and in the heart and soul I have a lot of different master classes covering all kinds of different uh things from color mixing, composition, doing a series, collage, plus a whole, you know, a whole group of fabulous um intuitive prompts and ideas and examples to really expand your horizons on your painting to get the most from it, to enjoy it the most. Because, you know, that's why we're doing it, isn't it? We're doing it because it gives us a lot of pleasure and it's so relaxing. It's very healing. You know, for me, my painting uh particularly at the moment is very much a healing journey and you know to see what um comes up and that's one of the wonderful things. We don't know what's going to um arise when we start this kind of um this kind of work. And it's it's beautiful to see. So within the heart and soul um art academy, we capitalize on this to help you and give you um some really fantastic prompts and ideas and inspiration to expand your horizons. And I've now put up a video which is explaining everything that's in there and you can do the first month for free to come and see if it's a good fit. You know, you've got nothing to lose, everything to gain and to see if it's something that, you know, you could really benefit from and uh so it's worthwhile going to have a look and having a play around with it. So, back to this uh painting. You can see that I'm adding um a lot more depth and color with the acrylic and getting some lovely textures and um ideas for uh you know, focal points up here with the red. Um you know, your eye can't help but go there. And obviously the two darker points here with the darker blue green. Um, so the idea is for the eye to stay within the painting to read the story. And it's interesting to know, you know, when you look at it, what you get from the painting, what what's your feeling about it. So let me know in the comments because it's always interesting, you know, could it be a landscape? Is it just shapes to you? Tell me what you feel. Um because everybody sees it differently and I think that's really um magical. [snorts] So, I've really enjoyed doing um doing this in two parts, you know, with the watercolor and then with the acrylic. And it's been a really enjoyable experience for me. So, now I'm I'm going to add some finishing touches. It's all dry. Um I've got a few um Stabillo crayons here, which I might use. And I've got um two black um this one is a Sharpie and this one is a uh fine nib uh MP pen. So I just want to um do a few of the finishing touches. So it's it's all done. So I've gone over, you know, this painting um with, you know, with the acrylic. So, it's actually quite nice to add in some detail. You know, all the detail always comes, you know, later. You don't want to be doing detail right at the beginning. Um, you know, as it changes, you can do add things as you go. I'm not going to do very much, but I kind of feel that there's a, you know, a few things that um I can add, which again adds some interest. And uh what we're looking at is, as we mentioned before, the composition, you know, where is the eye going and are you staying within the picture? So doing these little extras, you know, helps that on its way. So, um just adding a few different uh marks in here just to define some edges. You know, there's not very much, but again, it it draws you in and it helps with um you know, to help you move around the picture. And the bit that I'm not massively happy with is this. And I'm going to just do some scribble over here just to make it more obvious and add a bit of interest to it. You know, it's wonderful to just do a little bit of playing when you're um you know, when you're at this stage. It it helps to just add some fun things, make it really pop, [laughter] which is what we want to do, and um add some extra interest. Let's come over here a little. Add some black here. Okay, I think we could say that that was now finished. So, I'm very happy with how that's turned out and um I hope you've enjoyed watching it. Again, you know, you can say how you feel about this process. Do you know give me some feedback in the comments which would be fantastic. And now it's quite good to have a look at the comparison. This is what it was in the watercolor and now here it is with the acrylic. So you can see there's quite a difference. And now you see if I turn it around the other way, it looks different again. And it's always worth doing this with your paintings, you know, looking at them from different angles and seeing how it looks. And here's one um, [clears throat] you know, horizontally again. and it looks very different. And then I've put this in a print. And I think this is something that you can consider with the paintings that you like that you can um you know put them into prints. You can have them at any different sizes and um you can really change it up. So, if you take one of your paintings that you really like, that you've done in your sketchbook, if you take a good photograph of it, you can put it in a print and uh you can make it all different sizes, which is brilliant. So, as we've done quite a lot already in this video, I'm going to save the next one for the next video coming up. And because I think there's been quite a lot to absorb and take in. And if you'd like to like and subscribe, that would be fantastic. And then you'd be lined up to watch the video when it comes out. And don't forget the link in in the description for the heart and soul. And I look forward to seeing you next time. Thanks for watching. Take care. Lots of love. Bye for now.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>@simplyjanet Joining Heart and Soul was one of the best gifts to myself. Great to get some really positive feedback Thanks Janet! - Could it be your special gift to yourself too? Check it out at https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout || Thank you before start watching videos ❤❤❤❤ || Thank you for watching! I hope you enjoy the process. ❤️🎨 || The painting really came alive and got depth when you added the acrylic. || I’m so glad you enjoyed that layering process and how the depth came together! ✨🎨 || Am enjoying your videos very much. Your painting feels like a big toppling, we haven’t crashed yet but things are teetering. You are inspiring indeed. 🩵💙 || Thank you so much, I love that description of the painting process! 🎨💙 || Fascinating to watch and a stunningly beautiful outcome Joy!  I can sense the catharsis happening.  Thanks for sharing your process.  Wishing you all the best on your healing journey, and the motivation and energy to continue to create beautiful gifts to the world. ❤❤❤ || Thank you so much for your lovely comment and for wishing me well on my journey! ❤️🎨 || Hi Joy, new sub who just found your channel today and am enjoying your videos tremendously! I was so sorry to hear you had such a difficult year last year, art too is my therapy 😊 
+I'm a beginner with no formal understanding at all. I am enjoying this mini series immensely, but could I ask why in this two parter you taped the watercolour paper down? I've heard of taping it to a board etc so as it dries it doesn't warp, but you did it in your watercolour paper book, is it the same principle?
+Many thanks and best wishes 😊 || Welcome to the channel, and thank you! Yes, taping it down in the book helps prevent warping while it dries. 😊🎨 || What u mean by Let's finish this with Exclamation Mark? I suppose u are a perverted zio.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>fPv9OkVg_Xg</t>
+          <t>p8Qfzzpq2pM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>⛳️. Swing Plane Perfector: Fix Low Point AND Swing Path at the Same Time 🧨 #shorts</t>
+          <t>2 Simple Ways of Starting an Abstract Painting and Finding Your Creative Compass</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>⛳️. Swing Plane Perfector: Fix Low Point AND Swing Path at the Same Time 🧨
-🏌️ Most golfers I see have one major problem — their low point is behind the golf ball. That means no compression, no forward shaft lean, and no consistency. In this video, I show you a different way to use the Swing Plane Perfector that I haven't seen anyone else teach — fixing your low point AND your swing path at the same time. Kill two birds with one stone.
-This is how I train golfers at EJS Golf in Scottsdale, Arizona — using real cause-and-effect coaching, not band-aids.
-🔗 Get a Swing Plane Perfector with a discount code: EJSGolf.com/gear
-🔗 Grab my free drills guide: EJSGolf.com/my-drills
-🔗 Learn more about The Science of Better Golf: EJSGolf.com
-🔗 Read the blog: EJSGolf.com/blog
-📍 In-person lessons: McCormick Ranch Golf Club, Scottsdale, AZ
-🌐 Online coaching available worldwide
-#golf #golfswing #golftips #golflesson #ballstriking #swingplaneperfector #lowpoint #ejsgolf</t>
+          <t>⭐Here's Your Heart &amp; Soul Art Academy1 Month FREE Trial https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout
+Do you ever sit down to paint and feel completely stuck, unsure where to start, or worried you’ll do it “wrong”? In this video I share a gentle, practical way to start an abstract painting using what I call a Creative Compass, a simple method to help you feel confident, choose colours you love, and begin painting without overwhelm.
+This step-by-step abstract art tutorial is suitable for beginners and returning artists, and works in watercolour or acrylic painting. It’s especially helpful if you’re looking to rebuild creative confidence, find your personal style, or simply enjoy painting again.
+In this lesson we explore:
+• how to start an abstract painting
+• overcoming fear of the blank page
+• building creative confidence
+• choosing colours and shapes you love
+• small painting exercises for beginners
+• finding your artistic voice later in life
+If you enjoy this calm, supportive way of learning, you’re very welcome to try a free month inside the Heart &amp; Soul Art Academy, where we paint together each month with gentle guidance, masterclasses, prompts, and a friendly art community.
+👉 Join here: https://www.joyfaheyclasses.com/offers/w4Grz46J/checkout
+This channel is for anyone who wants to paint with more joy, confidence, and freedom, especially women returning to art after a long break or a difficult time.
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Gaudi Gallery Madrid. and selling a painting to an Arabian Princess! 
+🌼 Chapters 
+00:00 How to start an abstract painting
+02:30 Finding your Creative Compass
+08:00 First watercolour demonstration
+18:00 Painting through doubt
+28:00 Second demo &amp; next steps
+36:00 How paintings develop over time
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#AbstractPainting #WatercolourTutorial #AcrylicPainting #HowToStartPainting #BeginnerPainting #CreativeConfidence #artforbeginners  #AbstractArtTutorial #PaintingForRelaxation #ArtAfter50
+About - Abstract Painting in Acrylics &amp; Watercolour tutorials and demonstration</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-02T19:03:59Z</t>
+          <t>2026-02-21T17:34:31Z</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>949</t>
+          <t>2037</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>169</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.001054</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+        <v>0.097202</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Joining HeartandSoul was one of the best gifts to myself. || I'm so happy to hear that, what a lovely gift to yourself! 😊🎨 || I love the idea of looking at my scarves for inspiration! Thank you! I really needed that.❤ || I'm so glad that tip was helpful for your creative process! ❤️🎨 || Thank you so much Joy! Your videos are very inspiring and I really like your way of showing and explaining. I find it very difficult to start painting, and I had never thought about starting with watercolors. It's like you gave me the right key. || Thank you, I'm so glad I could help you find the key to starting! 🎨🔑 || This is so inspiring, Joy. I love how you took a seemingly simple scarf and used it to reimagine the shapes and colours. I'm really enjoying the Heart &amp; Soul Academy too - it's such a safe space to share and learn. Thank you!🙏 || So happy you are enjoying the Academy and finding inspiration in the process! 😊🎨 || This is the first time I’ve seen your channel. I appreciate what you have to say, but four minutes in and I’m curious why the camera keeps bobbing back and forth. It’s distracting and dizzying. But I will try to watch it through and hope that it doesn’t continue throughout the video. Thank you. || I’m so sorry the camera movement was distracting, I’ll work on keeping it steadier next time! 🎥🎨 || Ive missed you Joy. Im happy to see you back. || Ah thanks, I missed you too, so happy to be back sharing art with you again! 😊🎨 || Who keeps moving the camera!!! Stop it! || I’m so sorry for the camera movement, I will work on keeping it steadier next time! 🎥🎨 || I've just started in the Heart and Soul Circle, and I am finding real value in it. I can share my processes without worry and get some clear feedback. || Thanks so much Rose and I'm so happy you're enjoying the Heart and Soul Art Academy, I love how it's growing and gathering so many wonderful like minded folks who share their love of art 🎨🖌️😘 || Thank you ⚘️ I think this will help a lot. || You are so welcome, I'm glad it will help! 😊🎨 || Thank you for a watercolor exploration || Glad you enjoyed the exploration! 🎨✨ || Thank you Joy, I always come back to your videos. I love your soft, gentle approach. I'm definitely going to try this as I feel attracted to abstract painting like yours, but I'm very unsure. || So happy you find my approach gentle and helpful for starting abstract painting! 😊🎨 || Thanks for sharing your clever methods to find inspiration, we all get blocked now and then || So glad you found the methods helpful for getting unblocked! 😊🎨 || Thank you Joy, you have inspired me to experiment with the watercolour and oil pastel combination. || That's a wonderful combination to explore! 😊🎨 || I enjoyed watching you make the watercolour abstract paintings! I also sometimes use watercolours as a starting point for paintplaying. I love to let the watercolours bleed and create surprises during drying. I then go over with acrylics and finalize the sketch. || I love that approach, letting the watercolors lead the way is so fun! 😊🎨 || “What colour feels like home to you? I’d love to hear what your Creative Compass might be this week.”</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>69zdsNCQG30</t>
+          <t>Cdly8AaqkQo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>🔥 Stop Flipping the Club! This Simple Drill Forces Body Rotation Through Impact ⛳ #shorts</t>
+          <t>The Messy Middle - How to Finish an Abstract Painting Without Forcing It</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🔥 Stop Flipping the Club! This Simple Drill Forces Body Rotation Through Impact ⛳
-🏌🏿♂️ Are you all arms through impact? If you're flipping the club and never rotating through the ball, this drill is for you.
-HI. I'm coach Erik Schjolberg, founder of EJS Golf in Scottsdale, Arizona. In this video, I show you a simple silicon band drill that forces your body to rotate through impact instead of relying on your hands and the small muscles. When you rotate correctly, you move your low point forward, deliver the club with forward shaft lean, and produce controllable spin with a predictable launch angle. This is how you become a great chipper.
-This is not a swing thought. This is a constraint that makes your body do the right thing. You should feel improvement on the first rep 💥
-Get my FREE DRILLS guide at EJSGolf.com/my-drills
-🏌️ Work with me in person in Scottsdale, AZ at McCormick Ranch Golf Club or online:
-👉 https://EJSGolf.com
-👉 Learn more about me: https://EJSGolf.com/about
-👉 Get my drills guide: https://EJSGolf.com/my-drills
-👉 Read the blog: https://EJSGolf.com/blog
-#GolfDrill #BodyRotation #StopFlipping #BallStriking #ForwardShaftLean #LowPointControl #GolfInstruction #ScottsdaleGolf #EJSGolf #TheScienceOfBetterGolf #GolfTips</t>
+          <t>⭐Here's Your  Free Abstract Painting Tutorial - https://www.joyfaheyclasses.com/offers/zKznsbqH/checkout
+Have you ever started a painting feeling free and inspired… only to reach a point where it feels messy, uncertain, and you’re not sure what to do next?
+That “messy middle” stage is one of the most important parts of the abstract painting process and often the most uncomfortable.
+In this video, I share 6 things to notice when your painting feels unfinished, so you can move through that stage with more clarity and confidence instead of abandoning it or overworking it.
+If you’d like to see this entire process demonstrated step by step — from playful beginning, through the uncertain middle, to a more resolved painting,  I’ve created a free abstract painting tutorial where I guide you through each stage in real time.
+You’re very welcome to explore it here:
+👉 https://www.joyfaheyclasses.com/offers/zKznsbqH/checkout
+🔥 Don’t forget to like, comment, and subscribe for more creative inspiration!
+Perfect for beginners and intermediate artists looking to enhance their abstract painting skills. Whether you're working with acrylics, or mixed media, these principles will transform your creative process.
+🔥Discover my HEART &amp; SOUL Art Academy - FREE Week Trial to explore it all! Go To - https://www.joyfaheyclasses.com/offers/7LTV2GNo/checkout
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️See My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Gaudi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#PaintingProcess #arttipsandtricks #creativeconfidence  #abstractacrylicpaintingtechniques . #acrylicabstractarttutorials . #IntuitiveAbstractart.
+About - Abstract Painting in Acrylics, Abstract tutorials and Acrylic demonstrations</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-02-26T16:32:05Z</t>
+          <t>2026-02-14T16:17:04Z</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>548</t>
+          <t>640</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>77</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.009124</v>
+        <v>0.142187</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>The content is amazing I will come back to watch it again. || Get my FREE DRILLS guide at EJSGolf.com/my-drills</t>
+          <t>That's an interesting idea about interpreting the 'stuck' feeling as the time between freedom and structure. 😊 || Exactly, it's all about finding that balance without forcing it! 😊🎨 || Very informative Joy, thank you, I really needed this x || I'm so happy you found it informative and helpful! 😊🎨 || As usual, I can't seem to do anything right. It always tells me, invalid password. But yes, this is exactly where I'm at, 2 and 1/2 yrs later. || Hi Diane not sure I understand please feel free to email me at joyfaheyart@gmail.com  and I'm happy to help 😊 || Im so happy to see you again Joy. This is prob exactly what i need to see. || I'm so happy to hear that! 😊🎨 || a very insightful talk. Thanks!
+It sure resonated with me. || So happy it resonated with you! 😊🎨 || Great video with really helpful advice, the middle bit is always tricky!  I´ve signed up for the course and I think the Heart &amp; Soul Art Academy looks very interesting so I will definitely do the free trial for that too. Many thanks, D || So happy you found the advice helpful and signed up for the course! 😊🎨 || I love the work behind you Joy, especially the figurative one over your shoulder. || Thanks so much, I'm happy you like the paintings! 😊🎨</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>bRzUXlu5ILA</t>
+          <t>qAsqukJc11c</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>INSTANT Low Point Fix (Yoga Wedge Drill) | Stop Chunking Irons + Compress It</t>
+          <t>Seeing Colour Differently - Abstract Painting Inspiration from Nature &amp; Light</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Most golfers don’t need another “swing tip.” They need low point control. In this video I show you my favorite cheap training aid: a simple foam yoga wedge that trains a descending angle of attack and a low point in front of the ball—exactly how you create compression and stop hitting behind it.
-How to use it: place the wedge just ahead of the ball, make small swings, rotate through impact, and finish without flipping/scooping. I like the feel of my trail wrist staying extended in the finish because it confirms my body delivered the strike instead of my hands saving it.
-Want my full drill library and practice plan? Get my FREE Drills Guide at EJSGolf.com/my-drills.
-Coach Erik Schjolberg
-The Science of Better Golf
-#golf #golftips #golfdrills #ballstriking #compression #ironplay #lowpoint #impact #scottsdalegolf #ejsgolf</t>
+          <t>⭐Join The Heart &amp; Soul Art Circle for Free,  Create a New Vision for Your Painting - if you’d like to explore further, check it out at
+https://www.joyfaheyclasses.com/offers/7LTV2GNo/checkout
+⭐I filmed this video at Abbotsbury Tropical Gardens, Dorset, UK during one of their illumination evenings — an immersive experience of light, colour, and atmosphere. Walking through the gardens felt like stepping inside a living painting.
+As an abstract painter, I’m continually inspired by colour relationships, shifting light, and the emotional response they evoke. Rather than copying what I see, I allow these moments to inform my painting intuitively — letting colour, feeling, and movement lead the way.
+This way of working forms the foundation of my Heart &amp; Soul Art Circle, where I explore intuitive, colour-led abstract painting rooted in connection rather than rules. If this video resonates with you, the Art Circle is currently open to try free for seven days. You’ll find a link below  gently and in your own time.
+For now, enjoy this magnificent world of nature, light, and colour.
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering  'A New Vision for Your Art and a Creative Sanctuary if You are Ready to Paint from the Heart' with the Heart &amp; Soul Art Circle which also incudes 14  Masterclasses and the Artist Diary 
+  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Gaudi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+To see more of Abbotsbury Tropical Garden - https://www.youtube.com/@livinginweymouth
+#AbstractAcrylicPainting. #AcrylicAbstractArtTutorials. #IntuitiveAbstractart. #abstract painting #inspiration  #colour inspiration, #abstract art #intuitive painting #nature and colour #light and colour, #women artists #creative inspiration
+About - Intuitive Abstract Painting in Acrylics tutorials and demonstrations</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-02-17T17:13:16Z</t>
+          <t>2026-01-01T16:01:15Z</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>515</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+        <v>0.087379</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Jardín Botánico La Concepción! Jag var inte där på vintern och såg dessa fina belysningar, men det är en park att beundra när man väl kommer || It truly is an amazing place to admire no matter the season! 🌿🎨 || WOW! Thank you Joy, for sharing that.  What an amazing sight for an artist's eyes. || So happy you enjoyed the inspiration from nature! 🎨✨ || Hi Joy! I'm so happy you were able to experience that. The first part of the garden really looks abstract.  So beautiful.  Thanks for sharing this with us.  ✌️ || Thanks so much for your kind words! Happy you found the garden beautiful. 🙏😊</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>qVSu1aAhowo</t>
+          <t>s9DBjNkmQFg</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Stop Chunking | Blading Chips and add Spin Today:   Simple Techniques that Anyone Can Do!</t>
+          <t>Art Therapy in Real Life - How Creativity Helped Me Heal After Loss</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>If your chips feel random—one checks, one releases, one gets bladed—that’s not “touch.” That’s missing impact conditions. In this video I walk you through my chipping procedures that make the strike measurable and repeatable: ball first, turf second, with a PREDICTABLE amount of spin so you can actually trust what happens when it lands.
-Here’s the foundation. I build a stock chip shot that covers roughly 85–90% of what you’ll face around the green. Feet closer together, shoulders level (most golfers “get left” by shoving left and popping the lead shoulder up—don’t do that), lead foot flared to make rotation easier, and a descending strike. Then I show you the #1 DEADLY SIN that wrecks contact:
-I show you how I create spin without getting wristy or feel like you have to drive the ball into the ground.  With a wide, pivot-driven swing,  I can change distance by changing pivot speed—not by flipping my hands. I also teach the “float” action: the club head doesn’t dive down immediately. Finish matters too. I hold the finish because it tells the truth—face the target, handle pointing back at you, club face staying semi - open unless you’re intentionally running it.
-If you want this measured with TrackMan (dynamic loft + attack angle = the spin/launch window you’re actually delivering), book a session with me and I’ll build your stock chip around your clubs and your matchups.
-To find out how to book a lesson with me in Scottsdale, AZ at McCormick Ranch or online, go to my website, EJSGolf.com.  
-If you want me to cover the “runner” version (how I intentionally close the face to launch lower and release), comment “RUNNER” and I’ll film it for you.
-YouTube tags (comma-separated)
-Coach Erik Schjolberg
-The Science of Better Golf
-EJSGolf.com
-Scottsdale Golf Lessons
-Online Golf Lessons  
-#Golf #Chipping #ShortGame #BallStriking #EJSGolf</t>
+          <t>⭐The Heart &amp; Soul Art Circle - Now you can join for FREE for a month and then only $10 per month Click the Link to Learn More -  https://www.joyfaheyclasses.com/offers/7LTV2GNo/checkout
+____________________________________________________________
+After eight months away from YouTube, I’m finally returning — and today I’m sharing the truth behind why I stepped back, how creativity, painting in watercolour and acrylics  helped me heal after profound loss, and the new vision that has grown from that journey.
+In this video, I open up about how using art as a therapy became a source of grounding, expression, and emotional release when life changed in ways I never expected. Painting  and art therapy — whether abstract, intuitive, with watercolours or acrylics — became a place where I could breathe again, feel again, and gently rebuild my inner world one brushstroke at a time.
+This experience led me to create something deeply meaningful:
+✨ The Heart &amp; Soul Art Circle — a creative sanctuary for anyone ready to paint from emotion, rediscover themselves through art, and explore a new approach to creativity.
+Inside the Circle, you’ll find monthly Heart &amp; Soul lessons, creative downloads, a full library of masterclasses, the Artist’s Diary, and a warm community of like-minded artists. It’s a space for healing, discovery, and reconnecting with your artistic voice — especially after life changes.
+Whether you're exploring abstract art, intuitive painting, creative healing, emotional expression, watercolours, acrylics, or just want to reconnect with your creative spirit… you’re in the right place.
+✨ Join the Heart &amp; Soul Art Circle for FREE here:
+ https://www.joyfaheyclasses.com/offers/7LTV2GNo/checkout
+Thank you for being here. I’m so grateful to walk this new chapter with you.
+Let’s paint from the heart — and rediscover our spark together. 💛
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the the Heart&amp; Soul Art Circle .  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Gaudi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational intuitive Soulful Painting Tutorials
+Thanks for watching 💝
+#AbstractAcrylicPainting. #arttherapyideas  #AcrylicAbstractArtTutorials. #IntuitiveAbstractart. #watercolours #griefjourney</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-01-30T20:29:34Z</t>
+          <t>2025-11-23T18:04:22Z</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>261</t>
+          <t>857</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>117</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.003831</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
+        <v>0.183197</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Thank you so much for watching 💛
+If this message resonates with you — whether you’re exploring abstract art, intuitive painting, watercolours, acrylics, creative healing, or simply looking for a fresh start — I’d love to welcome you into the Heart &amp; Soul Art Circle.
+✨ Join here - https://www.joyfaheyclasses.com/offers/7LTV2GNo/checkout || So sorry for your loss Joy,  your courage is amazing,  you were missed. Your spirit is strong and its wonderful that 
+You are back sharing your gift in art.  God bless you. || Thank you for your incredibly kind words and support during this time. ❤️🎨 || Hej Joy! Jag är väldigt ledsen och delar din sorg över förlusten av din älskade son. Jag fick meddelande från din vän när det hände och tänkte på dig mycket. Ingen kan föreställa sig vilken smärta en sådan förlust är. Jag önskar att följa med dig på min resa genom målande. Tack! || Thanks for your kind words Hannah, my painting and my Heart and Soul Academy helps me tremendously and gives me so much support. I go one day at a time and slowly finding my new life. I really appreciate your heart felt message 🙏 ❤️🎨 || I am very sorry for the loss of your son and sending you best wishes during your healing journey!  Very happy to see you back on YT. || Thank you so much for your kindness and for welcoming me back! ❤️🎨 || Thanks for sharing your story, Joy, and for setting up the Heart and Soul Circle which I'm really enjoying. 💖 || So happy to hear you are enjoying the Circle and finding comfort in it! 💖🎨 || We are members of a terrible and fierce sorority, Joy. I lost my daughter at age 20, a little over 15 years ago. My heart goes out to yours. We owe it to those precious ones to shine brightly for the love they gave to us. || Thanks so much for sharing and your understanding, and my heart goes out to you too. And yes I dedicate my work to my son and thankfully have painting to share love and healing. Bless you ❤ || My deepest sympathy, Joy! I lost 2 very good friends last year, and then my brother in November. Painting helped me through the dark parts, I think the Heart and Soul Art Circle is a very good idea, so I may see you there. || Thanks so much for sharing your experience, so sorry to hear of your losses. Painting can be so healing 🙏🎨 || Hi! I’m so sorry for your loss! May your heart heal.
+I so much wanto join this circle. However, I’m an absolute beginner. I know nothing about abstract painting. The only thing I have is a strong desire to learn this. Will you teach us how to paint step by step? I so much wanto be able to create beautiful abstract paintings. || I'm so pleased you're interested in joining and I do teach step-by-step! There's everything you'll need to start your exciting painting journey. It would be lovely to see you there! 😃🎨🖌️ || @JoyFaheyArtist
+How many hours a week will I need to invest? || Thank you for being so transparent. You help me to realize all that I’ve been through in the past 2 years. I’ve begun to paint, for the first time in my life, after my loss and I’m beginning to realize, with your help, how transformative &amp; healing this journey has been. I’m so sorry for your loss and so thankful for your courage. God bless you and all you do. Thank you - I’m so grateful i found you. || Thanks so much for your beautiful comment, I'm so pleased painting is helping you too! 🙏🎨🖌️ || Joy, like so many I am so sorry to hear of your loss.  I cannot imagine the internal processing you are dealing with.  Creating this safe space is a testament to who you are as an artist and how you leverage your creativity in the most positive ways.  Please continue to be kind to yourself as you move forward.  ❤❤❤ || Thanks so much Paul for your kind comment I really appreciate it. Having something to focus on is helping me to process what has happened. One day at a time! 🙏😊 || 😥💔❤❤❤ || I'm so deeply sorry for the loss of your dear son Joy. I don't think there is a more devastating loss to move on from. May art continue to nurture your heart and soul. || Thanks so much for your lovely message and thank God for painting 🎨🖌️😊 || My deepest condolences for the passing of your son.  My father passed away 4 months ago and painting has helped me so much. || Thanks for your kind message and sorry for your loss also. Yes painting certainly helps with the grieving process doesn't it? One day at a time. Much love 💕 || Condolences for your loss. God bless you || Deepest Condolences on Your loss, Joy🤍🌹Sending You much Love, Peace, Healing, Grace, and Nurturance during this time🙏🏽💓🌈 || Thanks so much for your kind words I really appreciate it 🙏😊 || @JoyFaheyArtist 🤗Thank You for All the Beauty You Share in the World💝💞💝 || Good to see you  back online || Welcome back Joy. You have been truly missed. I think the circle is a marvellous idea and offering so much value for money. I know personally how therapeutic art can be so this will be such a fantastic opportunity for so many others. See you in the circle ! || Many thanks, I'm so pleased you enjoyed the video! 😃🎨🖌️ || So sorry for your loss Joy, I have lost a husband and grandson and almost lost my son also, but praise God, he is still here with us.  Praying for you. || so so sorry about the loss of your son. || Hugs to you. ❤ || It really is a lovely space and jam packed with well thought out rich lessons. || That's great to hear 😊 Thanks so much 🙏 || I feel so privileged to be in the circle. A truely wonderful space.❤ || Thanks so much 🙏 I'm so pleased you're enjoying the Circle 😊 || ​@JoyFaheyArtist I've been booking for something like the circle for the longest time. Finally, I feel that I have found my tribe. Im really enjoying the content. A huge thankyou ❤</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B5wDtzaY4MI</t>
+          <t>IF7Ur-b8VHY</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Stop Flipping: Split-Hand HOCKEY DRILL to FIX Casting and GAIN Compression, Rotation and Shaft Lean!</t>
+          <t>OLD Paintings TURN into STUNNING Abstract Flowers!</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>If you’re tired of flipping at impact with negative shaft lean—hands behind the ball, club head passing early, and zero compression—this is the drill I go to. It’s a hockey-style split-hand grip that forces the correct sequencing: rotation delivers the strike, not a last-second hand throw. The goal is simple and non-negotiable: ball first contact, then turf, with real shaft lean and a stable club face.
-Here’s the key: split your hands on the grip, rehearse without a ball first, then hit small shots. If your body tries to “save it” by casting, you’ll feel it immediately. When you do it right, your hands work left through rotation while the club head stays out in front of your chest longer—exactly what clean ball strikers do.
-Want the full breakdown on why you cast (and how to fix your impact fast)? Watch more on my YouTube channel and grab my free drills guide here: EJSGolf.com/my-drills
-If you want me to diagnose your swing and give you the fastest fix for your impact, send me your swing video for a FREE analysis.
-Coach Erik Schjolberg
-The Science of Better Golf
-EJSGolf.com
-Scottsdale Golf Lessons
-Online Golf Lessons  
-#SGL #golfswing #EJSGolfAcademy #CoachErik #golftechnique #ejsgolf #golf #golfgear #shallow #Rotation #shaftlean</t>
+          <t>⭐Get my Free Abstract Painting Mini Course - https://www.joyfaheyclasses.com/opt-in
+💥Prints of paintings - https://www.joyfaheyartist.com/store-1-2
+_______________________________________________________________________
+About this video -
+🎨 Unlock the hidden beauty in old paintings! In this mesmerizing video, we'll show you how to transform vintage artwork into stunning abstract flowers that will leave you breathless. From faded landscapes to vibrant masterpieces, get ready to be amazed by the power of creativity and imagination. Watch as old paintings come alive with new life and color, and discover the magic that happens when art meets transformation.
+🌟 What You’ll Learn:
+✔️ How to your old paintings into new modern abstract flower paintings
+✔️ Creative ways to combine abstracts and flowers
+✔️ Simple techniques to add rhythm, movement, and contrast
+✔️ Working in a series
+If you love abstract art, mixed media, or expressive painting, this video is for you! Grab your markers, pens and crayons and let’s transform your artwork with vibrant, impactful details.
+🔥 Don’t forget to like, comment, and subscribe for more creative inspiration! #PoscaPens #AbstractArt #PaintingTips #MixedMedia #ArtDetails
+Perfect for beginners and intermediate artists looking to enhance their abstract painting skills. Whether you're working with acrylics, or mixed media, these principles will transform your creative process.
+__________________________
+💝 Dive deep into intuitive painting and discover the power of how to connect your art with your heart and soul  "THE ULTIMATE ART CONNECTION"  4 Week Immersive Online Course,  at - https://joyfahey.com/4-week-abstract-art-course/ and you can *TRY IT Before You BUY !"
+💝*FREE MONTH TRIAL of The ARTIST CONNECTION GROUP - https://www.joyfaheyclasses.com/
+💝 Get a Solid Foundation  from start to finish in your abstracts paintings with "The Complete Abstract Painting Course" for just $27 Click - https://joyfahey.com/the-complete-abstract-art-painting-course/ 
+💝*FREE PDF's and more at - https://www.joyfahey.com
+___________________________
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Guadi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#AbstractAcrylicPainting. #AbstractFlowers. #AcrylicAbstractArtTutorials. #IntuitiveAbstractart.
+About - Abstract Painting in Acrylics tutorial and demonstration</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-01-26T00:05:44Z</t>
+          <t>2025-04-13T18:23:54Z</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>956</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>165</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.018828</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
+        <v>0.09170499999999999</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Hi Joy. I miss your videos. I hope you are well and can come back soon. ✌️ || Many thanks, it's been awhile but I've just posted a new video. https://youtu.be/s9DBjNkmQFg?si=EXon0jp5BW6q4djC 🙏😊 || ​@JoyFaheyArtistOh goody!  Thanks for letting me know.  ❤ || Dear Joy, I’m thinking about you and sending you prayers for healing. I will be thrilled when you are able to return. Blessings, Bonnie in California || Thanks so much 🙏😊 || Hi Joy  I’m a beginner in acrylic however I do like your colour palette can recommend which acrylics to purchase to achieve a similar colour palette.  Thank you . || Hi I mainly use Amsterdam paint however there are many different makes you can try. Golden are wonderful top! Happy painting 🎨🖌️😊 || Very nice Joy. || Thank you! 😊 || You are always so inspiring Miss Joy. Love the spring colors. I am going to give this a try 😊 || Have fun!🎨🖌️😄 || Fun free and easy thanks || Glad you like it! 😊🎨🖌️</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>C7EvmfEoZNU</t>
+          <t>9LEy5BgBoD0</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>How to Gain Speed, Distance, Shaft Lean and More in your Golf Swing with these 2 Drills</t>
+          <t>AWESOME Transformation Of An Old Abstract Painting Into A Modern New One!</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Most golfers don’t need a swing rebuild to hit it farther and compress the ball. They need better impact conditions—more forward shaft lean, better low point control, and a body that actually supports speed instead of stalling so the hands can “catch up.” In this video I show two simple drills you can do with what you already own: a golf club and an alignment stick (or training club).
-Drill #1 fixes the most common speed killer I see: the “pull-down gap” where the arms separate, the club gets yanked down, and the body has to stall to survive impact. I use an under-the-armpit connection constraint so you stop ripping from the top and learn how to rotate through with structure. If you can keep your lead arm connected longer, your sequencing improves and your impact starts looking like a ball striker—hands forward, club head delivered with intention, and compression you can actually feel.
-Drill #2 is my favorite speed producer before a round: swing as fast as you can and STOP in a controlled “impact checkpoint.” If you can’t stop it, your body isn’t supporting your speed—period. When you learn to stop it, your body organizes itself automatically: you clear space, you get the hands forward, and you find the kind of impact position golfers chase for years by thinking about ten different swing thoughts. I’m not interested in thoughts. I’m interested in measurable outcomes.
-Coach Erik Schjolberg
-The Science of Better Golf
-EJSGolf.com
-Scottsdale Golf Lessons
-Online Golf Lessons  
-#GolfDrills #ShaftLean #GolfSpeed #Compression #BallStriking #IncreaseDistance #ImpactPosition</t>
+          <t>⭐Get my Free Abstract Painting Mini Course - https://www.joyfaheyclasses.com/opt-in
+💥 SCROLL DOWN FOR MORE GREAT Art Courses and FREEBIES👇🏽👇🏽👇🏽👇🏽
+_______________________________________________________________________
+About this video -
+🎨 Transforming an old painting into a new modern one is a great way to use your play abstract play paintings🖊️✨
+In this video, I take an old play painting that’s been sitting around and give it a fresh new life! You'll see my full process—how I approach reworking a piece, what I keep, what I let go of, and how I find new energy in something familiar. It's all about transformation, intuition, and having fun with the layers. Hope it inspires you to revisit some of your own old work!
+🌟 What You’ll Learn:
+✔️ How to let go of old paintings
+✔️ Creative ways to think out of the box
+✔️ Simple techniques to add rhythm, movement, and contrast
+✔️ Have fun and enjoy a new lease of creativity!
+If you love abstract art, or expressive painting, this video is for you! Grab your markers, and paints and let’s transform your artwork with vibrant, impactful details.
+🔥 Don’t forget to like, comment, and subscribe for more creative inspiration! #PoscaPens #AbstractArt #PaintingTips #MixedMedia #ArtDetails
+Perfect for beginners and intermediate artists looking to enhance their abstract painting skills. Whether you're working with acrylics, or mixed media, these principles will transform your creative process.
+__________________________
+💝 Dive deep into intuitive painting and discover the power of how to connect your art with your heart and soul  "THE ULTIMATE ART CONNECTION"  4 Week Immersive Online Course,  at - https://joyfahey.com/4-week-abstract-art-course/ and you can *TRY IT Before You BUY !"
+💝*FREE MONTH TRIAL of The ARTIST CONNECTION GROUP - https://www.joyfaheyclasses.com/
+💝 Get a Solid Foundation  from start to finish in your abstracts paintings with "The Complete Abstract Painting Course" for just $27 Click - https://joyfahey.com/the-complete-abstract-art-painting-course/ 
+💝*FREE PDF's and more at - https://www.joyfahey.com
+___________________________
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Guadi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#AbstractAcrylicPainting. #AcrylicAbstractArtTutorials. #IntuitiveAbstractart.
+About - Abstract Painting in Acrylics tutorial and demonstration</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-01-25T07:09:14Z</t>
+          <t>2025-04-06T17:25:16Z</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>3284</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>213</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.054545</v>
+        <v>0.069123</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>1 MORE is LESS Skill applications being accepted || Thanks for the comment!</t>
+          <t>So glad I found you Joy. You create amazing art. I love your relaxed natural processes. || Thanks so much for your great feedback I'm so happy you're enjoying the videos 😊🎨🖌️ || hi joy, What paper are you using? || Watercolor paper 📜🙏😊 || Awesome tutorial, thanks. Sending you love and hugs || Really enjoyed your tutorial thank you so much for sharing and having us experiment with old paintings
+Fun to see how they come alive in their transformation || Thanks so much 😊 I'm very pleased you enjoyed the video 😊🖌️🎨 || Some great tips.  Thank you || Glad it was helpful! 😊🎨🖌️ || Having watched your videos a few times I am intrigued wondering why you pronounce yellow ochre as Yellow "Okra" which is a vegetable! Ochre is pronounced 'Oker' with emphasis on the O. May be helpful for viewers too. || She speaks it as it’s spelled - we can figure it out. Location, country, culture means we need to give grace here including pronunciation   I don’t expect anyone in the US or beyond to speak as I do. || Interesting! Thanks for the observation 😄🖌️🎨 || That really was a great tutorial!!! It’s beautiful! Thank you || Thank you so much! I'm so pleased you enjoyed it 😄🖌️🎨</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>QigOaULFjv8</t>
+          <t>PjRZaKH09Ew</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nail the Jump Move for Perfect Golf Rotation! #shorts</t>
+          <t>FINISHING My Abstract Shape Painting With GREAT Results!</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>🏌🏿♂️Nail the Jump Move for Perfect Golf Rotation!
-🏃♂️ Ready to elevate your golf game? The jump move is your key to crushing rotation, shaft lean, power, speed, compresion andd reducing early extension! ⛳ Feel the difference with my jump drill! 🙌 Let's go!
-Coach Erik Schjolberg
-EJS Golf
-The Science of Better Golf
-Scottsdale Golf Lesson
-Online Golf Lessons
- #Golf #SwingTips #JumpMove #Golfers #Training</t>
+          <t>⭐Here's Your Complete Abstract Painting Course - https://joyfahey.com/the-complete-abstract-art-painting-course/
+_______________________________________________________________________
+🎨 Elevate Your Art! Finishing Touches with Posca Pens, Coloured crayons and Collage 🖊️✨
+Your painting is almost there—but now it’s time to make it pop! In this video, I’ll show you how to use pens and collage to add bold details, crisp lines, and eye-catching contrast to your artwork. Whether you’re refining shapes, adding texture, or enhancing focal points, these techniques will bring depth, energy, and personality to your painting.
+🌟 What You’ll Learn:
+✔️ How to assess your painting for the perfect finishing touches
+✔️ Creative ways to use pens for mark-making, outlining, and layering with collage
+✔️ Simple techniques to add rhythm, movement, and contrast
+✔️ When to stop—so you don’t overwork your piece!
+If you love abstract art, mixed media, or expressive painting, this video is for you! Grab your markers, pens and crayons and let’s transform your artwork with vibrant, impactful details.
+🔥 Don’t forget to like, comment, and subscribe for more creative inspiration! #PoscaPens #AbstractArt #PaintingTips #MixedMedia #ArtDetails
+Learn how to 
+🎨 What you'll learn:
+*How to create a composition using large shapes
+*Techniques for adding layers of visual interest
+*Professional tips for creating depth and movement
+*Ways to know when your painting is complete
+Perfect for beginners and intermediate artists looking to enhance their abstract painting skills. Whether you're working with acrylics, or mixed media, these principles will transform your creative process.
+__________________________
+💝 Dive deep into intuitive painting and discover the power of how to connect your art with your heart and soul  "THE ULTIMATE ART CONNECTION"  4 Week Immersive Online Course,  at - https://joyfahey.com/4-week-abstract-art-course/ and you can *TRY IT Before You BUY !"
+💝*FREE MONTH TRIAL of The ARTIST CONNECTION GROUP - https://www.joyfaheyclasses.com/
+💝*FREE PDF's and more at - https://www.joyfahey.com
+___________________________
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Guadi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#AbstractAcrylicPainting. #AcrylicAbstractArtTutorials. #IntuitiveAbstractart.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-01-11T18:03:28Z</t>
+          <t>2025-03-30T15:30:08Z</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1083</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>211</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.003693</v>
+        <v>0.108182</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Get my FREE DRILLS guide at EJSGolf.com/my-drills</t>
+          <t>❤ Who will be my 10,000th  subscriber!? 🎉😂 || I love the way the 4 pieces came together! || I'm so glad you loved how they came together! 😊🎨 || Very Nice to see || Thank you, I'm so pleased you enjoyed the video! 😃🎨🖌️ || Loved it! || Thanks 🙏🎨🖌️ || Very nice, I LOVE your work😍😍😍 || This was a wonderful video.  Like your process and the final pieces.  Thank you. || Thank you so much! I'm so happy you enjoyed it 😄🖌️🎨 || Really great Joy and would love to see more of this type of video. Making abstracts accessible as they are not easy!! The small paintings in frames at the end look gorgeous together and I think they are very sellable small, yet affordable, pieces of original art. || Thanks Rachel I'm so pleased you enjoyed the video 😄 Yes it's a great way to gain your confidence with abstracts and slowly but surely increase the size! Happy Painting! 🖌️🎨 😄 || I really love your videos, you are so enjoyable to listen to and so encouraging!  I am always inspired by your work!💕🇨🇦 || Thanks so much Cindy 🙏 I'm so happy you're enjoying the videos 😊 || Doodling flowers w water pencils || I just painted a mat, to a big vintage piece I bought for my livingroom. It was white and I wanted it to be framed with black. || Awesome! 🎨🖌️😊 || Wow! Those are amazing. Thank you for the idea. || You are so welcome! 😊 || I love the one with the yellow triangle in the center of the painting. The one next to your hand with the ring. || Thanks for sharing. It's so interesting how these little paintings turn out isn't it? 🖌️🎨😊 || These are lovely. I really want to try this project. Thank you for sharing. || Thanks Barbara I'm really happy you enjoyed the video 😊🎨🖌️ || Bonsoir Joy, Quel superbe résultat, de ravissants mini abstraits 👍👌. Mon dada, c’est la peinture semi-abstraite à l’huile sur toile de lin 80*80 cm a minima mais, pour me détendre, m’amuser &amp; expérimenter, j’applique VOTRE process avec l’acrylique: c’est génial pour de belles découvertes! Et oui, les Posca sont les meilleurs feutres sur le marché. Merci 🙏🫶 à vous pour ce partage. Belle &amp; douce soirée. Abstraitement vôtre, Nathalie || Merci beaucoup 😊 I'm so pleased you enjoyed the video 🖌️🎨😊 || Love this idea! They really are cute and affordable to make. Thank you for sharing. Will give this a try!😊 || You are so welcome! Yes it's a great way to use your play paintings 😊🖌️🎨</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UCIdaiMpZGQ-SPvjBXhmpw8A</t>
+          <t>UCaCGKJVPW-z7gNXLJUThsNg</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Coach Erik Schjolberg - The Science of Better Golf</t>
+          <t>Joy Fahey Artist</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PJNm8Wq2wJY</t>
+          <t>cfSouigKbmg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>🏌🏿‍♂️Nail the Jump Move for Perfect Golf Rotation!</t>
+          <t>Beginners Guide To Creating Beautiful Abstract Paintings Easily</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>🏌🏿‍♂️Nail the Jump Move for Perfect Golf Rotation!
-🏃‍♂️ Ready to elevate your golf game? The jump move is your key to crushing rotation, shaft lean, power, speed, compresion andd reducing early extension! ⛳ Feel the difference with my jump drill! 🙌 Let's go!
-Coach Erik Schjolberg
-EJS Golf
-The Science of Better Golf
-Scottsdale Golf Lesson
-Online Golf Lessons
- #Golf #SwingTips #JumpMove #Golfers #Training</t>
+          <t>⭐Here's Your Complete Abstract Painting Course - https://joyfahey.com/the-complete-abstract-art-painting-course/
+💥 SCROLL DOWN FOR Extra Inspiration👇🏽👇🏽👇🏽👇🏽
+_______________________________________________________________________
+ABOUT THIS VIDEO - A great opportunity to really learn the basics of Abstract Painting from start to finish. If You're ready to dive into the world of abstract painting 🎨 I’ll show you how to create bold, expressive abstracts with confidence—no perfection required! Whether you're a beginner or looking to refine your skills, this is your chance to break free and let your creativity flow.
+🎨 Perfect for beginners and intermediate artists looking to enhance their abstract painting skills. Whether you're working with acrylics, or mixed media, these principles will transform your creative process.
+__________________________
+💥Learn more about INTUITIVE Painting in my Art Connection Course at https://www.joyfaheyartist.com💥 
+💝*FREE MONTH TRIAL of The ARTIST CONNECTION GROUP - https://www.joyfaheyclasses.com/
+💝*FREE PDF's and more at - https://www.joyfahey.com
+💝*FREE TRIAL of "THE ULTIMATE ART CONNECTION"  4 Week Immersive Online Course  at - https://joyfahey.com/4-week-abstract-art-course/
+___________________________
+⭐Check Out My 14 ONLINE PAINTING COURSES at
+https://joyfahey.com
+🖼️Check out My Paintings &amp; Art Prints for Sale
+https://joyfaheyartist.com
+⭐CONNECT WITH ME ON
+Instagram - https://www.instagram.com/joyfahey_arist
+Facebook - https://www.facebook.com/joyfaheyart  
+Pinterest - https://www.pinterest.com/joyfaheyart 
+Skillshare - https://skl.sh/3OT24XJ i  
+_______________________________________________________________________
+⭐ABOUT JOY Fahey
+I’m an English artist based in Malaga, Spain with over 30 years of painting experience. I’m passionate about teaching both beginners and seasoned painters looking to express themselves creatively and get maximum satisfaction from the abstract art practice offering Online courses, and Masterclasses and the Artist Diary in my Artists Connection Group.  My artwork has been featured in galleries across the Europe, i Some of my proudest moments were having my work showcased in the CAC Museum Malaga, and the Guadi Gallery Madrid. and selling a painting to an Arabian Princess! 
+💝Subscribe and LIKE for lots more inspirational Abstract Painting Tutorials
+Thanks for watching 💝
+#AbstractAcrylicPainting. #AcrylicAbstractArtTutorials. #IntuitiveAbstractart.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-01-11T17:57:28Z</t>
+          <t>2025-03-25T16:00:46Z</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>718</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1326,7 +1646,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.008357</v>
+        <v>0.01666</v>
       </c>
       <c r="M13" t="inlineStr"/>
     </row>

</xml_diff>